<commit_message>
Perbarui data SE2026 24/08/2026  7:48:08,26
</commit_message>
<xml_diff>
--- a/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
+++ b/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
@@ -16,7 +16,7 @@
     <t>DATA RADAR ANOMALI USAHA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 23 Agu 2026, 20.23</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 24 Agu 2026, 07.47</t>
   </si>
   <si>
     <t>Kode</t>
@@ -334,646 +334,646 @@
     <t>0,08</t>
   </si>
   <si>
-    <t>19,4</t>
-  </si>
-  <si>
-    <t>1,79</t>
-  </si>
-  <si>
-    <t>4,84</t>
-  </si>
-  <si>
-    <t>32,1</t>
-  </si>
-  <si>
-    <t>10,31</t>
+    <t>19,53</t>
+  </si>
+  <si>
+    <t>1,75</t>
+  </si>
+  <si>
+    <t>4,69</t>
+  </si>
+  <si>
+    <t>32,41</t>
+  </si>
+  <si>
+    <t>10,34</t>
+  </si>
+  <si>
+    <t>0,48</t>
+  </si>
+  <si>
+    <t>7,11</t>
+  </si>
+  <si>
+    <t>0,09</t>
+  </si>
+  <si>
+    <t>0,04</t>
+  </si>
+  <si>
+    <t>0,13</t>
+  </si>
+  <si>
+    <t>0,02</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>0,27</t>
+  </si>
+  <si>
+    <t>0,62</t>
+  </si>
+  <si>
+    <t>0,11</t>
+  </si>
+  <si>
+    <t>2,48</t>
+  </si>
+  <si>
+    <t>5,47</t>
+  </si>
+  <si>
+    <t>14,03</t>
+  </si>
+  <si>
+    <t>1801</t>
+  </si>
+  <si>
+    <t>LAMPUNG BARAT</t>
+  </si>
+  <si>
+    <t>0,18</t>
+  </si>
+  <si>
+    <t>22,15</t>
+  </si>
+  <si>
+    <t>1,43</t>
+  </si>
+  <si>
+    <t>4,97</t>
+  </si>
+  <si>
+    <t>38,13</t>
+  </si>
+  <si>
+    <t>2,51</t>
+  </si>
+  <si>
+    <t>0,61</t>
+  </si>
+  <si>
+    <t>4,06</t>
+  </si>
+  <si>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>0,14</t>
+  </si>
+  <si>
+    <t>0,24</t>
+  </si>
+  <si>
+    <t>0,34</t>
+  </si>
+  <si>
+    <t>0,06</t>
+  </si>
+  <si>
+    <t>11,17</t>
+  </si>
+  <si>
+    <t>3,62</t>
+  </si>
+  <si>
+    <t>9,96</t>
+  </si>
+  <si>
+    <t>1802</t>
+  </si>
+  <si>
+    <t>TANGGAMUS</t>
+  </si>
+  <si>
+    <t>12,63</t>
+  </si>
+  <si>
+    <t>0,46</t>
+  </si>
+  <si>
+    <t>21,35</t>
+  </si>
+  <si>
+    <t>29,97</t>
+  </si>
+  <si>
+    <t>5,29</t>
+  </si>
+  <si>
+    <t>0,07</t>
   </si>
   <si>
     <t>0,5</t>
   </si>
   <si>
-    <t>7,14</t>
-  </si>
-  <si>
-    <t>0,04</t>
-  </si>
-  <si>
-    <t>0,13</t>
-  </si>
-  <si>
-    <t>0,02</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>0,28</t>
-  </si>
-  <si>
-    <t>0,14</t>
-  </si>
-  <si>
-    <t>0,63</t>
-  </si>
-  <si>
-    <t>0,11</t>
-  </si>
-  <si>
-    <t>2,53</t>
-  </si>
-  <si>
-    <t>5,49</t>
+    <t>0,29</t>
+  </si>
+  <si>
+    <t>5,44</t>
+  </si>
+  <si>
+    <t>18,24</t>
+  </si>
+  <si>
+    <t>1803</t>
+  </si>
+  <si>
+    <t>LAMPUNG SELATAN</t>
+  </si>
+  <si>
+    <t>17,17</t>
+  </si>
+  <si>
+    <t>2,69</t>
+  </si>
+  <si>
+    <t>40,47</t>
+  </si>
+  <si>
+    <t>14,72</t>
+  </si>
+  <si>
+    <t>9,36</t>
+  </si>
+  <si>
+    <t>0,33</t>
+  </si>
+  <si>
+    <t>0,01</t>
+  </si>
+  <si>
+    <t>0,77</t>
+  </si>
+  <si>
+    <t>1,12</t>
+  </si>
+  <si>
+    <t>0,03</t>
+  </si>
+  <si>
+    <t>4,33</t>
+  </si>
+  <si>
+    <t>8,58</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>0,32</t>
+  </si>
+  <si>
+    <t>18,94</t>
+  </si>
+  <si>
+    <t>0,38</t>
+  </si>
+  <si>
+    <t>16,21</t>
+  </si>
+  <si>
+    <t>26,56</t>
+  </si>
+  <si>
+    <t>9,73</t>
+  </si>
+  <si>
+    <t>1,21</t>
+  </si>
+  <si>
+    <t>5,9</t>
+  </si>
+  <si>
+    <t>0,05</t>
+  </si>
+  <si>
+    <t>0,45</t>
+  </si>
+  <si>
+    <t>0,15</t>
+  </si>
+  <si>
+    <t>2,64</t>
+  </si>
+  <si>
+    <t>14,43</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>15,42</t>
+  </si>
+  <si>
+    <t>2,5</t>
+  </si>
+  <si>
+    <t>1,22</t>
+  </si>
+  <si>
+    <t>44,8</t>
+  </si>
+  <si>
+    <t>5,08</t>
+  </si>
+  <si>
+    <t>0,92</t>
+  </si>
+  <si>
+    <t>12,92</t>
+  </si>
+  <si>
+    <t>0,68</t>
+  </si>
+  <si>
+    <t>0,72</t>
+  </si>
+  <si>
+    <t>3,22</t>
+  </si>
+  <si>
+    <t>11,48</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>18,69</t>
+  </si>
+  <si>
+    <t>0,79</t>
+  </si>
+  <si>
+    <t>1,5</t>
+  </si>
+  <si>
+    <t>36,71</t>
   </si>
   <si>
     <t>14,21</t>
   </si>
   <si>
-    <t>1801</t>
-  </si>
-  <si>
-    <t>LAMPUNG BARAT</t>
+    <t>7,85</t>
+  </si>
+  <si>
+    <t>0,59</t>
+  </si>
+  <si>
+    <t>1,11</t>
+  </si>
+  <si>
+    <t>6,83</t>
+  </si>
+  <si>
+    <t>10,48</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>18,09</t>
+  </si>
+  <si>
+    <t>0,65</t>
+  </si>
+  <si>
+    <t>5,89</t>
+  </si>
+  <si>
+    <t>38,09</t>
+  </si>
+  <si>
+    <t>16,17</t>
+  </si>
+  <si>
+    <t>0,3</t>
+  </si>
+  <si>
+    <t>0,25</t>
+  </si>
+  <si>
+    <t>0,81</t>
+  </si>
+  <si>
+    <t>0,53</t>
+  </si>
+  <si>
+    <t>4,74</t>
+  </si>
+  <si>
+    <t>7,51</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>24,01</t>
+  </si>
+  <si>
+    <t>0,42</t>
+  </si>
+  <si>
+    <t>2,61</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>15,16</t>
+  </si>
+  <si>
+    <t>0,16</t>
+  </si>
+  <si>
+    <t>5,65</t>
+  </si>
+  <si>
+    <t>0,19</t>
+  </si>
+  <si>
+    <t>0,26</t>
+  </si>
+  <si>
+    <t>0,66</t>
+  </si>
+  <si>
+    <t>2,42</t>
+  </si>
+  <si>
+    <t>7,58</t>
+  </si>
+  <si>
+    <t>13,51</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>28,19</t>
+  </si>
+  <si>
+    <t>0,8</t>
+  </si>
+  <si>
+    <t>0,83</t>
+  </si>
+  <si>
+    <t>27,39</t>
+  </si>
+  <si>
+    <t>3,48</t>
+  </si>
+  <si>
+    <t>6,18</t>
+  </si>
+  <si>
+    <t>2,47</t>
+  </si>
+  <si>
+    <t>9,47</t>
+  </si>
+  <si>
+    <t>19,45</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>17,47</t>
+  </si>
+  <si>
+    <t>0,51</t>
+  </si>
+  <si>
+    <t>2,67</t>
+  </si>
+  <si>
+    <t>28,18</t>
+  </si>
+  <si>
+    <t>3,13</t>
+  </si>
+  <si>
+    <t>4,49</t>
+  </si>
+  <si>
+    <t>0,44</t>
+  </si>
+  <si>
+    <t>5,76</t>
+  </si>
+  <si>
+    <t>7,82</t>
+  </si>
+  <si>
+    <t>27,53</t>
+  </si>
+  <si>
+    <t>1811</t>
+  </si>
+  <si>
+    <t>MESUJI</t>
+  </si>
+  <si>
+    <t>29,98</t>
+  </si>
+  <si>
+    <t>7,39</t>
+  </si>
+  <si>
+    <t>3,31</t>
+  </si>
+  <si>
+    <t>26,18</t>
+  </si>
+  <si>
+    <t>7,24</t>
+  </si>
+  <si>
+    <t>0,36</t>
+  </si>
+  <si>
+    <t>3,41</t>
+  </si>
+  <si>
+    <t>0,2</t>
+  </si>
+  <si>
+    <t>4,77</t>
+  </si>
+  <si>
+    <t>9,41</t>
+  </si>
+  <si>
+    <t>6,3</t>
+  </si>
+  <si>
+    <t>1812</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG BARAT</t>
+  </si>
+  <si>
+    <t>16,98</t>
+  </si>
+  <si>
+    <t>2,33</t>
+  </si>
+  <si>
+    <t>10,76</t>
+  </si>
+  <si>
+    <t>23,23</t>
+  </si>
+  <si>
+    <t>14,08</t>
+  </si>
+  <si>
+    <t>5,25</t>
+  </si>
+  <si>
+    <t>3,67</t>
+  </si>
+  <si>
+    <t>3,38</t>
+  </si>
+  <si>
+    <t>18,5</t>
+  </si>
+  <si>
+    <t>1813</t>
+  </si>
+  <si>
+    <t>PESISIR BARAT</t>
+  </si>
+  <si>
+    <t>13,28</t>
   </si>
   <si>
     <t>0,17</t>
   </si>
   <si>
-    <t>22,71</t>
-  </si>
-  <si>
-    <t>1,6</t>
-  </si>
-  <si>
-    <t>5,27</t>
-  </si>
-  <si>
-    <t>36,34</t>
-  </si>
-  <si>
-    <t>2,58</t>
-  </si>
-  <si>
-    <t>0,65</t>
-  </si>
-  <si>
-    <t>3,75</t>
-  </si>
-  <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>0,15</t>
-  </si>
-  <si>
-    <t>0,27</t>
-  </si>
-  <si>
-    <t>0,35</t>
-  </si>
-  <si>
-    <t>0,06</t>
-  </si>
-  <si>
-    <t>11,8</t>
-  </si>
-  <si>
-    <t>3,45</t>
-  </si>
-  <si>
-    <t>10,43</t>
-  </si>
-  <si>
-    <t>1802</t>
-  </si>
-  <si>
-    <t>TANGGAMUS</t>
-  </si>
-  <si>
-    <t>12,62</t>
-  </si>
-  <si>
-    <t>0,46</t>
-  </si>
-  <si>
-    <t>5,51</t>
-  </si>
-  <si>
-    <t>21,34</t>
-  </si>
-  <si>
-    <t>29,96</t>
-  </si>
-  <si>
-    <t>5,29</t>
-  </si>
-  <si>
-    <t>0,07</t>
-  </si>
-  <si>
-    <t>0,18</t>
-  </si>
-  <si>
-    <t>0,29</t>
-  </si>
-  <si>
-    <t>5,47</t>
-  </si>
-  <si>
-    <t>18,2</t>
-  </si>
-  <si>
-    <t>1803</t>
-  </si>
-  <si>
-    <t>LAMPUNG SELATAN</t>
-  </si>
-  <si>
-    <t>17,2</t>
-  </si>
-  <si>
-    <t>2,7</t>
-  </si>
-  <si>
-    <t>40,37</t>
-  </si>
-  <si>
-    <t>14,72</t>
-  </si>
-  <si>
-    <t>0,01</t>
-  </si>
-  <si>
-    <t>9,33</t>
+    <t>36,25</t>
+  </si>
+  <si>
+    <t>20,56</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>0,22</t>
+  </si>
+  <si>
+    <t>0,69</t>
+  </si>
+  <si>
+    <t>7,57</t>
+  </si>
+  <si>
+    <t>10,97</t>
+  </si>
+  <si>
+    <t>1871</t>
+  </si>
+  <si>
+    <t>BANDAR LAMPUNG</t>
+  </si>
+  <si>
+    <t>15,73</t>
+  </si>
+  <si>
+    <t>0,6</t>
+  </si>
+  <si>
+    <t>3,71</t>
+  </si>
+  <si>
+    <t>30,26</t>
+  </si>
+  <si>
+    <t>4,81</t>
+  </si>
+  <si>
+    <t>16,33</t>
+  </si>
+  <si>
+    <t>0,9</t>
+  </si>
+  <si>
+    <t>1,8</t>
+  </si>
+  <si>
+    <t>0,4</t>
+  </si>
+  <si>
+    <t>4,61</t>
+  </si>
+  <si>
+    <t>18,34</t>
+  </si>
+  <si>
+    <t>1872</t>
+  </si>
+  <si>
+    <t>METRO</t>
+  </si>
+  <si>
+    <t>16,5</t>
+  </si>
+  <si>
+    <t>6,78</t>
+  </si>
+  <si>
+    <t>0,7</t>
+  </si>
+  <si>
+    <t>27,09</t>
+  </si>
+  <si>
+    <t>4,46</t>
   </si>
   <si>
     <t>0,31</t>
   </si>
   <si>
-    <t>0,77</t>
-  </si>
-  <si>
-    <t>1,12</t>
-  </si>
-  <si>
-    <t>0,03</t>
-  </si>
-  <si>
-    <t>4,31</t>
-  </si>
-  <si>
-    <t>8,58</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>0,34</t>
-  </si>
-  <si>
-    <t>17,64</t>
-  </si>
-  <si>
-    <t>0,37</t>
-  </si>
-  <si>
-    <t>17,71</t>
-  </si>
-  <si>
-    <t>25,76</t>
-  </si>
-  <si>
-    <t>9,05</t>
-  </si>
-  <si>
-    <t>1,35</t>
-  </si>
-  <si>
-    <t>5,98</t>
-  </si>
-  <si>
-    <t>0,47</t>
-  </si>
-  <si>
-    <t>2,74</t>
-  </si>
-  <si>
-    <t>2,57</t>
-  </si>
-  <si>
-    <t>15,32</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>15,35</t>
-  </si>
-  <si>
-    <t>1,17</t>
-  </si>
-  <si>
-    <t>44,81</t>
-  </si>
-  <si>
-    <t>5,09</t>
-  </si>
-  <si>
-    <t>0,92</t>
-  </si>
-  <si>
-    <t>12,93</t>
-  </si>
-  <si>
-    <t>0,24</t>
-  </si>
-  <si>
-    <t>0,68</t>
-  </si>
-  <si>
-    <t>0,73</t>
-  </si>
-  <si>
-    <t>3,23</t>
-  </si>
-  <si>
-    <t>11,49</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>18,7</t>
-  </si>
-  <si>
-    <t>0,79</t>
-  </si>
-  <si>
-    <t>1,58</t>
-  </si>
-  <si>
-    <t>36,53</t>
-  </si>
-  <si>
-    <t>14,28</t>
-  </si>
-  <si>
-    <t>7,85</t>
-  </si>
-  <si>
-    <t>0,59</t>
-  </si>
-  <si>
-    <t>6,84</t>
-  </si>
-  <si>
-    <t>10,49</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>0,05</t>
-  </si>
-  <si>
-    <t>18,1</t>
-  </si>
-  <si>
-    <t>5,87</t>
-  </si>
-  <si>
-    <t>38,11</t>
-  </si>
-  <si>
-    <t>16,18</t>
-  </si>
-  <si>
-    <t>0,3</t>
-  </si>
-  <si>
-    <t>5,48</t>
-  </si>
-  <si>
-    <t>0,25</t>
-  </si>
-  <si>
-    <t>0,81</t>
-  </si>
-  <si>
-    <t>0,53</t>
-  </si>
-  <si>
-    <t>0,44</t>
-  </si>
-  <si>
-    <t>4,74</t>
-  </si>
-  <si>
-    <t>7,51</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>0,42</t>
-  </si>
-  <si>
-    <t>2,64</t>
-  </si>
-  <si>
-    <t>26,9</t>
-  </si>
-  <si>
-    <t>15,19</t>
-  </si>
-  <si>
-    <t>0,19</t>
-  </si>
-  <si>
-    <t>5,64</t>
-  </si>
-  <si>
-    <t>0,26</t>
-  </si>
-  <si>
-    <t>0,66</t>
-  </si>
-  <si>
-    <t>2,5</t>
-  </si>
-  <si>
-    <t>7,55</t>
-  </si>
-  <si>
-    <t>13,51</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>28,26</t>
-  </si>
-  <si>
-    <t>0,8</t>
-  </si>
-  <si>
-    <t>0,85</t>
-  </si>
-  <si>
-    <t>27,23</t>
-  </si>
-  <si>
-    <t>3,49</t>
-  </si>
-  <si>
-    <t>6,2</t>
-  </si>
-  <si>
-    <t>0,39</t>
-  </si>
-  <si>
-    <t>0,16</t>
-  </si>
-  <si>
-    <t>2,47</t>
-  </si>
-  <si>
-    <t>9,5</t>
-  </si>
-  <si>
-    <t>19,49</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>17,46</t>
-  </si>
-  <si>
-    <t>0,51</t>
-  </si>
-  <si>
-    <t>28,18</t>
-  </si>
-  <si>
-    <t>3,13</t>
-  </si>
-  <si>
-    <t>4,49</t>
-  </si>
-  <si>
-    <t>0,61</t>
-  </si>
-  <si>
-    <t>5,76</t>
-  </si>
-  <si>
-    <t>7,82</t>
-  </si>
-  <si>
-    <t>27,52</t>
-  </si>
-  <si>
-    <t>1811</t>
-  </si>
-  <si>
-    <t>MESUJI</t>
-  </si>
-  <si>
-    <t>30,07</t>
-  </si>
-  <si>
-    <t>7,41</t>
-  </si>
-  <si>
-    <t>3,42</t>
-  </si>
-  <si>
-    <t>26,02</t>
-  </si>
-  <si>
-    <t>7,17</t>
-  </si>
-  <si>
-    <t>0,2</t>
-  </si>
-  <si>
-    <t>9,38</t>
-  </si>
-  <si>
-    <t>6,27</t>
-  </si>
-  <si>
-    <t>1812</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG BARAT</t>
-  </si>
-  <si>
-    <t>16,94</t>
-  </si>
-  <si>
-    <t>2,38</t>
-  </si>
-  <si>
-    <t>10,76</t>
-  </si>
-  <si>
-    <t>23,19</t>
-  </si>
-  <si>
-    <t>14,12</t>
-  </si>
-  <si>
-    <t>0,83</t>
-  </si>
-  <si>
-    <t>5,25</t>
-  </si>
-  <si>
-    <t>0,09</t>
-  </si>
-  <si>
-    <t>3,67</t>
-  </si>
-  <si>
-    <t>3,38</t>
-  </si>
-  <si>
-    <t>18,5</t>
-  </si>
-  <si>
-    <t>1813</t>
-  </si>
-  <si>
-    <t>PESISIR BARAT</t>
-  </si>
-  <si>
-    <t>13,37</t>
-  </si>
-  <si>
-    <t>0,55</t>
-  </si>
-  <si>
-    <t>35,19</t>
-  </si>
-  <si>
-    <t>21,06</t>
-  </si>
-  <si>
-    <t>9,18</t>
-  </si>
-  <si>
-    <t>0,23</t>
-  </si>
-  <si>
-    <t>0,71</t>
-  </si>
-  <si>
-    <t>0,6</t>
-  </si>
-  <si>
-    <t>7,54</t>
-  </si>
-  <si>
-    <t>11,13</t>
-  </si>
-  <si>
-    <t>1871</t>
-  </si>
-  <si>
-    <t>BANDAR LAMPUNG</t>
-  </si>
-  <si>
-    <t>15,76</t>
-  </si>
-  <si>
-    <t>3,61</t>
-  </si>
-  <si>
-    <t>30,22</t>
-  </si>
-  <si>
-    <t>4,82</t>
-  </si>
-  <si>
-    <t>16,37</t>
-  </si>
-  <si>
-    <t>0,9</t>
-  </si>
-  <si>
-    <t>1,81</t>
-  </si>
-  <si>
-    <t>0,4</t>
-  </si>
-  <si>
-    <t>4,62</t>
-  </si>
-  <si>
-    <t>18,37</t>
-  </si>
-  <si>
-    <t>1872</t>
-  </si>
-  <si>
-    <t>METRO</t>
-  </si>
-  <si>
-    <t>16,48</t>
-  </si>
-  <si>
-    <t>0,7</t>
-  </si>
-  <si>
-    <t>26,99</t>
-  </si>
-  <si>
-    <t>4,47</t>
-  </si>
-  <si>
-    <t>2,94</t>
-  </si>
-  <si>
-    <t>0,22</t>
-  </si>
-  <si>
-    <t>0,48</t>
-  </si>
-  <si>
-    <t>2,19</t>
-  </si>
-  <si>
-    <t>3,51</t>
-  </si>
-  <si>
-    <t>33,79</t>
+    <t>2,93</t>
+  </si>
+  <si>
+    <t>2,14</t>
+  </si>
+  <si>
+    <t>3,68</t>
+  </si>
+  <si>
+    <t>33,61</t>
   </si>
   <si>
     <t/>
@@ -1953,7 +1953,7 @@
         <v>105</v>
       </c>
       <c r="C6" s="6">
-        <v>91291</v>
+        <v>92539</v>
       </c>
       <c r="D6" s="6">
         <v>74</v>
@@ -1962,79 +1962,79 @@
         <v>106</v>
       </c>
       <c r="F6" s="6">
-        <v>17711</v>
+        <v>18071</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>107</v>
       </c>
       <c r="H6" s="6">
-        <v>1633</v>
+        <v>1619</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>108</v>
       </c>
       <c r="J6" s="6">
-        <v>4421</v>
+        <v>4342</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>109</v>
       </c>
       <c r="L6" s="6">
-        <v>29301</v>
+        <v>29995</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>110</v>
       </c>
       <c r="N6" s="6">
-        <v>9410</v>
+        <v>9571</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>111</v>
       </c>
       <c r="P6" s="6">
-        <v>455</v>
+        <v>443</v>
       </c>
       <c r="Q6" s="7" t="s">
         <v>112</v>
       </c>
       <c r="R6" s="6">
-        <v>6514</v>
+        <v>6582</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>113</v>
       </c>
       <c r="T6" s="6">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="U6" s="7" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="V6" s="6">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="W6" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="X6" s="6">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="Y6" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Z6" s="6">
         <v>15</v>
       </c>
       <c r="AA6" s="7" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AB6" s="6">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="AC6" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AD6" s="6">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AE6" s="7" t="s">
         <v>106</v>
@@ -2043,34 +2043,34 @@
         <v>1</v>
       </c>
       <c r="AG6" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH6" s="6">
         <v>35</v>
       </c>
       <c r="AI6" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AJ6" s="6">
         <v>253</v>
       </c>
       <c r="AK6" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AL6" s="6">
         <v>33</v>
       </c>
       <c r="AM6" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AN6" s="6">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="AO6" s="7" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="AP6" s="6">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="AQ6" s="7" t="s">
         <v>120</v>
@@ -2082,19 +2082,19 @@
         <v>121</v>
       </c>
       <c r="AT6" s="6">
-        <v>2309</v>
+        <v>2297</v>
       </c>
       <c r="AU6" s="7" t="s">
         <v>122</v>
       </c>
       <c r="AV6" s="6">
-        <v>5010</v>
+        <v>5065</v>
       </c>
       <c r="AW6" s="7" t="s">
         <v>123</v>
       </c>
       <c r="AX6" s="6">
-        <v>12970</v>
+        <v>12982</v>
       </c>
       <c r="AY6" s="7" t="s">
         <v>124</v>
@@ -2108,40 +2108,40 @@
         <v>126</v>
       </c>
       <c r="C7" s="9">
-        <v>4805</v>
+        <v>5051</v>
       </c>
       <c r="D7" s="9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>127</v>
       </c>
       <c r="F7" s="9">
-        <v>1091</v>
+        <v>1119</v>
       </c>
       <c r="G7" s="10" t="s">
         <v>128</v>
       </c>
       <c r="H7" s="9">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="I7" s="10" t="s">
         <v>129</v>
       </c>
       <c r="J7" s="9">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="K7" s="10" t="s">
         <v>130</v>
       </c>
       <c r="L7" s="9">
-        <v>1746</v>
+        <v>1926</v>
       </c>
       <c r="M7" s="10" t="s">
         <v>131</v>
       </c>
       <c r="N7" s="9">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="O7" s="10" t="s">
         <v>132</v>
@@ -2153,7 +2153,7 @@
         <v>133</v>
       </c>
       <c r="R7" s="9">
-        <v>180</v>
+        <v>205</v>
       </c>
       <c r="S7" s="10" t="s">
         <v>134</v>
@@ -2162,16 +2162,16 @@
         <v>0</v>
       </c>
       <c r="U7" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V7" s="9">
         <v>2</v>
       </c>
       <c r="W7" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="X7" s="9">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y7" s="10" t="s">
         <v>135</v>
@@ -2180,31 +2180,31 @@
         <v>1</v>
       </c>
       <c r="AA7" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AB7" s="9">
         <v>6</v>
       </c>
       <c r="AC7" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AD7" s="9">
         <v>5</v>
       </c>
       <c r="AE7" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AF7" s="9">
         <v>0</v>
       </c>
       <c r="AG7" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH7" s="9">
         <v>2</v>
       </c>
       <c r="AI7" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AJ7" s="9">
         <v>7</v>
@@ -2216,10 +2216,10 @@
         <v>0</v>
       </c>
       <c r="AM7" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AN7" s="9">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="AO7" s="10" t="s">
         <v>138</v>
@@ -2237,19 +2237,19 @@
         <v>140</v>
       </c>
       <c r="AT7" s="9">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="AU7" s="10" t="s">
         <v>141</v>
       </c>
       <c r="AV7" s="9">
-        <v>166</v>
+        <v>183</v>
       </c>
       <c r="AW7" s="10" t="s">
         <v>142</v>
       </c>
       <c r="AX7" s="9">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="AY7" s="10" t="s">
         <v>143</v>
@@ -2263,13 +2263,13 @@
         <v>145</v>
       </c>
       <c r="C8" s="9">
-        <v>2797</v>
+        <v>2796</v>
       </c>
       <c r="D8" s="9">
         <v>0</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F8" s="9">
         <v>353</v>
@@ -2284,356 +2284,356 @@
         <v>147</v>
       </c>
       <c r="J8" s="9">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>148</v>
+        <v>123</v>
       </c>
       <c r="L8" s="9">
         <v>597</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="N8" s="9">
         <v>838</v>
       </c>
       <c r="O8" s="10" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="P8" s="9">
         <v>0</v>
       </c>
       <c r="Q8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="R8" s="9">
         <v>148</v>
       </c>
       <c r="S8" s="10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="T8" s="9">
         <v>0</v>
       </c>
       <c r="U8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V8" s="9">
         <v>0</v>
       </c>
       <c r="W8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X8" s="9">
         <v>2</v>
       </c>
       <c r="Y8" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="Z8" s="9">
         <v>0</v>
       </c>
       <c r="AA8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AB8" s="9">
         <v>0</v>
       </c>
       <c r="AC8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD8" s="9">
         <v>1</v>
       </c>
       <c r="AE8" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AF8" s="9">
         <v>0</v>
       </c>
       <c r="AG8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH8" s="9">
         <v>0</v>
       </c>
       <c r="AI8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ8" s="9">
         <v>5</v>
       </c>
       <c r="AK8" s="10" t="s">
-        <v>153</v>
+        <v>127</v>
       </c>
       <c r="AL8" s="9">
         <v>0</v>
       </c>
       <c r="AM8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AN8" s="9">
         <v>0</v>
       </c>
       <c r="AO8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AP8" s="9">
         <v>14</v>
       </c>
       <c r="AQ8" s="10" t="s">
-        <v>112</v>
+        <v>152</v>
       </c>
       <c r="AR8" s="9">
         <v>2</v>
       </c>
       <c r="AS8" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AT8" s="9">
         <v>8</v>
       </c>
       <c r="AU8" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="AV8" s="9">
+        <v>152</v>
+      </c>
+      <c r="AW8" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="AV8" s="9">
-        <v>153</v>
-      </c>
-      <c r="AW8" s="10" t="s">
+      <c r="AX8" s="9">
+        <v>510</v>
+      </c>
+      <c r="AY8" s="10" t="s">
         <v>155</v>
-      </c>
-      <c r="AX8" s="9">
-        <v>509</v>
-      </c>
-      <c r="AY8" s="10" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="C9" s="9">
+        <v>7683</v>
+      </c>
+      <c r="D9" s="9">
+        <v>0</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F9" s="9">
+        <v>1319</v>
+      </c>
+      <c r="G9" s="10" t="s">
         <v>158</v>
-      </c>
-      <c r="C9" s="9">
-        <v>7655</v>
-      </c>
-      <c r="D9" s="9">
-        <v>0</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="F9" s="9">
-        <v>1317</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>159</v>
       </c>
       <c r="H9" s="9">
         <v>207</v>
       </c>
       <c r="I9" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="J9" s="9">
+        <v>7</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="L9" s="9">
+        <v>3109</v>
+      </c>
+      <c r="M9" s="10" t="s">
         <v>160</v>
       </c>
-      <c r="J9" s="9">
-        <v>10</v>
-      </c>
-      <c r="K9" s="10" t="s">
-        <v>115</v>
-      </c>
-      <c r="L9" s="9">
-        <v>3090</v>
-      </c>
-      <c r="M9" s="10" t="s">
+      <c r="N9" s="9">
+        <v>1131</v>
+      </c>
+      <c r="O9" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="N9" s="9">
-        <v>1127</v>
-      </c>
-      <c r="O9" s="10" t="s">
+      <c r="P9" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="R9" s="9">
+        <v>719</v>
+      </c>
+      <c r="S9" s="10" t="s">
         <v>162</v>
-      </c>
-      <c r="P9" s="9">
-        <v>1</v>
-      </c>
-      <c r="Q9" s="10" t="s">
-        <v>163</v>
-      </c>
-      <c r="R9" s="9">
-        <v>714</v>
-      </c>
-      <c r="S9" s="10" t="s">
-        <v>164</v>
       </c>
       <c r="T9" s="9">
         <v>8</v>
       </c>
       <c r="U9" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="V9" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W9" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="X9" s="9">
+        <v>25</v>
+      </c>
+      <c r="Y9" s="10" t="s">
         <v>163</v>
       </c>
-      <c r="X9" s="9">
-        <v>24</v>
-      </c>
-      <c r="Y9" s="10" t="s">
-        <v>165</v>
-      </c>
       <c r="Z9" s="9">
         <v>0</v>
       </c>
       <c r="AA9" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AB9" s="9">
         <v>0</v>
       </c>
       <c r="AC9" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD9" s="9">
         <v>8</v>
       </c>
       <c r="AE9" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AF9" s="9">
         <v>1</v>
       </c>
       <c r="AG9" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="AH9" s="9">
         <v>1</v>
       </c>
       <c r="AI9" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="AJ9" s="9">
         <v>59</v>
       </c>
       <c r="AK9" s="10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="AL9" s="9">
         <v>0</v>
       </c>
       <c r="AM9" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AN9" s="9">
         <v>1</v>
       </c>
       <c r="AO9" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="AP9" s="9">
         <v>86</v>
       </c>
       <c r="AQ9" s="10" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="AR9" s="9">
         <v>2</v>
       </c>
       <c r="AS9" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="AT9" s="9">
+        <v>8</v>
+      </c>
+      <c r="AU9" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="AV9" s="9">
+        <v>333</v>
+      </c>
+      <c r="AW9" s="10" t="s">
         <v>168</v>
       </c>
-      <c r="AT9" s="9">
-        <v>11</v>
-      </c>
-      <c r="AU9" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="AV9" s="9">
-        <v>330</v>
-      </c>
-      <c r="AW9" s="10" t="s">
+      <c r="AX9" s="9">
+        <v>659</v>
+      </c>
+      <c r="AY9" s="10" t="s">
         <v>169</v>
-      </c>
-      <c r="AX9" s="9">
-        <v>657</v>
-      </c>
-      <c r="AY9" s="10" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="C10" s="9">
+        <v>13010</v>
+      </c>
+      <c r="D10" s="9">
+        <v>41</v>
+      </c>
+      <c r="E10" s="10" t="s">
         <v>172</v>
       </c>
-      <c r="C10" s="9">
-        <v>12279</v>
-      </c>
-      <c r="D10" s="9">
-        <v>42</v>
-      </c>
-      <c r="E10" s="10" t="s">
+      <c r="F10" s="9">
+        <v>2464</v>
+      </c>
+      <c r="G10" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="F10" s="9">
-        <v>2166</v>
-      </c>
-      <c r="G10" s="10" t="s">
+      <c r="H10" s="9">
+        <v>49</v>
+      </c>
+      <c r="I10" s="10" t="s">
         <v>174</v>
       </c>
-      <c r="H10" s="9">
-        <v>45</v>
-      </c>
-      <c r="I10" s="10" t="s">
+      <c r="J10" s="9">
+        <v>2109</v>
+      </c>
+      <c r="K10" s="10" t="s">
         <v>175</v>
       </c>
-      <c r="J10" s="9">
-        <v>2175</v>
-      </c>
-      <c r="K10" s="10" t="s">
+      <c r="L10" s="9">
+        <v>3455</v>
+      </c>
+      <c r="M10" s="10" t="s">
         <v>176</v>
       </c>
-      <c r="L10" s="9">
-        <v>3163</v>
-      </c>
-      <c r="M10" s="10" t="s">
+      <c r="N10" s="9">
+        <v>1266</v>
+      </c>
+      <c r="O10" s="10" t="s">
         <v>177</v>
       </c>
-      <c r="N10" s="9">
-        <v>1111</v>
-      </c>
-      <c r="O10" s="10" t="s">
+      <c r="P10" s="9">
+        <v>157</v>
+      </c>
+      <c r="Q10" s="10" t="s">
         <v>178</v>
       </c>
-      <c r="P10" s="9">
-        <v>166</v>
-      </c>
-      <c r="Q10" s="10" t="s">
+      <c r="R10" s="9">
+        <v>768</v>
+      </c>
+      <c r="S10" s="10" t="s">
         <v>179</v>
       </c>
-      <c r="R10" s="9">
-        <v>734</v>
-      </c>
-      <c r="S10" s="10" t="s">
-        <v>180</v>
-      </c>
       <c r="T10" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U10" s="10" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="V10" s="9">
         <v>9</v>
       </c>
       <c r="W10" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="X10" s="9">
         <v>10</v>
@@ -2645,31 +2645,31 @@
         <v>0</v>
       </c>
       <c r="AA10" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AB10" s="9">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AC10" s="10" t="s">
-        <v>121</v>
+        <v>136</v>
       </c>
       <c r="AD10" s="9">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AE10" s="10" t="s">
-        <v>114</v>
+        <v>180</v>
       </c>
       <c r="AF10" s="9">
         <v>0</v>
       </c>
       <c r="AG10" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH10" s="9">
         <v>12</v>
       </c>
       <c r="AI10" s="10" t="s">
-        <v>135</v>
+        <v>114</v>
       </c>
       <c r="AJ10" s="9">
         <v>10</v>
@@ -2681,7 +2681,7 @@
         <v>1</v>
       </c>
       <c r="AM10" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="AN10" s="9">
         <v>58</v>
@@ -2693,28 +2693,28 @@
         <v>19</v>
       </c>
       <c r="AQ10" s="10" t="s">
-        <v>137</v>
+        <v>182</v>
       </c>
       <c r="AR10" s="9">
         <v>5</v>
       </c>
       <c r="AS10" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AT10" s="9">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="AU10" s="10" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="AV10" s="9">
-        <v>316</v>
+        <v>327</v>
       </c>
       <c r="AW10" s="10" t="s">
-        <v>183</v>
+        <v>132</v>
       </c>
       <c r="AX10" s="9">
-        <v>1881</v>
+        <v>1877</v>
       </c>
       <c r="AY10" s="10" t="s">
         <v>184</v>
@@ -2728,67 +2728,67 @@
         <v>186</v>
       </c>
       <c r="C11" s="9">
-        <v>12269</v>
+        <v>12280</v>
       </c>
       <c r="D11" s="9">
         <v>3</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F11" s="9">
-        <v>1883</v>
+        <v>1893</v>
       </c>
       <c r="G11" s="10" t="s">
         <v>187</v>
       </c>
       <c r="H11" s="9">
-        <v>316</v>
+        <v>307</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>132</v>
+        <v>188</v>
       </c>
       <c r="J11" s="9">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="L11" s="9">
-        <v>5498</v>
+        <v>5502</v>
       </c>
       <c r="M11" s="10" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="N11" s="9">
         <v>624</v>
       </c>
       <c r="O11" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="P11" s="9">
         <v>113</v>
       </c>
       <c r="Q11" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="R11" s="9">
         <v>1586</v>
       </c>
       <c r="S11" s="10" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="T11" s="9">
         <v>18</v>
       </c>
       <c r="U11" s="10" t="s">
-        <v>137</v>
+        <v>182</v>
       </c>
       <c r="V11" s="9">
         <v>5</v>
       </c>
       <c r="W11" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="X11" s="9">
         <v>10</v>
@@ -2800,52 +2800,52 @@
         <v>5</v>
       </c>
       <c r="AA11" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AB11" s="9">
         <v>3</v>
       </c>
       <c r="AC11" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AD11" s="9">
         <v>22</v>
       </c>
       <c r="AE11" s="10" t="s">
-        <v>153</v>
+        <v>127</v>
       </c>
       <c r="AF11" s="9">
         <v>0</v>
       </c>
       <c r="AG11" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH11" s="9">
         <v>5</v>
       </c>
       <c r="AI11" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AJ11" s="9">
         <v>29</v>
       </c>
       <c r="AK11" s="10" t="s">
-        <v>193</v>
+        <v>138</v>
       </c>
       <c r="AL11" s="9">
         <v>3</v>
       </c>
       <c r="AM11" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AN11" s="9">
         <v>8</v>
       </c>
       <c r="AO11" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AP11" s="9">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="AQ11" s="10" t="s">
         <v>194</v>
@@ -2854,10 +2854,10 @@
         <v>15</v>
       </c>
       <c r="AS11" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AT11" s="9">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="AU11" s="10" t="s">
         <v>195</v>
@@ -2883,13 +2883,13 @@
         <v>199</v>
       </c>
       <c r="C12" s="9">
-        <v>4930</v>
+        <v>4933</v>
       </c>
       <c r="D12" s="9">
         <v>0</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F12" s="9">
         <v>922</v>
@@ -2904,19 +2904,19 @@
         <v>201</v>
       </c>
       <c r="J12" s="9">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="K12" s="10" t="s">
         <v>202</v>
       </c>
       <c r="L12" s="9">
-        <v>1801</v>
+        <v>1811</v>
       </c>
       <c r="M12" s="10" t="s">
         <v>203</v>
       </c>
       <c r="N12" s="9">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="O12" s="10" t="s">
         <v>204</v>
@@ -2937,7 +2937,7 @@
         <v>0</v>
       </c>
       <c r="U12" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V12" s="9">
         <v>3</v>
@@ -2949,13 +2949,13 @@
         <v>6</v>
       </c>
       <c r="Y12" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="Z12" s="9">
         <v>1</v>
       </c>
       <c r="AA12" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AB12" s="9">
         <v>3</v>
@@ -2967,19 +2967,19 @@
         <v>9</v>
       </c>
       <c r="AE12" s="10" t="s">
-        <v>153</v>
+        <v>127</v>
       </c>
       <c r="AF12" s="9">
         <v>0</v>
       </c>
       <c r="AG12" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH12" s="9">
         <v>2</v>
       </c>
       <c r="AI12" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AJ12" s="9">
         <v>29</v>
@@ -2991,7 +2991,7 @@
         <v>0</v>
       </c>
       <c r="AM12" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AN12" s="9">
         <v>4</v>
@@ -3003,13 +3003,13 @@
         <v>55</v>
       </c>
       <c r="AQ12" s="10" t="s">
-        <v>167</v>
+        <v>207</v>
       </c>
       <c r="AR12" s="9">
         <v>1</v>
       </c>
       <c r="AS12" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AT12" s="9">
         <v>29</v>
@@ -3021,30 +3021,30 @@
         <v>337</v>
       </c>
       <c r="AW12" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AX12" s="9">
         <v>517</v>
       </c>
       <c r="AY12" s="10" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C13" s="9">
-        <v>4327</v>
+        <v>4329</v>
       </c>
       <c r="D13" s="9">
         <v>2</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>211</v>
+        <v>180</v>
       </c>
       <c r="F13" s="9">
         <v>783</v>
@@ -3056,91 +3056,91 @@
         <v>28</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>133</v>
+        <v>213</v>
       </c>
       <c r="J13" s="9">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="L13" s="9">
         <v>1649</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="N13" s="9">
         <v>700</v>
       </c>
       <c r="O13" s="10" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="P13" s="9">
         <v>13</v>
       </c>
       <c r="Q13" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="R13" s="9">
         <v>237</v>
       </c>
       <c r="S13" s="10" t="s">
-        <v>217</v>
+        <v>123</v>
       </c>
       <c r="T13" s="9">
         <v>0</v>
       </c>
       <c r="U13" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V13" s="9">
         <v>1</v>
       </c>
       <c r="W13" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="X13" s="9">
         <v>3</v>
       </c>
       <c r="Y13" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="Z13" s="9">
         <v>0</v>
       </c>
       <c r="AA13" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AB13" s="9">
         <v>1</v>
       </c>
       <c r="AC13" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AD13" s="9">
         <v>6</v>
       </c>
       <c r="AE13" s="10" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
       <c r="AF13" s="9">
         <v>0</v>
       </c>
       <c r="AG13" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH13" s="9">
         <v>1</v>
       </c>
       <c r="AI13" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AJ13" s="9">
         <v>28</v>
       </c>
       <c r="AK13" s="10" t="s">
-        <v>133</v>
+        <v>213</v>
       </c>
       <c r="AL13" s="9">
         <v>11</v>
@@ -3152,7 +3152,7 @@
         <v>3</v>
       </c>
       <c r="AO13" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AP13" s="9">
         <v>35</v>
@@ -3167,129 +3167,129 @@
         <v>220</v>
       </c>
       <c r="AT13" s="9">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="AU13" s="10" t="s">
-        <v>221</v>
+        <v>147</v>
       </c>
       <c r="AV13" s="9">
         <v>205</v>
       </c>
       <c r="AW13" s="10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="AX13" s="9">
         <v>325</v>
       </c>
       <c r="AY13" s="10" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="C14" s="9">
+        <v>4248</v>
+      </c>
+      <c r="D14" s="9">
+        <v>0</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F14" s="9">
+        <v>1020</v>
+      </c>
+      <c r="G14" s="10" t="s">
         <v>225</v>
-      </c>
-      <c r="C14" s="9">
-        <v>4241</v>
-      </c>
-      <c r="D14" s="9">
-        <v>0</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="F14" s="9">
-        <v>1018</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>226</v>
       </c>
       <c r="H14" s="9">
         <v>18</v>
       </c>
       <c r="I14" s="10" t="s">
+        <v>226</v>
+      </c>
+      <c r="J14" s="9">
+        <v>111</v>
+      </c>
+      <c r="K14" s="10" t="s">
         <v>227</v>
       </c>
-      <c r="J14" s="9">
-        <v>112</v>
-      </c>
-      <c r="K14" s="10" t="s">
+      <c r="L14" s="9">
+        <v>1147</v>
+      </c>
+      <c r="M14" s="10" t="s">
         <v>228</v>
-      </c>
-      <c r="L14" s="9">
-        <v>1141</v>
-      </c>
-      <c r="M14" s="10" t="s">
-        <v>229</v>
       </c>
       <c r="N14" s="9">
         <v>644</v>
       </c>
       <c r="O14" s="10" t="s">
+        <v>229</v>
+      </c>
+      <c r="P14" s="9">
+        <v>7</v>
+      </c>
+      <c r="Q14" s="10" t="s">
         <v>230</v>
       </c>
-      <c r="P14" s="9">
-        <v>8</v>
-      </c>
-      <c r="Q14" s="10" t="s">
+      <c r="R14" s="9">
+        <v>240</v>
+      </c>
+      <c r="S14" s="10" t="s">
         <v>231</v>
-      </c>
-      <c r="R14" s="9">
-        <v>239</v>
-      </c>
-      <c r="S14" s="10" t="s">
-        <v>232</v>
       </c>
       <c r="T14" s="9">
         <v>2</v>
       </c>
       <c r="U14" s="10" t="s">
-        <v>211</v>
+        <v>180</v>
       </c>
       <c r="V14" s="9">
         <v>0</v>
       </c>
       <c r="W14" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X14" s="9">
         <v>8</v>
       </c>
       <c r="Y14" s="10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="Z14" s="9">
         <v>1</v>
       </c>
       <c r="AA14" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AB14" s="9">
         <v>1</v>
       </c>
       <c r="AC14" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AD14" s="9">
         <v>5</v>
       </c>
       <c r="AE14" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AF14" s="9">
         <v>0</v>
       </c>
       <c r="AG14" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH14" s="9">
         <v>1</v>
       </c>
       <c r="AI14" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AJ14" s="9">
         <v>11</v>
@@ -3301,13 +3301,13 @@
         <v>1</v>
       </c>
       <c r="AM14" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AN14" s="9">
         <v>3</v>
       </c>
       <c r="AO14" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AP14" s="9">
         <v>28</v>
@@ -3319,22 +3319,22 @@
         <v>1</v>
       </c>
       <c r="AS14" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AT14" s="9">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="AU14" s="10" t="s">
         <v>235</v>
       </c>
       <c r="AV14" s="9">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="AW14" s="10" t="s">
         <v>236</v>
       </c>
       <c r="AX14" s="9">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="AY14" s="10" t="s">
         <v>237</v>
@@ -3348,13 +3348,13 @@
         <v>239</v>
       </c>
       <c r="C15" s="9">
-        <v>10644</v>
+        <v>10671</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F15" s="9">
         <v>3008</v>
@@ -3369,28 +3369,28 @@
         <v>241</v>
       </c>
       <c r="J15" s="9">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="K15" s="10" t="s">
         <v>242</v>
       </c>
       <c r="L15" s="9">
-        <v>2898</v>
+        <v>2923</v>
       </c>
       <c r="M15" s="10" t="s">
         <v>243</v>
       </c>
       <c r="N15" s="9">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="O15" s="10" t="s">
         <v>244</v>
       </c>
       <c r="P15" s="9">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="R15" s="9">
         <v>660</v>
@@ -3399,320 +3399,320 @@
         <v>245</v>
       </c>
       <c r="T15" s="9">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>246</v>
+        <v>226</v>
       </c>
       <c r="V15" s="9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W15" s="10" t="s">
-        <v>114</v>
+        <v>167</v>
       </c>
       <c r="X15" s="9">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Y15" s="10" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="Z15" s="9">
         <v>0</v>
       </c>
       <c r="AA15" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AB15" s="9">
         <v>0</v>
       </c>
       <c r="AC15" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD15" s="9">
         <v>3</v>
       </c>
       <c r="AE15" s="10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AF15" s="9">
         <v>0</v>
       </c>
       <c r="AG15" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH15" s="9">
         <v>1</v>
       </c>
       <c r="AI15" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="AJ15" s="9">
         <v>11</v>
       </c>
       <c r="AK15" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AL15" s="9">
         <v>2</v>
       </c>
       <c r="AM15" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AN15" s="9">
         <v>7</v>
       </c>
       <c r="AO15" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AP15" s="9">
         <v>69</v>
       </c>
       <c r="AQ15" s="10" t="s">
-        <v>133</v>
+        <v>213</v>
       </c>
       <c r="AR15" s="9">
         <v>17</v>
       </c>
       <c r="AS15" s="10" t="s">
-        <v>247</v>
+        <v>230</v>
       </c>
       <c r="AT15" s="9">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="AU15" s="10" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="AV15" s="9">
         <v>1011</v>
       </c>
       <c r="AW15" s="10" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="AX15" s="9">
-        <v>2074</v>
+        <v>2076</v>
       </c>
       <c r="AY15" s="10" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C16" s="9">
-        <v>4117</v>
+        <v>4116</v>
       </c>
       <c r="D16" s="9">
         <v>8</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F16" s="9">
         <v>719</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="H16" s="9">
         <v>21</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="J16" s="9">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>160</v>
+        <v>253</v>
       </c>
       <c r="L16" s="9">
         <v>1160</v>
       </c>
       <c r="M16" s="10" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="N16" s="9">
         <v>129</v>
       </c>
       <c r="O16" s="10" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="P16" s="9">
         <v>14</v>
       </c>
       <c r="Q16" s="10" t="s">
-        <v>173</v>
+        <v>139</v>
       </c>
       <c r="R16" s="9">
         <v>185</v>
       </c>
       <c r="S16" s="10" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="T16" s="9">
         <v>0</v>
       </c>
       <c r="U16" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V16" s="9">
         <v>2</v>
       </c>
       <c r="W16" s="10" t="s">
-        <v>211</v>
+        <v>180</v>
       </c>
       <c r="X16" s="9">
         <v>2</v>
       </c>
       <c r="Y16" s="10" t="s">
-        <v>211</v>
+        <v>180</v>
       </c>
       <c r="Z16" s="9">
         <v>0</v>
       </c>
       <c r="AA16" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AB16" s="9">
         <v>3</v>
       </c>
       <c r="AC16" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AD16" s="9">
         <v>1</v>
       </c>
       <c r="AE16" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AF16" s="9">
         <v>0</v>
       </c>
       <c r="AG16" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH16" s="9">
         <v>1</v>
       </c>
       <c r="AI16" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AJ16" s="9">
         <v>18</v>
       </c>
       <c r="AK16" s="10" t="s">
-        <v>221</v>
+        <v>257</v>
       </c>
       <c r="AL16" s="9">
         <v>8</v>
       </c>
       <c r="AM16" s="10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="AN16" s="9">
         <v>6</v>
       </c>
       <c r="AO16" s="10" t="s">
-        <v>137</v>
+        <v>182</v>
       </c>
       <c r="AP16" s="9">
         <v>25</v>
       </c>
       <c r="AQ16" s="10" t="s">
-        <v>258</v>
+        <v>133</v>
       </c>
       <c r="AR16" s="9">
         <v>12</v>
       </c>
       <c r="AS16" s="10" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="AT16" s="9">
         <v>237</v>
       </c>
       <c r="AU16" s="10" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AV16" s="9">
         <v>322</v>
       </c>
       <c r="AW16" s="10" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="AX16" s="9">
         <v>1133</v>
       </c>
       <c r="AY16" s="10" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>262</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>263</v>
-      </c>
       <c r="C17" s="9">
-        <v>6015</v>
+        <v>6034</v>
       </c>
       <c r="D17" s="9">
         <v>1</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F17" s="9">
         <v>1809</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="H17" s="9">
         <v>446</v>
       </c>
       <c r="I17" s="10" t="s">
+        <v>264</v>
+      </c>
+      <c r="J17" s="9">
+        <v>200</v>
+      </c>
+      <c r="K17" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="J17" s="9">
-        <v>206</v>
-      </c>
-      <c r="K17" s="10" t="s">
+      <c r="L17" s="9">
+        <v>1580</v>
+      </c>
+      <c r="M17" s="10" t="s">
         <v>266</v>
       </c>
-      <c r="L17" s="9">
-        <v>1565</v>
-      </c>
-      <c r="M17" s="10" t="s">
+      <c r="N17" s="9">
+        <v>437</v>
+      </c>
+      <c r="O17" s="10" t="s">
         <v>267</v>
-      </c>
-      <c r="N17" s="9">
-        <v>431</v>
-      </c>
-      <c r="O17" s="10" t="s">
-        <v>268</v>
       </c>
       <c r="P17" s="9">
         <v>22</v>
       </c>
       <c r="Q17" s="10" t="s">
-        <v>175</v>
+        <v>268</v>
       </c>
       <c r="R17" s="9">
         <v>206</v>
       </c>
       <c r="S17" s="10" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="T17" s="9">
         <v>1</v>
       </c>
       <c r="U17" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="V17" s="9">
         <v>5</v>
@@ -3730,37 +3730,37 @@
         <v>2</v>
       </c>
       <c r="AA17" s="10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AB17" s="9">
         <v>2</v>
       </c>
       <c r="AC17" s="10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AD17" s="9">
         <v>4</v>
       </c>
       <c r="AE17" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AF17" s="9">
         <v>0</v>
       </c>
       <c r="AG17" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH17" s="9">
         <v>2</v>
       </c>
       <c r="AI17" s="10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AJ17" s="9">
         <v>12</v>
       </c>
       <c r="AK17" s="10" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="AL17" s="9">
         <v>5</v>
@@ -3772,45 +3772,45 @@
         <v>9</v>
       </c>
       <c r="AO17" s="10" t="s">
-        <v>137</v>
+        <v>182</v>
       </c>
       <c r="AP17" s="9">
         <v>39</v>
       </c>
       <c r="AQ17" s="10" t="s">
-        <v>133</v>
+        <v>213</v>
       </c>
       <c r="AR17" s="9">
         <v>11</v>
       </c>
       <c r="AS17" s="10" t="s">
-        <v>153</v>
+        <v>127</v>
       </c>
       <c r="AT17" s="9">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="AU17" s="10" t="s">
-        <v>109</v>
+        <v>271</v>
       </c>
       <c r="AV17" s="9">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="AW17" s="10" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="AX17" s="9">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="AY17" s="10" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C18" s="9">
         <v>6896</v>
@@ -3819,115 +3819,115 @@
         <v>8</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F18" s="9">
-        <v>1168</v>
+        <v>1171</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="H18" s="9">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="J18" s="9">
         <v>742</v>
       </c>
       <c r="K18" s="10" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="L18" s="9">
-        <v>1599</v>
+        <v>1602</v>
       </c>
       <c r="M18" s="10" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="N18" s="9">
-        <v>974</v>
+        <v>971</v>
       </c>
       <c r="O18" s="10" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="P18" s="9">
         <v>57</v>
       </c>
       <c r="Q18" s="10" t="s">
-        <v>279</v>
+        <v>242</v>
       </c>
       <c r="R18" s="9">
         <v>362</v>
       </c>
       <c r="S18" s="10" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="T18" s="9">
         <v>3</v>
       </c>
       <c r="U18" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="V18" s="9">
         <v>2</v>
       </c>
       <c r="W18" s="10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="X18" s="9">
         <v>3</v>
       </c>
       <c r="Y18" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Z18" s="9">
         <v>0</v>
       </c>
       <c r="AA18" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AB18" s="9">
         <v>3</v>
       </c>
       <c r="AC18" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AD18" s="9">
         <v>1</v>
       </c>
       <c r="AE18" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="AF18" s="9">
         <v>0</v>
       </c>
       <c r="AG18" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH18" s="9">
         <v>6</v>
       </c>
       <c r="AI18" s="10" t="s">
-        <v>281</v>
+        <v>114</v>
       </c>
       <c r="AJ18" s="9">
         <v>9</v>
       </c>
       <c r="AK18" s="10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AL18" s="9">
         <v>0</v>
       </c>
       <c r="AM18" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AN18" s="9">
         <v>11</v>
       </c>
       <c r="AO18" s="10" t="s">
-        <v>247</v>
+        <v>230</v>
       </c>
       <c r="AP18" s="9">
         <v>17</v>
@@ -3939,7 +3939,7 @@
         <v>5</v>
       </c>
       <c r="AS18" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AT18" s="9">
         <v>253</v>
@@ -3968,16 +3968,16 @@
         <v>286</v>
       </c>
       <c r="C19" s="9">
-        <v>7038</v>
+        <v>7209</v>
       </c>
       <c r="D19" s="9">
         <v>1</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F19" s="9">
-        <v>941</v>
+        <v>957</v>
       </c>
       <c r="G19" s="10" t="s">
         <v>287</v>
@@ -3986,16 +3986,16 @@
         <v>12</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>127</v>
+        <v>288</v>
       </c>
       <c r="J19" s="9">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="K19" s="10" t="s">
-        <v>288</v>
+        <v>220</v>
       </c>
       <c r="L19" s="9">
-        <v>2477</v>
+        <v>2613</v>
       </c>
       <c r="M19" s="10" t="s">
         <v>289</v>
@@ -4010,10 +4010,10 @@
         <v>0</v>
       </c>
       <c r="Q19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="R19" s="9">
-        <v>646</v>
+        <v>649</v>
       </c>
       <c r="S19" s="10" t="s">
         <v>291</v>
@@ -4022,49 +4022,49 @@
         <v>0</v>
       </c>
       <c r="U19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V19" s="9">
         <v>1</v>
       </c>
       <c r="W19" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="X19" s="9">
         <v>12</v>
       </c>
       <c r="Y19" s="10" t="s">
-        <v>127</v>
+        <v>288</v>
       </c>
       <c r="Z19" s="9">
         <v>0</v>
       </c>
       <c r="AA19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AB19" s="9">
         <v>0</v>
       </c>
       <c r="AC19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD19" s="9">
         <v>3</v>
       </c>
       <c r="AE19" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AF19" s="9">
         <v>0</v>
       </c>
       <c r="AG19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH19" s="9">
         <v>0</v>
       </c>
       <c r="AI19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ19" s="9">
         <v>16</v>
@@ -4076,13 +4076,13 @@
         <v>0</v>
       </c>
       <c r="AM19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AN19" s="9">
         <v>1</v>
       </c>
       <c r="AO19" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="AP19" s="9">
         <v>50</v>
@@ -4094,63 +4094,63 @@
         <v>1</v>
       </c>
       <c r="AS19" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="AT19" s="9">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AU19" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="AV19" s="9">
+        <v>546</v>
+      </c>
+      <c r="AW19" s="10" t="s">
         <v>294</v>
       </c>
-      <c r="AV19" s="9">
-        <v>531</v>
-      </c>
-      <c r="AW19" s="10" t="s">
+      <c r="AX19" s="9">
+        <v>791</v>
+      </c>
+      <c r="AY19" s="10" t="s">
         <v>295</v>
-      </c>
-      <c r="AX19" s="9">
-        <v>783</v>
-      </c>
-      <c r="AY19" s="10" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
+        <v>296</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>297</v>
       </c>
-      <c r="B20" s="8" t="s">
-        <v>298</v>
-      </c>
       <c r="C20" s="9">
-        <v>996</v>
+        <v>998</v>
       </c>
       <c r="D20" s="9">
         <v>1</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F20" s="9">
         <v>157</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H20" s="9">
         <v>6</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="J20" s="9">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="K20" s="10" t="s">
         <v>300</v>
       </c>
       <c r="L20" s="9">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="M20" s="10" t="s">
         <v>301</v>
@@ -4165,7 +4165,7 @@
         <v>5</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>112</v>
+        <v>152</v>
       </c>
       <c r="R20" s="9">
         <v>163</v>
@@ -4177,13 +4177,13 @@
         <v>0</v>
       </c>
       <c r="U20" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V20" s="9">
         <v>0</v>
       </c>
       <c r="W20" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X20" s="9">
         <v>9</v>
@@ -4195,49 +4195,49 @@
         <v>3</v>
       </c>
       <c r="AA20" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="AB20" s="9">
         <v>0</v>
       </c>
       <c r="AC20" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD20" s="9">
         <v>0</v>
       </c>
       <c r="AE20" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AF20" s="9">
         <v>0</v>
       </c>
       <c r="AG20" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH20" s="9">
         <v>1</v>
       </c>
       <c r="AI20" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AJ20" s="9">
         <v>6</v>
       </c>
       <c r="AK20" s="10" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="AL20" s="9">
         <v>2</v>
       </c>
       <c r="AM20" s="10" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="AN20" s="9">
         <v>1</v>
       </c>
       <c r="AO20" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AP20" s="9">
         <v>18</v>
@@ -4255,7 +4255,7 @@
         <v>6</v>
       </c>
       <c r="AU20" s="10" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="AV20" s="9">
         <v>46</v>
@@ -4278,121 +4278,121 @@
         <v>310</v>
       </c>
       <c r="C21" s="9">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="D21" s="9">
         <v>0</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F21" s="9">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="G21" s="10" t="s">
         <v>311</v>
       </c>
       <c r="H21" s="9">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>207</v>
+        <v>312</v>
       </c>
       <c r="J21" s="9">
         <v>16</v>
       </c>
       <c r="K21" s="10" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="L21" s="9">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="N21" s="9">
         <v>102</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="P21" s="9">
         <v>7</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>165</v>
+        <v>316</v>
       </c>
       <c r="R21" s="9">
         <v>67</v>
       </c>
       <c r="S21" s="10" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="T21" s="9">
         <v>0</v>
       </c>
       <c r="U21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V21" s="9">
         <v>5</v>
       </c>
       <c r="W21" s="10" t="s">
-        <v>316</v>
+        <v>292</v>
       </c>
       <c r="X21" s="9">
         <v>11</v>
       </c>
       <c r="Y21" s="10" t="s">
-        <v>317</v>
+        <v>112</v>
       </c>
       <c r="Z21" s="9">
         <v>2</v>
       </c>
       <c r="AA21" s="10" t="s">
-        <v>281</v>
+        <v>114</v>
       </c>
       <c r="AB21" s="9">
         <v>0</v>
       </c>
       <c r="AC21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD21" s="9">
         <v>1</v>
       </c>
       <c r="AE21" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AF21" s="9">
         <v>0</v>
       </c>
       <c r="AG21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH21" s="9">
         <v>0</v>
       </c>
       <c r="AI21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ21" s="9">
         <v>3</v>
       </c>
       <c r="AK21" s="10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AL21" s="9">
         <v>0</v>
       </c>
       <c r="AM21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AN21" s="9">
         <v>0</v>
       </c>
       <c r="AO21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AP21" s="9">
         <v>18</v>
@@ -4404,22 +4404,22 @@
         <v>1</v>
       </c>
       <c r="AS21" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AT21" s="9">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="AU21" s="10" t="s">
         <v>318</v>
       </c>
       <c r="AV21" s="9">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="AW21" s="10" t="s">
         <v>319</v>
       </c>
       <c r="AX21" s="9">
-        <v>771</v>
+        <v>768</v>
       </c>
       <c r="AY21" s="10" t="s">
         <v>320</v>
@@ -4433,7 +4433,7 @@
         <v>322</v>
       </c>
       <c r="C22" s="12">
-        <v>91291</v>
+        <v>92539</v>
       </c>
       <c r="D22" s="12">
         <v>74</v>
@@ -4442,79 +4442,79 @@
         <v>106</v>
       </c>
       <c r="F22" s="12">
-        <v>17711</v>
+        <v>18071</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>107</v>
       </c>
       <c r="H22" s="12">
-        <v>1633</v>
+        <v>1619</v>
       </c>
       <c r="I22" s="13" t="s">
         <v>108</v>
       </c>
       <c r="J22" s="12">
-        <v>4421</v>
+        <v>4342</v>
       </c>
       <c r="K22" s="13" t="s">
         <v>109</v>
       </c>
       <c r="L22" s="12">
-        <v>29301</v>
+        <v>29995</v>
       </c>
       <c r="M22" s="13" t="s">
         <v>110</v>
       </c>
       <c r="N22" s="12">
-        <v>9410</v>
+        <v>9571</v>
       </c>
       <c r="O22" s="13" t="s">
         <v>111</v>
       </c>
       <c r="P22" s="12">
-        <v>455</v>
+        <v>443</v>
       </c>
       <c r="Q22" s="13" t="s">
         <v>112</v>
       </c>
       <c r="R22" s="12">
-        <v>6514</v>
+        <v>6582</v>
       </c>
       <c r="S22" s="13" t="s">
         <v>113</v>
       </c>
       <c r="T22" s="12">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="U22" s="13" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="V22" s="12">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="W22" s="13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="X22" s="12">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="Y22" s="13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Z22" s="12">
         <v>15</v>
       </c>
       <c r="AA22" s="13" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AB22" s="12">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="AC22" s="13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AD22" s="12">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AE22" s="13" t="s">
         <v>106</v>
@@ -4523,34 +4523,34 @@
         <v>1</v>
       </c>
       <c r="AG22" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH22" s="12">
         <v>35</v>
       </c>
       <c r="AI22" s="13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AJ22" s="12">
         <v>253</v>
       </c>
       <c r="AK22" s="13" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AL22" s="12">
         <v>33</v>
       </c>
       <c r="AM22" s="13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AN22" s="12">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="AO22" s="13" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="AP22" s="12">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="AQ22" s="13" t="s">
         <v>120</v>
@@ -4562,19 +4562,19 @@
         <v>121</v>
       </c>
       <c r="AT22" s="12">
-        <v>2309</v>
+        <v>2297</v>
       </c>
       <c r="AU22" s="13" t="s">
         <v>122</v>
       </c>
       <c r="AV22" s="12">
-        <v>5010</v>
+        <v>5065</v>
       </c>
       <c r="AW22" s="13" t="s">
         <v>123</v>
       </c>
       <c r="AX22" s="12">
-        <v>12970</v>
+        <v>12982</v>
       </c>
       <c r="AY22" s="13" t="s">
         <v>124</v>

</xml_diff>

<commit_message>
Perbarui data SE2026 25/08/2026  8:00:00,49
</commit_message>
<xml_diff>
--- a/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
+++ b/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
@@ -16,7 +16,7 @@
     <t>DATA RADAR ANOMALI USAHA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 24 Agu 2026, 21.08</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 25 Agu 2026, 07.58</t>
   </si>
   <si>
     <t>Kode</t>
@@ -334,502 +334,505 @@
     <t>0,08</t>
   </si>
   <si>
-    <t>19,53</t>
-  </si>
-  <si>
-    <t>1,75</t>
-  </si>
-  <si>
-    <t>4,69</t>
-  </si>
-  <si>
-    <t>32,41</t>
-  </si>
-  <si>
-    <t>10,34</t>
+    <t>19,72</t>
+  </si>
+  <si>
+    <t>1,69</t>
+  </si>
+  <si>
+    <t>4,45</t>
+  </si>
+  <si>
+    <t>32,84</t>
+  </si>
+  <si>
+    <t>10,31</t>
+  </si>
+  <si>
+    <t>0,47</t>
+  </si>
+  <si>
+    <t>7,09</t>
+  </si>
+  <si>
+    <t>0,09</t>
+  </si>
+  <si>
+    <t>0,03</t>
+  </si>
+  <si>
+    <t>0,14</t>
+  </si>
+  <si>
+    <t>0,02</t>
+  </si>
+  <si>
+    <t>0,04</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>0,27</t>
+  </si>
+  <si>
+    <t>0,13</t>
+  </si>
+  <si>
+    <t>0,62</t>
+  </si>
+  <si>
+    <t>0,11</t>
+  </si>
+  <si>
+    <t>2,34</t>
+  </si>
+  <si>
+    <t>5,45</t>
+  </si>
+  <si>
+    <t>13,97</t>
+  </si>
+  <si>
+    <t>1801</t>
+  </si>
+  <si>
+    <t>LAMPUNG BARAT</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>1,42</t>
+  </si>
+  <si>
+    <t>4,92</t>
+  </si>
+  <si>
+    <t>38,56</t>
+  </si>
+  <si>
+    <t>2,5</t>
+  </si>
+  <si>
+    <t>0,61</t>
+  </si>
+  <si>
+    <t>4,09</t>
+  </si>
+  <si>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>0,24</t>
+  </si>
+  <si>
+    <t>0,33</t>
+  </si>
+  <si>
+    <t>0,06</t>
+  </si>
+  <si>
+    <t>11,09</t>
+  </si>
+  <si>
+    <t>3,6</t>
+  </si>
+  <si>
+    <t>9,89</t>
+  </si>
+  <si>
+    <t>1802</t>
+  </si>
+  <si>
+    <t>TANGGAMUS</t>
+  </si>
+  <si>
+    <t>12,62</t>
+  </si>
+  <si>
+    <t>0,46</t>
+  </si>
+  <si>
+    <t>5,42</t>
+  </si>
+  <si>
+    <t>21,33</t>
+  </si>
+  <si>
+    <t>30,03</t>
+  </si>
+  <si>
+    <t>5,28</t>
+  </si>
+  <si>
+    <t>0,07</t>
+  </si>
+  <si>
+    <t>0,18</t>
+  </si>
+  <si>
+    <t>0,5</t>
+  </si>
+  <si>
+    <t>0,29</t>
+  </si>
+  <si>
+    <t>18,3</t>
+  </si>
+  <si>
+    <t>1803</t>
+  </si>
+  <si>
+    <t>LAMPUNG SELATAN</t>
+  </si>
+  <si>
+    <t>17,24</t>
+  </si>
+  <si>
+    <t>2,68</t>
+  </si>
+  <si>
+    <t>40,61</t>
+  </si>
+  <si>
+    <t>14,63</t>
+  </si>
+  <si>
+    <t>9,31</t>
+  </si>
+  <si>
+    <t>0,32</t>
+  </si>
+  <si>
+    <t>0,01</t>
+  </si>
+  <si>
+    <t>0,76</t>
+  </si>
+  <si>
+    <t>1,11</t>
+  </si>
+  <si>
+    <t>4,31</t>
+  </si>
+  <si>
+    <t>8,54</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>0,28</t>
+  </si>
+  <si>
+    <t>20,42</t>
+  </si>
+  <si>
+    <t>0,34</t>
+  </si>
+  <si>
+    <t>14,38</t>
+  </si>
+  <si>
+    <t>28,2</t>
+  </si>
+  <si>
+    <t>10,08</t>
+  </si>
+  <si>
+    <t>1,09</t>
+  </si>
+  <si>
+    <t>5,96</t>
+  </si>
+  <si>
+    <t>0,41</t>
+  </si>
+  <si>
+    <t>2,48</t>
+  </si>
+  <si>
+    <t>2,47</t>
+  </si>
+  <si>
+    <t>13,2</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>15,43</t>
+  </si>
+  <si>
+    <t>2,49</t>
+  </si>
+  <si>
+    <t>1,14</t>
+  </si>
+  <si>
+    <t>44,89</t>
+  </si>
+  <si>
+    <t>5,07</t>
+  </si>
+  <si>
+    <t>0,93</t>
+  </si>
+  <si>
+    <t>12,89</t>
+  </si>
+  <si>
+    <t>0,15</t>
+  </si>
+  <si>
+    <t>0,05</t>
+  </si>
+  <si>
+    <t>0,68</t>
+  </si>
+  <si>
+    <t>0,74</t>
+  </si>
+  <si>
+    <t>3,23</t>
+  </si>
+  <si>
+    <t>11,46</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>18,68</t>
+  </si>
+  <si>
+    <t>0,77</t>
+  </si>
+  <si>
+    <t>1,53</t>
+  </si>
+  <si>
+    <t>36,71</t>
+  </si>
+  <si>
+    <t>14,2</t>
+  </si>
+  <si>
+    <t>7,82</t>
+  </si>
+  <si>
+    <t>0,59</t>
+  </si>
+  <si>
+    <t>0,71</t>
+  </si>
+  <si>
+    <t>6,81</t>
+  </si>
+  <si>
+    <t>10,44</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>18,22</t>
+  </si>
+  <si>
+    <t>0,64</t>
+  </si>
+  <si>
+    <t>5,72</t>
+  </si>
+  <si>
+    <t>38,14</t>
+  </si>
+  <si>
+    <t>16,27</t>
+  </si>
+  <si>
+    <t>0,3</t>
+  </si>
+  <si>
+    <t>5,5</t>
+  </si>
+  <si>
+    <t>0,25</t>
+  </si>
+  <si>
+    <t>0,8</t>
+  </si>
+  <si>
+    <t>0,55</t>
   </si>
   <si>
     <t>0,48</t>
   </si>
   <si>
-    <t>7,11</t>
-  </si>
-  <si>
-    <t>0,09</t>
-  </si>
-  <si>
-    <t>0,04</t>
-  </si>
-  <si>
-    <t>0,13</t>
-  </si>
-  <si>
-    <t>0,02</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>0,27</t>
-  </si>
-  <si>
-    <t>0,62</t>
-  </si>
-  <si>
-    <t>0,11</t>
-  </si>
-  <si>
-    <t>2,48</t>
-  </si>
-  <si>
-    <t>5,47</t>
-  </si>
-  <si>
-    <t>14,03</t>
-  </si>
-  <si>
-    <t>1801</t>
-  </si>
-  <si>
-    <t>LAMPUNG BARAT</t>
-  </si>
-  <si>
-    <t>0,18</t>
-  </si>
-  <si>
-    <t>22,15</t>
-  </si>
-  <si>
-    <t>1,43</t>
-  </si>
-  <si>
-    <t>4,97</t>
-  </si>
-  <si>
-    <t>38,13</t>
-  </si>
-  <si>
-    <t>2,51</t>
-  </si>
-  <si>
-    <t>0,61</t>
-  </si>
-  <si>
-    <t>4,06</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>0,14</t>
-  </si>
-  <si>
-    <t>0,24</t>
-  </si>
-  <si>
-    <t>0,34</t>
-  </si>
-  <si>
-    <t>0,06</t>
-  </si>
-  <si>
-    <t>11,17</t>
+    <t>4,75</t>
+  </si>
+  <si>
+    <t>7,41</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>23,83</t>
+  </si>
+  <si>
+    <t>0,42</t>
+  </si>
+  <si>
+    <t>2,75</t>
+  </si>
+  <si>
+    <t>27,1</t>
+  </si>
+  <si>
+    <t>15,24</t>
+  </si>
+  <si>
+    <t>0,16</t>
+  </si>
+  <si>
+    <t>5,63</t>
+  </si>
+  <si>
+    <t>0,19</t>
+  </si>
+  <si>
+    <t>0,26</t>
+  </si>
+  <si>
+    <t>0,65</t>
+  </si>
+  <si>
+    <t>7,52</t>
+  </si>
+  <si>
+    <t>13,4</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>28,13</t>
+  </si>
+  <si>
+    <t>0,79</t>
+  </si>
+  <si>
+    <t>0,72</t>
+  </si>
+  <si>
+    <t>27,46</t>
   </si>
   <si>
     <t>3,62</t>
   </si>
   <si>
-    <t>9,96</t>
-  </si>
-  <si>
-    <t>1802</t>
-  </si>
-  <si>
-    <t>TANGGAMUS</t>
-  </si>
-  <si>
-    <t>12,63</t>
-  </si>
-  <si>
-    <t>0,46</t>
-  </si>
-  <si>
-    <t>21,35</t>
-  </si>
-  <si>
-    <t>29,97</t>
+    <t>6,23</t>
+  </si>
+  <si>
+    <t>9,46</t>
+  </si>
+  <si>
+    <t>19,35</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>17,68</t>
+  </si>
+  <si>
+    <t>2,43</t>
+  </si>
+  <si>
+    <t>28,55</t>
+  </si>
+  <si>
+    <t>3,1</t>
+  </si>
+  <si>
+    <t>4,47</t>
+  </si>
+  <si>
+    <t>0,43</t>
   </si>
   <si>
     <t>5,29</t>
   </si>
   <si>
-    <t>0,07</t>
-  </si>
-  <si>
-    <t>0,5</t>
-  </si>
-  <si>
-    <t>0,29</t>
-  </si>
-  <si>
-    <t>5,44</t>
-  </si>
-  <si>
-    <t>18,24</t>
-  </si>
-  <si>
-    <t>1803</t>
-  </si>
-  <si>
-    <t>LAMPUNG SELATAN</t>
-  </si>
-  <si>
-    <t>17,17</t>
-  </si>
-  <si>
-    <t>2,69</t>
-  </si>
-  <si>
-    <t>40,47</t>
-  </si>
-  <si>
-    <t>14,72</t>
-  </si>
-  <si>
-    <t>9,36</t>
-  </si>
-  <si>
-    <t>0,33</t>
-  </si>
-  <si>
-    <t>0,01</t>
-  </si>
-  <si>
-    <t>0,77</t>
-  </si>
-  <si>
-    <t>1,12</t>
-  </si>
-  <si>
-    <t>0,03</t>
-  </si>
-  <si>
-    <t>4,33</t>
-  </si>
-  <si>
-    <t>8,58</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>0,32</t>
-  </si>
-  <si>
-    <t>18,94</t>
-  </si>
-  <si>
-    <t>0,38</t>
-  </si>
-  <si>
-    <t>16,21</t>
-  </si>
-  <si>
-    <t>26,56</t>
-  </si>
-  <si>
-    <t>9,73</t>
-  </si>
-  <si>
-    <t>1,21</t>
-  </si>
-  <si>
-    <t>5,9</t>
-  </si>
-  <si>
-    <t>0,05</t>
-  </si>
-  <si>
-    <t>0,45</t>
-  </si>
-  <si>
-    <t>0,15</t>
-  </si>
-  <si>
-    <t>2,64</t>
-  </si>
-  <si>
-    <t>14,43</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>15,42</t>
-  </si>
-  <si>
-    <t>2,5</t>
-  </si>
-  <si>
-    <t>1,22</t>
-  </si>
-  <si>
-    <t>44,8</t>
-  </si>
-  <si>
-    <t>5,08</t>
-  </si>
-  <si>
-    <t>0,92</t>
-  </si>
-  <si>
-    <t>12,92</t>
-  </si>
-  <si>
-    <t>0,68</t>
-  </si>
-  <si>
-    <t>0,72</t>
-  </si>
-  <si>
-    <t>3,22</t>
-  </si>
-  <si>
-    <t>11,48</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>18,69</t>
-  </si>
-  <si>
-    <t>0,79</t>
-  </si>
-  <si>
-    <t>1,5</t>
-  </si>
-  <si>
-    <t>36,71</t>
-  </si>
-  <si>
-    <t>14,21</t>
-  </si>
-  <si>
-    <t>7,85</t>
-  </si>
-  <si>
-    <t>0,59</t>
-  </si>
-  <si>
-    <t>1,11</t>
-  </si>
-  <si>
-    <t>6,83</t>
-  </si>
-  <si>
-    <t>10,48</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>18,09</t>
-  </si>
-  <si>
-    <t>0,65</t>
-  </si>
-  <si>
-    <t>5,89</t>
-  </si>
-  <si>
-    <t>38,09</t>
-  </si>
-  <si>
-    <t>16,17</t>
-  </si>
-  <si>
-    <t>0,3</t>
-  </si>
-  <si>
-    <t>0,25</t>
-  </si>
-  <si>
-    <t>0,81</t>
-  </si>
-  <si>
-    <t>0,53</t>
-  </si>
-  <si>
-    <t>4,74</t>
-  </si>
-  <si>
-    <t>7,51</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>24,01</t>
-  </si>
-  <si>
-    <t>0,42</t>
-  </si>
-  <si>
-    <t>2,61</t>
-  </si>
-  <si>
-    <t>27</t>
-  </si>
-  <si>
-    <t>15,16</t>
-  </si>
-  <si>
-    <t>0,16</t>
-  </si>
-  <si>
-    <t>5,65</t>
-  </si>
-  <si>
-    <t>0,19</t>
-  </si>
-  <si>
-    <t>0,26</t>
+    <t>8,06</t>
+  </si>
+  <si>
+    <t>27,56</t>
+  </si>
+  <si>
+    <t>1811</t>
+  </si>
+  <si>
+    <t>MESUJI</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>7,36</t>
+  </si>
+  <si>
+    <t>3,08</t>
+  </si>
+  <si>
+    <t>26,67</t>
+  </si>
+  <si>
+    <t>6,99</t>
+  </si>
+  <si>
+    <t>0,36</t>
+  </si>
+  <si>
+    <t>3,41</t>
+  </si>
+  <si>
+    <t>0,2</t>
   </si>
   <si>
     <t>0,66</t>
   </si>
   <si>
-    <t>2,42</t>
-  </si>
-  <si>
-    <t>7,58</t>
-  </si>
-  <si>
-    <t>13,51</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>28,19</t>
-  </si>
-  <si>
-    <t>0,8</t>
-  </si>
-  <si>
-    <t>0,83</t>
-  </si>
-  <si>
-    <t>27,39</t>
-  </si>
-  <si>
-    <t>3,48</t>
-  </si>
-  <si>
-    <t>6,18</t>
-  </si>
-  <si>
-    <t>2,47</t>
-  </si>
-  <si>
-    <t>9,47</t>
-  </si>
-  <si>
-    <t>19,45</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>17,47</t>
-  </si>
-  <si>
-    <t>0,51</t>
-  </si>
-  <si>
-    <t>2,67</t>
-  </si>
-  <si>
-    <t>28,18</t>
-  </si>
-  <si>
-    <t>3,13</t>
-  </si>
-  <si>
-    <t>4,49</t>
-  </si>
-  <si>
-    <t>0,44</t>
-  </si>
-  <si>
-    <t>5,76</t>
-  </si>
-  <si>
-    <t>7,82</t>
-  </si>
-  <si>
-    <t>27,53</t>
-  </si>
-  <si>
-    <t>1811</t>
-  </si>
-  <si>
-    <t>MESUJI</t>
-  </si>
-  <si>
-    <t>29,98</t>
-  </si>
-  <si>
-    <t>7,39</t>
-  </si>
-  <si>
-    <t>3,31</t>
-  </si>
-  <si>
-    <t>26,18</t>
-  </si>
-  <si>
-    <t>7,24</t>
-  </si>
-  <si>
-    <t>0,36</t>
-  </si>
-  <si>
-    <t>3,41</t>
-  </si>
-  <si>
-    <t>0,2</t>
-  </si>
-  <si>
     <t>4,77</t>
   </si>
   <si>
-    <t>9,41</t>
+    <t>9,43</t>
   </si>
   <si>
     <t>6,3</t>
@@ -841,31 +844,34 @@
     <t>TULANG BAWANG BARAT</t>
   </si>
   <si>
-    <t>16,98</t>
-  </si>
-  <si>
-    <t>2,33</t>
-  </si>
-  <si>
-    <t>10,76</t>
-  </si>
-  <si>
-    <t>23,23</t>
-  </si>
-  <si>
-    <t>14,08</t>
-  </si>
-  <si>
-    <t>5,25</t>
-  </si>
-  <si>
-    <t>3,67</t>
-  </si>
-  <si>
-    <t>3,38</t>
-  </si>
-  <si>
-    <t>18,5</t>
+    <t>16,83</t>
+  </si>
+  <si>
+    <t>2,06</t>
+  </si>
+  <si>
+    <t>10,05</t>
+  </si>
+  <si>
+    <t>24,85</t>
+  </si>
+  <si>
+    <t>13,16</t>
+  </si>
+  <si>
+    <t>0,78</t>
+  </si>
+  <si>
+    <t>5,17</t>
+  </si>
+  <si>
+    <t>2,79</t>
+  </si>
+  <si>
+    <t>3,49</t>
+  </si>
+  <si>
+    <t>19,83</t>
   </si>
   <si>
     <t>1813</t>
@@ -874,19 +880,19 @@
     <t>PESISIR BARAT</t>
   </si>
   <si>
-    <t>13,28</t>
-  </si>
-  <si>
-    <t>0,17</t>
-  </si>
-  <si>
-    <t>36,25</t>
-  </si>
-  <si>
-    <t>20,56</t>
-  </si>
-  <si>
-    <t>9</t>
+    <t>13,36</t>
+  </si>
+  <si>
+    <t>0,56</t>
+  </si>
+  <si>
+    <t>36,47</t>
+  </si>
+  <si>
+    <t>20,36</t>
+  </si>
+  <si>
+    <t>8,98</t>
   </si>
   <si>
     <t>0,22</t>
@@ -895,10 +901,13 @@
     <t>0,69</t>
   </si>
   <si>
-    <t>7,57</t>
-  </si>
-  <si>
-    <t>10,97</t>
+    <t>0,49</t>
+  </si>
+  <si>
+    <t>7,59</t>
+  </si>
+  <si>
+    <t>10,85</t>
   </si>
   <si>
     <t>1871</t>
@@ -907,22 +916,22 @@
     <t>BANDAR LAMPUNG</t>
   </si>
   <si>
-    <t>15,73</t>
+    <t>15,72</t>
   </si>
   <si>
     <t>0,6</t>
   </si>
   <si>
-    <t>3,71</t>
-  </si>
-  <si>
-    <t>30,26</t>
-  </si>
-  <si>
-    <t>4,81</t>
-  </si>
-  <si>
-    <t>16,33</t>
+    <t>3,7</t>
+  </si>
+  <si>
+    <t>30,33</t>
+  </si>
+  <si>
+    <t>4,8</t>
+  </si>
+  <si>
+    <t>16,32</t>
   </si>
   <si>
     <t>0,9</t>
@@ -934,10 +943,10 @@
     <t>0,4</t>
   </si>
   <si>
-    <t>4,61</t>
-  </si>
-  <si>
-    <t>18,34</t>
+    <t>4,6</t>
+  </si>
+  <si>
+    <t>18,32</t>
   </si>
   <si>
     <t>1872</t>
@@ -946,34 +955,25 @@
     <t>METRO</t>
   </si>
   <si>
-    <t>16,5</t>
-  </si>
-  <si>
-    <t>6,78</t>
-  </si>
-  <si>
-    <t>0,7</t>
-  </si>
-  <si>
-    <t>27,09</t>
-  </si>
-  <si>
-    <t>4,46</t>
-  </si>
-  <si>
-    <t>0,31</t>
-  </si>
-  <si>
-    <t>2,93</t>
-  </si>
-  <si>
-    <t>2,14</t>
-  </si>
-  <si>
-    <t>3,68</t>
-  </si>
-  <si>
-    <t>33,61</t>
+    <t>16,55</t>
+  </si>
+  <si>
+    <t>6,43</t>
+  </si>
+  <si>
+    <t>28,77</t>
+  </si>
+  <si>
+    <t>3,32</t>
+  </si>
+  <si>
+    <t>0,67</t>
+  </si>
+  <si>
+    <t>4,03</t>
+  </si>
+  <si>
+    <t>34,1</t>
   </si>
   <si>
     <t/>
@@ -1953,52 +1953,52 @@
         <v>105</v>
       </c>
       <c r="C6" s="6">
-        <v>92539</v>
+        <v>94715</v>
       </c>
       <c r="D6" s="6">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>106</v>
       </c>
       <c r="F6" s="6">
-        <v>18071</v>
+        <v>18681</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>107</v>
       </c>
       <c r="H6" s="6">
-        <v>1619</v>
+        <v>1603</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>108</v>
       </c>
       <c r="J6" s="6">
-        <v>4342</v>
+        <v>4217</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>109</v>
       </c>
       <c r="L6" s="6">
-        <v>29995</v>
+        <v>31106</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>110</v>
       </c>
       <c r="N6" s="6">
-        <v>9571</v>
+        <v>9764</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>111</v>
       </c>
       <c r="P6" s="6">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="Q6" s="7" t="s">
         <v>112</v>
       </c>
       <c r="R6" s="6">
-        <v>6582</v>
+        <v>6716</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>113</v>
@@ -2010,31 +2010,31 @@
         <v>114</v>
       </c>
       <c r="V6" s="6">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="W6" s="7" t="s">
         <v>115</v>
       </c>
       <c r="X6" s="6">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="Y6" s="7" t="s">
         <v>116</v>
       </c>
       <c r="Z6" s="6">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="AA6" s="7" t="s">
         <v>117</v>
       </c>
       <c r="AB6" s="6">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AC6" s="7" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AD6" s="6">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AE6" s="7" t="s">
         <v>106</v>
@@ -2043,19 +2043,19 @@
         <v>1</v>
       </c>
       <c r="AG6" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="AH6" s="6">
+        <v>36</v>
+      </c>
+      <c r="AI6" s="7" t="s">
         <v>118</v>
-      </c>
-      <c r="AH6" s="6">
-        <v>35</v>
-      </c>
-      <c r="AI6" s="7" t="s">
-        <v>115</v>
       </c>
       <c r="AJ6" s="6">
         <v>253</v>
       </c>
       <c r="AK6" s="7" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AL6" s="6">
         <v>33</v>
@@ -2064,117 +2064,117 @@
         <v>115</v>
       </c>
       <c r="AN6" s="6">
+        <v>121</v>
+      </c>
+      <c r="AO6" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="AP6" s="6">
+        <v>583</v>
+      </c>
+      <c r="AQ6" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="AR6" s="6">
+        <v>104</v>
+      </c>
+      <c r="AS6" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="AT6" s="6">
+        <v>2216</v>
+      </c>
+      <c r="AU6" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="AO6" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="AP6" s="6">
-        <v>574</v>
-      </c>
-      <c r="AQ6" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="AR6" s="6">
-        <v>103</v>
-      </c>
-      <c r="AS6" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="AT6" s="6">
-        <v>2297</v>
-      </c>
-      <c r="AU6" s="7" t="s">
-        <v>122</v>
-      </c>
       <c r="AV6" s="6">
-        <v>5065</v>
+        <v>5158</v>
       </c>
       <c r="AW6" s="7" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="AX6" s="6">
-        <v>12982</v>
+        <v>13229</v>
       </c>
       <c r="AY6" s="7" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C7" s="9">
-        <v>5051</v>
+        <v>5086</v>
       </c>
       <c r="D7" s="9">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="F7" s="9">
         <v>1119</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H7" s="9">
         <v>72</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="J7" s="9">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="L7" s="9">
-        <v>1926</v>
+        <v>1961</v>
       </c>
       <c r="M7" s="10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="N7" s="9">
         <v>127</v>
       </c>
       <c r="O7" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="P7" s="9">
         <v>31</v>
       </c>
       <c r="Q7" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="R7" s="9">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="S7" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="T7" s="9">
         <v>0</v>
       </c>
       <c r="U7" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="V7" s="9">
         <v>2</v>
       </c>
       <c r="W7" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="X7" s="9">
         <v>6</v>
       </c>
       <c r="Y7" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Z7" s="9">
         <v>1</v>
@@ -2186,37 +2186,37 @@
         <v>6</v>
       </c>
       <c r="AC7" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AD7" s="9">
         <v>5</v>
       </c>
       <c r="AE7" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="AF7" s="9">
         <v>0</v>
       </c>
       <c r="AG7" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH7" s="9">
         <v>2</v>
       </c>
       <c r="AI7" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AJ7" s="9">
         <v>7</v>
       </c>
       <c r="AK7" s="10" t="s">
-        <v>137</v>
+        <v>116</v>
       </c>
       <c r="AL7" s="9">
         <v>0</v>
       </c>
       <c r="AM7" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AN7" s="9">
         <v>12</v>
@@ -2263,16 +2263,16 @@
         <v>145</v>
       </c>
       <c r="C8" s="9">
-        <v>2796</v>
+        <v>2804</v>
       </c>
       <c r="D8" s="9">
         <v>0</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F8" s="9">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>146</v>
@@ -2284,273 +2284,273 @@
         <v>147</v>
       </c>
       <c r="J8" s="9">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="L8" s="9">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="N8" s="9">
-        <v>838</v>
+        <v>842</v>
       </c>
       <c r="O8" s="10" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="P8" s="9">
         <v>0</v>
       </c>
       <c r="Q8" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="R8" s="9">
         <v>148</v>
       </c>
       <c r="S8" s="10" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="T8" s="9">
         <v>0</v>
       </c>
       <c r="U8" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="V8" s="9">
         <v>0</v>
       </c>
       <c r="W8" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="X8" s="9">
         <v>2</v>
       </c>
       <c r="Y8" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="Z8" s="9">
         <v>0</v>
       </c>
       <c r="AA8" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AB8" s="9">
         <v>0</v>
       </c>
       <c r="AC8" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AD8" s="9">
         <v>1</v>
       </c>
       <c r="AE8" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AF8" s="9">
         <v>0</v>
       </c>
       <c r="AG8" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH8" s="9">
         <v>0</v>
       </c>
       <c r="AI8" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AJ8" s="9">
         <v>5</v>
       </c>
       <c r="AK8" s="10" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="AL8" s="9">
         <v>0</v>
       </c>
       <c r="AM8" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AN8" s="9">
         <v>0</v>
       </c>
       <c r="AO8" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AP8" s="9">
         <v>14</v>
       </c>
       <c r="AQ8" s="10" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="AR8" s="9">
         <v>2</v>
       </c>
       <c r="AS8" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AT8" s="9">
         <v>8</v>
       </c>
       <c r="AU8" s="10" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="AV8" s="9">
         <v>152</v>
       </c>
       <c r="AW8" s="10" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="AX8" s="9">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="AY8" s="10" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C9" s="9">
-        <v>7683</v>
+        <v>7732</v>
       </c>
       <c r="D9" s="9">
         <v>0</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F9" s="9">
-        <v>1319</v>
+        <v>1333</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H9" s="9">
         <v>207</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J9" s="9">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>114</v>
+        <v>136</v>
       </c>
       <c r="L9" s="9">
-        <v>3109</v>
+        <v>3140</v>
       </c>
       <c r="M9" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="N9" s="9">
         <v>1131</v>
       </c>
       <c r="O9" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="P9" s="9">
         <v>0</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="R9" s="9">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="S9" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T9" s="9">
         <v>8</v>
       </c>
       <c r="U9" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="V9" s="9">
         <v>0</v>
       </c>
       <c r="W9" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="X9" s="9">
         <v>25</v>
       </c>
       <c r="Y9" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="Z9" s="9">
         <v>0</v>
       </c>
       <c r="AA9" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AB9" s="9">
         <v>0</v>
       </c>
       <c r="AC9" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AD9" s="9">
         <v>8</v>
       </c>
       <c r="AE9" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="AF9" s="9">
         <v>1</v>
       </c>
       <c r="AG9" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="AH9" s="9">
         <v>1</v>
       </c>
       <c r="AI9" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="AJ9" s="9">
         <v>59</v>
       </c>
       <c r="AK9" s="10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="AL9" s="9">
         <v>0</v>
       </c>
       <c r="AM9" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AN9" s="9">
         <v>1</v>
       </c>
       <c r="AO9" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="AP9" s="9">
         <v>86</v>
       </c>
       <c r="AQ9" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AR9" s="9">
         <v>2</v>
       </c>
       <c r="AS9" s="10" t="s">
-        <v>167</v>
+        <v>115</v>
       </c>
       <c r="AT9" s="9">
         <v>8</v>
       </c>
       <c r="AU9" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="AV9" s="9">
         <v>333</v>
@@ -2559,7 +2559,7 @@
         <v>168</v>
       </c>
       <c r="AX9" s="9">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="AY9" s="10" t="s">
         <v>169</v>
@@ -2573,16 +2573,16 @@
         <v>171</v>
       </c>
       <c r="C10" s="9">
-        <v>13010</v>
+        <v>14210</v>
       </c>
       <c r="D10" s="9">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>172</v>
       </c>
       <c r="F10" s="9">
-        <v>2464</v>
+        <v>2902</v>
       </c>
       <c r="G10" s="10" t="s">
         <v>173</v>
@@ -2594,31 +2594,31 @@
         <v>174</v>
       </c>
       <c r="J10" s="9">
-        <v>2109</v>
+        <v>2044</v>
       </c>
       <c r="K10" s="10" t="s">
         <v>175</v>
       </c>
       <c r="L10" s="9">
-        <v>3455</v>
+        <v>4007</v>
       </c>
       <c r="M10" s="10" t="s">
         <v>176</v>
       </c>
       <c r="N10" s="9">
-        <v>1266</v>
+        <v>1432</v>
       </c>
       <c r="O10" s="10" t="s">
         <v>177</v>
       </c>
       <c r="P10" s="9">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="Q10" s="10" t="s">
         <v>178</v>
       </c>
       <c r="R10" s="9">
-        <v>768</v>
+        <v>847</v>
       </c>
       <c r="S10" s="10" t="s">
         <v>179</v>
@@ -2627,168 +2627,168 @@
         <v>10</v>
       </c>
       <c r="U10" s="10" t="s">
-        <v>106</v>
+        <v>152</v>
       </c>
       <c r="V10" s="9">
         <v>9</v>
       </c>
       <c r="W10" s="10" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="X10" s="9">
         <v>10</v>
       </c>
       <c r="Y10" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="Z10" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA10" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="AB10" s="9">
+        <v>12</v>
+      </c>
+      <c r="AC10" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="Z10" s="9">
-        <v>0</v>
-      </c>
-      <c r="AA10" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="AB10" s="9">
-        <v>13</v>
-      </c>
-      <c r="AC10" s="10" t="s">
-        <v>136</v>
-      </c>
       <c r="AD10" s="9">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AE10" s="10" t="s">
-        <v>180</v>
+        <v>140</v>
       </c>
       <c r="AF10" s="9">
         <v>0</v>
       </c>
       <c r="AG10" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH10" s="9">
         <v>12</v>
       </c>
       <c r="AI10" s="10" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="AJ10" s="9">
         <v>10</v>
       </c>
       <c r="AK10" s="10" t="s">
-        <v>106</v>
+        <v>152</v>
       </c>
       <c r="AL10" s="9">
         <v>1</v>
       </c>
       <c r="AM10" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="AN10" s="9">
         <v>58</v>
       </c>
       <c r="AO10" s="10" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AP10" s="9">
         <v>19</v>
       </c>
       <c r="AQ10" s="10" t="s">
-        <v>182</v>
+        <v>121</v>
       </c>
       <c r="AR10" s="9">
         <v>5</v>
       </c>
       <c r="AS10" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AT10" s="9">
-        <v>343</v>
+        <v>352</v>
       </c>
       <c r="AU10" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="AV10" s="9">
+        <v>351</v>
+      </c>
+      <c r="AW10" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="AX10" s="9">
+        <v>1876</v>
+      </c>
+      <c r="AY10" s="10" t="s">
         <v>183</v>
-      </c>
-      <c r="AV10" s="9">
-        <v>327</v>
-      </c>
-      <c r="AW10" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="AX10" s="9">
-        <v>1877</v>
-      </c>
-      <c r="AY10" s="10" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>185</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="C11" s="9">
+        <v>12306</v>
+      </c>
+      <c r="D11" s="9">
+        <v>4</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="F11" s="9">
+        <v>1899</v>
+      </c>
+      <c r="G11" s="10" t="s">
         <v>186</v>
-      </c>
-      <c r="C11" s="9">
-        <v>12280</v>
-      </c>
-      <c r="D11" s="9">
-        <v>3</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="F11" s="9">
-        <v>1893</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>187</v>
       </c>
       <c r="H11" s="9">
         <v>307</v>
       </c>
       <c r="I11" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="J11" s="9">
+        <v>140</v>
+      </c>
+      <c r="K11" s="10" t="s">
         <v>188</v>
       </c>
-      <c r="J11" s="9">
-        <v>150</v>
-      </c>
-      <c r="K11" s="10" t="s">
+      <c r="L11" s="9">
+        <v>5524</v>
+      </c>
+      <c r="M11" s="10" t="s">
         <v>189</v>
-      </c>
-      <c r="L11" s="9">
-        <v>5502</v>
-      </c>
-      <c r="M11" s="10" t="s">
-        <v>190</v>
       </c>
       <c r="N11" s="9">
         <v>624</v>
       </c>
       <c r="O11" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="P11" s="9">
+        <v>114</v>
+      </c>
+      <c r="Q11" s="10" t="s">
         <v>191</v>
-      </c>
-      <c r="P11" s="9">
-        <v>113</v>
-      </c>
-      <c r="Q11" s="10" t="s">
-        <v>192</v>
       </c>
       <c r="R11" s="9">
         <v>1586</v>
       </c>
       <c r="S11" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="T11" s="9">
         <v>18</v>
       </c>
       <c r="U11" s="10" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="V11" s="9">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W11" s="10" t="s">
-        <v>115</v>
+        <v>194</v>
       </c>
       <c r="X11" s="9">
         <v>10</v>
@@ -2800,7 +2800,7 @@
         <v>5</v>
       </c>
       <c r="AA11" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AB11" s="9">
         <v>3</v>
@@ -2812,19 +2812,19 @@
         <v>22</v>
       </c>
       <c r="AE11" s="10" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="AF11" s="9">
         <v>0</v>
       </c>
       <c r="AG11" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH11" s="9">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AI11" s="10" t="s">
-        <v>115</v>
+        <v>194</v>
       </c>
       <c r="AJ11" s="9">
         <v>29</v>
@@ -2839,87 +2839,87 @@
         <v>117</v>
       </c>
       <c r="AN11" s="9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AO11" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AP11" s="9">
         <v>84</v>
       </c>
       <c r="AQ11" s="10" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AR11" s="9">
         <v>15</v>
       </c>
       <c r="AS11" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AT11" s="9">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AU11" s="10" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="AV11" s="9">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="AW11" s="10" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="AX11" s="9">
         <v>1410</v>
       </c>
       <c r="AY11" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C12" s="9">
-        <v>4933</v>
+        <v>4952</v>
       </c>
       <c r="D12" s="9">
         <v>0</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F12" s="9">
-        <v>922</v>
+        <v>925</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H12" s="9">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="J12" s="9">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="L12" s="9">
-        <v>1811</v>
+        <v>1818</v>
       </c>
       <c r="M12" s="10" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="N12" s="9">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="O12" s="10" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="P12" s="9">
         <v>3</v>
@@ -2931,13 +2931,13 @@
         <v>387</v>
       </c>
       <c r="S12" s="10" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="T12" s="9">
         <v>0</v>
       </c>
       <c r="U12" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="V12" s="9">
         <v>3</v>
@@ -2949,7 +2949,7 @@
         <v>6</v>
       </c>
       <c r="Y12" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Z12" s="9">
         <v>1</v>
@@ -2967,31 +2967,31 @@
         <v>9</v>
       </c>
       <c r="AE12" s="10" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="AF12" s="9">
         <v>0</v>
       </c>
       <c r="AG12" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH12" s="9">
         <v>2</v>
       </c>
       <c r="AI12" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AJ12" s="9">
         <v>29</v>
       </c>
       <c r="AK12" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AL12" s="9">
         <v>0</v>
       </c>
       <c r="AM12" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AN12" s="9">
         <v>4</v>
@@ -3003,7 +3003,7 @@
         <v>55</v>
       </c>
       <c r="AQ12" s="10" t="s">
-        <v>207</v>
+        <v>167</v>
       </c>
       <c r="AR12" s="9">
         <v>1</v>
@@ -3012,87 +3012,87 @@
         <v>117</v>
       </c>
       <c r="AT12" s="9">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="AU12" s="10" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="AV12" s="9">
         <v>337</v>
       </c>
       <c r="AW12" s="10" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AX12" s="9">
         <v>517</v>
       </c>
       <c r="AY12" s="10" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C13" s="9">
-        <v>4329</v>
+        <v>4402</v>
       </c>
       <c r="D13" s="9">
         <v>2</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>180</v>
+        <v>194</v>
       </c>
       <c r="F13" s="9">
-        <v>783</v>
+        <v>802</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H13" s="9">
         <v>28</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="J13" s="9">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="L13" s="9">
-        <v>1649</v>
+        <v>1679</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="N13" s="9">
-        <v>700</v>
+        <v>716</v>
       </c>
       <c r="O13" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="P13" s="9">
         <v>13</v>
       </c>
       <c r="Q13" s="10" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="R13" s="9">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="S13" s="10" t="s">
-        <v>123</v>
+        <v>219</v>
       </c>
       <c r="T13" s="9">
         <v>0</v>
       </c>
       <c r="U13" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="V13" s="9">
         <v>1</v>
@@ -3104,13 +3104,13 @@
         <v>3</v>
       </c>
       <c r="Y13" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="Z13" s="9">
         <v>0</v>
       </c>
       <c r="AA13" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AB13" s="9">
         <v>1</v>
@@ -3122,13 +3122,13 @@
         <v>6</v>
       </c>
       <c r="AE13" s="10" t="s">
-        <v>137</v>
+        <v>116</v>
       </c>
       <c r="AF13" s="9">
         <v>0</v>
       </c>
       <c r="AG13" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH13" s="9">
         <v>1</v>
@@ -3140,126 +3140,126 @@
         <v>28</v>
       </c>
       <c r="AK13" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AL13" s="9">
         <v>11</v>
       </c>
       <c r="AM13" s="10" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="AN13" s="9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AO13" s="10" t="s">
-        <v>151</v>
+        <v>194</v>
       </c>
       <c r="AP13" s="9">
         <v>35</v>
       </c>
       <c r="AQ13" s="10" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="AR13" s="9">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AS13" s="10" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="AT13" s="9">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="AU13" s="10" t="s">
-        <v>147</v>
+        <v>223</v>
       </c>
       <c r="AV13" s="9">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="AW13" s="10" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="AX13" s="9">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="AY13" s="10" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="C14" s="9">
-        <v>4248</v>
+        <v>4284</v>
       </c>
       <c r="D14" s="9">
         <v>0</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F14" s="9">
-        <v>1020</v>
+        <v>1021</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="H14" s="9">
         <v>18</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="J14" s="9">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="L14" s="9">
-        <v>1147</v>
+        <v>1161</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="N14" s="9">
-        <v>644</v>
+        <v>653</v>
       </c>
       <c r="O14" s="10" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="P14" s="9">
         <v>7</v>
       </c>
       <c r="Q14" s="10" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="R14" s="9">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="S14" s="10" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="T14" s="9">
         <v>2</v>
       </c>
       <c r="U14" s="10" t="s">
-        <v>180</v>
+        <v>194</v>
       </c>
       <c r="V14" s="9">
         <v>0</v>
       </c>
       <c r="W14" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="X14" s="9">
         <v>8</v>
       </c>
       <c r="Y14" s="10" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="Z14" s="9">
         <v>1</v>
@@ -3277,13 +3277,13 @@
         <v>5</v>
       </c>
       <c r="AE14" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AF14" s="9">
         <v>0</v>
       </c>
       <c r="AG14" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH14" s="9">
         <v>1</v>
@@ -3295,7 +3295,7 @@
         <v>11</v>
       </c>
       <c r="AK14" s="10" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="AL14" s="9">
         <v>1</v>
@@ -3307,13 +3307,13 @@
         <v>3</v>
       </c>
       <c r="AO14" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AP14" s="9">
         <v>28</v>
       </c>
       <c r="AQ14" s="10" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="AR14" s="9">
         <v>1</v>
@@ -3322,135 +3322,135 @@
         <v>117</v>
       </c>
       <c r="AT14" s="9">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="AU14" s="10" t="s">
-        <v>235</v>
+        <v>133</v>
       </c>
       <c r="AV14" s="9">
         <v>322</v>
       </c>
       <c r="AW14" s="10" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="AX14" s="9">
         <v>574</v>
       </c>
       <c r="AY14" s="10" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C15" s="9">
-        <v>10671</v>
+        <v>10730</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F15" s="9">
-        <v>3008</v>
+        <v>3018</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="H15" s="9">
         <v>85</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="J15" s="9">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="L15" s="9">
-        <v>2923</v>
+        <v>2946</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="N15" s="9">
-        <v>371</v>
+        <v>388</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="P15" s="9">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>116</v>
+        <v>136</v>
       </c>
       <c r="R15" s="9">
-        <v>660</v>
+        <v>669</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="T15" s="9">
         <v>45</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="V15" s="9">
         <v>3</v>
       </c>
       <c r="W15" s="10" t="s">
-        <v>167</v>
+        <v>115</v>
       </c>
       <c r="X15" s="9">
         <v>12</v>
       </c>
       <c r="Y15" s="10" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="Z15" s="9">
         <v>0</v>
       </c>
       <c r="AA15" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AB15" s="9">
         <v>0</v>
       </c>
       <c r="AC15" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AD15" s="9">
         <v>3</v>
       </c>
       <c r="AE15" s="10" t="s">
-        <v>167</v>
+        <v>115</v>
       </c>
       <c r="AF15" s="9">
         <v>0</v>
       </c>
       <c r="AG15" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH15" s="9">
         <v>1</v>
       </c>
       <c r="AI15" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="AJ15" s="9">
         <v>11</v>
       </c>
       <c r="AK15" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="AL15" s="9">
         <v>2</v>
@@ -3459,84 +3459,84 @@
         <v>117</v>
       </c>
       <c r="AN15" s="9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AO15" s="10" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="AP15" s="9">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AQ15" s="10" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="AR15" s="9">
         <v>17</v>
       </c>
       <c r="AS15" s="10" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="AT15" s="9">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="AU15" s="10" t="s">
-        <v>246</v>
+        <v>187</v>
       </c>
       <c r="AV15" s="9">
-        <v>1011</v>
+        <v>1015</v>
       </c>
       <c r="AW15" s="10" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="AX15" s="9">
         <v>2076</v>
       </c>
       <c r="AY15" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C16" s="9">
-        <v>4116</v>
+        <v>4231</v>
       </c>
       <c r="D16" s="9">
         <v>8</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="F16" s="9">
-        <v>719</v>
+        <v>748</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="H16" s="9">
         <v>21</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>252</v>
+        <v>154</v>
       </c>
       <c r="J16" s="9">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="K16" s="10" t="s">
         <v>253</v>
       </c>
       <c r="L16" s="9">
-        <v>1160</v>
+        <v>1208</v>
       </c>
       <c r="M16" s="10" t="s">
         <v>254</v>
       </c>
       <c r="N16" s="9">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="O16" s="10" t="s">
         <v>255</v>
@@ -3548,7 +3548,7 @@
         <v>139</v>
       </c>
       <c r="R16" s="9">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="S16" s="10" t="s">
         <v>256</v>
@@ -3557,31 +3557,31 @@
         <v>0</v>
       </c>
       <c r="U16" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="V16" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W16" s="10" t="s">
-        <v>180</v>
+        <v>117</v>
       </c>
       <c r="X16" s="9">
         <v>2</v>
       </c>
       <c r="Y16" s="10" t="s">
-        <v>180</v>
+        <v>194</v>
       </c>
       <c r="Z16" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA16" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AB16" s="9">
         <v>3</v>
       </c>
       <c r="AC16" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AD16" s="9">
         <v>1</v>
@@ -3593,7 +3593,7 @@
         <v>0</v>
       </c>
       <c r="AG16" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH16" s="9">
         <v>1</v>
@@ -3611,40 +3611,40 @@
         <v>8</v>
       </c>
       <c r="AM16" s="10" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="AN16" s="9">
         <v>6</v>
       </c>
       <c r="AO16" s="10" t="s">
-        <v>182</v>
+        <v>116</v>
       </c>
       <c r="AP16" s="9">
         <v>25</v>
       </c>
       <c r="AQ16" s="10" t="s">
-        <v>133</v>
+        <v>207</v>
       </c>
       <c r="AR16" s="9">
         <v>12</v>
       </c>
       <c r="AS16" s="10" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="AT16" s="9">
-        <v>237</v>
+        <v>224</v>
       </c>
       <c r="AU16" s="10" t="s">
         <v>258</v>
       </c>
       <c r="AV16" s="9">
-        <v>322</v>
+        <v>341</v>
       </c>
       <c r="AW16" s="10" t="s">
         <v>259</v>
       </c>
       <c r="AX16" s="9">
-        <v>1133</v>
+        <v>1166</v>
       </c>
       <c r="AY16" s="10" t="s">
         <v>260</v>
@@ -3658,40 +3658,40 @@
         <v>262</v>
       </c>
       <c r="C17" s="9">
-        <v>6034</v>
+        <v>6036</v>
       </c>
       <c r="D17" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F17" s="9">
-        <v>1809</v>
+        <v>1811</v>
       </c>
       <c r="G17" s="10" t="s">
         <v>263</v>
       </c>
       <c r="H17" s="9">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="I17" s="10" t="s">
         <v>264</v>
       </c>
       <c r="J17" s="9">
-        <v>200</v>
+        <v>186</v>
       </c>
       <c r="K17" s="10" t="s">
         <v>265</v>
       </c>
       <c r="L17" s="9">
-        <v>1580</v>
+        <v>1610</v>
       </c>
       <c r="M17" s="10" t="s">
         <v>266</v>
       </c>
       <c r="N17" s="9">
-        <v>437</v>
+        <v>422</v>
       </c>
       <c r="O17" s="10" t="s">
         <v>267</v>
@@ -3730,31 +3730,31 @@
         <v>2</v>
       </c>
       <c r="AA17" s="10" t="s">
-        <v>167</v>
+        <v>115</v>
       </c>
       <c r="AB17" s="9">
         <v>2</v>
       </c>
       <c r="AC17" s="10" t="s">
-        <v>167</v>
+        <v>115</v>
       </c>
       <c r="AD17" s="9">
         <v>4</v>
       </c>
       <c r="AE17" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AF17" s="9">
         <v>0</v>
       </c>
       <c r="AG17" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH17" s="9">
         <v>2</v>
       </c>
       <c r="AI17" s="10" t="s">
-        <v>167</v>
+        <v>115</v>
       </c>
       <c r="AJ17" s="9">
         <v>12</v>
@@ -3769,463 +3769,463 @@
         <v>106</v>
       </c>
       <c r="AN17" s="9">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AO17" s="10" t="s">
-        <v>182</v>
+        <v>136</v>
       </c>
       <c r="AP17" s="9">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="AQ17" s="10" t="s">
-        <v>213</v>
+        <v>271</v>
       </c>
       <c r="AR17" s="9">
         <v>11</v>
       </c>
       <c r="AS17" s="10" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="AT17" s="9">
         <v>288</v>
       </c>
       <c r="AU17" s="10" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="AV17" s="9">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="AW17" s="10" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="AX17" s="9">
         <v>380</v>
       </c>
       <c r="AY17" s="10" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C18" s="9">
-        <v>6896</v>
+        <v>7272</v>
       </c>
       <c r="D18" s="9">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>135</v>
+        <v>116</v>
       </c>
       <c r="F18" s="9">
-        <v>1171</v>
+        <v>1224</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="H18" s="9">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J18" s="9">
-        <v>742</v>
+        <v>731</v>
       </c>
       <c r="K18" s="10" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="L18" s="9">
-        <v>1602</v>
+        <v>1807</v>
       </c>
       <c r="M18" s="10" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="N18" s="9">
-        <v>971</v>
+        <v>957</v>
       </c>
       <c r="O18" s="10" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="P18" s="9">
         <v>57</v>
       </c>
       <c r="Q18" s="10" t="s">
-        <v>242</v>
+        <v>282</v>
       </c>
       <c r="R18" s="9">
-        <v>362</v>
+        <v>376</v>
       </c>
       <c r="S18" s="10" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="T18" s="9">
         <v>3</v>
       </c>
       <c r="U18" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="V18" s="9">
         <v>2</v>
       </c>
       <c r="W18" s="10" t="s">
-        <v>167</v>
+        <v>115</v>
       </c>
       <c r="X18" s="9">
         <v>3</v>
       </c>
       <c r="Y18" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="Z18" s="9">
         <v>0</v>
       </c>
       <c r="AA18" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AB18" s="9">
         <v>3</v>
       </c>
       <c r="AC18" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AD18" s="9">
         <v>1</v>
       </c>
       <c r="AE18" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="AF18" s="9">
         <v>0</v>
       </c>
       <c r="AG18" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH18" s="9">
         <v>6</v>
       </c>
       <c r="AI18" s="10" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="AJ18" s="9">
         <v>9</v>
       </c>
       <c r="AK18" s="10" t="s">
-        <v>116</v>
+        <v>136</v>
       </c>
       <c r="AL18" s="9">
         <v>0</v>
       </c>
       <c r="AM18" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AN18" s="9">
         <v>11</v>
       </c>
       <c r="AO18" s="10" t="s">
-        <v>230</v>
+        <v>193</v>
       </c>
       <c r="AP18" s="9">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AQ18" s="10" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="AR18" s="9">
         <v>5</v>
       </c>
       <c r="AS18" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AT18" s="9">
-        <v>253</v>
+        <v>203</v>
       </c>
       <c r="AU18" s="10" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="AV18" s="9">
-        <v>233</v>
+        <v>254</v>
       </c>
       <c r="AW18" s="10" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="AX18" s="9">
-        <v>1276</v>
+        <v>1442</v>
       </c>
       <c r="AY18" s="10" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C19" s="9">
-        <v>7209</v>
+        <v>7290</v>
       </c>
       <c r="D19" s="9">
         <v>1</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F19" s="9">
-        <v>957</v>
+        <v>974</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="H19" s="9">
         <v>12</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>288</v>
+        <v>233</v>
       </c>
       <c r="J19" s="9">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="K19" s="10" t="s">
-        <v>220</v>
+        <v>290</v>
       </c>
       <c r="L19" s="9">
-        <v>2613</v>
+        <v>2659</v>
       </c>
       <c r="M19" s="10" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="N19" s="9">
-        <v>1482</v>
+        <v>1484</v>
       </c>
       <c r="O19" s="10" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="P19" s="9">
         <v>0</v>
       </c>
       <c r="Q19" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="R19" s="9">
-        <v>649</v>
+        <v>655</v>
       </c>
       <c r="S19" s="10" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="T19" s="9">
         <v>0</v>
       </c>
       <c r="U19" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="V19" s="9">
         <v>1</v>
       </c>
       <c r="W19" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="X19" s="9">
         <v>12</v>
       </c>
       <c r="Y19" s="10" t="s">
-        <v>288</v>
+        <v>233</v>
       </c>
       <c r="Z19" s="9">
         <v>0</v>
       </c>
       <c r="AA19" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AB19" s="9">
         <v>0</v>
       </c>
       <c r="AC19" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AD19" s="9">
         <v>3</v>
       </c>
       <c r="AE19" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AF19" s="9">
         <v>0</v>
       </c>
       <c r="AG19" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH19" s="9">
         <v>0</v>
       </c>
       <c r="AI19" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AJ19" s="9">
         <v>16</v>
       </c>
       <c r="AK19" s="10" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="AL19" s="9">
         <v>0</v>
       </c>
       <c r="AM19" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AN19" s="9">
         <v>1</v>
       </c>
       <c r="AO19" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="AP19" s="9">
         <v>50</v>
       </c>
       <c r="AQ19" s="10" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="AR19" s="9">
         <v>1</v>
       </c>
       <c r="AS19" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="AT19" s="9">
         <v>36</v>
       </c>
       <c r="AU19" s="10" t="s">
-        <v>152</v>
+        <v>296</v>
       </c>
       <c r="AV19" s="9">
-        <v>546</v>
+        <v>553</v>
       </c>
       <c r="AW19" s="10" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="AX19" s="9">
         <v>791</v>
       </c>
       <c r="AY19" s="10" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="C20" s="9">
-        <v>998</v>
+        <v>999</v>
       </c>
       <c r="D20" s="9">
         <v>1</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F20" s="9">
         <v>157</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="H20" s="9">
         <v>6</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="J20" s="9">
         <v>37</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="L20" s="9">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="M20" s="10" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="N20" s="9">
         <v>48</v>
       </c>
       <c r="O20" s="10" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="P20" s="9">
         <v>5</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="R20" s="9">
         <v>163</v>
       </c>
       <c r="S20" s="10" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="T20" s="9">
         <v>0</v>
       </c>
       <c r="U20" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="V20" s="9">
         <v>0</v>
       </c>
       <c r="W20" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="X20" s="9">
         <v>9</v>
       </c>
       <c r="Y20" s="10" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="Z20" s="9">
         <v>3</v>
       </c>
       <c r="AA20" s="10" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AB20" s="9">
         <v>0</v>
       </c>
       <c r="AC20" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AD20" s="9">
         <v>0</v>
       </c>
       <c r="AE20" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AF20" s="9">
         <v>0</v>
       </c>
       <c r="AG20" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH20" s="9">
         <v>1</v>
       </c>
       <c r="AI20" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="AJ20" s="9">
         <v>6</v>
       </c>
       <c r="AK20" s="10" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="AL20" s="9">
         <v>2</v>
@@ -4237,93 +4237,93 @@
         <v>1</v>
       </c>
       <c r="AO20" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="AP20" s="9">
         <v>18</v>
       </c>
       <c r="AQ20" s="10" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="AR20" s="9">
         <v>4</v>
       </c>
       <c r="AS20" s="10" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="AT20" s="9">
         <v>6</v>
       </c>
       <c r="AU20" s="10" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="AV20" s="9">
         <v>46</v>
       </c>
       <c r="AW20" s="10" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="AX20" s="9">
         <v>183</v>
       </c>
       <c r="AY20" s="10" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="C21" s="9">
-        <v>2285</v>
+        <v>2381</v>
       </c>
       <c r="D21" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>118</v>
       </c>
       <c r="F21" s="9">
-        <v>377</v>
+        <v>394</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="H21" s="9">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="J21" s="9">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="K21" s="10" t="s">
-        <v>313</v>
+        <v>118</v>
       </c>
       <c r="L21" s="9">
-        <v>619</v>
+        <v>685</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="N21" s="9">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>315</v>
+        <v>109</v>
       </c>
       <c r="P21" s="9">
         <v>7</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>316</v>
+        <v>155</v>
       </c>
       <c r="R21" s="9">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="S21" s="10" t="s">
         <v>317</v>
@@ -4332,94 +4332,94 @@
         <v>0</v>
       </c>
       <c r="U21" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="V21" s="9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="W21" s="10" t="s">
-        <v>292</v>
+        <v>119</v>
       </c>
       <c r="X21" s="9">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="Y21" s="10" t="s">
-        <v>112</v>
+        <v>318</v>
       </c>
       <c r="Z21" s="9">
         <v>2</v>
       </c>
       <c r="AA21" s="10" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="AB21" s="9">
         <v>0</v>
       </c>
       <c r="AC21" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AD21" s="9">
         <v>1</v>
       </c>
       <c r="AE21" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AF21" s="9">
         <v>0</v>
       </c>
       <c r="AG21" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH21" s="9">
         <v>0</v>
       </c>
       <c r="AI21" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AJ21" s="9">
         <v>3</v>
       </c>
       <c r="AK21" s="10" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="AL21" s="9">
         <v>0</v>
       </c>
       <c r="AM21" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AN21" s="9">
         <v>0</v>
       </c>
       <c r="AO21" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AP21" s="9">
         <v>18</v>
       </c>
       <c r="AQ21" s="10" t="s">
-        <v>201</v>
+        <v>166</v>
       </c>
       <c r="AR21" s="9">
         <v>1</v>
       </c>
       <c r="AS21" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AT21" s="9">
-        <v>49</v>
+        <v>6</v>
       </c>
       <c r="AU21" s="10" t="s">
-        <v>318</v>
+        <v>220</v>
       </c>
       <c r="AV21" s="9">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="AW21" s="10" t="s">
         <v>319</v>
       </c>
       <c r="AX21" s="9">
-        <v>768</v>
+        <v>812</v>
       </c>
       <c r="AY21" s="10" t="s">
         <v>320</v>
@@ -4433,52 +4433,52 @@
         <v>322</v>
       </c>
       <c r="C22" s="12">
-        <v>92539</v>
+        <v>94715</v>
       </c>
       <c r="D22" s="12">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>106</v>
       </c>
       <c r="F22" s="12">
-        <v>18071</v>
+        <v>18681</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>107</v>
       </c>
       <c r="H22" s="12">
-        <v>1619</v>
+        <v>1603</v>
       </c>
       <c r="I22" s="13" t="s">
         <v>108</v>
       </c>
       <c r="J22" s="12">
-        <v>4342</v>
+        <v>4217</v>
       </c>
       <c r="K22" s="13" t="s">
         <v>109</v>
       </c>
       <c r="L22" s="12">
-        <v>29995</v>
+        <v>31106</v>
       </c>
       <c r="M22" s="13" t="s">
         <v>110</v>
       </c>
       <c r="N22" s="12">
-        <v>9571</v>
+        <v>9764</v>
       </c>
       <c r="O22" s="13" t="s">
         <v>111</v>
       </c>
       <c r="P22" s="12">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="Q22" s="13" t="s">
         <v>112</v>
       </c>
       <c r="R22" s="12">
-        <v>6582</v>
+        <v>6716</v>
       </c>
       <c r="S22" s="13" t="s">
         <v>113</v>
@@ -4490,31 +4490,31 @@
         <v>114</v>
       </c>
       <c r="V22" s="12">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="W22" s="13" t="s">
         <v>115</v>
       </c>
       <c r="X22" s="12">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="Y22" s="13" t="s">
         <v>116</v>
       </c>
       <c r="Z22" s="12">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="AA22" s="13" t="s">
         <v>117</v>
       </c>
       <c r="AB22" s="12">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AC22" s="13" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AD22" s="12">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AE22" s="13" t="s">
         <v>106</v>
@@ -4523,19 +4523,19 @@
         <v>1</v>
       </c>
       <c r="AG22" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="AH22" s="12">
+        <v>36</v>
+      </c>
+      <c r="AI22" s="13" t="s">
         <v>118</v>
-      </c>
-      <c r="AH22" s="12">
-        <v>35</v>
-      </c>
-      <c r="AI22" s="13" t="s">
-        <v>115</v>
       </c>
       <c r="AJ22" s="12">
         <v>253</v>
       </c>
       <c r="AK22" s="13" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AL22" s="12">
         <v>33</v>
@@ -4544,40 +4544,40 @@
         <v>115</v>
       </c>
       <c r="AN22" s="12">
+        <v>121</v>
+      </c>
+      <c r="AO22" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="AP22" s="12">
+        <v>583</v>
+      </c>
+      <c r="AQ22" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="AR22" s="12">
+        <v>104</v>
+      </c>
+      <c r="AS22" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="AT22" s="12">
+        <v>2216</v>
+      </c>
+      <c r="AU22" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="AO22" s="13" t="s">
-        <v>116</v>
-      </c>
-      <c r="AP22" s="12">
-        <v>574</v>
-      </c>
-      <c r="AQ22" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="AR22" s="12">
-        <v>103</v>
-      </c>
-      <c r="AS22" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="AT22" s="12">
-        <v>2297</v>
-      </c>
-      <c r="AU22" s="13" t="s">
-        <v>122</v>
-      </c>
       <c r="AV22" s="12">
-        <v>5065</v>
+        <v>5158</v>
       </c>
       <c r="AW22" s="13" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="AX22" s="12">
-        <v>12982</v>
+        <v>13229</v>
       </c>
       <c r="AY22" s="13" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Perbarui data SE2026 28/08/2026 10:24:04,26
</commit_message>
<xml_diff>
--- a/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
+++ b/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="316">
   <si>
     <t>DATA RADAR ANOMALI USAHA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 27 Agu 2026, 12.59</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 28 Agu 2026, 10.22</t>
   </si>
   <si>
     <t>Kode</t>
@@ -331,460 +331,457 @@
     <t>LAMPUNG</t>
   </si>
   <si>
+    <t>0,07</t>
+  </si>
+  <si>
+    <t>19,76</t>
+  </si>
+  <si>
+    <t>1,6</t>
+  </si>
+  <si>
+    <t>3,65</t>
+  </si>
+  <si>
+    <t>33,89</t>
+  </si>
+  <si>
+    <t>10,54</t>
+  </si>
+  <si>
+    <t>0,39</t>
+  </si>
+  <si>
+    <t>7,18</t>
+  </si>
+  <si>
     <t>0,08</t>
   </si>
   <si>
-    <t>19,78</t>
-  </si>
-  <si>
-    <t>1,64</t>
-  </si>
-  <si>
-    <t>3,94</t>
-  </si>
-  <si>
-    <t>33,46</t>
-  </si>
-  <si>
-    <t>10,5</t>
+    <t>0,03</t>
+  </si>
+  <si>
+    <t>0,14</t>
+  </si>
+  <si>
+    <t>0,02</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>0,26</t>
+  </si>
+  <si>
+    <t>0,04</t>
+  </si>
+  <si>
+    <t>0,11</t>
+  </si>
+  <si>
+    <t>0,59</t>
+  </si>
+  <si>
+    <t>1,9</t>
+  </si>
+  <si>
+    <t>5,43</t>
+  </si>
+  <si>
+    <t>14,06</t>
+  </si>
+  <si>
+    <t>1801</t>
+  </si>
+  <si>
+    <t>LAMPUNG BARAT</t>
+  </si>
+  <si>
+    <t>22,08</t>
+  </si>
+  <si>
+    <t>1,34</t>
+  </si>
+  <si>
+    <t>4,85</t>
+  </si>
+  <si>
+    <t>38,68</t>
+  </si>
+  <si>
+    <t>2,5</t>
+  </si>
+  <si>
+    <t>4,09</t>
+  </si>
+  <si>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>0,2</t>
+  </si>
+  <si>
+    <t>0,33</t>
+  </si>
+  <si>
+    <t>0,06</t>
+  </si>
+  <si>
+    <t>11,02</t>
+  </si>
+  <si>
+    <t>3,69</t>
+  </si>
+  <si>
+    <t>9,86</t>
+  </si>
+  <si>
+    <t>1802</t>
+  </si>
+  <si>
+    <t>TANGGAMUS</t>
+  </si>
+  <si>
+    <t>13,58</t>
   </si>
   <si>
     <t>0,43</t>
   </si>
   <si>
-    <t>7,1</t>
+    <t>1,38</t>
+  </si>
+  <si>
+    <t>25,44</t>
+  </si>
+  <si>
+    <t>30,86</t>
+  </si>
+  <si>
+    <t>6,61</t>
   </si>
   <si>
     <t>0,09</t>
   </si>
   <si>
-    <t>0,03</t>
-  </si>
-  <si>
-    <t>0,14</t>
-  </si>
-  <si>
-    <t>0,02</t>
-  </si>
-  <si>
-    <t>0,04</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>0,26</t>
-  </si>
-  <si>
-    <t>0,12</t>
+    <t>0,15</t>
+  </si>
+  <si>
+    <t>0,18</t>
+  </si>
+  <si>
+    <t>4,74</t>
+  </si>
+  <si>
+    <t>16,02</t>
+  </si>
+  <si>
+    <t>1803</t>
+  </si>
+  <si>
+    <t>LAMPUNG SELATAN</t>
+  </si>
+  <si>
+    <t>17,22</t>
+  </si>
+  <si>
+    <t>2,55</t>
+  </si>
+  <si>
+    <t>0,05</t>
+  </si>
+  <si>
+    <t>41,25</t>
+  </si>
+  <si>
+    <t>14,04</t>
+  </si>
+  <si>
+    <t>0,01</t>
+  </si>
+  <si>
+    <t>9,69</t>
+  </si>
+  <si>
+    <t>0,75</t>
+  </si>
+  <si>
+    <t>1,09</t>
+  </si>
+  <si>
+    <t>4,26</t>
+  </si>
+  <si>
+    <t>8,38</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>0,25</t>
+  </si>
+  <si>
+    <t>21,39</t>
+  </si>
+  <si>
+    <t>0,32</t>
+  </si>
+  <si>
+    <t>12,38</t>
+  </si>
+  <si>
+    <t>28,83</t>
+  </si>
+  <si>
+    <t>11,96</t>
+  </si>
+  <si>
+    <t>0,97</t>
+  </si>
+  <si>
+    <t>5,93</t>
+  </si>
+  <si>
+    <t>0,36</t>
+  </si>
+  <si>
+    <t>2,4</t>
+  </si>
+  <si>
+    <t>2,38</t>
+  </si>
+  <si>
+    <t>12,19</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>15,51</t>
+  </si>
+  <si>
+    <t>2,41</t>
+  </si>
+  <si>
+    <t>1,17</t>
+  </si>
+  <si>
+    <t>45,06</t>
+  </si>
+  <si>
+    <t>5,03</t>
+  </si>
+  <si>
+    <t>0,8</t>
+  </si>
+  <si>
+    <t>12,86</t>
+  </si>
+  <si>
+    <t>0,23</t>
+  </si>
+  <si>
+    <t>0,68</t>
+  </si>
+  <si>
+    <t>0,67</t>
+  </si>
+  <si>
+    <t>3,26</t>
+  </si>
+  <si>
+    <t>11,48</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>18,73</t>
+  </si>
+  <si>
+    <t>1,25</t>
+  </si>
+  <si>
+    <t>36,94</t>
+  </si>
+  <si>
+    <t>14,34</t>
+  </si>
+  <si>
+    <t>7,86</t>
+  </si>
+  <si>
+    <t>0,58</t>
+  </si>
+  <si>
+    <t>0,62</t>
+  </si>
+  <si>
+    <t>6,77</t>
+  </si>
+  <si>
+    <t>10,39</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>18,41</t>
+  </si>
+  <si>
+    <t>0,63</t>
+  </si>
+  <si>
+    <t>4,4</t>
+  </si>
+  <si>
+    <t>39,02</t>
+  </si>
+  <si>
+    <t>16,78</t>
+  </si>
+  <si>
+    <t>0,29</t>
+  </si>
+  <si>
+    <t>5,5</t>
+  </si>
+  <si>
+    <t>0,13</t>
+  </si>
+  <si>
+    <t>0,76</t>
+  </si>
+  <si>
+    <t>0,54</t>
+  </si>
+  <si>
+    <t>0,31</t>
+  </si>
+  <si>
+    <t>4,72</t>
+  </si>
+  <si>
+    <t>7,46</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>23,56</t>
+  </si>
+  <si>
+    <t>0,41</t>
+  </si>
+  <si>
+    <t>2,71</t>
+  </si>
+  <si>
+    <t>27,12</t>
+  </si>
+  <si>
+    <t>15,69</t>
+  </si>
+  <si>
+    <t>5,67</t>
+  </si>
+  <si>
+    <t>0,64</t>
+  </si>
+  <si>
+    <t>2,39</t>
+  </si>
+  <si>
+    <t>7,41</t>
+  </si>
+  <si>
+    <t>13,42</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>27,5</t>
+  </si>
+  <si>
+    <t>0,45</t>
+  </si>
+  <si>
+    <t>28,97</t>
+  </si>
+  <si>
+    <t>3,54</t>
+  </si>
+  <si>
+    <t>6,18</t>
+  </si>
+  <si>
+    <t>0,37</t>
+  </si>
+  <si>
+    <t>0,16</t>
+  </si>
+  <si>
+    <t>8,89</t>
+  </si>
+  <si>
+    <t>21,44</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>17,81</t>
+  </si>
+  <si>
+    <t>0,46</t>
+  </si>
+  <si>
+    <t>1,46</t>
+  </si>
+  <si>
+    <t>30,95</t>
+  </si>
+  <si>
+    <t>3,09</t>
+  </si>
+  <si>
+    <t>0,44</t>
   </si>
   <si>
     <t>0,6</t>
   </si>
   <si>
-    <t>0,11</t>
-  </si>
-  <si>
-    <t>2,25</t>
-  </si>
-  <si>
-    <t>5,48</t>
-  </si>
-  <si>
-    <t>13,78</t>
-  </si>
-  <si>
-    <t>1801</t>
-  </si>
-  <si>
-    <t>LAMPUNG BARAT</t>
-  </si>
-  <si>
-    <t>22,12</t>
-  </si>
-  <si>
-    <t>1,34</t>
-  </si>
-  <si>
-    <t>4,9</t>
-  </si>
-  <si>
-    <t>38,58</t>
-  </si>
-  <si>
-    <t>2,5</t>
-  </si>
-  <si>
-    <t>0,59</t>
-  </si>
-  <si>
-    <t>4,09</t>
-  </si>
-  <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>0,24</t>
-  </si>
-  <si>
-    <t>0,33</t>
-  </si>
-  <si>
-    <t>0,06</t>
-  </si>
-  <si>
-    <t>11,09</t>
-  </si>
-  <si>
-    <t>3,7</t>
-  </si>
-  <si>
-    <t>9,77</t>
-  </si>
-  <si>
-    <t>1802</t>
-  </si>
-  <si>
-    <t>TANGGAMUS</t>
-  </si>
-  <si>
-    <t>13,62</t>
-  </si>
-  <si>
-    <t>1,46</t>
-  </si>
-  <si>
-    <t>25,39</t>
-  </si>
-  <si>
-    <t>30,81</t>
-  </si>
-  <si>
-    <t>6,64</t>
-  </si>
-  <si>
-    <t>0,15</t>
-  </si>
-  <si>
-    <t>0,18</t>
-  </si>
-  <si>
-    <t>4,72</t>
-  </si>
-  <si>
-    <t>15,97</t>
-  </si>
-  <si>
-    <t>1803</t>
-  </si>
-  <si>
-    <t>LAMPUNG SELATAN</t>
-  </si>
-  <si>
-    <t>17,22</t>
-  </si>
-  <si>
-    <t>2,67</t>
-  </si>
-  <si>
-    <t>0,05</t>
-  </si>
-  <si>
-    <t>40,69</t>
-  </si>
-  <si>
-    <t>14,64</t>
-  </si>
-  <si>
-    <t>0,01</t>
-  </si>
-  <si>
-    <t>9,29</t>
-  </si>
-  <si>
-    <t>0,32</t>
-  </si>
-  <si>
-    <t>0,76</t>
-  </si>
-  <si>
-    <t>1,11</t>
-  </si>
-  <si>
-    <t>0,13</t>
-  </si>
-  <si>
-    <t>4,33</t>
-  </si>
-  <si>
-    <t>8,5</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>21,17</t>
-  </si>
-  <si>
-    <t>13,34</t>
-  </si>
-  <si>
-    <t>28,63</t>
-  </si>
-  <si>
-    <t>10,78</t>
-  </si>
-  <si>
-    <t>1,03</t>
-  </si>
-  <si>
-    <t>5,79</t>
-  </si>
-  <si>
-    <t>0,07</t>
-  </si>
-  <si>
-    <t>0,38</t>
-  </si>
-  <si>
-    <t>2,48</t>
-  </si>
-  <si>
-    <t>2,44</t>
-  </si>
-  <si>
-    <t>12,7</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>15,47</t>
-  </si>
-  <si>
-    <t>2,42</t>
-  </si>
-  <si>
-    <t>1,17</t>
-  </si>
-  <si>
-    <t>44,95</t>
-  </si>
-  <si>
-    <t>5,04</t>
-  </si>
-  <si>
-    <t>0,93</t>
-  </si>
-  <si>
-    <t>12,87</t>
-  </si>
-  <si>
-    <t>0,23</t>
-  </si>
-  <si>
-    <t>0,68</t>
-  </si>
-  <si>
-    <t>0,73</t>
-  </si>
-  <si>
-    <t>3,25</t>
-  </si>
-  <si>
-    <t>11,41</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>18,7</t>
-  </si>
-  <si>
-    <t>1,54</t>
-  </si>
-  <si>
-    <t>36,87</t>
-  </si>
-  <si>
-    <t>14,06</t>
-  </si>
-  <si>
-    <t>7,94</t>
-  </si>
-  <si>
-    <t>0,58</t>
-  </si>
-  <si>
-    <t>1,1</t>
-  </si>
-  <si>
-    <t>6,8</t>
-  </si>
-  <si>
-    <t>10,43</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>18,29</t>
-  </si>
-  <si>
-    <t>0,63</t>
-  </si>
-  <si>
-    <t>5,26</t>
-  </si>
-  <si>
-    <t>38,42</t>
-  </si>
-  <si>
-    <t>16,51</t>
-  </si>
-  <si>
-    <t>0,29</t>
-  </si>
-  <si>
-    <t>5,53</t>
-  </si>
-  <si>
-    <t>0,25</t>
-  </si>
-  <si>
-    <t>0,79</t>
-  </si>
-  <si>
-    <t>0,54</t>
-  </si>
-  <si>
-    <t>4,76</t>
-  </si>
-  <si>
-    <t>7,4</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>23,63</t>
-  </si>
-  <si>
-    <t>0,41</t>
-  </si>
-  <si>
-    <t>2,76</t>
-  </si>
-  <si>
-    <t>27,05</t>
-  </si>
-  <si>
-    <t>15,71</t>
-  </si>
-  <si>
-    <t>5,68</t>
-  </si>
-  <si>
-    <t>0,64</t>
-  </si>
-  <si>
-    <t>2,46</t>
-  </si>
-  <si>
-    <t>7,43</t>
-  </si>
-  <si>
-    <t>13,23</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>28,1</t>
-  </si>
-  <si>
-    <t>27,71</t>
-  </si>
-  <si>
-    <t>3,66</t>
-  </si>
-  <si>
-    <t>6,29</t>
-  </si>
-  <si>
-    <t>0,39</t>
-  </si>
-  <si>
-    <t>0,72</t>
-  </si>
-  <si>
-    <t>0,16</t>
-  </si>
-  <si>
-    <t>2,47</t>
-  </si>
-  <si>
-    <t>9,44</t>
-  </si>
-  <si>
-    <t>19,28</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>17,76</t>
-  </si>
-  <si>
-    <t>0,48</t>
-  </si>
-  <si>
-    <t>2,18</t>
-  </si>
-  <si>
-    <t>29,42</t>
-  </si>
-  <si>
-    <t>3,16</t>
-  </si>
-  <si>
-    <t>0,27</t>
-  </si>
-  <si>
-    <t>4,58</t>
-  </si>
-  <si>
-    <t>0,57</t>
-  </si>
-  <si>
-    <t>4,61</t>
-  </si>
-  <si>
-    <t>8,23</t>
-  </si>
-  <si>
-    <t>27,34</t>
+    <t>3,36</t>
+  </si>
+  <si>
+    <t>8,48</t>
+  </si>
+  <si>
+    <t>27,37</t>
   </si>
   <si>
     <t>1811</t>
@@ -793,40 +790,34 @@
     <t>MESUJI</t>
   </si>
   <si>
-    <t>29,77</t>
-  </si>
-  <si>
-    <t>7,28</t>
-  </si>
-  <si>
-    <t>2,66</t>
-  </si>
-  <si>
-    <t>27,56</t>
-  </si>
-  <si>
-    <t>6,9</t>
-  </si>
-  <si>
-    <t>0,36</t>
-  </si>
-  <si>
-    <t>3,38</t>
-  </si>
-  <si>
-    <t>0,2</t>
+    <t>29,65</t>
+  </si>
+  <si>
+    <t>7,32</t>
+  </si>
+  <si>
+    <t>2,52</t>
+  </si>
+  <si>
+    <t>27,77</t>
+  </si>
+  <si>
+    <t>6,88</t>
+  </si>
+  <si>
+    <t>0,34</t>
+  </si>
+  <si>
+    <t>3,39</t>
   </si>
   <si>
     <t>0,66</t>
   </si>
   <si>
-    <t>4,77</t>
-  </si>
-  <si>
     <t>9,45</t>
   </si>
   <si>
-    <t>6,26</t>
+    <t>6,34</t>
   </si>
   <si>
     <t>1812</t>
@@ -835,34 +826,34 @@
     <t>TULANG BAWANG BARAT</t>
   </si>
   <si>
-    <t>16,86</t>
-  </si>
-  <si>
-    <t>1,92</t>
-  </si>
-  <si>
-    <t>7,63</t>
-  </si>
-  <si>
-    <t>28,35</t>
-  </si>
-  <si>
-    <t>12,5</t>
-  </si>
-  <si>
-    <t>0,55</t>
-  </si>
-  <si>
-    <t>5,12</t>
-  </si>
-  <si>
-    <t>2,26</t>
-  </si>
-  <si>
-    <t>4,28</t>
-  </si>
-  <si>
-    <t>19,64</t>
+    <t>16,6</t>
+  </si>
+  <si>
+    <t>1,84</t>
+  </si>
+  <si>
+    <t>6,84</t>
+  </si>
+  <si>
+    <t>29,91</t>
+  </si>
+  <si>
+    <t>11,89</t>
+  </si>
+  <si>
+    <t>0,49</t>
+  </si>
+  <si>
+    <t>5,39</t>
+  </si>
+  <si>
+    <t>1,52</t>
+  </si>
+  <si>
+    <t>4,53</t>
+  </si>
+  <si>
+    <t>20,1</t>
   </si>
   <si>
     <t>1813</t>
@@ -871,25 +862,34 @@
     <t>PESISIR BARAT</t>
   </si>
   <si>
-    <t>13,1</t>
-  </si>
-  <si>
-    <t>0,4</t>
-  </si>
-  <si>
-    <t>37,66</t>
-  </si>
-  <si>
-    <t>19,82</t>
-  </si>
-  <si>
-    <t>8,95</t>
+    <t>12,98</t>
+  </si>
+  <si>
+    <t>0,42</t>
+  </si>
+  <si>
+    <t>37,75</t>
+  </si>
+  <si>
+    <t>19,71</t>
+  </si>
+  <si>
+    <t>9,22</t>
   </si>
   <si>
     <t>0,21</t>
   </si>
   <si>
-    <t>10,82</t>
+    <t>0,65</t>
+  </si>
+  <si>
+    <t>0,3</t>
+  </si>
+  <si>
+    <t>7,54</t>
+  </si>
+  <si>
+    <t>10,79</t>
   </si>
   <si>
     <t>1871</t>
@@ -898,34 +898,31 @@
     <t>BANDAR LAMPUNG</t>
   </si>
   <si>
-    <t>15,56</t>
-  </si>
-  <si>
-    <t>3,87</t>
-  </si>
-  <si>
-    <t>30,03</t>
-  </si>
-  <si>
-    <t>16,55</t>
-  </si>
-  <si>
-    <t>0,89</t>
-  </si>
-  <si>
-    <t>0,3</t>
-  </si>
-  <si>
-    <t>1,78</t>
-  </si>
-  <si>
-    <t>1,09</t>
-  </si>
-  <si>
-    <t>4,56</t>
-  </si>
-  <si>
-    <t>18,14</t>
+    <t>15,44</t>
+  </si>
+  <si>
+    <t>3,83</t>
+  </si>
+  <si>
+    <t>30,19</t>
+  </si>
+  <si>
+    <t>16,42</t>
+  </si>
+  <si>
+    <t>0,88</t>
+  </si>
+  <si>
+    <t>1,77</t>
+  </si>
+  <si>
+    <t>1,28</t>
+  </si>
+  <si>
+    <t>4,62</t>
+  </si>
+  <si>
+    <t>17,99</t>
   </si>
   <si>
     <t>1872</t>
@@ -934,34 +931,28 @@
     <t>METRO</t>
   </si>
   <si>
-    <t>16,39</t>
-  </si>
-  <si>
-    <t>6,36</t>
-  </si>
-  <si>
-    <t>28,66</t>
-  </si>
-  <si>
-    <t>4,41</t>
-  </si>
-  <si>
-    <t>3,29</t>
-  </si>
-  <si>
-    <t>0,71</t>
-  </si>
-  <si>
-    <t>0,75</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>4,03</t>
-  </si>
-  <si>
-    <t>33,78</t>
+    <t>16,44</t>
+  </si>
+  <si>
+    <t>6,21</t>
+  </si>
+  <si>
+    <t>28,78</t>
+  </si>
+  <si>
+    <t>4,31</t>
+  </si>
+  <si>
+    <t>3,27</t>
+  </si>
+  <si>
+    <t>0,7</t>
+  </si>
+  <si>
+    <t>3,98</t>
+  </si>
+  <si>
+    <t>33,62</t>
   </si>
   <si>
     <t/>
@@ -1941,16 +1932,16 @@
         <v>105</v>
       </c>
       <c r="C6" s="6">
-        <v>96907</v>
+        <v>99157</v>
       </c>
       <c r="D6" s="6">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>106</v>
       </c>
       <c r="F6" s="6">
-        <v>19169</v>
+        <v>19592</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>107</v>
@@ -1962,31 +1953,31 @@
         <v>108</v>
       </c>
       <c r="J6" s="6">
-        <v>3818</v>
+        <v>3617</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>109</v>
       </c>
       <c r="L6" s="6">
-        <v>32427</v>
+        <v>33605</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>110</v>
       </c>
       <c r="N6" s="6">
-        <v>10172</v>
+        <v>10453</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>111</v>
       </c>
       <c r="P6" s="6">
-        <v>417</v>
+        <v>387</v>
       </c>
       <c r="Q6" s="7" t="s">
         <v>112</v>
       </c>
       <c r="R6" s="6">
-        <v>6884</v>
+        <v>7122</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>113</v>
@@ -1998,19 +1989,19 @@
         <v>114</v>
       </c>
       <c r="V6" s="6">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="W6" s="7" t="s">
         <v>115</v>
       </c>
       <c r="X6" s="6">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="Y6" s="7" t="s">
         <v>116</v>
       </c>
       <c r="Z6" s="6">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AA6" s="7" t="s">
         <v>117</v>
@@ -2019,84 +2010,84 @@
         <v>34</v>
       </c>
       <c r="AC6" s="7" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AD6" s="6">
         <v>78</v>
       </c>
       <c r="AE6" s="7" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="AF6" s="6">
         <v>1</v>
       </c>
       <c r="AG6" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="AH6" s="6">
+        <v>32</v>
+      </c>
+      <c r="AI6" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="AJ6" s="6">
+        <v>256</v>
+      </c>
+      <c r="AK6" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="AH6" s="6">
-        <v>34</v>
-      </c>
-      <c r="AI6" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="AJ6" s="6">
-        <v>253</v>
-      </c>
-      <c r="AK6" s="7" t="s">
+      <c r="AL6" s="6">
+        <v>37</v>
+      </c>
+      <c r="AM6" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="AL6" s="6">
-        <v>33</v>
-      </c>
-      <c r="AM6" s="7" t="s">
-        <v>115</v>
-      </c>
       <c r="AN6" s="6">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="AO6" s="7" t="s">
         <v>121</v>
       </c>
       <c r="AP6" s="6">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="AQ6" s="7" t="s">
         <v>122</v>
       </c>
       <c r="AR6" s="6">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="AS6" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="AT6" s="6">
+        <v>1885</v>
+      </c>
+      <c r="AU6" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="AT6" s="6">
-        <v>2180</v>
-      </c>
-      <c r="AU6" s="7" t="s">
+      <c r="AV6" s="6">
+        <v>5388</v>
+      </c>
+      <c r="AW6" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="AV6" s="6">
-        <v>5315</v>
-      </c>
-      <c r="AW6" s="7" t="s">
+      <c r="AX6" s="6">
+        <v>13938</v>
+      </c>
+      <c r="AY6" s="7" t="s">
         <v>125</v>
-      </c>
-      <c r="AX6" s="6">
-        <v>13356</v>
-      </c>
-      <c r="AY6" s="7" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="B7" s="8" t="s">
-        <v>128</v>
-      </c>
       <c r="C7" s="9">
-        <v>5086</v>
+        <v>5090</v>
       </c>
       <c r="D7" s="9">
         <v>7</v>
@@ -2105,64 +2096,64 @@
         <v>116</v>
       </c>
       <c r="F7" s="9">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H7" s="9">
         <v>68</v>
       </c>
       <c r="I7" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="J7" s="9">
+        <v>247</v>
+      </c>
+      <c r="K7" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="J7" s="9">
-        <v>249</v>
-      </c>
-      <c r="K7" s="10" t="s">
+      <c r="L7" s="9">
+        <v>1969</v>
+      </c>
+      <c r="M7" s="10" t="s">
         <v>131</v>
-      </c>
-      <c r="L7" s="9">
-        <v>1962</v>
-      </c>
-      <c r="M7" s="10" t="s">
-        <v>132</v>
       </c>
       <c r="N7" s="9">
         <v>127</v>
       </c>
       <c r="O7" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="P7" s="9">
         <v>30</v>
       </c>
       <c r="Q7" s="10" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="R7" s="9">
         <v>208</v>
       </c>
       <c r="S7" s="10" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="T7" s="9">
         <v>0</v>
       </c>
       <c r="U7" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="V7" s="9">
         <v>2</v>
       </c>
       <c r="W7" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="X7" s="9">
         <v>6</v>
       </c>
       <c r="Y7" s="10" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="Z7" s="9">
         <v>1</v>
@@ -2174,25 +2165,25 @@
         <v>6</v>
       </c>
       <c r="AC7" s="10" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="AD7" s="9">
         <v>5</v>
       </c>
       <c r="AE7" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AF7" s="9">
         <v>0</v>
       </c>
       <c r="AG7" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AH7" s="9">
         <v>2</v>
       </c>
       <c r="AI7" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="AJ7" s="9">
         <v>7</v>
@@ -2204,87 +2195,87 @@
         <v>0</v>
       </c>
       <c r="AM7" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AN7" s="9">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="AO7" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AP7" s="9">
         <v>17</v>
       </c>
       <c r="AQ7" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AR7" s="9">
         <v>3</v>
       </c>
       <c r="AS7" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="AT7" s="9">
+        <v>561</v>
+      </c>
+      <c r="AU7" s="10" t="s">
         <v>139</v>
-      </c>
-      <c r="AT7" s="9">
-        <v>564</v>
-      </c>
-      <c r="AU7" s="10" t="s">
-        <v>140</v>
       </c>
       <c r="AV7" s="9">
         <v>188</v>
       </c>
       <c r="AW7" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="AX7" s="9">
+        <v>502</v>
+      </c>
+      <c r="AY7" s="10" t="s">
         <v>141</v>
-      </c>
-      <c r="AX7" s="9">
-        <v>497</v>
-      </c>
-      <c r="AY7" s="10" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="C8" s="9">
+        <v>3270</v>
+      </c>
+      <c r="D8" s="9">
+        <v>0</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F8" s="9">
+        <v>444</v>
+      </c>
+      <c r="G8" s="10" t="s">
         <v>144</v>
-      </c>
-      <c r="C8" s="9">
-        <v>3281</v>
-      </c>
-      <c r="D8" s="9">
-        <v>0</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="F8" s="9">
-        <v>447</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>145</v>
       </c>
       <c r="H8" s="9">
         <v>14</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>112</v>
+        <v>145</v>
       </c>
       <c r="J8" s="9">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="K8" s="10" t="s">
         <v>146</v>
       </c>
       <c r="L8" s="9">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="M8" s="10" t="s">
         <v>147</v>
       </c>
       <c r="N8" s="9">
-        <v>1011</v>
+        <v>1009</v>
       </c>
       <c r="O8" s="10" t="s">
         <v>148</v>
@@ -2293,10 +2284,10 @@
         <v>0</v>
       </c>
       <c r="Q8" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="R8" s="9">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="S8" s="10" t="s">
         <v>149</v>
@@ -2305,31 +2296,31 @@
         <v>0</v>
       </c>
       <c r="U8" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="V8" s="9">
         <v>0</v>
       </c>
       <c r="W8" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="X8" s="9">
         <v>3</v>
       </c>
       <c r="Y8" s="10" t="s">
-        <v>114</v>
+        <v>150</v>
       </c>
       <c r="Z8" s="9">
         <v>0</v>
       </c>
       <c r="AA8" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AB8" s="9">
         <v>0</v>
       </c>
       <c r="AC8" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AD8" s="9">
         <v>1</v>
@@ -2341,171 +2332,171 @@
         <v>0</v>
       </c>
       <c r="AG8" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AH8" s="9">
         <v>0</v>
       </c>
       <c r="AI8" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AJ8" s="9">
         <v>5</v>
       </c>
       <c r="AK8" s="10" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AL8" s="9">
         <v>0</v>
       </c>
       <c r="AM8" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AN8" s="9">
         <v>0</v>
       </c>
       <c r="AO8" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AP8" s="9">
         <v>14</v>
       </c>
       <c r="AQ8" s="10" t="s">
-        <v>112</v>
+        <v>145</v>
       </c>
       <c r="AR8" s="9">
         <v>2</v>
       </c>
       <c r="AS8" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AT8" s="9">
         <v>6</v>
       </c>
       <c r="AU8" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AV8" s="9">
         <v>155</v>
       </c>
       <c r="AW8" s="10" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AX8" s="9">
         <v>524</v>
       </c>
       <c r="AY8" s="10" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C9" s="9">
-        <v>7752</v>
+        <v>7986</v>
       </c>
       <c r="D9" s="9">
         <v>0</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F9" s="9">
-        <v>1335</v>
+        <v>1375</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H9" s="9">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J9" s="9">
         <v>4</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="L9" s="9">
-        <v>3154</v>
+        <v>3294</v>
       </c>
       <c r="M9" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N9" s="9">
-        <v>1135</v>
+        <v>1121</v>
       </c>
       <c r="O9" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="P9" s="9">
         <v>1</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="R9" s="9">
-        <v>720</v>
+        <v>774</v>
       </c>
       <c r="S9" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T9" s="9">
         <v>8</v>
       </c>
       <c r="U9" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="V9" s="9">
         <v>0</v>
       </c>
       <c r="W9" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="X9" s="9">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="Y9" s="10" t="s">
-        <v>163</v>
+        <v>137</v>
       </c>
       <c r="Z9" s="9">
         <v>0</v>
       </c>
       <c r="AA9" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AB9" s="9">
         <v>0</v>
       </c>
       <c r="AC9" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AD9" s="9">
         <v>8</v>
       </c>
       <c r="AE9" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AF9" s="9">
         <v>1</v>
       </c>
       <c r="AG9" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AH9" s="9">
         <v>1</v>
       </c>
       <c r="AI9" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AJ9" s="9">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="AK9" s="10" t="s">
         <v>164</v>
@@ -2514,16 +2505,16 @@
         <v>0</v>
       </c>
       <c r="AM9" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AN9" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO9" s="10" t="s">
-        <v>161</v>
+        <v>118</v>
       </c>
       <c r="AP9" s="9">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AQ9" s="10" t="s">
         <v>165</v>
@@ -2535,42 +2526,42 @@
         <v>115</v>
       </c>
       <c r="AT9" s="9">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AU9" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="AV9" s="9">
+        <v>340</v>
+      </c>
+      <c r="AW9" s="10" t="s">
         <v>166</v>
       </c>
-      <c r="AV9" s="9">
-        <v>336</v>
-      </c>
-      <c r="AW9" s="10" t="s">
+      <c r="AX9" s="9">
+        <v>669</v>
+      </c>
+      <c r="AY9" s="10" t="s">
         <v>167</v>
-      </c>
-      <c r="AX9" s="9">
-        <v>659</v>
-      </c>
-      <c r="AY9" s="10" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="B10" s="8" t="s">
-        <v>170</v>
-      </c>
       <c r="C10" s="9">
-        <v>14794</v>
+        <v>15440</v>
       </c>
       <c r="D10" s="9">
         <v>38</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>120</v>
+        <v>170</v>
       </c>
       <c r="F10" s="9">
-        <v>3132</v>
+        <v>3303</v>
       </c>
       <c r="G10" s="10" t="s">
         <v>171</v>
@@ -2579,97 +2570,97 @@
         <v>49</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>138</v>
+        <v>172</v>
       </c>
       <c r="J10" s="9">
-        <v>1973</v>
+        <v>1911</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="L10" s="9">
-        <v>4235</v>
+        <v>4452</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="N10" s="9">
-        <v>1595</v>
+        <v>1846</v>
       </c>
       <c r="O10" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P10" s="9">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="Q10" s="10" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="R10" s="9">
-        <v>857</v>
+        <v>916</v>
       </c>
       <c r="S10" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="T10" s="9">
         <v>10</v>
       </c>
       <c r="U10" s="10" t="s">
-        <v>177</v>
+        <v>138</v>
       </c>
       <c r="V10" s="9">
         <v>9</v>
       </c>
       <c r="W10" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="X10" s="9">
         <v>10</v>
       </c>
       <c r="Y10" s="10" t="s">
-        <v>177</v>
+        <v>138</v>
       </c>
       <c r="Z10" s="9">
         <v>0</v>
       </c>
       <c r="AA10" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AB10" s="9">
         <v>12</v>
       </c>
       <c r="AC10" s="10" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="AD10" s="9">
         <v>9</v>
       </c>
       <c r="AE10" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AF10" s="9">
         <v>0</v>
       </c>
       <c r="AG10" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AH10" s="9">
         <v>11</v>
       </c>
       <c r="AI10" s="10" t="s">
-        <v>177</v>
+        <v>106</v>
       </c>
       <c r="AJ10" s="9">
         <v>10</v>
       </c>
       <c r="AK10" s="10" t="s">
-        <v>177</v>
+        <v>138</v>
       </c>
       <c r="AL10" s="9">
         <v>1</v>
       </c>
       <c r="AM10" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AN10" s="9">
         <v>56</v>
@@ -2681,28 +2672,28 @@
         <v>19</v>
       </c>
       <c r="AQ10" s="10" t="s">
-        <v>166</v>
+        <v>134</v>
       </c>
       <c r="AR10" s="9">
         <v>9</v>
       </c>
       <c r="AS10" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AT10" s="9">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="AU10" s="10" t="s">
         <v>179</v>
       </c>
       <c r="AV10" s="9">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="AW10" s="10" t="s">
         <v>180</v>
       </c>
       <c r="AX10" s="9">
-        <v>1879</v>
+        <v>1882</v>
       </c>
       <c r="AY10" s="10" t="s">
         <v>181</v>
@@ -2716,16 +2707,16 @@
         <v>183</v>
       </c>
       <c r="C11" s="9">
-        <v>12382</v>
+        <v>12427</v>
       </c>
       <c r="D11" s="9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>158</v>
+        <v>120</v>
       </c>
       <c r="F11" s="9">
-        <v>1915</v>
+        <v>1928</v>
       </c>
       <c r="G11" s="10" t="s">
         <v>184</v>
@@ -2737,31 +2728,31 @@
         <v>185</v>
       </c>
       <c r="J11" s="9">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="K11" s="10" t="s">
         <v>186</v>
       </c>
       <c r="L11" s="9">
-        <v>5566</v>
+        <v>5600</v>
       </c>
       <c r="M11" s="10" t="s">
         <v>187</v>
       </c>
       <c r="N11" s="9">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="O11" s="10" t="s">
         <v>188</v>
       </c>
       <c r="P11" s="9">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="Q11" s="10" t="s">
         <v>189</v>
       </c>
       <c r="R11" s="9">
-        <v>1594</v>
+        <v>1598</v>
       </c>
       <c r="S11" s="10" t="s">
         <v>190</v>
@@ -2770,25 +2761,25 @@
         <v>18</v>
       </c>
       <c r="U11" s="10" t="s">
-        <v>150</v>
+        <v>116</v>
       </c>
       <c r="V11" s="9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W11" s="10" t="s">
-        <v>158</v>
+        <v>138</v>
       </c>
       <c r="X11" s="9">
         <v>10</v>
       </c>
       <c r="Y11" s="10" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="Z11" s="9">
         <v>5</v>
       </c>
       <c r="AA11" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="AB11" s="9">
         <v>3</v>
@@ -2800,19 +2791,19 @@
         <v>22</v>
       </c>
       <c r="AE11" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AF11" s="9">
         <v>0</v>
       </c>
       <c r="AG11" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AH11" s="9">
         <v>6</v>
       </c>
       <c r="AI11" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="AJ11" s="9">
         <v>29</v>
@@ -2830,7 +2821,7 @@
         <v>9</v>
       </c>
       <c r="AO11" s="10" t="s">
-        <v>177</v>
+        <v>106</v>
       </c>
       <c r="AP11" s="9">
         <v>84</v>
@@ -2842,22 +2833,22 @@
         <v>15</v>
       </c>
       <c r="AS11" s="10" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="AT11" s="9">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="AU11" s="10" t="s">
         <v>193</v>
       </c>
       <c r="AV11" s="9">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="AW11" s="10" t="s">
         <v>194</v>
       </c>
       <c r="AX11" s="9">
-        <v>1413</v>
+        <v>1427</v>
       </c>
       <c r="AY11" s="10" t="s">
         <v>195</v>
@@ -2871,16 +2862,16 @@
         <v>197</v>
       </c>
       <c r="C12" s="9">
-        <v>5015</v>
+        <v>5035</v>
       </c>
       <c r="D12" s="9">
         <v>0</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F12" s="9">
-        <v>938</v>
+        <v>943</v>
       </c>
       <c r="G12" s="10" t="s">
         <v>198</v>
@@ -2892,31 +2883,31 @@
         <v>164</v>
       </c>
       <c r="J12" s="9">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="K12" s="10" t="s">
         <v>199</v>
       </c>
       <c r="L12" s="9">
-        <v>1849</v>
+        <v>1860</v>
       </c>
       <c r="M12" s="10" t="s">
         <v>200</v>
       </c>
       <c r="N12" s="9">
-        <v>705</v>
+        <v>722</v>
       </c>
       <c r="O12" s="10" t="s">
         <v>201</v>
       </c>
       <c r="P12" s="9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q12" s="10" t="s">
-        <v>139</v>
+        <v>114</v>
       </c>
       <c r="R12" s="9">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="S12" s="10" t="s">
         <v>202</v>
@@ -2925,13 +2916,13 @@
         <v>0</v>
       </c>
       <c r="U12" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="V12" s="9">
         <v>3</v>
       </c>
       <c r="W12" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="X12" s="9">
         <v>7</v>
@@ -2949,25 +2940,25 @@
         <v>3</v>
       </c>
       <c r="AC12" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AD12" s="9">
         <v>9</v>
       </c>
       <c r="AE12" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AF12" s="9">
         <v>0</v>
       </c>
       <c r="AG12" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AH12" s="9">
         <v>2</v>
       </c>
       <c r="AI12" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="AJ12" s="9">
         <v>29</v>
@@ -2979,19 +2970,19 @@
         <v>0</v>
       </c>
       <c r="AM12" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AN12" s="9">
         <v>4</v>
       </c>
       <c r="AO12" s="10" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="AP12" s="9">
         <v>55</v>
       </c>
       <c r="AQ12" s="10" t="s">
-        <v>204</v>
+        <v>165</v>
       </c>
       <c r="AR12" s="9">
         <v>1</v>
@@ -3000,10 +2991,10 @@
         <v>117</v>
       </c>
       <c r="AT12" s="9">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="AU12" s="10" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AV12" s="9">
         <v>341</v>
@@ -3026,16 +3017,16 @@
         <v>208</v>
       </c>
       <c r="C13" s="9">
-        <v>4433</v>
+        <v>4475</v>
       </c>
       <c r="D13" s="9">
         <v>2</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>158</v>
+        <v>120</v>
       </c>
       <c r="F13" s="9">
-        <v>811</v>
+        <v>824</v>
       </c>
       <c r="G13" s="10" t="s">
         <v>209</v>
@@ -3047,19 +3038,19 @@
         <v>210</v>
       </c>
       <c r="J13" s="9">
-        <v>233</v>
+        <v>197</v>
       </c>
       <c r="K13" s="10" t="s">
         <v>211</v>
       </c>
       <c r="L13" s="9">
-        <v>1703</v>
+        <v>1746</v>
       </c>
       <c r="M13" s="10" t="s">
         <v>212</v>
       </c>
       <c r="N13" s="9">
-        <v>732</v>
+        <v>751</v>
       </c>
       <c r="O13" s="10" t="s">
         <v>213</v>
@@ -3071,7 +3062,7 @@
         <v>214</v>
       </c>
       <c r="R13" s="9">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="S13" s="10" t="s">
         <v>215</v>
@@ -3080,7 +3071,7 @@
         <v>0</v>
       </c>
       <c r="U13" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="V13" s="9">
         <v>1</v>
@@ -3092,13 +3083,13 @@
         <v>3</v>
       </c>
       <c r="Y13" s="10" t="s">
-        <v>177</v>
+        <v>106</v>
       </c>
       <c r="Z13" s="9">
         <v>0</v>
       </c>
       <c r="AA13" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AB13" s="9">
         <v>1</v>
@@ -3110,19 +3101,19 @@
         <v>6</v>
       </c>
       <c r="AE13" s="10" t="s">
-        <v>116</v>
+        <v>216</v>
       </c>
       <c r="AF13" s="9">
         <v>0</v>
       </c>
       <c r="AG13" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AH13" s="9">
         <v>0</v>
       </c>
       <c r="AI13" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AJ13" s="9">
         <v>28</v>
@@ -3134,7 +3125,7 @@
         <v>11</v>
       </c>
       <c r="AM13" s="10" t="s">
-        <v>216</v>
+        <v>170</v>
       </c>
       <c r="AN13" s="9">
         <v>1</v>
@@ -3143,7 +3134,7 @@
         <v>117</v>
       </c>
       <c r="AP13" s="9">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AQ13" s="10" t="s">
         <v>217</v>
@@ -3155,87 +3146,87 @@
         <v>218</v>
       </c>
       <c r="AT13" s="9">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="AU13" s="10" t="s">
-        <v>178</v>
+        <v>219</v>
       </c>
       <c r="AV13" s="9">
         <v>211</v>
       </c>
       <c r="AW13" s="10" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AX13" s="9">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="AY13" s="10" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C14" s="9">
-        <v>4347</v>
+        <v>4359</v>
       </c>
       <c r="D14" s="9">
         <v>0</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F14" s="9">
         <v>1027</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H14" s="9">
         <v>18</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="J14" s="9">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="L14" s="9">
-        <v>1176</v>
+        <v>1182</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="N14" s="9">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="O14" s="10" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="P14" s="9">
         <v>8</v>
       </c>
       <c r="Q14" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="R14" s="9">
         <v>247</v>
       </c>
       <c r="S14" s="10" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="T14" s="9">
         <v>2</v>
       </c>
       <c r="U14" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="V14" s="9">
         <v>1</v>
@@ -3247,7 +3238,7 @@
         <v>8</v>
       </c>
       <c r="Y14" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="Z14" s="9">
         <v>1</v>
@@ -3271,7 +3262,7 @@
         <v>0</v>
       </c>
       <c r="AG14" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AH14" s="9">
         <v>1</v>
@@ -3283,7 +3274,7 @@
         <v>11</v>
       </c>
       <c r="AK14" s="10" t="s">
-        <v>216</v>
+        <v>170</v>
       </c>
       <c r="AL14" s="9">
         <v>1</v>
@@ -3295,13 +3286,13 @@
         <v>3</v>
       </c>
       <c r="AO14" s="10" t="s">
-        <v>177</v>
+        <v>106</v>
       </c>
       <c r="AP14" s="9">
         <v>28</v>
       </c>
       <c r="AQ14" s="10" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="AR14" s="9">
         <v>1</v>
@@ -3310,111 +3301,111 @@
         <v>117</v>
       </c>
       <c r="AT14" s="9">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="AU14" s="10" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="AV14" s="9">
         <v>323</v>
       </c>
       <c r="AW14" s="10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="AX14" s="9">
-        <v>575</v>
+        <v>585</v>
       </c>
       <c r="AY14" s="10" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C15" s="9">
-        <v>10764</v>
+        <v>11434</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F15" s="9">
-        <v>3025</v>
+        <v>3144</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H15" s="9">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="I15" s="10" t="s">
         <v>217</v>
       </c>
       <c r="J15" s="9">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>203</v>
+        <v>237</v>
       </c>
       <c r="L15" s="9">
-        <v>2983</v>
+        <v>3312</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="N15" s="9">
-        <v>394</v>
+        <v>405</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="P15" s="9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>177</v>
+        <v>138</v>
       </c>
       <c r="R15" s="9">
-        <v>677</v>
+        <v>707</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="T15" s="9">
         <v>42</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="V15" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W15" s="10" t="s">
-        <v>161</v>
+        <v>118</v>
       </c>
       <c r="X15" s="9">
         <v>14</v>
       </c>
       <c r="Y15" s="10" t="s">
-        <v>166</v>
+        <v>134</v>
       </c>
       <c r="Z15" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA15" s="10" t="s">
-        <v>119</v>
+        <v>162</v>
       </c>
       <c r="AB15" s="9">
         <v>0</v>
       </c>
       <c r="AC15" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AD15" s="9">
         <v>3</v>
@@ -3426,19 +3417,19 @@
         <v>0</v>
       </c>
       <c r="AG15" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AH15" s="9">
         <v>1</v>
       </c>
       <c r="AI15" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AJ15" s="9">
         <v>11</v>
       </c>
       <c r="AK15" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AL15" s="9">
         <v>2</v>
@@ -3447,37 +3438,37 @@
         <v>117</v>
       </c>
       <c r="AN15" s="9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AO15" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AP15" s="9">
         <v>78</v>
       </c>
       <c r="AQ15" s="10" t="s">
-        <v>240</v>
+        <v>192</v>
       </c>
       <c r="AR15" s="9">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AS15" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AT15" s="9">
-        <v>266</v>
+        <v>78</v>
       </c>
       <c r="AU15" s="10" t="s">
-        <v>242</v>
+        <v>192</v>
       </c>
       <c r="AV15" s="9">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="AW15" s="10" t="s">
         <v>243</v>
       </c>
       <c r="AX15" s="9">
-        <v>2075</v>
+        <v>2452</v>
       </c>
       <c r="AY15" s="10" t="s">
         <v>244</v>
@@ -3491,16 +3482,16 @@
         <v>246</v>
       </c>
       <c r="C16" s="9">
-        <v>4364</v>
+        <v>4530</v>
       </c>
       <c r="D16" s="9">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>151</v>
+        <v>216</v>
       </c>
       <c r="F16" s="9">
-        <v>775</v>
+        <v>807</v>
       </c>
       <c r="G16" s="10" t="s">
         <v>247</v>
@@ -3512,52 +3503,52 @@
         <v>248</v>
       </c>
       <c r="J16" s="9">
-        <v>95</v>
+        <v>66</v>
       </c>
       <c r="K16" s="10" t="s">
         <v>249</v>
       </c>
       <c r="L16" s="9">
-        <v>1284</v>
+        <v>1402</v>
       </c>
       <c r="M16" s="10" t="s">
         <v>250</v>
       </c>
       <c r="N16" s="9">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="O16" s="10" t="s">
         <v>251</v>
       </c>
       <c r="P16" s="9">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="Q16" s="10" t="s">
-        <v>252</v>
+        <v>106</v>
       </c>
       <c r="R16" s="9">
-        <v>200</v>
+        <v>228</v>
       </c>
       <c r="S16" s="10" t="s">
-        <v>253</v>
+        <v>188</v>
       </c>
       <c r="T16" s="9">
         <v>0</v>
       </c>
       <c r="U16" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="V16" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W16" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X16" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y16" s="10" t="s">
-        <v>158</v>
+        <v>106</v>
       </c>
       <c r="Z16" s="9">
         <v>1</v>
@@ -3569,7 +3560,7 @@
         <v>3</v>
       </c>
       <c r="AC16" s="10" t="s">
-        <v>177</v>
+        <v>106</v>
       </c>
       <c r="AD16" s="9">
         <v>1</v>
@@ -3581,7 +3572,7 @@
         <v>0</v>
       </c>
       <c r="AG16" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AH16" s="9">
         <v>1</v>
@@ -3590,63 +3581,63 @@
         <v>117</v>
       </c>
       <c r="AJ16" s="9">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="AK16" s="10" t="s">
-        <v>224</v>
+        <v>252</v>
       </c>
       <c r="AL16" s="9">
         <v>8</v>
       </c>
       <c r="AM16" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AN16" s="9">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AO16" s="10" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="AP16" s="9">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="AQ16" s="10" t="s">
+        <v>253</v>
+      </c>
+      <c r="AR16" s="9">
+        <v>14</v>
+      </c>
+      <c r="AS16" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="AT16" s="9">
+        <v>152</v>
+      </c>
+      <c r="AU16" s="10" t="s">
         <v>254</v>
       </c>
-      <c r="AR16" s="9">
-        <v>12</v>
-      </c>
-      <c r="AS16" s="10" t="s">
-        <v>252</v>
-      </c>
-      <c r="AT16" s="9">
-        <v>201</v>
-      </c>
-      <c r="AU16" s="10" t="s">
+      <c r="AV16" s="9">
+        <v>384</v>
+      </c>
+      <c r="AW16" s="10" t="s">
         <v>255</v>
       </c>
-      <c r="AV16" s="9">
-        <v>359</v>
-      </c>
-      <c r="AW16" s="10" t="s">
+      <c r="AX16" s="9">
+        <v>1240</v>
+      </c>
+      <c r="AY16" s="10" t="s">
         <v>256</v>
-      </c>
-      <c r="AX16" s="9">
-        <v>1193</v>
-      </c>
-      <c r="AY16" s="10" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>258</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>259</v>
-      </c>
       <c r="C17" s="9">
-        <v>6086</v>
+        <v>6104</v>
       </c>
       <c r="D17" s="9">
         <v>2</v>
@@ -3655,46 +3646,46 @@
         <v>115</v>
       </c>
       <c r="F17" s="9">
-        <v>1812</v>
+        <v>1810</v>
       </c>
       <c r="G17" s="10" t="s">
+        <v>259</v>
+      </c>
+      <c r="H17" s="9">
+        <v>447</v>
+      </c>
+      <c r="I17" s="10" t="s">
         <v>260</v>
       </c>
-      <c r="H17" s="9">
-        <v>443</v>
-      </c>
-      <c r="I17" s="10" t="s">
+      <c r="J17" s="9">
+        <v>154</v>
+      </c>
+      <c r="K17" s="10" t="s">
         <v>261</v>
       </c>
-      <c r="J17" s="9">
-        <v>162</v>
-      </c>
-      <c r="K17" s="10" t="s">
+      <c r="L17" s="9">
+        <v>1695</v>
+      </c>
+      <c r="M17" s="10" t="s">
         <v>262</v>
-      </c>
-      <c r="L17" s="9">
-        <v>1677</v>
-      </c>
-      <c r="M17" s="10" t="s">
-        <v>263</v>
       </c>
       <c r="N17" s="9">
         <v>420</v>
       </c>
       <c r="O17" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="P17" s="9">
+        <v>21</v>
+      </c>
+      <c r="Q17" s="10" t="s">
         <v>264</v>
       </c>
-      <c r="P17" s="9">
-        <v>22</v>
-      </c>
-      <c r="Q17" s="10" t="s">
+      <c r="R17" s="9">
+        <v>207</v>
+      </c>
+      <c r="S17" s="10" t="s">
         <v>265</v>
-      </c>
-      <c r="R17" s="9">
-        <v>206</v>
-      </c>
-      <c r="S17" s="10" t="s">
-        <v>266</v>
       </c>
       <c r="T17" s="9">
         <v>1</v>
@@ -3706,13 +3697,13 @@
         <v>5</v>
       </c>
       <c r="W17" s="10" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="X17" s="9">
         <v>5</v>
       </c>
       <c r="Y17" s="10" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="Z17" s="9">
         <v>2</v>
@@ -3730,13 +3721,13 @@
         <v>4</v>
       </c>
       <c r="AE17" s="10" t="s">
-        <v>177</v>
+        <v>106</v>
       </c>
       <c r="AF17" s="9">
         <v>0</v>
       </c>
       <c r="AG17" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AH17" s="9">
         <v>2</v>
@@ -3748,13 +3739,13 @@
         <v>12</v>
       </c>
       <c r="AK17" s="10" t="s">
-        <v>267</v>
+        <v>136</v>
       </c>
       <c r="AL17" s="9">
         <v>5</v>
       </c>
       <c r="AM17" s="10" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="AN17" s="9">
         <v>7</v>
@@ -3766,138 +3757,138 @@
         <v>40</v>
       </c>
       <c r="AQ17" s="10" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="AR17" s="9">
         <v>11</v>
       </c>
       <c r="AS17" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AT17" s="9">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="AU17" s="10" t="s">
-        <v>269</v>
+        <v>220</v>
       </c>
       <c r="AV17" s="9">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="AW17" s="10" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="AX17" s="9">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="AY17" s="10" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="C18" s="9">
-        <v>7602</v>
+        <v>7920</v>
       </c>
       <c r="D18" s="9">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="F18" s="9">
-        <v>1282</v>
+        <v>1315</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="H18" s="9">
         <v>146</v>
       </c>
       <c r="I18" s="10" t="s">
+        <v>272</v>
+      </c>
+      <c r="J18" s="9">
+        <v>542</v>
+      </c>
+      <c r="K18" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="L18" s="9">
+        <v>2369</v>
+      </c>
+      <c r="M18" s="10" t="s">
+        <v>274</v>
+      </c>
+      <c r="N18" s="9">
+        <v>942</v>
+      </c>
+      <c r="O18" s="10" t="s">
         <v>275</v>
       </c>
-      <c r="J18" s="9">
-        <v>580</v>
-      </c>
-      <c r="K18" s="10" t="s">
+      <c r="P18" s="9">
+        <v>39</v>
+      </c>
+      <c r="Q18" s="10" t="s">
         <v>276</v>
       </c>
-      <c r="L18" s="9">
-        <v>2155</v>
-      </c>
-      <c r="M18" s="10" t="s">
+      <c r="R18" s="9">
+        <v>427</v>
+      </c>
+      <c r="S18" s="10" t="s">
         <v>277</v>
-      </c>
-      <c r="N18" s="9">
-        <v>950</v>
-      </c>
-      <c r="O18" s="10" t="s">
-        <v>278</v>
-      </c>
-      <c r="P18" s="9">
-        <v>42</v>
-      </c>
-      <c r="Q18" s="10" t="s">
-        <v>279</v>
-      </c>
-      <c r="R18" s="9">
-        <v>389</v>
-      </c>
-      <c r="S18" s="10" t="s">
-        <v>280</v>
       </c>
       <c r="T18" s="9">
         <v>3</v>
       </c>
       <c r="U18" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="V18" s="9">
         <v>1</v>
       </c>
       <c r="W18" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="X18" s="9">
         <v>3</v>
       </c>
       <c r="Y18" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="Z18" s="9">
         <v>0</v>
       </c>
       <c r="AA18" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AB18" s="9">
         <v>3</v>
       </c>
       <c r="AC18" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="AD18" s="9">
         <v>1</v>
       </c>
       <c r="AE18" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AF18" s="9">
         <v>0</v>
       </c>
       <c r="AG18" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AH18" s="9">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AI18" s="10" t="s">
-        <v>106</v>
+        <v>159</v>
       </c>
       <c r="AJ18" s="9">
         <v>9</v>
@@ -3906,57 +3897,57 @@
         <v>121</v>
       </c>
       <c r="AL18" s="9">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AM18" s="10" t="s">
-        <v>119</v>
+        <v>159</v>
       </c>
       <c r="AN18" s="9">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AO18" s="10" t="s">
-        <v>166</v>
+        <v>121</v>
       </c>
       <c r="AP18" s="9">
         <v>18</v>
       </c>
       <c r="AQ18" s="10" t="s">
-        <v>137</v>
+        <v>191</v>
       </c>
       <c r="AR18" s="9">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AS18" s="10" t="s">
-        <v>177</v>
+        <v>135</v>
       </c>
       <c r="AT18" s="9">
-        <v>172</v>
+        <v>120</v>
       </c>
       <c r="AU18" s="10" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="AV18" s="9">
-        <v>325</v>
+        <v>359</v>
       </c>
       <c r="AW18" s="10" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="AX18" s="9">
-        <v>1493</v>
+        <v>1592</v>
       </c>
       <c r="AY18" s="10" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="C19" s="9">
-        <v>7588</v>
+        <v>7655</v>
       </c>
       <c r="D19" s="9">
         <v>2</v>
@@ -3968,136 +3959,136 @@
         <v>994</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="H19" s="9">
         <v>12</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J19" s="9">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="K19" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="L19" s="9">
+        <v>2890</v>
+      </c>
+      <c r="M19" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="N19" s="9">
+        <v>1509</v>
+      </c>
+      <c r="O19" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="P19" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="R19" s="9">
+        <v>706</v>
+      </c>
+      <c r="S19" s="10" t="s">
         <v>287</v>
       </c>
-      <c r="L19" s="9">
-        <v>2858</v>
-      </c>
-      <c r="M19" s="10" t="s">
-        <v>288</v>
-      </c>
-      <c r="N19" s="9">
-        <v>1504</v>
-      </c>
-      <c r="O19" s="10" t="s">
-        <v>289</v>
-      </c>
-      <c r="P19" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="R19" s="9">
-        <v>679</v>
-      </c>
-      <c r="S19" s="10" t="s">
-        <v>290</v>
-      </c>
       <c r="T19" s="9">
         <v>0</v>
       </c>
       <c r="U19" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="V19" s="9">
         <v>1</v>
       </c>
       <c r="W19" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="X19" s="9">
         <v>12</v>
       </c>
       <c r="Y19" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="Z19" s="9">
         <v>0</v>
       </c>
       <c r="AA19" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AB19" s="9">
         <v>0</v>
       </c>
       <c r="AC19" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AD19" s="9">
         <v>3</v>
       </c>
       <c r="AE19" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="AF19" s="9">
         <v>0</v>
       </c>
       <c r="AG19" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AH19" s="9">
         <v>0</v>
       </c>
       <c r="AI19" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AJ19" s="9">
         <v>16</v>
       </c>
       <c r="AK19" s="10" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="AL19" s="9">
         <v>0</v>
       </c>
       <c r="AM19" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AN19" s="9">
         <v>1</v>
       </c>
       <c r="AO19" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AP19" s="9">
         <v>50</v>
       </c>
       <c r="AQ19" s="10" t="s">
-        <v>268</v>
+        <v>289</v>
       </c>
       <c r="AR19" s="9">
         <v>1</v>
       </c>
       <c r="AS19" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AT19" s="9">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="AU19" s="10" t="s">
-        <v>138</v>
+        <v>290</v>
       </c>
       <c r="AV19" s="9">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="AW19" s="10" t="s">
-        <v>276</v>
+        <v>291</v>
       </c>
       <c r="AX19" s="9">
-        <v>821</v>
+        <v>826</v>
       </c>
       <c r="AY19" s="10" t="s">
         <v>292</v>
@@ -4111,13 +4102,13 @@
         <v>294</v>
       </c>
       <c r="C20" s="9">
-        <v>1009</v>
+        <v>1017</v>
       </c>
       <c r="D20" s="9">
         <v>1</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F20" s="9">
         <v>157</v>
@@ -4129,7 +4120,7 @@
         <v>6</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="J20" s="9">
         <v>39</v>
@@ -4138,7 +4129,7 @@
         <v>296</v>
       </c>
       <c r="L20" s="9">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="M20" s="10" t="s">
         <v>297</v>
@@ -4147,13 +4138,13 @@
         <v>48</v>
       </c>
       <c r="O20" s="10" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="P20" s="9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>287</v>
+        <v>276</v>
       </c>
       <c r="R20" s="9">
         <v>167</v>
@@ -4165,13 +4156,13 @@
         <v>0</v>
       </c>
       <c r="U20" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="V20" s="9">
         <v>0</v>
       </c>
       <c r="W20" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="X20" s="9">
         <v>9</v>
@@ -4183,254 +4174,254 @@
         <v>3</v>
       </c>
       <c r="AA20" s="10" t="s">
-        <v>300</v>
+        <v>214</v>
       </c>
       <c r="AB20" s="9">
         <v>0</v>
       </c>
       <c r="AC20" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AD20" s="9">
         <v>0</v>
       </c>
       <c r="AE20" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AF20" s="9">
         <v>0</v>
       </c>
       <c r="AG20" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AH20" s="9">
         <v>1</v>
       </c>
       <c r="AI20" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AJ20" s="9">
         <v>6</v>
       </c>
       <c r="AK20" s="10" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="AL20" s="9">
         <v>2</v>
       </c>
       <c r="AM20" s="10" t="s">
-        <v>267</v>
+        <v>136</v>
       </c>
       <c r="AN20" s="9">
         <v>1</v>
       </c>
       <c r="AO20" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AP20" s="9">
         <v>18</v>
       </c>
       <c r="AQ20" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="AR20" s="9">
         <v>4</v>
       </c>
       <c r="AS20" s="10" t="s">
-        <v>287</v>
+        <v>112</v>
       </c>
       <c r="AT20" s="9">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="AU20" s="10" t="s">
+        <v>301</v>
+      </c>
+      <c r="AV20" s="9">
+        <v>47</v>
+      </c>
+      <c r="AW20" s="10" t="s">
         <v>302</v>
-      </c>
-      <c r="AV20" s="9">
-        <v>46</v>
-      </c>
-      <c r="AW20" s="10" t="s">
-        <v>303</v>
       </c>
       <c r="AX20" s="9">
         <v>183</v>
       </c>
       <c r="AY20" s="10" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
+        <v>304</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>305</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="C21" s="9">
+        <v>2415</v>
+      </c>
+      <c r="D21" s="9">
+        <v>0</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F21" s="9">
+        <v>397</v>
+      </c>
+      <c r="G21" s="10" t="s">
         <v>306</v>
       </c>
-      <c r="C21" s="9">
-        <v>2404</v>
-      </c>
-      <c r="D21" s="9">
-        <v>0</v>
-      </c>
-      <c r="E21" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="F21" s="9">
-        <v>394</v>
-      </c>
-      <c r="G21" s="10" t="s">
+      <c r="H21" s="9">
+        <v>150</v>
+      </c>
+      <c r="I21" s="10" t="s">
         <v>307</v>
-      </c>
-      <c r="H21" s="9">
-        <v>153</v>
-      </c>
-      <c r="I21" s="10" t="s">
-        <v>308</v>
       </c>
       <c r="J21" s="9">
         <v>1</v>
       </c>
       <c r="K21" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="L21" s="9">
-        <v>689</v>
+        <v>695</v>
       </c>
       <c r="M21" s="10" t="s">
+        <v>308</v>
+      </c>
+      <c r="N21" s="9">
+        <v>104</v>
+      </c>
+      <c r="O21" s="10" t="s">
         <v>309</v>
       </c>
-      <c r="N21" s="9">
-        <v>106</v>
-      </c>
-      <c r="O21" s="10" t="s">
-        <v>310</v>
-      </c>
       <c r="P21" s="9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>214</v>
+        <v>137</v>
       </c>
       <c r="R21" s="9">
         <v>79</v>
       </c>
       <c r="S21" s="10" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="T21" s="9">
         <v>0</v>
       </c>
       <c r="U21" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="V21" s="9">
         <v>0</v>
       </c>
       <c r="W21" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="X21" s="9">
         <v>17</v>
       </c>
       <c r="Y21" s="10" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="Z21" s="9">
         <v>2</v>
       </c>
       <c r="AA21" s="10" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="AB21" s="9">
         <v>0</v>
       </c>
       <c r="AC21" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AD21" s="9">
         <v>1</v>
       </c>
       <c r="AE21" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="AF21" s="9">
         <v>0</v>
       </c>
       <c r="AG21" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AH21" s="9">
         <v>0</v>
       </c>
       <c r="AI21" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AJ21" s="9">
         <v>3</v>
       </c>
       <c r="AK21" s="10" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="AL21" s="9">
         <v>0</v>
       </c>
       <c r="AM21" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AN21" s="9">
         <v>0</v>
       </c>
       <c r="AO21" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AP21" s="9">
         <v>18</v>
       </c>
       <c r="AQ21" s="10" t="s">
-        <v>313</v>
+        <v>164</v>
       </c>
       <c r="AR21" s="9">
         <v>1</v>
       </c>
       <c r="AS21" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="AT21" s="9">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="AU21" s="10" t="s">
-        <v>314</v>
+        <v>301</v>
       </c>
       <c r="AV21" s="9">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="AW21" s="10" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="AX21" s="9">
         <v>812</v>
       </c>
       <c r="AY21" s="10" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="C22" s="12">
-        <v>96907</v>
+        <v>99157</v>
       </c>
       <c r="D22" s="12">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>106</v>
       </c>
       <c r="F22" s="12">
-        <v>19169</v>
+        <v>19592</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>107</v>
@@ -4442,31 +4433,31 @@
         <v>108</v>
       </c>
       <c r="J22" s="12">
-        <v>3818</v>
+        <v>3617</v>
       </c>
       <c r="K22" s="13" t="s">
         <v>109</v>
       </c>
       <c r="L22" s="12">
-        <v>32427</v>
+        <v>33605</v>
       </c>
       <c r="M22" s="13" t="s">
         <v>110</v>
       </c>
       <c r="N22" s="12">
-        <v>10172</v>
+        <v>10453</v>
       </c>
       <c r="O22" s="13" t="s">
         <v>111</v>
       </c>
       <c r="P22" s="12">
-        <v>417</v>
+        <v>387</v>
       </c>
       <c r="Q22" s="13" t="s">
         <v>112</v>
       </c>
       <c r="R22" s="12">
-        <v>6884</v>
+        <v>7122</v>
       </c>
       <c r="S22" s="13" t="s">
         <v>113</v>
@@ -4478,19 +4469,19 @@
         <v>114</v>
       </c>
       <c r="V22" s="12">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="W22" s="13" t="s">
         <v>115</v>
       </c>
       <c r="X22" s="12">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="Y22" s="13" t="s">
         <v>116</v>
       </c>
       <c r="Z22" s="12">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AA22" s="13" t="s">
         <v>117</v>
@@ -4499,73 +4490,73 @@
         <v>34</v>
       </c>
       <c r="AC22" s="13" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AD22" s="12">
         <v>78</v>
       </c>
       <c r="AE22" s="13" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="AF22" s="12">
         <v>1</v>
       </c>
       <c r="AG22" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="AH22" s="12">
+        <v>32</v>
+      </c>
+      <c r="AI22" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="AJ22" s="12">
+        <v>256</v>
+      </c>
+      <c r="AK22" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="AH22" s="12">
-        <v>34</v>
-      </c>
-      <c r="AI22" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="AJ22" s="12">
-        <v>253</v>
-      </c>
-      <c r="AK22" s="13" t="s">
+      <c r="AL22" s="12">
+        <v>37</v>
+      </c>
+      <c r="AM22" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="AL22" s="12">
-        <v>33</v>
-      </c>
-      <c r="AM22" s="13" t="s">
-        <v>115</v>
-      </c>
       <c r="AN22" s="12">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="AO22" s="13" t="s">
         <v>121</v>
       </c>
       <c r="AP22" s="12">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="AQ22" s="13" t="s">
         <v>122</v>
       </c>
       <c r="AR22" s="12">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="AS22" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="AT22" s="12">
+        <v>1885</v>
+      </c>
+      <c r="AU22" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="AT22" s="12">
-        <v>2180</v>
-      </c>
-      <c r="AU22" s="13" t="s">
+      <c r="AV22" s="12">
+        <v>5388</v>
+      </c>
+      <c r="AW22" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="AV22" s="12">
-        <v>5315</v>
-      </c>
-      <c r="AW22" s="13" t="s">
+      <c r="AX22" s="12">
+        <v>13938</v>
+      </c>
+      <c r="AY22" s="13" t="s">
         <v>125</v>
-      </c>
-      <c r="AX22" s="12">
-        <v>13356</v>
-      </c>
-      <c r="AY22" s="13" t="s">
-        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Perbarui data SE2026 01/09/2026 13:02:59,09
</commit_message>
<xml_diff>
--- a/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
+++ b/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="313">
   <si>
     <t>DATA RADAR ANOMALI USAHA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 31 Agu 2026, 08.56</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 1 Sep 2026, 13.02</t>
   </si>
   <si>
     <t>Kode</t>
@@ -331,634 +331,613 @@
     <t>LAMPUNG</t>
   </si>
   <si>
+    <t>0,06</t>
+  </si>
+  <si>
+    <t>20,35</t>
+  </si>
+  <si>
+    <t>1,31</t>
+  </si>
+  <si>
+    <t>2,43</t>
+  </si>
+  <si>
+    <t>36,48</t>
+  </si>
+  <si>
+    <t>10,35</t>
+  </si>
+  <si>
+    <t>0,25</t>
+  </si>
+  <si>
+    <t>7,36</t>
+  </si>
+  <si>
+    <t>0,09</t>
+  </si>
+  <si>
+    <t>0,03</t>
+  </si>
+  <si>
+    <t>0,15</t>
+  </si>
+  <si>
+    <t>0,02</t>
+  </si>
+  <si>
+    <t>0,08</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>0,26</t>
+  </si>
+  <si>
+    <t>0,58</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>1,17</t>
+  </si>
+  <si>
+    <t>5,18</t>
+  </si>
+  <si>
+    <t>13,6</t>
+  </si>
+  <si>
+    <t>1801</t>
+  </si>
+  <si>
+    <t>LAMPUNG BARAT</t>
+  </si>
+  <si>
+    <t>0,04</t>
+  </si>
+  <si>
+    <t>19,58</t>
+  </si>
+  <si>
+    <t>0,98</t>
+  </si>
+  <si>
+    <t>1,44</t>
+  </si>
+  <si>
+    <t>45,01</t>
+  </si>
+  <si>
+    <t>5,43</t>
+  </si>
+  <si>
+    <t>0,24</t>
+  </si>
+  <si>
+    <t>4,49</t>
+  </si>
+  <si>
+    <t>0,01</t>
+  </si>
+  <si>
+    <t>0,2</t>
+  </si>
+  <si>
     <t>0,07</t>
   </si>
   <si>
-    <t>20,15</t>
-  </si>
-  <si>
-    <t>1,39</t>
-  </si>
-  <si>
-    <t>2,78</t>
-  </si>
-  <si>
-    <t>35,73</t>
-  </si>
-  <si>
-    <t>10,45</t>
+    <t>0,14</t>
+  </si>
+  <si>
+    <t>0,13</t>
+  </si>
+  <si>
+    <t>0,36</t>
+  </si>
+  <si>
+    <t>4,22</t>
+  </si>
+  <si>
+    <t>3,48</t>
+  </si>
+  <si>
+    <t>13,93</t>
+  </si>
+  <si>
+    <t>1802</t>
+  </si>
+  <si>
+    <t>TANGGAMUS</t>
+  </si>
+  <si>
+    <t>13,76</t>
+  </si>
+  <si>
+    <t>0,42</t>
+  </si>
+  <si>
+    <t>1,32</t>
+  </si>
+  <si>
+    <t>26,07</t>
+  </si>
+  <si>
+    <t>30,37</t>
+  </si>
+  <si>
+    <t>6,5</t>
+  </si>
+  <si>
+    <t>0,18</t>
+  </si>
+  <si>
+    <t>4,67</t>
+  </si>
+  <si>
+    <t>15,77</t>
+  </si>
+  <si>
+    <t>1803</t>
+  </si>
+  <si>
+    <t>LAMPUNG SELATAN</t>
+  </si>
+  <si>
+    <t>17,24</t>
+  </si>
+  <si>
+    <t>2,36</t>
+  </si>
+  <si>
+    <t>42,73</t>
+  </si>
+  <si>
+    <t>12,9</t>
+  </si>
+  <si>
+    <t>9,62</t>
+  </si>
+  <si>
+    <t>0,33</t>
+  </si>
+  <si>
+    <t>0,76</t>
+  </si>
+  <si>
+    <t>4,25</t>
+  </si>
+  <si>
+    <t>8,19</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>0,19</t>
+  </si>
+  <si>
+    <t>22,84</t>
+  </si>
+  <si>
+    <t>0,27</t>
+  </si>
+  <si>
+    <t>9,18</t>
+  </si>
+  <si>
+    <t>32,35</t>
+  </si>
+  <si>
+    <t>11,87</t>
+  </si>
+  <si>
+    <t>0,81</t>
+  </si>
+  <si>
+    <t>6,83</t>
+  </si>
+  <si>
+    <t>0,05</t>
+  </si>
+  <si>
+    <t>0,29</t>
+  </si>
+  <si>
+    <t>2,07</t>
+  </si>
+  <si>
+    <t>2,26</t>
+  </si>
+  <si>
+    <t>10,39</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>15,36</t>
+  </si>
+  <si>
+    <t>2,33</t>
+  </si>
+  <si>
+    <t>1,13</t>
+  </si>
+  <si>
+    <t>45,78</t>
+  </si>
+  <si>
+    <t>4,88</t>
+  </si>
+  <si>
+    <t>0,17</t>
+  </si>
+  <si>
+    <t>13,41</t>
+  </si>
+  <si>
+    <t>0,23</t>
+  </si>
+  <si>
+    <t>0,65</t>
+  </si>
+  <si>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>3,18</t>
+  </si>
+  <si>
+    <t>11,88</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>18,8</t>
+  </si>
+  <si>
+    <t>0,74</t>
+  </si>
+  <si>
+    <t>0,96</t>
+  </si>
+  <si>
+    <t>37,35</t>
+  </si>
+  <si>
+    <t>14,28</t>
+  </si>
+  <si>
+    <t>7,85</t>
+  </si>
+  <si>
+    <t>0,57</t>
+  </si>
+  <si>
+    <t>1,08</t>
+  </si>
+  <si>
+    <t>0,63</t>
+  </si>
+  <si>
+    <t>6,68</t>
+  </si>
+  <si>
+    <t>10,24</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>18,17</t>
+  </si>
+  <si>
+    <t>0,64</t>
+  </si>
+  <si>
+    <t>0,83</t>
+  </si>
+  <si>
+    <t>42,44</t>
+  </si>
+  <si>
+    <t>17,41</t>
+  </si>
+  <si>
+    <t>5,82</t>
+  </si>
+  <si>
+    <t>0,66</t>
+  </si>
+  <si>
+    <t>0,79</t>
+  </si>
+  <si>
+    <t>0,49</t>
+  </si>
+  <si>
+    <t>4,62</t>
+  </si>
+  <si>
+    <t>7,2</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>23,51</t>
+  </si>
+  <si>
+    <t>0,41</t>
+  </si>
+  <si>
+    <t>2,6</t>
+  </si>
+  <si>
+    <t>27,35</t>
+  </si>
+  <si>
+    <t>15,67</t>
+  </si>
+  <si>
+    <t>5,64</t>
+  </si>
+  <si>
+    <t>0,11</t>
+  </si>
+  <si>
+    <t>2,42</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>30,68</t>
+  </si>
+  <si>
+    <t>0,45</t>
+  </si>
+  <si>
+    <t>30,51</t>
+  </si>
+  <si>
+    <t>1,88</t>
+  </si>
+  <si>
+    <t>5,85</t>
+  </si>
+  <si>
+    <t>8,4</t>
+  </si>
+  <si>
+    <t>20,76</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>18,03</t>
+  </si>
+  <si>
+    <t>0,51</t>
+  </si>
+  <si>
+    <t>1,06</t>
+  </si>
+  <si>
+    <t>31,81</t>
+  </si>
+  <si>
+    <t>3,04</t>
+  </si>
+  <si>
+    <t>4,99</t>
+  </si>
+  <si>
+    <t>0,62</t>
+  </si>
+  <si>
+    <t>0,93</t>
+  </si>
+  <si>
+    <t>2,12</t>
+  </si>
+  <si>
+    <t>8,41</t>
+  </si>
+  <si>
+    <t>27,88</t>
+  </si>
+  <si>
+    <t>1811</t>
+  </si>
+  <si>
+    <t>MESUJI</t>
+  </si>
+  <si>
+    <t>0,21</t>
+  </si>
+  <si>
+    <t>30,06</t>
+  </si>
+  <si>
+    <t>4,09</t>
+  </si>
+  <si>
+    <t>1,57</t>
+  </si>
+  <si>
+    <t>35,88</t>
+  </si>
+  <si>
+    <t>5,76</t>
+  </si>
+  <si>
+    <t>3,62</t>
+  </si>
+  <si>
+    <t>0,54</t>
+  </si>
+  <si>
+    <t>3,17</t>
+  </si>
+  <si>
+    <t>8,59</t>
+  </si>
+  <si>
+    <t>5,55</t>
+  </si>
+  <si>
+    <t>1812</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG BARAT</t>
+  </si>
+  <si>
+    <t>16,84</t>
+  </si>
+  <si>
+    <t>1,6</t>
+  </si>
+  <si>
+    <t>2,93</t>
+  </si>
+  <si>
+    <t>31,43</t>
+  </si>
+  <si>
+    <t>16,02</t>
   </si>
   <si>
     <t>0,32</t>
   </si>
   <si>
-    <t>7,38</t>
-  </si>
-  <si>
-    <t>0,09</t>
-  </si>
-  <si>
-    <t>0,03</t>
-  </si>
-  <si>
-    <t>0,15</t>
-  </si>
-  <si>
-    <t>0,02</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>0,25</t>
-  </si>
-  <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>0,56</t>
-  </si>
-  <si>
-    <t>0,11</t>
-  </si>
-  <si>
-    <t>1,61</t>
-  </si>
-  <si>
-    <t>5,25</t>
-  </si>
-  <si>
-    <t>13,39</t>
-  </si>
-  <si>
-    <t>1801</t>
-  </si>
-  <si>
-    <t>LAMPUNG BARAT</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>20,11</t>
-  </si>
-  <si>
-    <t>0,96</t>
-  </si>
-  <si>
-    <t>3,61</t>
-  </si>
-  <si>
-    <t>45,02</t>
-  </si>
-  <si>
-    <t>2,83</t>
-  </si>
-  <si>
-    <t>0,41</t>
-  </si>
-  <si>
-    <t>4,72</t>
-  </si>
-  <si>
-    <t>0,08</t>
-  </si>
-  <si>
-    <t>0,22</t>
-  </si>
-  <si>
-    <t>0,3</t>
-  </si>
-  <si>
-    <t>9,12</t>
-  </si>
-  <si>
-    <t>3,56</t>
-  </si>
-  <si>
-    <t>8,47</t>
-  </si>
-  <si>
-    <t>1802</t>
-  </si>
-  <si>
-    <t>TANGGAMUS</t>
-  </si>
-  <si>
-    <t>13,8</t>
-  </si>
-  <si>
-    <t>0,42</t>
-  </si>
-  <si>
-    <t>1,3</t>
-  </si>
-  <si>
-    <t>26</t>
-  </si>
-  <si>
-    <t>30,46</t>
-  </si>
-  <si>
-    <t>6,52</t>
-  </si>
-  <si>
-    <t>0,06</t>
-  </si>
-  <si>
-    <t>0,24</t>
-  </si>
-  <si>
-    <t>4,68</t>
-  </si>
-  <si>
-    <t>15,82</t>
-  </si>
-  <si>
-    <t>1803</t>
-  </si>
-  <si>
-    <t>LAMPUNG SELATAN</t>
-  </si>
-  <si>
-    <t>0,01</t>
-  </si>
-  <si>
-    <t>17,33</t>
-  </si>
-  <si>
-    <t>2,47</t>
-  </si>
-  <si>
-    <t>41,62</t>
-  </si>
-  <si>
-    <t>13,5</t>
-  </si>
-  <si>
-    <t>9,7</t>
-  </si>
-  <si>
-    <t>0,34</t>
-  </si>
-  <si>
-    <t>0,74</t>
-  </si>
-  <si>
-    <t>1,07</t>
-  </si>
-  <si>
-    <t>4,32</t>
-  </si>
-  <si>
-    <t>8,41</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>0,2</t>
-  </si>
-  <si>
-    <t>22,03</t>
+    <t>5,77</t>
   </si>
   <si>
     <t>0,28</t>
   </si>
   <si>
-    <t>9,75</t>
-  </si>
-  <si>
-    <t>31,31</t>
-  </si>
-  <si>
-    <t>12,45</t>
-  </si>
-  <si>
-    <t>0,85</t>
-  </si>
-  <si>
-    <t>6,92</t>
-  </si>
-  <si>
-    <t>0,04</t>
-  </si>
-  <si>
-    <t>0,05</t>
-  </si>
-  <si>
-    <t>0,33</t>
-  </si>
-  <si>
-    <t>2,16</t>
-  </si>
-  <si>
-    <t>2,22</t>
-  </si>
-  <si>
-    <t>10,89</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>15,52</t>
-  </si>
-  <si>
-    <t>2,38</t>
-  </si>
-  <si>
-    <t>1,16</t>
-  </si>
-  <si>
-    <t>45,42</t>
-  </si>
-  <si>
-    <t>4,95</t>
-  </si>
-  <si>
-    <t>0,57</t>
-  </si>
-  <si>
-    <t>12,88</t>
-  </si>
-  <si>
-    <t>0,14</t>
-  </si>
-  <si>
-    <t>0,17</t>
-  </si>
-  <si>
-    <t>0,23</t>
-  </si>
-  <si>
-    <t>0,67</t>
-  </si>
-  <si>
-    <t>0,31</t>
-  </si>
-  <si>
-    <t>3,23</t>
-  </si>
-  <si>
-    <t>11,88</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>18,84</t>
-  </si>
-  <si>
-    <t>0,75</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>37,2</t>
-  </si>
-  <si>
-    <t>14,32</t>
-  </si>
-  <si>
-    <t>7,79</t>
-  </si>
-  <si>
-    <t>0,26</t>
-  </si>
-  <si>
-    <t>0,18</t>
-  </si>
-  <si>
-    <t>1,08</t>
-  </si>
-  <si>
-    <t>0,63</t>
-  </si>
-  <si>
-    <t>6,71</t>
-  </si>
-  <si>
-    <t>10,27</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>18,23</t>
-  </si>
-  <si>
-    <t>0,65</t>
-  </si>
-  <si>
-    <t>1,97</t>
-  </si>
-  <si>
-    <t>41,5</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>5,78</t>
-  </si>
-  <si>
-    <t>0,76</t>
-  </si>
-  <si>
-    <t>0,5</t>
+    <t>4,2</t>
+  </si>
+  <si>
+    <t>19,81</t>
+  </si>
+  <si>
+    <t>1813</t>
+  </si>
+  <si>
+    <t>PESISIR BARAT</t>
+  </si>
+  <si>
+    <t>12,13</t>
+  </si>
+  <si>
+    <t>0,38</t>
+  </si>
+  <si>
+    <t>42,76</t>
+  </si>
+  <si>
+    <t>16,95</t>
+  </si>
+  <si>
+    <t>10,14</t>
+  </si>
+  <si>
+    <t>6,95</t>
+  </si>
+  <si>
+    <t>9,33</t>
+  </si>
+  <si>
+    <t>1871</t>
+  </si>
+  <si>
+    <t>BANDAR LAMPUNG</t>
+  </si>
+  <si>
+    <t>15,56</t>
+  </si>
+  <si>
+    <t>3,46</t>
+  </si>
+  <si>
+    <t>31,41</t>
   </si>
   <si>
     <t>4,61</t>
   </si>
   <si>
-    <t>7,25</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>23,51</t>
-  </si>
-  <si>
-    <t>2,61</t>
-  </si>
-  <si>
-    <t>27,35</t>
-  </si>
-  <si>
-    <t>15,68</t>
-  </si>
-  <si>
-    <t>5,64</t>
-  </si>
-  <si>
-    <t>0,64</t>
-  </si>
-  <si>
-    <t>2,45</t>
-  </si>
-  <si>
-    <t>7,36</t>
-  </si>
-  <si>
-    <t>13,37</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>30,69</t>
-  </si>
-  <si>
-    <t>0,45</t>
-  </si>
-  <si>
-    <t>30,26</t>
-  </si>
-  <si>
-    <t>1,88</t>
-  </si>
-  <si>
-    <t>5,84</t>
-  </si>
-  <si>
-    <t>0,16</t>
-  </si>
-  <si>
-    <t>8,42</t>
-  </si>
-  <si>
-    <t>20,67</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>17,87</t>
-  </si>
-  <si>
-    <t>0,46</t>
-  </si>
-  <si>
-    <t>1,18</t>
-  </si>
-  <si>
-    <t>31,35</t>
-  </si>
-  <si>
-    <t>3,1</t>
-  </si>
-  <si>
-    <t>5,02</t>
-  </si>
-  <si>
-    <t>0,61</t>
-  </si>
-  <si>
-    <t>3,32</t>
-  </si>
-  <si>
-    <t>8,38</t>
-  </si>
-  <si>
-    <t>27,29</t>
-  </si>
-  <si>
-    <t>1811</t>
-  </si>
-  <si>
-    <t>MESUJI</t>
-  </si>
-  <si>
-    <t>29,29</t>
-  </si>
-  <si>
-    <t>5,24</t>
-  </si>
-  <si>
-    <t>1,91</t>
-  </si>
-  <si>
-    <t>33,17</t>
-  </si>
-  <si>
-    <t>6,18</t>
-  </si>
-  <si>
-    <t>0,29</t>
-  </si>
-  <si>
-    <t>3,67</t>
-  </si>
-  <si>
-    <t>0,13</t>
-  </si>
-  <si>
-    <t>3,71</t>
-  </si>
-  <si>
-    <t>8,89</t>
-  </si>
-  <si>
-    <t>6,09</t>
-  </si>
-  <si>
-    <t>1812</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG BARAT</t>
-  </si>
-  <si>
-    <t>16,79</t>
-  </si>
-  <si>
-    <t>1,68</t>
-  </si>
-  <si>
-    <t>3,57</t>
-  </si>
-  <si>
-    <t>30,27</t>
-  </si>
-  <si>
-    <t>16,32</t>
-  </si>
-  <si>
-    <t>0,35</t>
-  </si>
-  <si>
-    <t>5,68</t>
-  </si>
-  <si>
-    <t>4,37</t>
-  </si>
-  <si>
-    <t>19,03</t>
-  </si>
-  <si>
-    <t>1813</t>
-  </si>
-  <si>
-    <t>PESISIR BARAT</t>
-  </si>
-  <si>
-    <t>12,2</t>
-  </si>
-  <si>
-    <t>42,48</t>
-  </si>
-  <si>
-    <t>10,17</t>
-  </si>
-  <si>
-    <t>0,19</t>
-  </si>
-  <si>
-    <t>0,21</t>
-  </si>
-  <si>
-    <t>6,99</t>
-  </si>
-  <si>
-    <t>9,35</t>
-  </si>
-  <si>
-    <t>1871</t>
-  </si>
-  <si>
-    <t>BANDAR LAMPUNG</t>
-  </si>
-  <si>
-    <t>15,38</t>
-  </si>
-  <si>
-    <t>0,58</t>
-  </si>
-  <si>
-    <t>3,87</t>
-  </si>
-  <si>
-    <t>30,85</t>
-  </si>
-  <si>
-    <t>4,64</t>
-  </si>
-  <si>
-    <t>0,68</t>
-  </si>
-  <si>
-    <t>16,15</t>
-  </si>
-  <si>
-    <t>0,87</t>
+    <t>16,14</t>
+  </si>
+  <si>
+    <t>0,86</t>
+  </si>
+  <si>
+    <t>1,73</t>
+  </si>
+  <si>
+    <t>4,51</t>
+  </si>
+  <si>
+    <t>17,77</t>
+  </si>
+  <si>
+    <t>1872</t>
+  </si>
+  <si>
+    <t>METRO</t>
+  </si>
+  <si>
+    <t>16,07</t>
+  </si>
+  <si>
+    <t>6,22</t>
+  </si>
+  <si>
+    <t>29,44</t>
+  </si>
+  <si>
+    <t>4,12</t>
+  </si>
+  <si>
+    <t>3,19</t>
+  </si>
+  <si>
+    <t>0,69</t>
+  </si>
+  <si>
+    <t>0,73</t>
   </si>
   <si>
     <t>1,74</t>
-  </si>
-  <si>
-    <t>0,39</t>
-  </si>
-  <si>
-    <t>1,26</t>
-  </si>
-  <si>
-    <t>4,55</t>
-  </si>
-  <si>
-    <t>17,7</t>
-  </si>
-  <si>
-    <t>1872</t>
-  </si>
-  <si>
-    <t>METRO</t>
-  </si>
-  <si>
-    <t>16,07</t>
-  </si>
-  <si>
-    <t>6,22</t>
-  </si>
-  <si>
-    <t>29,4</t>
-  </si>
-  <si>
-    <t>4,12</t>
-  </si>
-  <si>
-    <t>3,19</t>
-  </si>
-  <si>
-    <t>0,69</t>
-  </si>
-  <si>
-    <t>0,73</t>
-  </si>
-  <si>
-    <t>1,78</t>
   </si>
   <si>
     <t>3,88</t>
@@ -1944,148 +1923,148 @@
         <v>105</v>
       </c>
       <c r="C6" s="6">
-        <v>106882</v>
+        <v>111025</v>
       </c>
       <c r="D6" s="6">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>106</v>
       </c>
       <c r="F6" s="6">
-        <v>21538</v>
+        <v>22589</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>107</v>
       </c>
       <c r="H6" s="6">
-        <v>1482</v>
+        <v>1450</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>108</v>
       </c>
       <c r="J6" s="6">
-        <v>2973</v>
+        <v>2698</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>109</v>
       </c>
       <c r="L6" s="6">
-        <v>38187</v>
+        <v>40497</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>110</v>
       </c>
       <c r="N6" s="6">
-        <v>11171</v>
+        <v>11488</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>111</v>
       </c>
       <c r="P6" s="6">
-        <v>344</v>
+        <v>276</v>
       </c>
       <c r="Q6" s="7" t="s">
         <v>112</v>
       </c>
       <c r="R6" s="6">
-        <v>7893</v>
+        <v>8174</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>113</v>
       </c>
       <c r="T6" s="6">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="U6" s="7" t="s">
         <v>114</v>
       </c>
       <c r="V6" s="6">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="W6" s="7" t="s">
         <v>115</v>
       </c>
       <c r="X6" s="6">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="Y6" s="7" t="s">
         <v>116</v>
       </c>
       <c r="Z6" s="6">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="AA6" s="7" t="s">
         <v>117</v>
       </c>
       <c r="AB6" s="6">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="AC6" s="7" t="s">
         <v>115</v>
       </c>
       <c r="AD6" s="6">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="AE6" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="AF6" s="6">
         <v>1</v>
       </c>
       <c r="AG6" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH6" s="6">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="AI6" s="7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AJ6" s="6">
-        <v>264</v>
+        <v>284</v>
       </c>
       <c r="AK6" s="7" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AL6" s="6">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="AM6" s="7" t="s">
         <v>115</v>
       </c>
       <c r="AN6" s="6">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="AO6" s="7" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="AP6" s="6">
-        <v>601</v>
+        <v>649</v>
       </c>
       <c r="AQ6" s="7" t="s">
         <v>121</v>
       </c>
       <c r="AR6" s="6">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="AS6" s="7" t="s">
         <v>122</v>
       </c>
       <c r="AT6" s="6">
-        <v>1723</v>
+        <v>1296</v>
       </c>
       <c r="AU6" s="7" t="s">
         <v>123</v>
       </c>
       <c r="AV6" s="6">
-        <v>5607</v>
+        <v>5755</v>
       </c>
       <c r="AW6" s="7" t="s">
         <v>124</v>
       </c>
       <c r="AX6" s="6">
-        <v>14316</v>
+        <v>15094</v>
       </c>
       <c r="AY6" s="7" t="s">
         <v>125</v>
@@ -2099,240 +2078,240 @@
         <v>127</v>
       </c>
       <c r="C7" s="9">
-        <v>6042</v>
+        <v>7012</v>
       </c>
       <c r="D7" s="9">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>128</v>
       </c>
       <c r="F7" s="9">
-        <v>1215</v>
+        <v>1373</v>
       </c>
       <c r="G7" s="10" t="s">
         <v>129</v>
       </c>
       <c r="H7" s="9">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="I7" s="10" t="s">
         <v>130</v>
       </c>
       <c r="J7" s="9">
-        <v>218</v>
+        <v>101</v>
       </c>
       <c r="K7" s="10" t="s">
         <v>131</v>
       </c>
       <c r="L7" s="9">
-        <v>2720</v>
+        <v>3156</v>
       </c>
       <c r="M7" s="10" t="s">
         <v>132</v>
       </c>
       <c r="N7" s="9">
-        <v>171</v>
+        <v>381</v>
       </c>
       <c r="O7" s="10" t="s">
         <v>133</v>
       </c>
       <c r="P7" s="9">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="Q7" s="10" t="s">
         <v>134</v>
       </c>
       <c r="R7" s="9">
-        <v>285</v>
+        <v>315</v>
       </c>
       <c r="S7" s="10" t="s">
         <v>135</v>
       </c>
       <c r="T7" s="9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U7" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="V7" s="9">
+        <v>1</v>
+      </c>
+      <c r="W7" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="X7" s="9">
+        <v>14</v>
+      </c>
+      <c r="Y7" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="Z7" s="9">
         <v>2</v>
       </c>
-      <c r="W7" s="10" t="s">
+      <c r="AA7" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="X7" s="9">
-        <v>9</v>
-      </c>
-      <c r="Y7" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="Z7" s="9">
-        <v>1</v>
-      </c>
-      <c r="AA7" s="10" t="s">
-        <v>117</v>
-      </c>
       <c r="AB7" s="9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AC7" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="AD7" s="9">
         <v>5</v>
       </c>
       <c r="AE7" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="AF7" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG7" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="AH7" s="9">
+        <v>1</v>
+      </c>
+      <c r="AI7" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="AF7" s="9">
-        <v>0</v>
-      </c>
-      <c r="AG7" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="AH7" s="9">
-        <v>2</v>
-      </c>
-      <c r="AI7" s="10" t="s">
-        <v>115</v>
-      </c>
       <c r="AJ7" s="9">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="AK7" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="AL7" s="9">
+        <v>1</v>
+      </c>
+      <c r="AM7" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="AN7" s="9">
+        <v>9</v>
+      </c>
+      <c r="AO7" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="AP7" s="9">
+        <v>25</v>
+      </c>
+      <c r="AQ7" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="AR7" s="9">
+        <v>3</v>
+      </c>
+      <c r="AS7" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="AL7" s="9">
-        <v>0</v>
-      </c>
-      <c r="AM7" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="AN7" s="9">
-        <v>13</v>
-      </c>
-      <c r="AO7" s="10" t="s">
-        <v>137</v>
-      </c>
-      <c r="AP7" s="9">
-        <v>18</v>
-      </c>
-      <c r="AQ7" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="AR7" s="9">
-        <v>2</v>
-      </c>
-      <c r="AS7" s="10" t="s">
-        <v>115</v>
-      </c>
       <c r="AT7" s="9">
-        <v>551</v>
+        <v>296</v>
       </c>
       <c r="AU7" s="10" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="AV7" s="9">
-        <v>215</v>
+        <v>244</v>
       </c>
       <c r="AW7" s="10" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="AX7" s="9">
-        <v>512</v>
+        <v>977</v>
       </c>
       <c r="AY7" s="10" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="C8" s="9">
-        <v>3312</v>
+        <v>3322</v>
       </c>
       <c r="D8" s="9">
         <v>0</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F8" s="9">
         <v>457</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="H8" s="9">
         <v>14</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="J8" s="9">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="L8" s="9">
-        <v>861</v>
+        <v>866</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="N8" s="9">
         <v>1009</v>
       </c>
       <c r="O8" s="10" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="P8" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q8" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="R8" s="9">
         <v>216</v>
       </c>
       <c r="S8" s="10" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="T8" s="9">
         <v>0</v>
       </c>
       <c r="U8" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="V8" s="9">
         <v>0</v>
       </c>
       <c r="W8" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="X8" s="9">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Y8" s="10" t="s">
-        <v>114</v>
+        <v>153</v>
       </c>
       <c r="Z8" s="9">
         <v>0</v>
       </c>
       <c r="AA8" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AB8" s="9">
         <v>0</v>
       </c>
       <c r="AC8" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AD8" s="9">
         <v>1</v>
@@ -2344,13 +2323,13 @@
         <v>0</v>
       </c>
       <c r="AG8" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH8" s="9">
         <v>0</v>
       </c>
       <c r="AI8" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AJ8" s="9">
         <v>5</v>
@@ -2362,174 +2341,174 @@
         <v>0</v>
       </c>
       <c r="AM8" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AN8" s="9">
         <v>0</v>
       </c>
       <c r="AO8" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AP8" s="9">
         <v>14</v>
       </c>
       <c r="AQ8" s="10" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="AR8" s="9">
         <v>2</v>
       </c>
       <c r="AS8" s="10" t="s">
-        <v>150</v>
+        <v>106</v>
       </c>
       <c r="AT8" s="9">
         <v>8</v>
       </c>
       <c r="AU8" s="10" t="s">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="AV8" s="9">
         <v>155</v>
       </c>
       <c r="AW8" s="10" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="AX8" s="9">
         <v>524</v>
       </c>
       <c r="AY8" s="10" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C9" s="9">
-        <v>8125</v>
+        <v>8380</v>
       </c>
       <c r="D9" s="9">
         <v>1</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>156</v>
+        <v>136</v>
       </c>
       <c r="F9" s="9">
-        <v>1408</v>
+        <v>1445</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H9" s="9">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J9" s="9">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="L9" s="9">
-        <v>3382</v>
+        <v>3581</v>
       </c>
       <c r="M9" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N9" s="9">
-        <v>1097</v>
+        <v>1081</v>
       </c>
       <c r="O9" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="P9" s="9">
         <v>1</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>156</v>
+        <v>136</v>
       </c>
       <c r="R9" s="9">
-        <v>788</v>
+        <v>806</v>
       </c>
       <c r="S9" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T9" s="9">
         <v>8</v>
       </c>
       <c r="U9" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="V9" s="9">
         <v>1</v>
       </c>
       <c r="W9" s="10" t="s">
-        <v>156</v>
+        <v>136</v>
       </c>
       <c r="X9" s="9">
         <v>28</v>
       </c>
       <c r="Y9" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="Z9" s="9">
         <v>0</v>
       </c>
       <c r="AA9" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AB9" s="9">
         <v>0</v>
       </c>
       <c r="AC9" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AD9" s="9">
         <v>8</v>
       </c>
       <c r="AE9" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="AF9" s="9">
         <v>1</v>
       </c>
       <c r="AG9" s="10" t="s">
-        <v>156</v>
+        <v>136</v>
       </c>
       <c r="AH9" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI9" s="10" t="s">
-        <v>156</v>
+        <v>119</v>
       </c>
       <c r="AJ9" s="9">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="AK9" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="AL9" s="9">
         <v>0</v>
       </c>
       <c r="AM9" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AN9" s="9">
         <v>0</v>
       </c>
       <c r="AO9" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AP9" s="9">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="AQ9" s="10" t="s">
-        <v>164</v>
+        <v>123</v>
       </c>
       <c r="AR9" s="9">
         <v>2</v>
@@ -2541,16 +2520,16 @@
         <v>7</v>
       </c>
       <c r="AU9" s="10" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="AV9" s="9">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="AW9" s="10" t="s">
         <v>165</v>
       </c>
       <c r="AX9" s="9">
-        <v>683</v>
+        <v>686</v>
       </c>
       <c r="AY9" s="10" t="s">
         <v>166</v>
@@ -2564,7 +2543,7 @@
         <v>168</v>
       </c>
       <c r="C10" s="9">
-        <v>17324</v>
+        <v>18227</v>
       </c>
       <c r="D10" s="9">
         <v>35</v>
@@ -2573,7 +2552,7 @@
         <v>169</v>
       </c>
       <c r="F10" s="9">
-        <v>3817</v>
+        <v>4163</v>
       </c>
       <c r="G10" s="10" t="s">
         <v>170</v>
@@ -2585,31 +2564,31 @@
         <v>171</v>
       </c>
       <c r="J10" s="9">
-        <v>1689</v>
+        <v>1673</v>
       </c>
       <c r="K10" s="10" t="s">
         <v>172</v>
       </c>
       <c r="L10" s="9">
-        <v>5424</v>
+        <v>5897</v>
       </c>
       <c r="M10" s="10" t="s">
         <v>173</v>
       </c>
       <c r="N10" s="9">
-        <v>2156</v>
+        <v>2164</v>
       </c>
       <c r="O10" s="10" t="s">
         <v>174</v>
       </c>
       <c r="P10" s="9">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="Q10" s="10" t="s">
         <v>175</v>
       </c>
       <c r="R10" s="9">
-        <v>1199</v>
+        <v>1245</v>
       </c>
       <c r="S10" s="10" t="s">
         <v>176</v>
@@ -2618,180 +2597,180 @@
         <v>10</v>
       </c>
       <c r="U10" s="10" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="V10" s="9">
         <v>7</v>
       </c>
       <c r="W10" s="10" t="s">
-        <v>177</v>
+        <v>128</v>
       </c>
       <c r="X10" s="9">
         <v>14</v>
       </c>
       <c r="Y10" s="10" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z10" s="9">
         <v>2</v>
       </c>
       <c r="AA10" s="10" t="s">
-        <v>156</v>
+        <v>136</v>
       </c>
       <c r="AB10" s="9">
         <v>12</v>
       </c>
       <c r="AC10" s="10" t="s">
-        <v>106</v>
+        <v>138</v>
       </c>
       <c r="AD10" s="9">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="AE10" s="10" t="s">
-        <v>178</v>
+        <v>138</v>
       </c>
       <c r="AF10" s="9">
         <v>0</v>
       </c>
       <c r="AG10" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH10" s="9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AI10" s="10" t="s">
-        <v>178</v>
+        <v>128</v>
       </c>
       <c r="AJ10" s="9">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="AK10" s="10" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="AL10" s="9">
         <v>1</v>
       </c>
       <c r="AM10" s="10" t="s">
-        <v>156</v>
+        <v>136</v>
       </c>
       <c r="AN10" s="9">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="AO10" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="AP10" s="9">
+        <v>28</v>
+      </c>
+      <c r="AQ10" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="AR10" s="9">
+        <v>10</v>
+      </c>
+      <c r="AS10" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="AT10" s="9">
+        <v>378</v>
+      </c>
+      <c r="AU10" s="10" t="s">
         <v>179</v>
       </c>
-      <c r="AP10" s="9">
-        <v>20</v>
-      </c>
-      <c r="AQ10" s="10" t="s">
-        <v>128</v>
-      </c>
-      <c r="AR10" s="9">
-        <v>9</v>
-      </c>
-      <c r="AS10" s="10" t="s">
-        <v>178</v>
-      </c>
-      <c r="AT10" s="9">
-        <v>375</v>
-      </c>
-      <c r="AU10" s="10" t="s">
+      <c r="AV10" s="9">
+        <v>412</v>
+      </c>
+      <c r="AW10" s="10" t="s">
         <v>180</v>
       </c>
-      <c r="AV10" s="9">
-        <v>385</v>
-      </c>
-      <c r="AW10" s="10" t="s">
+      <c r="AX10" s="9">
+        <v>1894</v>
+      </c>
+      <c r="AY10" s="10" t="s">
         <v>181</v>
-      </c>
-      <c r="AX10" s="9">
-        <v>1887</v>
-      </c>
-      <c r="AY10" s="10" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>184</v>
-      </c>
       <c r="C11" s="9">
-        <v>12624</v>
+        <v>12842</v>
       </c>
       <c r="D11" s="9">
         <v>5</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>177</v>
+        <v>128</v>
       </c>
       <c r="F11" s="9">
-        <v>1959</v>
+        <v>1973</v>
       </c>
       <c r="G11" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="H11" s="9">
+        <v>299</v>
+      </c>
+      <c r="I11" s="10" t="s">
         <v>185</v>
       </c>
-      <c r="H11" s="9">
-        <v>300</v>
-      </c>
-      <c r="I11" s="10" t="s">
+      <c r="J11" s="9">
+        <v>145</v>
+      </c>
+      <c r="K11" s="10" t="s">
         <v>186</v>
       </c>
-      <c r="J11" s="9">
-        <v>147</v>
-      </c>
-      <c r="K11" s="10" t="s">
+      <c r="L11" s="9">
+        <v>5879</v>
+      </c>
+      <c r="M11" s="10" t="s">
         <v>187</v>
       </c>
-      <c r="L11" s="9">
-        <v>5734</v>
-      </c>
-      <c r="M11" s="10" t="s">
+      <c r="N11" s="9">
+        <v>627</v>
+      </c>
+      <c r="O11" s="10" t="s">
         <v>188</v>
       </c>
-      <c r="N11" s="9">
-        <v>625</v>
-      </c>
-      <c r="O11" s="10" t="s">
+      <c r="P11" s="9">
+        <v>22</v>
+      </c>
+      <c r="Q11" s="10" t="s">
         <v>189</v>
       </c>
-      <c r="P11" s="9">
-        <v>72</v>
-      </c>
-      <c r="Q11" s="10" t="s">
+      <c r="R11" s="9">
+        <v>1722</v>
+      </c>
+      <c r="S11" s="10" t="s">
         <v>190</v>
-      </c>
-      <c r="R11" s="9">
-        <v>1626</v>
-      </c>
-      <c r="S11" s="10" t="s">
-        <v>191</v>
       </c>
       <c r="T11" s="9">
         <v>18</v>
       </c>
       <c r="U11" s="10" t="s">
-        <v>192</v>
+        <v>139</v>
       </c>
       <c r="V11" s="9">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="W11" s="10" t="s">
-        <v>150</v>
+        <v>128</v>
       </c>
       <c r="X11" s="9">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Y11" s="10" t="s">
-        <v>136</v>
+        <v>114</v>
       </c>
       <c r="Z11" s="9">
         <v>5</v>
       </c>
       <c r="AA11" s="10" t="s">
-        <v>177</v>
+        <v>128</v>
       </c>
       <c r="AB11" s="9">
         <v>3</v>
@@ -2803,16 +2782,16 @@
         <v>22</v>
       </c>
       <c r="AE11" s="10" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="AF11" s="9">
         <v>0</v>
       </c>
       <c r="AG11" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH11" s="9">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AI11" s="10" t="s">
         <v>177</v>
@@ -2821,7 +2800,7 @@
         <v>29</v>
       </c>
       <c r="AK11" s="10" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="AL11" s="9">
         <v>3</v>
@@ -2830,171 +2809,171 @@
         <v>117</v>
       </c>
       <c r="AN11" s="9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AO11" s="10" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="AP11" s="9">
         <v>84</v>
       </c>
       <c r="AQ11" s="10" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="AR11" s="9">
         <v>15</v>
       </c>
       <c r="AS11" s="10" t="s">
-        <v>128</v>
+        <v>193</v>
       </c>
       <c r="AT11" s="9">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="AU11" s="10" t="s">
-        <v>196</v>
+        <v>137</v>
       </c>
       <c r="AV11" s="9">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AW11" s="10" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="AX11" s="9">
-        <v>1500</v>
+        <v>1525</v>
       </c>
       <c r="AY11" s="10" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="C12" s="9">
-        <v>5084</v>
+        <v>5106</v>
       </c>
       <c r="D12" s="9">
         <v>0</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F12" s="9">
-        <v>958</v>
+        <v>960</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="H12" s="9">
         <v>38</v>
       </c>
       <c r="I12" s="10" t="s">
+        <v>199</v>
+      </c>
+      <c r="J12" s="9">
+        <v>49</v>
+      </c>
+      <c r="K12" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="L12" s="9">
+        <v>1907</v>
+      </c>
+      <c r="M12" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="N12" s="9">
+        <v>729</v>
+      </c>
+      <c r="O12" s="10" t="s">
         <v>202</v>
       </c>
-      <c r="J12" s="9">
-        <v>51</v>
-      </c>
-      <c r="K12" s="10" t="s">
+      <c r="P12" s="9">
+        <v>3</v>
+      </c>
+      <c r="Q12" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="R12" s="9">
+        <v>401</v>
+      </c>
+      <c r="S12" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="L12" s="9">
-        <v>1891</v>
-      </c>
-      <c r="M12" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="N12" s="9">
-        <v>728</v>
-      </c>
-      <c r="O12" s="10" t="s">
-        <v>205</v>
-      </c>
-      <c r="P12" s="9">
-        <v>4</v>
-      </c>
-      <c r="Q12" s="10" t="s">
-        <v>136</v>
-      </c>
-      <c r="R12" s="9">
-        <v>396</v>
-      </c>
-      <c r="S12" s="10" t="s">
-        <v>206</v>
-      </c>
       <c r="T12" s="9">
         <v>0</v>
       </c>
       <c r="U12" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="V12" s="9">
         <v>5</v>
       </c>
       <c r="W12" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="X12" s="9">
         <v>13</v>
       </c>
       <c r="Y12" s="10" t="s">
-        <v>207</v>
+        <v>112</v>
       </c>
       <c r="Z12" s="9">
         <v>2</v>
       </c>
       <c r="AA12" s="10" t="s">
-        <v>177</v>
+        <v>128</v>
       </c>
       <c r="AB12" s="9">
         <v>3</v>
       </c>
       <c r="AC12" s="10" t="s">
-        <v>150</v>
+        <v>106</v>
       </c>
       <c r="AD12" s="9">
         <v>9</v>
       </c>
       <c r="AE12" s="10" t="s">
-        <v>208</v>
+        <v>153</v>
       </c>
       <c r="AF12" s="9">
         <v>0</v>
       </c>
       <c r="AG12" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH12" s="9">
         <v>2</v>
       </c>
       <c r="AI12" s="10" t="s">
-        <v>177</v>
+        <v>128</v>
       </c>
       <c r="AJ12" s="9">
         <v>29</v>
       </c>
       <c r="AK12" s="10" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="AL12" s="9">
         <v>0</v>
       </c>
       <c r="AM12" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AN12" s="9">
         <v>4</v>
       </c>
       <c r="AO12" s="10" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="AP12" s="9">
         <v>55</v>
       </c>
       <c r="AQ12" s="10" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="AR12" s="9">
         <v>1</v>
@@ -3006,120 +2985,120 @@
         <v>32</v>
       </c>
       <c r="AU12" s="10" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="AV12" s="9">
         <v>341</v>
       </c>
       <c r="AW12" s="10" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="AX12" s="9">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AY12" s="10" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="C13" s="9">
-        <v>4619</v>
+        <v>4694</v>
       </c>
       <c r="D13" s="9">
         <v>0</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F13" s="9">
-        <v>842</v>
+        <v>853</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="H13" s="9">
         <v>30</v>
       </c>
       <c r="I13" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="J13" s="9">
+        <v>39</v>
+      </c>
+      <c r="K13" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="L13" s="9">
+        <v>1992</v>
+      </c>
+      <c r="M13" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="N13" s="9">
+        <v>817</v>
+      </c>
+      <c r="O13" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="P13" s="9">
+        <v>9</v>
+      </c>
+      <c r="Q13" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="R13" s="9">
+        <v>273</v>
+      </c>
+      <c r="S13" s="10" t="s">
         <v>216</v>
       </c>
-      <c r="J13" s="9">
-        <v>91</v>
-      </c>
-      <c r="K13" s="10" t="s">
-        <v>217</v>
-      </c>
-      <c r="L13" s="9">
-        <v>1917</v>
-      </c>
-      <c r="M13" s="10" t="s">
-        <v>218</v>
-      </c>
-      <c r="N13" s="9">
-        <v>785</v>
-      </c>
-      <c r="O13" s="10" t="s">
-        <v>219</v>
-      </c>
-      <c r="P13" s="9">
-        <v>11</v>
-      </c>
-      <c r="Q13" s="10" t="s">
-        <v>151</v>
-      </c>
-      <c r="R13" s="9">
-        <v>267</v>
-      </c>
-      <c r="S13" s="10" t="s">
-        <v>220</v>
-      </c>
       <c r="T13" s="9">
         <v>0</v>
       </c>
       <c r="U13" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="V13" s="9">
         <v>2</v>
       </c>
       <c r="W13" s="10" t="s">
-        <v>177</v>
+        <v>128</v>
       </c>
       <c r="X13" s="9">
         <v>3</v>
       </c>
       <c r="Y13" s="10" t="s">
-        <v>150</v>
+        <v>106</v>
       </c>
       <c r="Z13" s="9">
         <v>0</v>
       </c>
       <c r="AA13" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AB13" s="9">
         <v>0</v>
       </c>
       <c r="AC13" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AD13" s="9">
         <v>8</v>
       </c>
       <c r="AE13" s="10" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="AF13" s="9">
         <v>0</v>
       </c>
       <c r="AG13" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH13" s="9">
         <v>1</v>
@@ -3128,117 +3107,117 @@
         <v>117</v>
       </c>
       <c r="AJ13" s="9">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="AK13" s="10" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="AL13" s="9">
         <v>11</v>
       </c>
       <c r="AM13" s="10" t="s">
-        <v>151</v>
+        <v>191</v>
       </c>
       <c r="AN13" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AO13" s="10" t="s">
-        <v>177</v>
+        <v>117</v>
       </c>
       <c r="AP13" s="9">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="AQ13" s="10" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="AR13" s="9">
         <v>23</v>
       </c>
       <c r="AS13" s="10" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="AT13" s="9">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="AU13" s="10" t="s">
-        <v>138</v>
+        <v>169</v>
       </c>
       <c r="AV13" s="9">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="AW13" s="10" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="AX13" s="9">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="AY13" s="10" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="C14" s="9">
-        <v>4376</v>
+        <v>4377</v>
       </c>
       <c r="D14" s="9">
         <v>0</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F14" s="9">
         <v>1029</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="H14" s="9">
         <v>18</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>134</v>
+        <v>225</v>
       </c>
       <c r="J14" s="9">
         <v>114</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="L14" s="9">
         <v>1197</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="N14" s="9">
         <v>686</v>
       </c>
       <c r="O14" s="10" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="P14" s="9">
         <v>8</v>
       </c>
       <c r="Q14" s="10" t="s">
-        <v>208</v>
+        <v>153</v>
       </c>
       <c r="R14" s="9">
         <v>247</v>
       </c>
       <c r="S14" s="10" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="T14" s="9">
         <v>2</v>
       </c>
       <c r="U14" s="10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="V14" s="9">
         <v>1</v>
@@ -3250,7 +3229,7 @@
         <v>8</v>
       </c>
       <c r="Y14" s="10" t="s">
-        <v>208</v>
+        <v>153</v>
       </c>
       <c r="Z14" s="9">
         <v>1</v>
@@ -3268,13 +3247,13 @@
         <v>5</v>
       </c>
       <c r="AE14" s="10" t="s">
-        <v>122</v>
+        <v>230</v>
       </c>
       <c r="AF14" s="9">
         <v>0</v>
       </c>
       <c r="AG14" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH14" s="9">
         <v>1</v>
@@ -3286,7 +3265,7 @@
         <v>11</v>
       </c>
       <c r="AK14" s="10" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="AL14" s="9">
         <v>1</v>
@@ -3298,13 +3277,13 @@
         <v>3</v>
       </c>
       <c r="AO14" s="10" t="s">
-        <v>106</v>
+        <v>138</v>
       </c>
       <c r="AP14" s="9">
         <v>28</v>
       </c>
       <c r="AQ14" s="10" t="s">
-        <v>232</v>
+        <v>212</v>
       </c>
       <c r="AR14" s="9">
         <v>1</v>
@@ -3313,111 +3292,111 @@
         <v>117</v>
       </c>
       <c r="AT14" s="9">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="AU14" s="10" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="AV14" s="9">
         <v>322</v>
       </c>
       <c r="AW14" s="10" t="s">
-        <v>234</v>
+        <v>113</v>
       </c>
       <c r="AX14" s="9">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="AY14" s="10" t="s">
-        <v>235</v>
+        <v>190</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="C15" s="9">
-        <v>12421</v>
+        <v>12522</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F15" s="9">
-        <v>3812</v>
+        <v>3842</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="H15" s="9">
         <v>56</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="J15" s="9">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="L15" s="9">
-        <v>3758</v>
+        <v>3821</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="N15" s="9">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="P15" s="9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>115</v>
+        <v>136</v>
       </c>
       <c r="R15" s="9">
-        <v>726</v>
+        <v>733</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="T15" s="9">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>196</v>
+        <v>163</v>
       </c>
       <c r="V15" s="9">
         <v>0</v>
       </c>
       <c r="W15" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="X15" s="9">
         <v>15</v>
       </c>
       <c r="Y15" s="10" t="s">
-        <v>128</v>
+        <v>193</v>
       </c>
       <c r="Z15" s="9">
         <v>0</v>
       </c>
       <c r="AA15" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AB15" s="9">
         <v>0</v>
       </c>
       <c r="AC15" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AD15" s="9">
         <v>3</v>
@@ -3429,13 +3408,13 @@
         <v>0</v>
       </c>
       <c r="AG15" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH15" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AI15" s="10" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="AJ15" s="9">
         <v>11</v>
@@ -3444,272 +3423,272 @@
         <v>114</v>
       </c>
       <c r="AL15" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AM15" s="10" t="s">
         <v>117</v>
       </c>
       <c r="AN15" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AO15" s="10" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="AP15" s="9">
         <v>79</v>
       </c>
       <c r="AQ15" s="10" t="s">
-        <v>232</v>
+        <v>206</v>
       </c>
       <c r="AR15" s="9">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AS15" s="10" t="s">
-        <v>192</v>
+        <v>116</v>
       </c>
       <c r="AT15" s="9">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="AU15" s="10" t="s">
-        <v>243</v>
+        <v>117</v>
       </c>
       <c r="AV15" s="9">
-        <v>1046</v>
+        <v>1052</v>
       </c>
       <c r="AW15" s="10" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="AX15" s="9">
-        <v>2568</v>
+        <v>2600</v>
       </c>
       <c r="AY15" s="10" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="C16" s="9">
+        <v>4709</v>
+      </c>
+      <c r="D16" s="9">
+        <v>2</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="F16" s="9">
+        <v>849</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="H16" s="9">
+        <v>24</v>
+      </c>
+      <c r="I16" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="J16" s="9">
+        <v>50</v>
+      </c>
+      <c r="K16" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="L16" s="9">
+        <v>1498</v>
+      </c>
+      <c r="M16" s="10" t="s">
         <v>246</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="N16" s="9">
+        <v>143</v>
+      </c>
+      <c r="O16" s="10" t="s">
         <v>247</v>
       </c>
-      <c r="C16" s="9">
-        <v>4584</v>
-      </c>
-      <c r="D16" s="9">
+      <c r="P16" s="9">
+        <v>2</v>
+      </c>
+      <c r="Q16" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="R16" s="9">
+        <v>235</v>
+      </c>
+      <c r="S16" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="T16" s="9">
+        <v>0</v>
+      </c>
+      <c r="U16" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="V16" s="9">
+        <v>2</v>
+      </c>
+      <c r="W16" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="X16" s="9">
         <v>4</v>
       </c>
-      <c r="E16" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="F16" s="9">
-        <v>819</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>248</v>
-      </c>
-      <c r="H16" s="9">
-        <v>21</v>
-      </c>
-      <c r="I16" s="10" t="s">
-        <v>249</v>
-      </c>
-      <c r="J16" s="9">
-        <v>54</v>
-      </c>
-      <c r="K16" s="10" t="s">
-        <v>250</v>
-      </c>
-      <c r="L16" s="9">
-        <v>1437</v>
-      </c>
-      <c r="M16" s="10" t="s">
-        <v>251</v>
-      </c>
-      <c r="N16" s="9">
-        <v>142</v>
-      </c>
-      <c r="O16" s="10" t="s">
-        <v>252</v>
-      </c>
-      <c r="P16" s="9">
-        <v>4</v>
-      </c>
-      <c r="Q16" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="R16" s="9">
-        <v>230</v>
-      </c>
-      <c r="S16" s="10" t="s">
-        <v>253</v>
-      </c>
-      <c r="T16" s="9">
-        <v>0</v>
-      </c>
-      <c r="U16" s="10" t="s">
+      <c r="Y16" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="V16" s="9">
-        <v>4</v>
-      </c>
-      <c r="W16" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="X16" s="9">
+      <c r="Z16" s="9">
+        <v>2</v>
+      </c>
+      <c r="AA16" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="AB16" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC16" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="AD16" s="9">
         <v>3</v>
       </c>
-      <c r="Y16" s="10" t="s">
+      <c r="AE16" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="Z16" s="9">
-        <v>1</v>
-      </c>
-      <c r="AA16" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="AB16" s="9">
-        <v>2</v>
-      </c>
-      <c r="AC16" s="10" t="s">
-        <v>177</v>
-      </c>
-      <c r="AD16" s="9">
-        <v>2</v>
-      </c>
-      <c r="AE16" s="10" t="s">
-        <v>177</v>
-      </c>
       <c r="AF16" s="9">
         <v>0</v>
       </c>
       <c r="AG16" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH16" s="9">
         <v>0</v>
       </c>
       <c r="AI16" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AJ16" s="9">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="AK16" s="10" t="s">
         <v>249</v>
       </c>
       <c r="AL16" s="9">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AM16" s="10" t="s">
-        <v>193</v>
+        <v>118</v>
       </c>
       <c r="AN16" s="9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AO16" s="10" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="AP16" s="9">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="AQ16" s="10" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="AR16" s="9">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="AS16" s="10" t="s">
-        <v>196</v>
+        <v>116</v>
       </c>
       <c r="AT16" s="9">
-        <v>152</v>
+        <v>100</v>
       </c>
       <c r="AU16" s="10" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="AV16" s="9">
-        <v>384</v>
+        <v>396</v>
       </c>
       <c r="AW16" s="10" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="AX16" s="9">
-        <v>1251</v>
+        <v>1313</v>
       </c>
       <c r="AY16" s="10" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="C17" s="9">
+        <v>8127</v>
+      </c>
+      <c r="D17" s="9">
+        <v>17</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="F17" s="9">
+        <v>2443</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>257</v>
+      </c>
+      <c r="H17" s="9">
+        <v>332</v>
+      </c>
+      <c r="I17" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="J17" s="9">
+        <v>128</v>
+      </c>
+      <c r="K17" s="10" t="s">
         <v>259</v>
       </c>
-      <c r="C17" s="9">
-        <v>7190</v>
-      </c>
-      <c r="D17" s="9">
-        <v>12</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>193</v>
-      </c>
-      <c r="F17" s="9">
-        <v>2106</v>
-      </c>
-      <c r="G17" s="10" t="s">
+      <c r="L17" s="9">
+        <v>2916</v>
+      </c>
+      <c r="M17" s="10" t="s">
         <v>260</v>
       </c>
-      <c r="H17" s="9">
-        <v>377</v>
-      </c>
-      <c r="I17" s="10" t="s">
+      <c r="N17" s="9">
+        <v>468</v>
+      </c>
+      <c r="O17" s="10" t="s">
         <v>261</v>
-      </c>
-      <c r="J17" s="9">
-        <v>137</v>
-      </c>
-      <c r="K17" s="10" t="s">
-        <v>262</v>
-      </c>
-      <c r="L17" s="9">
-        <v>2385</v>
-      </c>
-      <c r="M17" s="10" t="s">
-        <v>263</v>
-      </c>
-      <c r="N17" s="9">
-        <v>444</v>
-      </c>
-      <c r="O17" s="10" t="s">
-        <v>264</v>
       </c>
       <c r="P17" s="9">
         <v>21</v>
       </c>
       <c r="Q17" s="10" t="s">
-        <v>265</v>
+        <v>120</v>
       </c>
       <c r="R17" s="9">
-        <v>264</v>
+        <v>294</v>
       </c>
       <c r="S17" s="10" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="T17" s="9">
         <v>1</v>
       </c>
       <c r="U17" s="10" t="s">
-        <v>156</v>
+        <v>136</v>
       </c>
       <c r="V17" s="9">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W17" s="10" t="s">
-        <v>106</v>
+        <v>138</v>
       </c>
       <c r="X17" s="9">
         <v>5</v>
@@ -3721,31 +3700,31 @@
         <v>2</v>
       </c>
       <c r="AA17" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AB17" s="9">
         <v>2</v>
       </c>
       <c r="AC17" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AD17" s="9">
         <v>4</v>
       </c>
       <c r="AE17" s="10" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AF17" s="9">
         <v>0</v>
       </c>
       <c r="AG17" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH17" s="9">
         <v>2</v>
       </c>
       <c r="AI17" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AJ17" s="9">
         <v>16</v>
@@ -3757,144 +3736,144 @@
         <v>3</v>
       </c>
       <c r="AM17" s="10" t="s">
-        <v>177</v>
+        <v>128</v>
       </c>
       <c r="AN17" s="9">
         <v>7</v>
       </c>
       <c r="AO17" s="10" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="AP17" s="9">
         <v>44</v>
       </c>
       <c r="AQ17" s="10" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="AR17" s="9">
         <v>9</v>
       </c>
       <c r="AS17" s="10" t="s">
-        <v>267</v>
+        <v>230</v>
       </c>
       <c r="AT17" s="9">
-        <v>267</v>
+        <v>258</v>
       </c>
       <c r="AU17" s="10" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="AV17" s="9">
-        <v>639</v>
+        <v>698</v>
       </c>
       <c r="AW17" s="10" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="AX17" s="9">
-        <v>438</v>
+        <v>451</v>
       </c>
       <c r="AY17" s="10" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="C18" s="9">
-        <v>8785</v>
+        <v>9245</v>
       </c>
       <c r="D18" s="9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F18" s="9">
-        <v>1475</v>
+        <v>1557</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="H18" s="9">
         <v>148</v>
       </c>
       <c r="I18" s="10" t="s">
+        <v>270</v>
+      </c>
+      <c r="J18" s="9">
+        <v>271</v>
+      </c>
+      <c r="K18" s="10" t="s">
+        <v>271</v>
+      </c>
+      <c r="L18" s="9">
+        <v>2906</v>
+      </c>
+      <c r="M18" s="10" t="s">
+        <v>272</v>
+      </c>
+      <c r="N18" s="9">
+        <v>1481</v>
+      </c>
+      <c r="O18" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="P18" s="9">
+        <v>30</v>
+      </c>
+      <c r="Q18" s="10" t="s">
         <v>274</v>
       </c>
-      <c r="J18" s="9">
-        <v>314</v>
-      </c>
-      <c r="K18" s="10" t="s">
+      <c r="R18" s="9">
+        <v>533</v>
+      </c>
+      <c r="S18" s="10" t="s">
         <v>275</v>
-      </c>
-      <c r="L18" s="9">
-        <v>2659</v>
-      </c>
-      <c r="M18" s="10" t="s">
-        <v>276</v>
-      </c>
-      <c r="N18" s="9">
-        <v>1434</v>
-      </c>
-      <c r="O18" s="10" t="s">
-        <v>277</v>
-      </c>
-      <c r="P18" s="9">
-        <v>31</v>
-      </c>
-      <c r="Q18" s="10" t="s">
-        <v>278</v>
-      </c>
-      <c r="R18" s="9">
-        <v>499</v>
-      </c>
-      <c r="S18" s="10" t="s">
-        <v>279</v>
       </c>
       <c r="T18" s="9">
         <v>22</v>
       </c>
       <c r="U18" s="10" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="V18" s="9">
         <v>0</v>
       </c>
       <c r="W18" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="X18" s="9">
         <v>5</v>
       </c>
       <c r="Y18" s="10" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Z18" s="9">
         <v>1</v>
       </c>
       <c r="AA18" s="10" t="s">
-        <v>156</v>
+        <v>136</v>
       </c>
       <c r="AB18" s="9">
+        <v>2</v>
+      </c>
+      <c r="AC18" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="AD18" s="9">
         <v>3</v>
       </c>
-      <c r="AC18" s="10" t="s">
+      <c r="AE18" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="AD18" s="9">
-        <v>1</v>
-      </c>
-      <c r="AE18" s="10" t="s">
-        <v>156</v>
-      </c>
       <c r="AF18" s="9">
         <v>0</v>
       </c>
       <c r="AG18" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH18" s="9">
         <v>2</v>
@@ -3906,138 +3885,138 @@
         <v>11</v>
       </c>
       <c r="AK18" s="10" t="s">
-        <v>267</v>
+        <v>193</v>
       </c>
       <c r="AL18" s="9">
         <v>5</v>
       </c>
       <c r="AM18" s="10" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AN18" s="9">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AO18" s="10" t="s">
-        <v>136</v>
+        <v>177</v>
       </c>
       <c r="AP18" s="9">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="AQ18" s="10" t="s">
-        <v>119</v>
+        <v>276</v>
       </c>
       <c r="AR18" s="9">
         <v>12</v>
       </c>
       <c r="AS18" s="10" t="s">
-        <v>192</v>
+        <v>140</v>
       </c>
       <c r="AT18" s="9">
-        <v>75</v>
+        <v>4</v>
       </c>
       <c r="AU18" s="10" t="s">
-        <v>175</v>
+        <v>128</v>
       </c>
       <c r="AV18" s="9">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="AW18" s="10" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="AX18" s="9">
-        <v>1672</v>
+        <v>1831</v>
       </c>
       <c r="AY18" s="10" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="C19" s="9">
+        <v>8945</v>
+      </c>
+      <c r="D19" s="9">
+        <v>1</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="F19" s="9">
+        <v>1085</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="H19" s="9">
+        <v>15</v>
+      </c>
+      <c r="I19" s="10" t="s">
+        <v>189</v>
+      </c>
+      <c r="J19" s="9">
+        <v>34</v>
+      </c>
+      <c r="K19" s="10" t="s">
         <v>282</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="L19" s="9">
+        <v>3825</v>
+      </c>
+      <c r="M19" s="10" t="s">
         <v>283</v>
       </c>
-      <c r="C19" s="9">
-        <v>8886</v>
-      </c>
-      <c r="D19" s="9">
-        <v>2</v>
-      </c>
-      <c r="E19" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="F19" s="9">
-        <v>1084</v>
-      </c>
-      <c r="G19" s="10" t="s">
+      <c r="N19" s="9">
+        <v>1516</v>
+      </c>
+      <c r="O19" s="10" t="s">
         <v>284</v>
       </c>
-      <c r="H19" s="9">
-        <v>12</v>
-      </c>
-      <c r="I19" s="10" t="s">
-        <v>192</v>
-      </c>
-      <c r="J19" s="9">
-        <v>37</v>
-      </c>
-      <c r="K19" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="L19" s="9">
-        <v>3775</v>
-      </c>
-      <c r="M19" s="10" t="s">
+      <c r="P19" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="R19" s="9">
+        <v>907</v>
+      </c>
+      <c r="S19" s="10" t="s">
         <v>285</v>
       </c>
-      <c r="N19" s="9">
-        <v>1511</v>
-      </c>
-      <c r="O19" s="10" t="s">
-        <v>219</v>
-      </c>
-      <c r="P19" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="R19" s="9">
-        <v>904</v>
-      </c>
-      <c r="S19" s="10" t="s">
-        <v>286</v>
-      </c>
       <c r="T19" s="9">
         <v>0</v>
       </c>
       <c r="U19" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="V19" s="9">
         <v>1</v>
       </c>
       <c r="W19" s="10" t="s">
-        <v>156</v>
+        <v>136</v>
       </c>
       <c r="X19" s="9">
         <v>17</v>
       </c>
       <c r="Y19" s="10" t="s">
-        <v>287</v>
+        <v>169</v>
       </c>
       <c r="Z19" s="9">
         <v>0</v>
       </c>
       <c r="AA19" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AB19" s="9">
         <v>0</v>
       </c>
       <c r="AC19" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AD19" s="9">
         <v>3</v>
@@ -4049,224 +4028,224 @@
         <v>0</v>
       </c>
       <c r="AG19" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH19" s="9">
         <v>0</v>
       </c>
       <c r="AI19" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AJ19" s="9">
         <v>16</v>
       </c>
       <c r="AK19" s="10" t="s">
-        <v>208</v>
+        <v>153</v>
       </c>
       <c r="AL19" s="9">
         <v>0</v>
       </c>
       <c r="AM19" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AN19" s="9">
         <v>1</v>
       </c>
       <c r="AO19" s="10" t="s">
-        <v>156</v>
+        <v>136</v>
       </c>
       <c r="AP19" s="9">
         <v>51</v>
       </c>
       <c r="AQ19" s="10" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="AR19" s="9">
         <v>1</v>
       </c>
       <c r="AS19" s="10" t="s">
-        <v>156</v>
+        <v>136</v>
       </c>
       <c r="AT19" s="9">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="AU19" s="10" t="s">
-        <v>288</v>
+        <v>189</v>
       </c>
       <c r="AV19" s="9">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="AW19" s="10" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="AX19" s="9">
-        <v>831</v>
+        <v>835</v>
       </c>
       <c r="AY19" s="10" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="C20" s="9">
-        <v>1034</v>
+        <v>1041</v>
       </c>
       <c r="D20" s="9">
         <v>1</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F20" s="9">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="H20" s="9">
         <v>6</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>294</v>
+        <v>121</v>
       </c>
       <c r="J20" s="9">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="L20" s="9">
-        <v>319</v>
+        <v>327</v>
       </c>
       <c r="M20" s="10" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="N20" s="9">
         <v>48</v>
       </c>
       <c r="O20" s="10" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="P20" s="9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>298</v>
+        <v>121</v>
       </c>
       <c r="R20" s="9">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S20" s="10" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="T20" s="9">
         <v>0</v>
       </c>
       <c r="U20" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="V20" s="9">
         <v>0</v>
       </c>
       <c r="W20" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="X20" s="9">
         <v>9</v>
       </c>
       <c r="Y20" s="10" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="Z20" s="9">
         <v>3</v>
       </c>
       <c r="AA20" s="10" t="s">
-        <v>265</v>
+        <v>178</v>
       </c>
       <c r="AB20" s="9">
         <v>0</v>
       </c>
       <c r="AC20" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AD20" s="9">
         <v>0</v>
       </c>
       <c r="AE20" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AF20" s="9">
         <v>0</v>
       </c>
       <c r="AG20" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH20" s="9">
         <v>1</v>
       </c>
       <c r="AI20" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="AJ20" s="9">
         <v>6</v>
       </c>
       <c r="AK20" s="10" t="s">
-        <v>294</v>
+        <v>121</v>
       </c>
       <c r="AL20" s="9">
         <v>2</v>
       </c>
       <c r="AM20" s="10" t="s">
-        <v>287</v>
+        <v>169</v>
       </c>
       <c r="AN20" s="9">
         <v>1</v>
       </c>
       <c r="AO20" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="AP20" s="9">
         <v>18</v>
       </c>
       <c r="AQ20" s="10" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="AR20" s="9">
         <v>4</v>
       </c>
       <c r="AS20" s="10" t="s">
-        <v>302</v>
+        <v>282</v>
       </c>
       <c r="AT20" s="9">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="AU20" s="10" t="s">
-        <v>303</v>
+        <v>245</v>
       </c>
       <c r="AV20" s="9">
         <v>47</v>
       </c>
       <c r="AW20" s="10" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="AX20" s="9">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="AY20" s="10" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="C21" s="9">
         <v>2476</v>
@@ -4275,297 +4254,297 @@
         <v>0</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F21" s="9">
         <v>398</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="H21" s="9">
         <v>154</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="J21" s="9">
         <v>1</v>
       </c>
       <c r="K21" s="10" t="s">
-        <v>177</v>
+        <v>128</v>
       </c>
       <c r="L21" s="9">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="N21" s="9">
         <v>102</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="P21" s="9">
         <v>8</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>112</v>
+        <v>274</v>
       </c>
       <c r="R21" s="9">
         <v>79</v>
       </c>
       <c r="S21" s="10" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="T21" s="9">
         <v>0</v>
       </c>
       <c r="U21" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="V21" s="9">
         <v>0</v>
       </c>
       <c r="W21" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="X21" s="9">
         <v>17</v>
       </c>
       <c r="Y21" s="10" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="Z21" s="9">
         <v>2</v>
       </c>
       <c r="AA21" s="10" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="AB21" s="9">
         <v>0</v>
       </c>
       <c r="AC21" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AD21" s="9">
         <v>0</v>
       </c>
       <c r="AE21" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AF21" s="9">
         <v>0</v>
       </c>
       <c r="AG21" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH21" s="9">
         <v>0</v>
       </c>
       <c r="AI21" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AJ21" s="9">
         <v>3</v>
       </c>
       <c r="AK21" s="10" t="s">
-        <v>128</v>
+        <v>193</v>
       </c>
       <c r="AL21" s="9">
         <v>0</v>
       </c>
       <c r="AM21" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AN21" s="9">
         <v>0</v>
       </c>
       <c r="AO21" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AP21" s="9">
         <v>18</v>
       </c>
       <c r="AQ21" s="10" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="AR21" s="9">
         <v>1</v>
       </c>
       <c r="AS21" s="10" t="s">
-        <v>177</v>
+        <v>128</v>
       </c>
       <c r="AT21" s="9">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="AU21" s="10" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
       <c r="AV21" s="9">
         <v>96</v>
       </c>
       <c r="AW21" s="10" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="AX21" s="9">
         <v>825</v>
       </c>
       <c r="AY21" s="10" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="C22" s="12">
-        <v>106882</v>
+        <v>111025</v>
       </c>
       <c r="D22" s="12">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>106</v>
       </c>
       <c r="F22" s="12">
-        <v>21538</v>
+        <v>22589</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>107</v>
       </c>
       <c r="H22" s="12">
-        <v>1482</v>
+        <v>1450</v>
       </c>
       <c r="I22" s="13" t="s">
         <v>108</v>
       </c>
       <c r="J22" s="12">
-        <v>2973</v>
+        <v>2698</v>
       </c>
       <c r="K22" s="13" t="s">
         <v>109</v>
       </c>
       <c r="L22" s="12">
-        <v>38187</v>
+        <v>40497</v>
       </c>
       <c r="M22" s="13" t="s">
         <v>110</v>
       </c>
       <c r="N22" s="12">
-        <v>11171</v>
+        <v>11488</v>
       </c>
       <c r="O22" s="13" t="s">
         <v>111</v>
       </c>
       <c r="P22" s="12">
-        <v>344</v>
+        <v>276</v>
       </c>
       <c r="Q22" s="13" t="s">
         <v>112</v>
       </c>
       <c r="R22" s="12">
-        <v>7893</v>
+        <v>8174</v>
       </c>
       <c r="S22" s="13" t="s">
         <v>113</v>
       </c>
       <c r="T22" s="12">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="U22" s="13" t="s">
         <v>114</v>
       </c>
       <c r="V22" s="12">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="W22" s="13" t="s">
         <v>115</v>
       </c>
       <c r="X22" s="12">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="Y22" s="13" t="s">
         <v>116</v>
       </c>
       <c r="Z22" s="12">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="AA22" s="13" t="s">
         <v>117</v>
       </c>
       <c r="AB22" s="12">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="AC22" s="13" t="s">
         <v>115</v>
       </c>
       <c r="AD22" s="12">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="AE22" s="13" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="AF22" s="12">
         <v>1</v>
       </c>
       <c r="AG22" s="13" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AH22" s="12">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="AI22" s="13" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AJ22" s="12">
-        <v>264</v>
+        <v>284</v>
       </c>
       <c r="AK22" s="13" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AL22" s="12">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="AM22" s="13" t="s">
         <v>115</v>
       </c>
       <c r="AN22" s="12">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="AO22" s="13" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="AP22" s="12">
-        <v>601</v>
+        <v>649</v>
       </c>
       <c r="AQ22" s="13" t="s">
         <v>121</v>
       </c>
       <c r="AR22" s="12">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="AS22" s="13" t="s">
         <v>122</v>
       </c>
       <c r="AT22" s="12">
-        <v>1723</v>
+        <v>1296</v>
       </c>
       <c r="AU22" s="13" t="s">
         <v>123</v>
       </c>
       <c r="AV22" s="12">
-        <v>5607</v>
+        <v>5755</v>
       </c>
       <c r="AW22" s="13" t="s">
         <v>124</v>
       </c>
       <c r="AX22" s="12">
-        <v>14316</v>
+        <v>15094</v>
       </c>
       <c r="AY22" s="13" t="s">
         <v>125</v>

</xml_diff>

<commit_message>
Perbarui data SE2026 02/09/2026 10:05:53,34
</commit_message>
<xml_diff>
--- a/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
+++ b/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
@@ -16,7 +16,7 @@
     <t>DATA RADAR ANOMALI USAHA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 1 Sep 2026, 13.02</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 2 Sep 2026, 10.04</t>
   </si>
   <si>
     <t>Kode</t>
@@ -334,580 +334,586 @@
     <t>0,06</t>
   </si>
   <si>
-    <t>20,35</t>
-  </si>
-  <si>
-    <t>1,31</t>
-  </si>
-  <si>
-    <t>2,43</t>
-  </si>
-  <si>
-    <t>36,48</t>
-  </si>
-  <si>
-    <t>10,35</t>
+    <t>20,43</t>
+  </si>
+  <si>
+    <t>1,27</t>
+  </si>
+  <si>
+    <t>2,25</t>
+  </si>
+  <si>
+    <t>37</t>
+  </si>
+  <si>
+    <t>10,3</t>
+  </si>
+  <si>
+    <t>0,23</t>
+  </si>
+  <si>
+    <t>7,35</t>
+  </si>
+  <si>
+    <t>0,09</t>
+  </si>
+  <si>
+    <t>0,03</t>
+  </si>
+  <si>
+    <t>0,15</t>
+  </si>
+  <si>
+    <t>0,02</t>
+  </si>
+  <si>
+    <t>0,08</t>
+  </si>
+  <si>
+    <t>0</t>
   </si>
   <si>
     <t>0,25</t>
   </si>
   <si>
-    <t>7,36</t>
-  </si>
-  <si>
-    <t>0,09</t>
-  </si>
-  <si>
-    <t>0,03</t>
-  </si>
-  <si>
-    <t>0,15</t>
-  </si>
-  <si>
-    <t>0,02</t>
-  </si>
-  <si>
-    <t>0,08</t>
-  </si>
-  <si>
-    <t>0</t>
+    <t>0,58</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>5,12</t>
+  </si>
+  <si>
+    <t>13,51</t>
+  </si>
+  <si>
+    <t>1801</t>
+  </si>
+  <si>
+    <t>LAMPUNG BARAT</t>
+  </si>
+  <si>
+    <t>0,04</t>
+  </si>
+  <si>
+    <t>19,56</t>
+  </si>
+  <si>
+    <t>0,96</t>
+  </si>
+  <si>
+    <t>1,25</t>
+  </si>
+  <si>
+    <t>45,66</t>
+  </si>
+  <si>
+    <t>5,21</t>
+  </si>
+  <si>
+    <t>0,22</t>
+  </si>
+  <si>
+    <t>4,46</t>
+  </si>
+  <si>
+    <t>0,01</t>
+  </si>
+  <si>
+    <t>0,19</t>
+  </si>
+  <si>
+    <t>0,07</t>
+  </si>
+  <si>
+    <t>0,14</t>
+  </si>
+  <si>
+    <t>0,11</t>
+  </si>
+  <si>
+    <t>0,34</t>
+  </si>
+  <si>
+    <t>3,21</t>
+  </si>
+  <si>
+    <t>3,44</t>
+  </si>
+  <si>
+    <t>14,92</t>
+  </si>
+  <si>
+    <t>1802</t>
+  </si>
+  <si>
+    <t>TANGGAMUS</t>
+  </si>
+  <si>
+    <t>13,73</t>
+  </si>
+  <si>
+    <t>0,54</t>
+  </si>
+  <si>
+    <t>1,08</t>
+  </si>
+  <si>
+    <t>26,23</t>
+  </si>
+  <si>
+    <t>30,42</t>
+  </si>
+  <si>
+    <t>6,46</t>
+  </si>
+  <si>
+    <t>0,18</t>
+  </si>
+  <si>
+    <t>0,48</t>
+  </si>
+  <si>
+    <t>0,3</t>
+  </si>
+  <si>
+    <t>4,64</t>
+  </si>
+  <si>
+    <t>15,67</t>
+  </si>
+  <si>
+    <t>1803</t>
+  </si>
+  <si>
+    <t>LAMPUNG SELATAN</t>
+  </si>
+  <si>
+    <t>17,1</t>
+  </si>
+  <si>
+    <t>2,31</t>
+  </si>
+  <si>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>43,72</t>
+  </si>
+  <si>
+    <t>12,36</t>
+  </si>
+  <si>
+    <t>9,63</t>
+  </si>
+  <si>
+    <t>0,33</t>
+  </si>
+  <si>
+    <t>0,76</t>
+  </si>
+  <si>
+    <t>1,17</t>
+  </si>
+  <si>
+    <t>4,17</t>
+  </si>
+  <si>
+    <t>8,03</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>23,54</t>
   </si>
   <si>
     <t>0,26</t>
   </si>
   <si>
-    <t>0,58</t>
-  </si>
-  <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>1,17</t>
-  </si>
-  <si>
-    <t>5,18</t>
-  </si>
-  <si>
-    <t>13,6</t>
-  </si>
-  <si>
-    <t>1801</t>
-  </si>
-  <si>
-    <t>LAMPUNG BARAT</t>
-  </si>
-  <si>
-    <t>0,04</t>
-  </si>
-  <si>
-    <t>19,58</t>
-  </si>
-  <si>
-    <t>0,98</t>
-  </si>
-  <si>
-    <t>1,44</t>
-  </si>
-  <si>
-    <t>45,01</t>
-  </si>
-  <si>
-    <t>5,43</t>
-  </si>
-  <si>
-    <t>0,24</t>
+    <t>8,81</t>
+  </si>
+  <si>
+    <t>32,8</t>
+  </si>
+  <si>
+    <t>11,7</t>
+  </si>
+  <si>
+    <t>0,79</t>
+  </si>
+  <si>
+    <t>6,76</t>
+  </si>
+  <si>
+    <t>0,05</t>
+  </si>
+  <si>
+    <t>0,28</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>2,24</t>
+  </si>
+  <si>
+    <t>10,02</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>15,42</t>
+  </si>
+  <si>
+    <t>2,33</t>
+  </si>
+  <si>
+    <t>1,11</t>
+  </si>
+  <si>
+    <t>46,01</t>
+  </si>
+  <si>
+    <t>4,81</t>
+  </si>
+  <si>
+    <t>0,17</t>
+  </si>
+  <si>
+    <t>13,37</t>
+  </si>
+  <si>
+    <t>0,66</t>
+  </si>
+  <si>
+    <t>0,21</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>18,89</t>
+  </si>
+  <si>
+    <t>0,74</t>
+  </si>
+  <si>
+    <t>1,07</t>
+  </si>
+  <si>
+    <t>37,33</t>
+  </si>
+  <si>
+    <t>14,12</t>
+  </si>
+  <si>
+    <t>7,83</t>
+  </si>
+  <si>
+    <t>0,35</t>
+  </si>
+  <si>
+    <t>0,56</t>
+  </si>
+  <si>
+    <t>0,29</t>
+  </si>
+  <si>
+    <t>6,8</t>
+  </si>
+  <si>
+    <t>10,34</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>17,99</t>
+  </si>
+  <si>
+    <t>0,65</t>
+  </si>
+  <si>
+    <t>0,44</t>
+  </si>
+  <si>
+    <t>42,85</t>
+  </si>
+  <si>
+    <t>17,36</t>
+  </si>
+  <si>
+    <t>6,28</t>
+  </si>
+  <si>
+    <t>0,78</t>
+  </si>
+  <si>
+    <t>0,49</t>
+  </si>
+  <si>
+    <t>7,19</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>23,46</t>
+  </si>
+  <si>
+    <t>0,41</t>
+  </si>
+  <si>
+    <t>2,59</t>
+  </si>
+  <si>
+    <t>27,46</t>
+  </si>
+  <si>
+    <t>15,61</t>
+  </si>
+  <si>
+    <t>5,73</t>
+  </si>
+  <si>
+    <t>0,2</t>
+  </si>
+  <si>
+    <t>0,64</t>
+  </si>
+  <si>
+    <t>2,41</t>
+  </si>
+  <si>
+    <t>7,33</t>
+  </si>
+  <si>
+    <t>13,36</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>30,72</t>
+  </si>
+  <si>
+    <t>0,45</t>
+  </si>
+  <si>
+    <t>30,5</t>
+  </si>
+  <si>
+    <t>1,88</t>
+  </si>
+  <si>
+    <t>5,85</t>
+  </si>
+  <si>
+    <t>0,63</t>
+  </si>
+  <si>
+    <t>8,4</t>
+  </si>
+  <si>
+    <t>20,75</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>18,05</t>
+  </si>
+  <si>
+    <t>0,59</t>
+  </si>
+  <si>
+    <t>32,1</t>
+  </si>
+  <si>
+    <t>3,07</t>
+  </si>
+  <si>
+    <t>4,99</t>
+  </si>
+  <si>
+    <t>0,88</t>
+  </si>
+  <si>
+    <t>1,06</t>
+  </si>
+  <si>
+    <t>8,24</t>
+  </si>
+  <si>
+    <t>28,93</t>
+  </si>
+  <si>
+    <t>1811</t>
+  </si>
+  <si>
+    <t>MESUJI</t>
+  </si>
+  <si>
+    <t>30,21</t>
+  </si>
+  <si>
+    <t>3,8</t>
+  </si>
+  <si>
+    <t>1,51</t>
+  </si>
+  <si>
+    <t>36,72</t>
+  </si>
+  <si>
+    <t>5,6</t>
+  </si>
+  <si>
+    <t>3,62</t>
+  </si>
+  <si>
+    <t>0,52</t>
+  </si>
+  <si>
+    <t>3,09</t>
+  </si>
+  <si>
+    <t>8,37</t>
+  </si>
+  <si>
+    <t>5,4</t>
+  </si>
+  <si>
+    <t>1812</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG BARAT</t>
+  </si>
+  <si>
+    <t>16,87</t>
+  </si>
+  <si>
+    <t>1,58</t>
+  </si>
+  <si>
+    <t>1,98</t>
+  </si>
+  <si>
+    <t>31,17</t>
+  </si>
+  <si>
+    <t>17,63</t>
+  </si>
+  <si>
+    <t>0,31</t>
+  </si>
+  <si>
+    <t>0,13</t>
+  </si>
+  <si>
+    <t>4,19</t>
+  </si>
+  <si>
+    <t>19,52</t>
+  </si>
+  <si>
+    <t>1813</t>
+  </si>
+  <si>
+    <t>PESISIR BARAT</t>
+  </si>
+  <si>
+    <t>11,95</t>
+  </si>
+  <si>
+    <t>0,16</t>
+  </si>
+  <si>
+    <t>0,27</t>
+  </si>
+  <si>
+    <t>44,79</t>
+  </si>
+  <si>
+    <t>16,11</t>
+  </si>
+  <si>
+    <t>10,05</t>
+  </si>
+  <si>
+    <t>6,71</t>
+  </si>
+  <si>
+    <t>8,82</t>
+  </si>
+  <si>
+    <t>1871</t>
+  </si>
+  <si>
+    <t>BANDAR LAMPUNG</t>
+  </si>
+  <si>
+    <t>15,49</t>
+  </si>
+  <si>
+    <t>0,57</t>
+  </si>
+  <si>
+    <t>3,35</t>
+  </si>
+  <si>
+    <t>31,64</t>
+  </si>
+  <si>
+    <t>4,59</t>
+  </si>
+  <si>
+    <t>16,06</t>
+  </si>
+  <si>
+    <t>0,86</t>
+  </si>
+  <si>
+    <t>1,72</t>
+  </si>
+  <si>
+    <t>0,38</t>
+  </si>
+  <si>
+    <t>1,24</t>
   </si>
   <si>
     <t>4,49</t>
   </si>
   <si>
-    <t>0,01</t>
-  </si>
-  <si>
-    <t>0,2</t>
-  </si>
-  <si>
-    <t>0,07</t>
-  </si>
-  <si>
-    <t>0,14</t>
-  </si>
-  <si>
-    <t>0,13</t>
-  </si>
-  <si>
-    <t>0,36</t>
-  </si>
-  <si>
-    <t>4,22</t>
-  </si>
-  <si>
-    <t>3,48</t>
-  </si>
-  <si>
-    <t>13,93</t>
-  </si>
-  <si>
-    <t>1802</t>
-  </si>
-  <si>
-    <t>TANGGAMUS</t>
-  </si>
-  <si>
-    <t>13,76</t>
-  </si>
-  <si>
-    <t>0,42</t>
-  </si>
-  <si>
-    <t>1,32</t>
-  </si>
-  <si>
-    <t>26,07</t>
-  </si>
-  <si>
-    <t>30,37</t>
-  </si>
-  <si>
-    <t>6,5</t>
-  </si>
-  <si>
-    <t>0,18</t>
-  </si>
-  <si>
-    <t>4,67</t>
-  </si>
-  <si>
-    <t>15,77</t>
-  </si>
-  <si>
-    <t>1803</t>
-  </si>
-  <si>
-    <t>LAMPUNG SELATAN</t>
-  </si>
-  <si>
-    <t>17,24</t>
-  </si>
-  <si>
-    <t>2,36</t>
-  </si>
-  <si>
-    <t>42,73</t>
-  </si>
-  <si>
-    <t>12,9</t>
-  </si>
-  <si>
-    <t>9,62</t>
-  </si>
-  <si>
-    <t>0,33</t>
-  </si>
-  <si>
-    <t>0,76</t>
-  </si>
-  <si>
-    <t>4,25</t>
-  </si>
-  <si>
-    <t>8,19</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>0,19</t>
-  </si>
-  <si>
-    <t>22,84</t>
-  </si>
-  <si>
-    <t>0,27</t>
-  </si>
-  <si>
-    <t>9,18</t>
-  </si>
-  <si>
-    <t>32,35</t>
-  </si>
-  <si>
-    <t>11,87</t>
-  </si>
-  <si>
-    <t>0,81</t>
-  </si>
-  <si>
-    <t>6,83</t>
-  </si>
-  <si>
-    <t>0,05</t>
-  </si>
-  <si>
-    <t>0,29</t>
-  </si>
-  <si>
-    <t>2,07</t>
-  </si>
-  <si>
-    <t>2,26</t>
-  </si>
-  <si>
-    <t>10,39</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>15,36</t>
-  </si>
-  <si>
-    <t>2,33</t>
-  </si>
-  <si>
-    <t>1,13</t>
-  </si>
-  <si>
-    <t>45,78</t>
-  </si>
-  <si>
-    <t>4,88</t>
-  </si>
-  <si>
-    <t>0,17</t>
-  </si>
-  <si>
-    <t>13,41</t>
-  </si>
-  <si>
-    <t>0,23</t>
-  </si>
-  <si>
-    <t>0,65</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>3,18</t>
-  </si>
-  <si>
-    <t>11,88</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>18,8</t>
-  </si>
-  <si>
-    <t>0,74</t>
-  </si>
-  <si>
-    <t>0,96</t>
-  </si>
-  <si>
-    <t>37,35</t>
-  </si>
-  <si>
-    <t>14,28</t>
-  </si>
-  <si>
-    <t>7,85</t>
-  </si>
-  <si>
-    <t>0,57</t>
-  </si>
-  <si>
-    <t>1,08</t>
-  </si>
-  <si>
-    <t>0,63</t>
-  </si>
-  <si>
-    <t>6,68</t>
-  </si>
-  <si>
-    <t>10,24</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>18,17</t>
-  </si>
-  <si>
-    <t>0,64</t>
-  </si>
-  <si>
-    <t>0,83</t>
-  </si>
-  <si>
-    <t>42,44</t>
-  </si>
-  <si>
-    <t>17,41</t>
-  </si>
-  <si>
-    <t>5,82</t>
-  </si>
-  <si>
-    <t>0,66</t>
-  </si>
-  <si>
-    <t>0,79</t>
-  </si>
-  <si>
-    <t>0,49</t>
-  </si>
-  <si>
-    <t>4,62</t>
-  </si>
-  <si>
-    <t>7,2</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>23,51</t>
-  </si>
-  <si>
-    <t>0,41</t>
-  </si>
-  <si>
-    <t>2,6</t>
-  </si>
-  <si>
-    <t>27,35</t>
-  </si>
-  <si>
-    <t>15,67</t>
-  </si>
-  <si>
-    <t>5,64</t>
-  </si>
-  <si>
-    <t>0,11</t>
-  </si>
-  <si>
-    <t>2,42</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>30,68</t>
-  </si>
-  <si>
-    <t>0,45</t>
-  </si>
-  <si>
-    <t>30,51</t>
-  </si>
-  <si>
-    <t>1,88</t>
-  </si>
-  <si>
-    <t>5,85</t>
-  </si>
-  <si>
-    <t>8,4</t>
-  </si>
-  <si>
-    <t>20,76</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>18,03</t>
-  </si>
-  <si>
-    <t>0,51</t>
-  </si>
-  <si>
-    <t>1,06</t>
-  </si>
-  <si>
-    <t>31,81</t>
-  </si>
-  <si>
-    <t>3,04</t>
-  </si>
-  <si>
-    <t>4,99</t>
-  </si>
-  <si>
-    <t>0,62</t>
-  </si>
-  <si>
-    <t>0,93</t>
-  </si>
-  <si>
-    <t>2,12</t>
-  </si>
-  <si>
-    <t>8,41</t>
-  </si>
-  <si>
-    <t>27,88</t>
-  </si>
-  <si>
-    <t>1811</t>
-  </si>
-  <si>
-    <t>MESUJI</t>
-  </si>
-  <si>
-    <t>0,21</t>
-  </si>
-  <si>
-    <t>30,06</t>
-  </si>
-  <si>
-    <t>4,09</t>
-  </si>
-  <si>
-    <t>1,57</t>
-  </si>
-  <si>
-    <t>35,88</t>
-  </si>
-  <si>
-    <t>5,76</t>
-  </si>
-  <si>
-    <t>3,62</t>
-  </si>
-  <si>
-    <t>0,54</t>
-  </si>
-  <si>
-    <t>3,17</t>
-  </si>
-  <si>
-    <t>8,59</t>
-  </si>
-  <si>
-    <t>5,55</t>
-  </si>
-  <si>
-    <t>1812</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG BARAT</t>
-  </si>
-  <si>
-    <t>16,84</t>
-  </si>
-  <si>
-    <t>1,6</t>
-  </si>
-  <si>
-    <t>2,93</t>
-  </si>
-  <si>
-    <t>31,43</t>
-  </si>
-  <si>
-    <t>16,02</t>
-  </si>
-  <si>
-    <t>0,32</t>
-  </si>
-  <si>
-    <t>5,77</t>
-  </si>
-  <si>
-    <t>0,28</t>
-  </si>
-  <si>
-    <t>4,2</t>
-  </si>
-  <si>
-    <t>19,81</t>
-  </si>
-  <si>
-    <t>1813</t>
-  </si>
-  <si>
-    <t>PESISIR BARAT</t>
-  </si>
-  <si>
-    <t>12,13</t>
-  </si>
-  <si>
-    <t>0,38</t>
-  </si>
-  <si>
-    <t>42,76</t>
-  </si>
-  <si>
-    <t>16,95</t>
-  </si>
-  <si>
-    <t>10,14</t>
-  </si>
-  <si>
-    <t>6,95</t>
-  </si>
-  <si>
-    <t>9,33</t>
-  </si>
-  <si>
-    <t>1871</t>
-  </si>
-  <si>
-    <t>BANDAR LAMPUNG</t>
-  </si>
-  <si>
-    <t>15,56</t>
-  </si>
-  <si>
-    <t>3,46</t>
-  </si>
-  <si>
-    <t>31,41</t>
-  </si>
-  <si>
-    <t>4,61</t>
-  </si>
-  <si>
-    <t>16,14</t>
-  </si>
-  <si>
-    <t>0,86</t>
-  </si>
-  <si>
-    <t>1,73</t>
-  </si>
-  <si>
-    <t>4,51</t>
-  </si>
-  <si>
-    <t>17,77</t>
+    <t>17,69</t>
   </si>
   <si>
     <t>1872</t>
@@ -916,34 +922,28 @@
     <t>METRO</t>
   </si>
   <si>
-    <t>16,07</t>
-  </si>
-  <si>
-    <t>6,22</t>
-  </si>
-  <si>
-    <t>29,44</t>
-  </si>
-  <si>
-    <t>4,12</t>
-  </si>
-  <si>
-    <t>3,19</t>
-  </si>
-  <si>
-    <t>0,69</t>
-  </si>
-  <si>
-    <t>0,73</t>
-  </si>
-  <si>
-    <t>1,74</t>
-  </si>
-  <si>
-    <t>3,88</t>
-  </si>
-  <si>
-    <t>33,32</t>
+    <t>16,45</t>
+  </si>
+  <si>
+    <t>5,88</t>
+  </si>
+  <si>
+    <t>30,32</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>0,67</t>
+  </si>
+  <si>
+    <t>0,71</t>
+  </si>
+  <si>
+    <t>3,76</t>
+  </si>
+  <si>
+    <t>33,8</t>
   </si>
   <si>
     <t/>
@@ -1923,16 +1923,16 @@
         <v>105</v>
       </c>
       <c r="C6" s="6">
-        <v>111025</v>
+        <v>113814</v>
       </c>
       <c r="D6" s="6">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>106</v>
       </c>
       <c r="F6" s="6">
-        <v>22589</v>
+        <v>23252</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>107</v>
@@ -1944,31 +1944,31 @@
         <v>108</v>
       </c>
       <c r="J6" s="6">
-        <v>2698</v>
+        <v>2565</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>109</v>
       </c>
       <c r="L6" s="6">
-        <v>40497</v>
+        <v>42111</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>110</v>
       </c>
       <c r="N6" s="6">
-        <v>11488</v>
+        <v>11727</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>111</v>
       </c>
       <c r="P6" s="6">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="Q6" s="7" t="s">
         <v>112</v>
       </c>
       <c r="R6" s="6">
-        <v>8174</v>
+        <v>8364</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>113</v>
@@ -1980,19 +1980,19 @@
         <v>114</v>
       </c>
       <c r="V6" s="6">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="W6" s="7" t="s">
         <v>115</v>
       </c>
       <c r="X6" s="6">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="Y6" s="7" t="s">
         <v>116</v>
       </c>
       <c r="Z6" s="6">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="AA6" s="7" t="s">
         <v>117</v>
@@ -2022,7 +2022,7 @@
         <v>117</v>
       </c>
       <c r="AJ6" s="6">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="AK6" s="7" t="s">
         <v>120</v>
@@ -2034,13 +2034,13 @@
         <v>115</v>
       </c>
       <c r="AN6" s="6">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="AO6" s="7" t="s">
         <v>118</v>
       </c>
       <c r="AP6" s="6">
-        <v>649</v>
+        <v>659</v>
       </c>
       <c r="AQ6" s="7" t="s">
         <v>121</v>
@@ -2052,19 +2052,19 @@
         <v>122</v>
       </c>
       <c r="AT6" s="6">
-        <v>1296</v>
+        <v>1143</v>
       </c>
       <c r="AU6" s="7" t="s">
         <v>123</v>
       </c>
       <c r="AV6" s="6">
-        <v>5755</v>
+        <v>5832</v>
       </c>
       <c r="AW6" s="7" t="s">
         <v>124</v>
       </c>
       <c r="AX6" s="6">
-        <v>15094</v>
+        <v>15378</v>
       </c>
       <c r="AY6" s="7" t="s">
         <v>125</v>
@@ -2078,7 +2078,7 @@
         <v>127</v>
       </c>
       <c r="C7" s="9">
-        <v>7012</v>
+        <v>7374</v>
       </c>
       <c r="D7" s="9">
         <v>3</v>
@@ -2087,43 +2087,43 @@
         <v>128</v>
       </c>
       <c r="F7" s="9">
-        <v>1373</v>
+        <v>1442</v>
       </c>
       <c r="G7" s="10" t="s">
         <v>129</v>
       </c>
       <c r="H7" s="9">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I7" s="10" t="s">
         <v>130</v>
       </c>
       <c r="J7" s="9">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="K7" s="10" t="s">
         <v>131</v>
       </c>
       <c r="L7" s="9">
-        <v>3156</v>
+        <v>3367</v>
       </c>
       <c r="M7" s="10" t="s">
         <v>132</v>
       </c>
       <c r="N7" s="9">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="O7" s="10" t="s">
         <v>133</v>
       </c>
       <c r="P7" s="9">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="Q7" s="10" t="s">
         <v>134</v>
       </c>
       <c r="R7" s="9">
-        <v>315</v>
+        <v>329</v>
       </c>
       <c r="S7" s="10" t="s">
         <v>135</v>
@@ -2156,7 +2156,7 @@
         <v>7</v>
       </c>
       <c r="AC7" s="10" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="AD7" s="9">
         <v>5</v>
@@ -2189,7 +2189,7 @@
         <v>136</v>
       </c>
       <c r="AN7" s="9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AO7" s="10" t="s">
         <v>140</v>
@@ -2207,19 +2207,19 @@
         <v>128</v>
       </c>
       <c r="AT7" s="9">
-        <v>296</v>
+        <v>237</v>
       </c>
       <c r="AU7" s="10" t="s">
         <v>142</v>
       </c>
       <c r="AV7" s="9">
-        <v>244</v>
+        <v>254</v>
       </c>
       <c r="AW7" s="10" t="s">
         <v>143</v>
       </c>
       <c r="AX7" s="9">
-        <v>977</v>
+        <v>1100</v>
       </c>
       <c r="AY7" s="10" t="s">
         <v>144</v>
@@ -2233,7 +2233,7 @@
         <v>146</v>
       </c>
       <c r="C8" s="9">
-        <v>3322</v>
+        <v>3343</v>
       </c>
       <c r="D8" s="9">
         <v>0</v>
@@ -2242,31 +2242,31 @@
         <v>119</v>
       </c>
       <c r="F8" s="9">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>147</v>
       </c>
       <c r="H8" s="9">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="I8" s="10" t="s">
         <v>148</v>
       </c>
       <c r="J8" s="9">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="K8" s="10" t="s">
         <v>149</v>
       </c>
       <c r="L8" s="9">
-        <v>866</v>
+        <v>877</v>
       </c>
       <c r="M8" s="10" t="s">
         <v>150</v>
       </c>
       <c r="N8" s="9">
-        <v>1009</v>
+        <v>1017</v>
       </c>
       <c r="O8" s="10" t="s">
         <v>151</v>
@@ -2350,10 +2350,10 @@
         <v>119</v>
       </c>
       <c r="AP8" s="9">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="AQ8" s="10" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="AR8" s="9">
         <v>2</v>
@@ -2362,87 +2362,87 @@
         <v>106</v>
       </c>
       <c r="AT8" s="9">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AU8" s="10" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
       <c r="AV8" s="9">
         <v>155</v>
       </c>
       <c r="AW8" s="10" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="AX8" s="9">
         <v>524</v>
       </c>
       <c r="AY8" s="10" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C9" s="9">
-        <v>8380</v>
+        <v>8559</v>
       </c>
       <c r="D9" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>136</v>
+        <v>119</v>
       </c>
       <c r="F9" s="9">
-        <v>1445</v>
+        <v>1464</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H9" s="9">
         <v>198</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="J9" s="9">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>122</v>
+        <v>162</v>
       </c>
       <c r="L9" s="9">
-        <v>3581</v>
+        <v>3742</v>
       </c>
       <c r="M9" s="10" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="N9" s="9">
-        <v>1081</v>
+        <v>1058</v>
       </c>
       <c r="O9" s="10" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="P9" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>136</v>
+        <v>119</v>
       </c>
       <c r="R9" s="9">
-        <v>806</v>
+        <v>824</v>
       </c>
       <c r="S9" s="10" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T9" s="9">
         <v>8</v>
       </c>
       <c r="U9" s="10" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="V9" s="9">
         <v>1</v>
@@ -2454,7 +2454,7 @@
         <v>28</v>
       </c>
       <c r="Y9" s="10" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="Z9" s="9">
         <v>0</v>
@@ -2472,7 +2472,7 @@
         <v>8</v>
       </c>
       <c r="AE9" s="10" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="AF9" s="9">
         <v>1</v>
@@ -2487,10 +2487,10 @@
         <v>119</v>
       </c>
       <c r="AJ9" s="9">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AK9" s="10" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="AL9" s="9">
         <v>0</v>
@@ -2505,10 +2505,10 @@
         <v>119</v>
       </c>
       <c r="AP9" s="9">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AQ9" s="10" t="s">
-        <v>123</v>
+        <v>168</v>
       </c>
       <c r="AR9" s="9">
         <v>2</v>
@@ -2517,87 +2517,87 @@
         <v>117</v>
       </c>
       <c r="AT9" s="9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AU9" s="10" t="s">
-        <v>118</v>
+        <v>138</v>
       </c>
       <c r="AV9" s="9">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="AW9" s="10" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="AX9" s="9">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="AY9" s="10" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="C10" s="9">
-        <v>18227</v>
+        <v>18900</v>
       </c>
       <c r="D10" s="9">
         <v>35</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>169</v>
+        <v>137</v>
       </c>
       <c r="F10" s="9">
-        <v>4163</v>
+        <v>4449</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="H10" s="9">
         <v>49</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="J10" s="9">
-        <v>1673</v>
+        <v>1665</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="L10" s="9">
-        <v>5897</v>
+        <v>6199</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="N10" s="9">
-        <v>2164</v>
+        <v>2212</v>
       </c>
       <c r="O10" s="10" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="P10" s="9">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="Q10" s="10" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="R10" s="9">
-        <v>1245</v>
+        <v>1278</v>
       </c>
       <c r="S10" s="10" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="T10" s="9">
         <v>10</v>
       </c>
       <c r="U10" s="10" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="V10" s="9">
         <v>7</v>
@@ -2609,7 +2609,7 @@
         <v>14</v>
       </c>
       <c r="Y10" s="10" t="s">
-        <v>118</v>
+        <v>138</v>
       </c>
       <c r="Z10" s="9">
         <v>2</v>
@@ -2621,7 +2621,7 @@
         <v>12</v>
       </c>
       <c r="AC10" s="10" t="s">
-        <v>138</v>
+        <v>106</v>
       </c>
       <c r="AD10" s="9">
         <v>13</v>
@@ -2657,7 +2657,7 @@
         <v>52</v>
       </c>
       <c r="AO10" s="10" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="AP10" s="9">
         <v>28</v>
@@ -2669,36 +2669,36 @@
         <v>10</v>
       </c>
       <c r="AS10" s="10" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="AT10" s="9">
         <v>378</v>
       </c>
       <c r="AU10" s="10" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="AV10" s="9">
-        <v>412</v>
+        <v>423</v>
       </c>
       <c r="AW10" s="10" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="AX10" s="9">
-        <v>1894</v>
+        <v>1893</v>
       </c>
       <c r="AY10" s="10" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C11" s="9">
-        <v>12842</v>
+        <v>13038</v>
       </c>
       <c r="D11" s="9">
         <v>5</v>
@@ -2707,46 +2707,46 @@
         <v>128</v>
       </c>
       <c r="F11" s="9">
-        <v>1973</v>
+        <v>2010</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="H11" s="9">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="J11" s="9">
         <v>145</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="L11" s="9">
-        <v>5879</v>
+        <v>5999</v>
       </c>
       <c r="M11" s="10" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="N11" s="9">
         <v>627</v>
       </c>
       <c r="O11" s="10" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="P11" s="9">
         <v>22</v>
       </c>
       <c r="Q11" s="10" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="R11" s="9">
-        <v>1722</v>
+        <v>1743</v>
       </c>
       <c r="S11" s="10" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="T11" s="9">
         <v>18</v>
@@ -2764,7 +2764,7 @@
         <v>11</v>
       </c>
       <c r="Y11" s="10" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="Z11" s="9">
         <v>5</v>
@@ -2782,7 +2782,7 @@
         <v>22</v>
       </c>
       <c r="AE11" s="10" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="AF11" s="9">
         <v>0</v>
@@ -2794,13 +2794,13 @@
         <v>6</v>
       </c>
       <c r="AI11" s="10" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="AJ11" s="9">
         <v>29</v>
       </c>
       <c r="AK11" s="10" t="s">
-        <v>191</v>
+        <v>134</v>
       </c>
       <c r="AL11" s="9">
         <v>3</v>
@@ -2815,34 +2815,34 @@
         <v>138</v>
       </c>
       <c r="AP11" s="9">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="AQ11" s="10" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="AR11" s="9">
         <v>15</v>
       </c>
       <c r="AS11" s="10" t="s">
-        <v>193</v>
+        <v>162</v>
       </c>
       <c r="AT11" s="9">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AU11" s="10" t="s">
-        <v>137</v>
+        <v>195</v>
       </c>
       <c r="AV11" s="9">
-        <v>409</v>
+        <v>419</v>
       </c>
       <c r="AW11" s="10" t="s">
-        <v>194</v>
+        <v>142</v>
       </c>
       <c r="AX11" s="9">
         <v>1525</v>
       </c>
       <c r="AY11" s="10" t="s">
-        <v>195</v>
+        <v>177</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
@@ -2853,7 +2853,7 @@
         <v>197</v>
       </c>
       <c r="C12" s="9">
-        <v>5106</v>
+        <v>5162</v>
       </c>
       <c r="D12" s="9">
         <v>0</v>
@@ -2862,7 +2862,7 @@
         <v>119</v>
       </c>
       <c r="F12" s="9">
-        <v>960</v>
+        <v>975</v>
       </c>
       <c r="G12" s="10" t="s">
         <v>198</v>
@@ -2874,13 +2874,13 @@
         <v>199</v>
       </c>
       <c r="J12" s="9">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="K12" s="10" t="s">
         <v>200</v>
       </c>
       <c r="L12" s="9">
-        <v>1907</v>
+        <v>1927</v>
       </c>
       <c r="M12" s="10" t="s">
         <v>201</v>
@@ -2898,7 +2898,7 @@
         <v>106</v>
       </c>
       <c r="R12" s="9">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="S12" s="10" t="s">
         <v>203</v>
@@ -2910,16 +2910,16 @@
         <v>119</v>
       </c>
       <c r="V12" s="9">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="W12" s="10" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="X12" s="9">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="Y12" s="10" t="s">
-        <v>112</v>
+        <v>204</v>
       </c>
       <c r="Z12" s="9">
         <v>2</v>
@@ -2937,7 +2937,7 @@
         <v>9</v>
       </c>
       <c r="AE12" s="10" t="s">
-        <v>153</v>
+        <v>192</v>
       </c>
       <c r="AF12" s="9">
         <v>0</v>
@@ -2955,7 +2955,7 @@
         <v>29</v>
       </c>
       <c r="AK12" s="10" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AL12" s="9">
         <v>0</v>
@@ -2973,7 +2973,7 @@
         <v>55</v>
       </c>
       <c r="AQ12" s="10" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="AR12" s="9">
         <v>1</v>
@@ -2982,19 +2982,19 @@
         <v>117</v>
       </c>
       <c r="AT12" s="9">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="AU12" s="10" t="s">
         <v>206</v>
       </c>
       <c r="AV12" s="9">
-        <v>341</v>
+        <v>351</v>
       </c>
       <c r="AW12" s="10" t="s">
         <v>207</v>
       </c>
       <c r="AX12" s="9">
-        <v>523</v>
+        <v>534</v>
       </c>
       <c r="AY12" s="10" t="s">
         <v>208</v>
@@ -3008,7 +3008,7 @@
         <v>210</v>
       </c>
       <c r="C13" s="9">
-        <v>4694</v>
+        <v>4742</v>
       </c>
       <c r="D13" s="9">
         <v>0</v>
@@ -3023,37 +3023,37 @@
         <v>211</v>
       </c>
       <c r="H13" s="9">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I13" s="10" t="s">
         <v>212</v>
       </c>
       <c r="J13" s="9">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="K13" s="10" t="s">
         <v>213</v>
       </c>
       <c r="L13" s="9">
-        <v>1992</v>
+        <v>2032</v>
       </c>
       <c r="M13" s="10" t="s">
         <v>214</v>
       </c>
       <c r="N13" s="9">
-        <v>817</v>
+        <v>823</v>
       </c>
       <c r="O13" s="10" t="s">
         <v>215</v>
       </c>
       <c r="P13" s="9">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="Q13" s="10" t="s">
-        <v>169</v>
+        <v>117</v>
       </c>
       <c r="R13" s="9">
-        <v>273</v>
+        <v>298</v>
       </c>
       <c r="S13" s="10" t="s">
         <v>216</v>
@@ -3092,7 +3092,7 @@
         <v>8</v>
       </c>
       <c r="AE13" s="10" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="AF13" s="9">
         <v>0</v>
@@ -3110,13 +3110,13 @@
         <v>31</v>
       </c>
       <c r="AK13" s="10" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="AL13" s="9">
         <v>11</v>
       </c>
       <c r="AM13" s="10" t="s">
-        <v>191</v>
+        <v>112</v>
       </c>
       <c r="AN13" s="9">
         <v>1</v>
@@ -3128,78 +3128,78 @@
         <v>37</v>
       </c>
       <c r="AQ13" s="10" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="AR13" s="9">
         <v>23</v>
       </c>
       <c r="AS13" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="AT13" s="9">
+        <v>5</v>
+      </c>
+      <c r="AU13" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="AV13" s="9">
+        <v>220</v>
+      </c>
+      <c r="AW13" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="AX13" s="9">
+        <v>341</v>
+      </c>
+      <c r="AY13" s="10" t="s">
         <v>219</v>
-      </c>
-      <c r="AT13" s="9">
-        <v>9</v>
-      </c>
-      <c r="AU13" s="10" t="s">
-        <v>169</v>
-      </c>
-      <c r="AV13" s="9">
-        <v>217</v>
-      </c>
-      <c r="AW13" s="10" t="s">
-        <v>220</v>
-      </c>
-      <c r="AX13" s="9">
-        <v>338</v>
-      </c>
-      <c r="AY13" s="10" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="C14" s="9">
+        <v>4395</v>
+      </c>
+      <c r="D14" s="9">
+        <v>0</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="F14" s="9">
+        <v>1031</v>
+      </c>
+      <c r="G14" s="10" t="s">
         <v>222</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>223</v>
-      </c>
-      <c r="C14" s="9">
-        <v>4377</v>
-      </c>
-      <c r="D14" s="9">
-        <v>0</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="F14" s="9">
-        <v>1029</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>224</v>
       </c>
       <c r="H14" s="9">
         <v>18</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="J14" s="9">
         <v>114</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="L14" s="9">
-        <v>1197</v>
+        <v>1207</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="N14" s="9">
         <v>686</v>
       </c>
       <c r="O14" s="10" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="P14" s="9">
         <v>8</v>
@@ -3208,16 +3208,16 @@
         <v>153</v>
       </c>
       <c r="R14" s="9">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="S14" s="10" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="T14" s="9">
         <v>2</v>
       </c>
       <c r="U14" s="10" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="V14" s="9">
         <v>1</v>
@@ -3226,10 +3226,10 @@
         <v>117</v>
       </c>
       <c r="X14" s="9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Y14" s="10" t="s">
-        <v>153</v>
+        <v>228</v>
       </c>
       <c r="Z14" s="9">
         <v>1</v>
@@ -3247,7 +3247,7 @@
         <v>5</v>
       </c>
       <c r="AE14" s="10" t="s">
-        <v>230</v>
+        <v>140</v>
       </c>
       <c r="AF14" s="9">
         <v>0</v>
@@ -3265,7 +3265,7 @@
         <v>11</v>
       </c>
       <c r="AK14" s="10" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="AL14" s="9">
         <v>1</v>
@@ -3283,7 +3283,7 @@
         <v>28</v>
       </c>
       <c r="AQ14" s="10" t="s">
-        <v>212</v>
+        <v>229</v>
       </c>
       <c r="AR14" s="9">
         <v>1</v>
@@ -3295,30 +3295,30 @@
         <v>106</v>
       </c>
       <c r="AU14" s="10" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="AV14" s="9">
         <v>322</v>
       </c>
       <c r="AW14" s="10" t="s">
-        <v>113</v>
+        <v>231</v>
       </c>
       <c r="AX14" s="9">
         <v>587</v>
       </c>
       <c r="AY14" s="10" t="s">
-        <v>190</v>
+        <v>232</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C15" s="9">
-        <v>12522</v>
+        <v>12530</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
@@ -3327,16 +3327,16 @@
         <v>119</v>
       </c>
       <c r="F15" s="9">
-        <v>3842</v>
+        <v>3849</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="H15" s="9">
         <v>56</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="J15" s="9">
         <v>5</v>
@@ -3345,16 +3345,16 @@
         <v>128</v>
       </c>
       <c r="L15" s="9">
-        <v>3821</v>
+        <v>3822</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="N15" s="9">
         <v>236</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="P15" s="9">
         <v>1</v>
@@ -3366,13 +3366,13 @@
         <v>733</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="T15" s="9">
         <v>41</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="V15" s="9">
         <v>0</v>
@@ -3384,7 +3384,7 @@
         <v>15</v>
       </c>
       <c r="Y15" s="10" t="s">
-        <v>193</v>
+        <v>162</v>
       </c>
       <c r="Z15" s="9">
         <v>0</v>
@@ -3438,7 +3438,7 @@
         <v>79</v>
       </c>
       <c r="AQ15" s="10" t="s">
-        <v>206</v>
+        <v>240</v>
       </c>
       <c r="AR15" s="9">
         <v>19</v>
@@ -3456,24 +3456,24 @@
         <v>1052</v>
       </c>
       <c r="AW15" s="10" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="AX15" s="9">
         <v>2600</v>
       </c>
       <c r="AY15" s="10" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C16" s="9">
-        <v>4709</v>
+        <v>4891</v>
       </c>
       <c r="D16" s="9">
         <v>2</v>
@@ -3482,46 +3482,46 @@
         <v>128</v>
       </c>
       <c r="F16" s="9">
-        <v>849</v>
+        <v>883</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="H16" s="9">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="I16" s="10" t="s">
+        <v>246</v>
+      </c>
+      <c r="J16" s="9">
+        <v>47</v>
+      </c>
+      <c r="K16" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="L16" s="9">
+        <v>1570</v>
+      </c>
+      <c r="M16" s="10" t="s">
+        <v>247</v>
+      </c>
+      <c r="N16" s="9">
+        <v>150</v>
+      </c>
+      <c r="O16" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="P16" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="R16" s="9">
         <v>244</v>
       </c>
-      <c r="J16" s="9">
-        <v>50</v>
-      </c>
-      <c r="K16" s="10" t="s">
-        <v>245</v>
-      </c>
-      <c r="L16" s="9">
-        <v>1498</v>
-      </c>
-      <c r="M16" s="10" t="s">
-        <v>246</v>
-      </c>
-      <c r="N16" s="9">
-        <v>143</v>
-      </c>
-      <c r="O16" s="10" t="s">
-        <v>247</v>
-      </c>
-      <c r="P16" s="9">
-        <v>2</v>
-      </c>
-      <c r="Q16" s="10" t="s">
-        <v>128</v>
-      </c>
-      <c r="R16" s="9">
-        <v>235</v>
-      </c>
       <c r="S16" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="T16" s="9">
         <v>0</v>
@@ -3530,10 +3530,10 @@
         <v>119</v>
       </c>
       <c r="V16" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W16" s="10" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="X16" s="9">
         <v>4</v>
@@ -3542,10 +3542,10 @@
         <v>118</v>
       </c>
       <c r="Z16" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AA16" s="10" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="AB16" s="9">
         <v>1</v>
@@ -3575,7 +3575,7 @@
         <v>29</v>
       </c>
       <c r="AK16" s="10" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="AL16" s="9">
         <v>4</v>
@@ -3590,7 +3590,7 @@
         <v>117</v>
       </c>
       <c r="AP16" s="9">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="AQ16" s="10" t="s">
         <v>250</v>
@@ -3599,22 +3599,22 @@
         <v>7</v>
       </c>
       <c r="AS16" s="10" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
       <c r="AT16" s="9">
-        <v>100</v>
+        <v>52</v>
       </c>
       <c r="AU16" s="10" t="s">
         <v>251</v>
       </c>
       <c r="AV16" s="9">
-        <v>396</v>
+        <v>403</v>
       </c>
       <c r="AW16" s="10" t="s">
         <v>252</v>
       </c>
       <c r="AX16" s="9">
-        <v>1313</v>
+        <v>1415</v>
       </c>
       <c r="AY16" s="10" t="s">
         <v>253</v>
@@ -3628,55 +3628,55 @@
         <v>255</v>
       </c>
       <c r="C17" s="9">
-        <v>8127</v>
+        <v>8395</v>
       </c>
       <c r="D17" s="9">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E17" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="F17" s="9">
+        <v>2536</v>
+      </c>
+      <c r="G17" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="F17" s="9">
-        <v>2443</v>
-      </c>
-      <c r="G17" s="10" t="s">
+      <c r="H17" s="9">
+        <v>319</v>
+      </c>
+      <c r="I17" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="H17" s="9">
-        <v>332</v>
-      </c>
-      <c r="I17" s="10" t="s">
+      <c r="J17" s="9">
+        <v>127</v>
+      </c>
+      <c r="K17" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="J17" s="9">
-        <v>128</v>
-      </c>
-      <c r="K17" s="10" t="s">
+      <c r="L17" s="9">
+        <v>3083</v>
+      </c>
+      <c r="M17" s="10" t="s">
         <v>259</v>
       </c>
-      <c r="L17" s="9">
-        <v>2916</v>
-      </c>
-      <c r="M17" s="10" t="s">
+      <c r="N17" s="9">
+        <v>470</v>
+      </c>
+      <c r="O17" s="10" t="s">
         <v>260</v>
       </c>
-      <c r="N17" s="9">
-        <v>468</v>
-      </c>
-      <c r="O17" s="10" t="s">
+      <c r="P17" s="9">
+        <v>22</v>
+      </c>
+      <c r="Q17" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="R17" s="9">
+        <v>304</v>
+      </c>
+      <c r="S17" s="10" t="s">
         <v>261</v>
-      </c>
-      <c r="P17" s="9">
-        <v>21</v>
-      </c>
-      <c r="Q17" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="R17" s="9">
-        <v>294</v>
-      </c>
-      <c r="S17" s="10" t="s">
-        <v>262</v>
       </c>
       <c r="T17" s="9">
         <v>1</v>
@@ -3712,7 +3712,7 @@
         <v>4</v>
       </c>
       <c r="AE17" s="10" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="AF17" s="9">
         <v>0</v>
@@ -3742,102 +3742,102 @@
         <v>7</v>
       </c>
       <c r="AO17" s="10" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="AP17" s="9">
         <v>44</v>
       </c>
       <c r="AQ17" s="10" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="AR17" s="9">
         <v>9</v>
       </c>
       <c r="AS17" s="10" t="s">
-        <v>230</v>
+        <v>140</v>
       </c>
       <c r="AT17" s="9">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="AU17" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="AV17" s="9">
+        <v>703</v>
+      </c>
+      <c r="AW17" s="10" t="s">
         <v>264</v>
       </c>
-      <c r="AV17" s="9">
-        <v>698</v>
-      </c>
-      <c r="AW17" s="10" t="s">
+      <c r="AX17" s="9">
+        <v>453</v>
+      </c>
+      <c r="AY17" s="10" t="s">
         <v>265</v>
-      </c>
-      <c r="AX17" s="9">
-        <v>451</v>
-      </c>
-      <c r="AY17" s="10" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>267</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="C18" s="9">
+        <v>9389</v>
+      </c>
+      <c r="D18" s="9">
+        <v>1</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="F18" s="9">
+        <v>1584</v>
+      </c>
+      <c r="G18" s="10" t="s">
         <v>268</v>
-      </c>
-      <c r="C18" s="9">
-        <v>9245</v>
-      </c>
-      <c r="D18" s="9">
-        <v>2</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="F18" s="9">
-        <v>1557</v>
-      </c>
-      <c r="G18" s="10" t="s">
-        <v>269</v>
       </c>
       <c r="H18" s="9">
         <v>148</v>
       </c>
       <c r="I18" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="J18" s="9">
+        <v>186</v>
+      </c>
+      <c r="K18" s="10" t="s">
         <v>270</v>
       </c>
-      <c r="J18" s="9">
+      <c r="L18" s="9">
+        <v>2927</v>
+      </c>
+      <c r="M18" s="10" t="s">
         <v>271</v>
       </c>
-      <c r="K18" s="10" t="s">
-        <v>271</v>
-      </c>
-      <c r="L18" s="9">
-        <v>2906</v>
-      </c>
-      <c r="M18" s="10" t="s">
+      <c r="N18" s="9">
+        <v>1655</v>
+      </c>
+      <c r="O18" s="10" t="s">
         <v>272</v>
       </c>
-      <c r="N18" s="9">
-        <v>1481</v>
-      </c>
-      <c r="O18" s="10" t="s">
+      <c r="P18" s="9">
+        <v>29</v>
+      </c>
+      <c r="Q18" s="10" t="s">
         <v>273</v>
       </c>
-      <c r="P18" s="9">
-        <v>30</v>
-      </c>
-      <c r="Q18" s="10" t="s">
-        <v>274</v>
-      </c>
       <c r="R18" s="9">
-        <v>533</v>
+        <v>538</v>
       </c>
       <c r="S18" s="10" t="s">
-        <v>275</v>
+        <v>227</v>
       </c>
       <c r="T18" s="9">
         <v>22</v>
       </c>
       <c r="U18" s="10" t="s">
-        <v>134</v>
+        <v>112</v>
       </c>
       <c r="V18" s="9">
         <v>0</v>
@@ -3849,7 +3849,7 @@
         <v>5</v>
       </c>
       <c r="Y18" s="10" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="Z18" s="9">
         <v>1</v>
@@ -3885,60 +3885,60 @@
         <v>11</v>
       </c>
       <c r="AK18" s="10" t="s">
-        <v>193</v>
+        <v>162</v>
       </c>
       <c r="AL18" s="9">
         <v>5</v>
       </c>
       <c r="AM18" s="10" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="AN18" s="9">
         <v>5</v>
       </c>
       <c r="AO18" s="10" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="AP18" s="9">
         <v>26</v>
       </c>
       <c r="AQ18" s="10" t="s">
-        <v>276</v>
+        <v>181</v>
       </c>
       <c r="AR18" s="9">
         <v>12</v>
       </c>
       <c r="AS18" s="10" t="s">
-        <v>140</v>
+        <v>274</v>
       </c>
       <c r="AT18" s="9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AU18" s="10" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="AV18" s="9">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="AW18" s="10" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="AX18" s="9">
-        <v>1831</v>
+        <v>1833</v>
       </c>
       <c r="AY18" s="10" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C19" s="9">
-        <v>8945</v>
+        <v>9497</v>
       </c>
       <c r="D19" s="9">
         <v>1</v>
@@ -3947,46 +3947,46 @@
         <v>136</v>
       </c>
       <c r="F19" s="9">
-        <v>1085</v>
+        <v>1135</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="H19" s="9">
         <v>15</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>189</v>
+        <v>280</v>
       </c>
       <c r="J19" s="9">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="K19" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="L19" s="9">
+        <v>4254</v>
+      </c>
+      <c r="M19" s="10" t="s">
         <v>282</v>
       </c>
-      <c r="L19" s="9">
-        <v>3825</v>
-      </c>
-      <c r="M19" s="10" t="s">
+      <c r="N19" s="9">
+        <v>1530</v>
+      </c>
+      <c r="O19" s="10" t="s">
         <v>283</v>
       </c>
-      <c r="N19" s="9">
-        <v>1516</v>
-      </c>
-      <c r="O19" s="10" t="s">
+      <c r="P19" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="R19" s="9">
+        <v>954</v>
+      </c>
+      <c r="S19" s="10" t="s">
         <v>284</v>
-      </c>
-      <c r="P19" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="R19" s="9">
-        <v>907</v>
-      </c>
-      <c r="S19" s="10" t="s">
-        <v>285</v>
       </c>
       <c r="T19" s="9">
         <v>0</v>
@@ -4004,7 +4004,7 @@
         <v>17</v>
       </c>
       <c r="Y19" s="10" t="s">
-        <v>169</v>
+        <v>153</v>
       </c>
       <c r="Z19" s="9">
         <v>0</v>
@@ -4040,7 +4040,7 @@
         <v>16</v>
       </c>
       <c r="AK19" s="10" t="s">
-        <v>153</v>
+        <v>192</v>
       </c>
       <c r="AL19" s="9">
         <v>0</v>
@@ -4055,10 +4055,10 @@
         <v>136</v>
       </c>
       <c r="AP19" s="9">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="AQ19" s="10" t="s">
-        <v>204</v>
+        <v>246</v>
       </c>
       <c r="AR19" s="9">
         <v>1</v>
@@ -4067,33 +4067,33 @@
         <v>136</v>
       </c>
       <c r="AT19" s="9">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="AU19" s="10" t="s">
-        <v>189</v>
+        <v>274</v>
       </c>
       <c r="AV19" s="9">
-        <v>622</v>
+        <v>637</v>
       </c>
       <c r="AW19" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="AX19" s="9">
+        <v>838</v>
+      </c>
+      <c r="AY19" s="10" t="s">
         <v>286</v>
-      </c>
-      <c r="AX19" s="9">
-        <v>835</v>
-      </c>
-      <c r="AY19" s="10" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
+        <v>287</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>288</v>
       </c>
-      <c r="B20" s="8" t="s">
-        <v>289</v>
-      </c>
       <c r="C20" s="9">
-        <v>1041</v>
+        <v>1046</v>
       </c>
       <c r="D20" s="9">
         <v>1</v>
@@ -4105,22 +4105,22 @@
         <v>162</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="H20" s="9">
         <v>6</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>121</v>
+        <v>290</v>
       </c>
       <c r="J20" s="9">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K20" s="10" t="s">
         <v>291</v>
       </c>
       <c r="L20" s="9">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="M20" s="10" t="s">
         <v>292</v>
@@ -4135,7 +4135,7 @@
         <v>6</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>121</v>
+        <v>290</v>
       </c>
       <c r="R20" s="9">
         <v>168</v>
@@ -4165,7 +4165,7 @@
         <v>3</v>
       </c>
       <c r="AA20" s="10" t="s">
-        <v>178</v>
+        <v>206</v>
       </c>
       <c r="AB20" s="9">
         <v>0</v>
@@ -4195,13 +4195,13 @@
         <v>6</v>
       </c>
       <c r="AK20" s="10" t="s">
-        <v>121</v>
+        <v>290</v>
       </c>
       <c r="AL20" s="9">
         <v>2</v>
       </c>
       <c r="AM20" s="10" t="s">
-        <v>169</v>
+        <v>137</v>
       </c>
       <c r="AN20" s="9">
         <v>1</v>
@@ -4219,36 +4219,36 @@
         <v>4</v>
       </c>
       <c r="AS20" s="10" t="s">
-        <v>282</v>
+        <v>297</v>
       </c>
       <c r="AT20" s="9">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="AU20" s="10" t="s">
-        <v>245</v>
+        <v>298</v>
       </c>
       <c r="AV20" s="9">
         <v>47</v>
       </c>
       <c r="AW20" s="10" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="AX20" s="9">
         <v>185</v>
       </c>
       <c r="AY20" s="10" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="C21" s="9">
-        <v>2476</v>
+        <v>2553</v>
       </c>
       <c r="D21" s="9">
         <v>0</v>
@@ -4257,16 +4257,16 @@
         <v>119</v>
       </c>
       <c r="F21" s="9">
-        <v>398</v>
+        <v>420</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="H21" s="9">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="J21" s="9">
         <v>1</v>
@@ -4275,28 +4275,28 @@
         <v>128</v>
       </c>
       <c r="L21" s="9">
-        <v>729</v>
+        <v>774</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="N21" s="9">
         <v>102</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="P21" s="9">
         <v>8</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R21" s="9">
         <v>79</v>
       </c>
       <c r="S21" s="10" t="s">
-        <v>305</v>
+        <v>263</v>
       </c>
       <c r="T21" s="9">
         <v>0</v>
@@ -4314,7 +4314,7 @@
         <v>17</v>
       </c>
       <c r="Y21" s="10" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="Z21" s="9">
         <v>2</v>
@@ -4350,7 +4350,7 @@
         <v>3</v>
       </c>
       <c r="AK21" s="10" t="s">
-        <v>193</v>
+        <v>162</v>
       </c>
       <c r="AL21" s="9">
         <v>0</v>
@@ -4368,7 +4368,7 @@
         <v>18</v>
       </c>
       <c r="AQ21" s="10" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="AR21" s="9">
         <v>1</v>
@@ -4377,10 +4377,10 @@
         <v>128</v>
       </c>
       <c r="AT21" s="9">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="AU21" s="10" t="s">
-        <v>308</v>
+        <v>199</v>
       </c>
       <c r="AV21" s="9">
         <v>96</v>
@@ -4389,7 +4389,7 @@
         <v>309</v>
       </c>
       <c r="AX21" s="9">
-        <v>825</v>
+        <v>863</v>
       </c>
       <c r="AY21" s="10" t="s">
         <v>310</v>
@@ -4403,16 +4403,16 @@
         <v>312</v>
       </c>
       <c r="C22" s="12">
-        <v>111025</v>
+        <v>113814</v>
       </c>
       <c r="D22" s="12">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>106</v>
       </c>
       <c r="F22" s="12">
-        <v>22589</v>
+        <v>23252</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>107</v>
@@ -4424,31 +4424,31 @@
         <v>108</v>
       </c>
       <c r="J22" s="12">
-        <v>2698</v>
+        <v>2565</v>
       </c>
       <c r="K22" s="13" t="s">
         <v>109</v>
       </c>
       <c r="L22" s="12">
-        <v>40497</v>
+        <v>42111</v>
       </c>
       <c r="M22" s="13" t="s">
         <v>110</v>
       </c>
       <c r="N22" s="12">
-        <v>11488</v>
+        <v>11727</v>
       </c>
       <c r="O22" s="13" t="s">
         <v>111</v>
       </c>
       <c r="P22" s="12">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="Q22" s="13" t="s">
         <v>112</v>
       </c>
       <c r="R22" s="12">
-        <v>8174</v>
+        <v>8364</v>
       </c>
       <c r="S22" s="13" t="s">
         <v>113</v>
@@ -4460,19 +4460,19 @@
         <v>114</v>
       </c>
       <c r="V22" s="12">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="W22" s="13" t="s">
         <v>115</v>
       </c>
       <c r="X22" s="12">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="Y22" s="13" t="s">
         <v>116</v>
       </c>
       <c r="Z22" s="12">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="AA22" s="13" t="s">
         <v>117</v>
@@ -4502,7 +4502,7 @@
         <v>117</v>
       </c>
       <c r="AJ22" s="12">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="AK22" s="13" t="s">
         <v>120</v>
@@ -4514,13 +4514,13 @@
         <v>115</v>
       </c>
       <c r="AN22" s="12">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="AO22" s="13" t="s">
         <v>118</v>
       </c>
       <c r="AP22" s="12">
-        <v>649</v>
+        <v>659</v>
       </c>
       <c r="AQ22" s="13" t="s">
         <v>121</v>
@@ -4532,19 +4532,19 @@
         <v>122</v>
       </c>
       <c r="AT22" s="12">
-        <v>1296</v>
+        <v>1143</v>
       </c>
       <c r="AU22" s="13" t="s">
         <v>123</v>
       </c>
       <c r="AV22" s="12">
-        <v>5755</v>
+        <v>5832</v>
       </c>
       <c r="AW22" s="13" t="s">
         <v>124</v>
       </c>
       <c r="AX22" s="12">
-        <v>15094</v>
+        <v>15378</v>
       </c>
       <c r="AY22" s="13" t="s">
         <v>125</v>

</xml_diff>

<commit_message>
Perbarui data SE2026 03/09/2026 13:28:48,17
</commit_message>
<xml_diff>
--- a/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
+++ b/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="312">
   <si>
     <t>DATA RADAR ANOMALI USAHA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 2 Sep 2026, 10.04</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 3 Sep 2026, 13.26</t>
   </si>
   <si>
     <t>Kode</t>
@@ -334,616 +334,613 @@
     <t>0,06</t>
   </si>
   <si>
-    <t>20,43</t>
-  </si>
-  <si>
-    <t>1,27</t>
-  </si>
-  <si>
-    <t>2,25</t>
-  </si>
-  <si>
-    <t>37</t>
-  </si>
-  <si>
-    <t>10,3</t>
+    <t>20,37</t>
+  </si>
+  <si>
+    <t>1,3</t>
+  </si>
+  <si>
+    <t>2,04</t>
+  </si>
+  <si>
+    <t>37,66</t>
+  </si>
+  <si>
+    <t>10,19</t>
+  </si>
+  <si>
+    <t>0,21</t>
+  </si>
+  <si>
+    <t>7,52</t>
+  </si>
+  <si>
+    <t>0,08</t>
+  </si>
+  <si>
+    <t>0,03</t>
+  </si>
+  <si>
+    <t>0,16</t>
+  </si>
+  <si>
+    <t>0,02</t>
+  </si>
+  <si>
+    <t>0,07</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>0,25</t>
+  </si>
+  <si>
+    <t>0,58</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>0,93</t>
+  </si>
+  <si>
+    <t>5,07</t>
+  </si>
+  <si>
+    <t>13,22</t>
+  </si>
+  <si>
+    <t>1801</t>
+  </si>
+  <si>
+    <t>LAMPUNG BARAT</t>
+  </si>
+  <si>
+    <t>0,09</t>
+  </si>
+  <si>
+    <t>19,23</t>
+  </si>
+  <si>
+    <t>0,96</t>
+  </si>
+  <si>
+    <t>1,02</t>
+  </si>
+  <si>
+    <t>47,57</t>
+  </si>
+  <si>
+    <t>4,04</t>
+  </si>
+  <si>
+    <t>0,18</t>
+  </si>
+  <si>
+    <t>4,55</t>
+  </si>
+  <si>
+    <t>0,01</t>
+  </si>
+  <si>
+    <t>0,19</t>
+  </si>
+  <si>
+    <t>0,13</t>
+  </si>
+  <si>
+    <t>0,35</t>
+  </si>
+  <si>
+    <t>0,04</t>
+  </si>
+  <si>
+    <t>2,82</t>
+  </si>
+  <si>
+    <t>3,52</t>
+  </si>
+  <si>
+    <t>14,99</t>
+  </si>
+  <si>
+    <t>1802</t>
+  </si>
+  <si>
+    <t>TANGGAMUS</t>
+  </si>
+  <si>
+    <t>13,71</t>
+  </si>
+  <si>
+    <t>0,54</t>
+  </si>
+  <si>
+    <t>1,08</t>
+  </si>
+  <si>
+    <t>26,37</t>
+  </si>
+  <si>
+    <t>30,38</t>
+  </si>
+  <si>
+    <t>6,45</t>
+  </si>
+  <si>
+    <t>0,15</t>
+  </si>
+  <si>
+    <t>0,48</t>
+  </si>
+  <si>
+    <t>0,3</t>
+  </si>
+  <si>
+    <t>4,63</t>
+  </si>
+  <si>
+    <t>15,65</t>
+  </si>
+  <si>
+    <t>1803</t>
+  </si>
+  <si>
+    <t>LAMPUNG SELATAN</t>
+  </si>
+  <si>
+    <t>16,52</t>
+  </si>
+  <si>
+    <t>2,2</t>
+  </si>
+  <si>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>44,83</t>
+  </si>
+  <si>
+    <t>11,37</t>
+  </si>
+  <si>
+    <t>10,82</t>
+  </si>
+  <si>
+    <t>0,4</t>
+  </si>
+  <si>
+    <t>0,72</t>
+  </si>
+  <si>
+    <t>1,11</t>
+  </si>
+  <si>
+    <t>4,01</t>
+  </si>
+  <si>
+    <t>7,7</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>0,17</t>
+  </si>
+  <si>
+    <t>23,32</t>
+  </si>
+  <si>
+    <t>0,77</t>
+  </si>
+  <si>
+    <t>8,5</t>
+  </si>
+  <si>
+    <t>33,28</t>
+  </si>
+  <si>
+    <t>11,68</t>
+  </si>
+  <si>
+    <t>0,76</t>
+  </si>
+  <si>
+    <t>6,72</t>
+  </si>
+  <si>
+    <t>0,05</t>
+  </si>
+  <si>
+    <t>0,27</t>
+  </si>
+  <si>
+    <t>0,14</t>
+  </si>
+  <si>
+    <t>1,96</t>
+  </si>
+  <si>
+    <t>2,22</t>
+  </si>
+  <si>
+    <t>9,73</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>15,54</t>
+  </si>
+  <si>
+    <t>2,29</t>
+  </si>
+  <si>
+    <t>46,17</t>
+  </si>
+  <si>
+    <t>4,72</t>
+  </si>
+  <si>
+    <t>13,23</t>
+  </si>
+  <si>
+    <t>0,22</t>
+  </si>
+  <si>
+    <t>0,65</t>
+  </si>
+  <si>
+    <t>0,11</t>
+  </si>
+  <si>
+    <t>3,24</t>
+  </si>
+  <si>
+    <t>11,63</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>18,92</t>
+  </si>
+  <si>
+    <t>0,74</t>
+  </si>
+  <si>
+    <t>1,04</t>
+  </si>
+  <si>
+    <t>37,31</t>
+  </si>
+  <si>
+    <t>14,1</t>
+  </si>
+  <si>
+    <t>7,81</t>
+  </si>
+  <si>
+    <t>0,56</t>
+  </si>
+  <si>
+    <t>1,06</t>
+  </si>
+  <si>
+    <t>0,37</t>
+  </si>
+  <si>
+    <t>6,79</t>
+  </si>
+  <si>
+    <t>10,33</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>17,99</t>
   </si>
   <si>
     <t>0,23</t>
   </si>
   <si>
-    <t>7,35</t>
-  </si>
-  <si>
-    <t>0,09</t>
-  </si>
-  <si>
-    <t>0,03</t>
-  </si>
-  <si>
-    <t>0,15</t>
-  </si>
-  <si>
-    <t>0,02</t>
-  </si>
-  <si>
-    <t>0,08</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>0,25</t>
-  </si>
-  <si>
-    <t>0,58</t>
-  </si>
-  <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>5,12</t>
-  </si>
-  <si>
-    <t>13,51</t>
-  </si>
-  <si>
-    <t>1801</t>
-  </si>
-  <si>
-    <t>LAMPUNG BARAT</t>
-  </si>
-  <si>
-    <t>0,04</t>
-  </si>
-  <si>
-    <t>19,56</t>
-  </si>
-  <si>
-    <t>0,96</t>
-  </si>
-  <si>
-    <t>1,25</t>
-  </si>
-  <si>
-    <t>45,66</t>
-  </si>
-  <si>
-    <t>5,21</t>
-  </si>
-  <si>
-    <t>0,22</t>
-  </si>
-  <si>
-    <t>4,46</t>
-  </si>
-  <si>
-    <t>0,01</t>
-  </si>
-  <si>
-    <t>0,19</t>
-  </si>
-  <si>
-    <t>0,07</t>
-  </si>
-  <si>
-    <t>0,14</t>
-  </si>
-  <si>
-    <t>0,11</t>
-  </si>
-  <si>
-    <t>0,34</t>
-  </si>
-  <si>
-    <t>3,21</t>
-  </si>
-  <si>
-    <t>3,44</t>
-  </si>
-  <si>
-    <t>14,92</t>
-  </si>
-  <si>
-    <t>1802</t>
-  </si>
-  <si>
-    <t>TANGGAMUS</t>
-  </si>
-  <si>
-    <t>13,73</t>
-  </si>
-  <si>
-    <t>0,54</t>
-  </si>
-  <si>
-    <t>1,08</t>
-  </si>
-  <si>
-    <t>26,23</t>
-  </si>
-  <si>
-    <t>30,42</t>
-  </si>
-  <si>
-    <t>6,46</t>
-  </si>
-  <si>
-    <t>0,18</t>
-  </si>
-  <si>
-    <t>0,48</t>
-  </si>
-  <si>
-    <t>0,3</t>
-  </si>
-  <si>
-    <t>4,64</t>
-  </si>
-  <si>
-    <t>15,67</t>
-  </si>
-  <si>
-    <t>1803</t>
-  </si>
-  <si>
-    <t>LAMPUNG SELATAN</t>
-  </si>
-  <si>
-    <t>17,1</t>
-  </si>
-  <si>
-    <t>2,31</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>43,72</t>
-  </si>
-  <si>
-    <t>12,36</t>
-  </si>
-  <si>
-    <t>9,63</t>
+    <t>43,08</t>
+  </si>
+  <si>
+    <t>17,34</t>
+  </si>
+  <si>
+    <t>6,37</t>
+  </si>
+  <si>
+    <t>0,78</t>
+  </si>
+  <si>
+    <t>4,62</t>
+  </si>
+  <si>
+    <t>7,23</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>23,22</t>
+  </si>
+  <si>
+    <t>27,9</t>
+  </si>
+  <si>
+    <t>15,94</t>
+  </si>
+  <si>
+    <t>5,87</t>
+  </si>
+  <si>
+    <t>0,2</t>
+  </si>
+  <si>
+    <t>0,31</t>
+  </si>
+  <si>
+    <t>0,68</t>
+  </si>
+  <si>
+    <t>1,89</t>
+  </si>
+  <si>
+    <t>7,45</t>
+  </si>
+  <si>
+    <t>13,57</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>30,79</t>
+  </si>
+  <si>
+    <t>0,44</t>
+  </si>
+  <si>
+    <t>30,57</t>
+  </si>
+  <si>
+    <t>1,8</t>
+  </si>
+  <si>
+    <t>5,84</t>
   </si>
   <si>
     <t>0,33</t>
   </si>
   <si>
-    <t>0,76</t>
-  </si>
-  <si>
-    <t>1,17</t>
-  </si>
-  <si>
-    <t>4,17</t>
-  </si>
-  <si>
-    <t>8,03</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>23,54</t>
-  </si>
-  <si>
-    <t>0,26</t>
-  </si>
-  <si>
-    <t>8,81</t>
-  </si>
-  <si>
-    <t>32,8</t>
-  </si>
-  <si>
-    <t>11,7</t>
-  </si>
-  <si>
-    <t>0,79</t>
-  </si>
-  <si>
-    <t>6,76</t>
-  </si>
-  <si>
-    <t>0,05</t>
-  </si>
-  <si>
-    <t>0,28</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>2,24</t>
-  </si>
-  <si>
-    <t>10,02</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>15,42</t>
-  </si>
-  <si>
-    <t>2,33</t>
-  </si>
-  <si>
-    <t>1,11</t>
-  </si>
-  <si>
-    <t>46,01</t>
-  </si>
-  <si>
-    <t>4,81</t>
-  </si>
-  <si>
-    <t>0,17</t>
-  </si>
-  <si>
-    <t>13,37</t>
+    <t>0,63</t>
+  </si>
+  <si>
+    <t>8,39</t>
+  </si>
+  <si>
+    <t>20,72</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>17,77</t>
+  </si>
+  <si>
+    <t>31,57</t>
+  </si>
+  <si>
+    <t>5,3</t>
+  </si>
+  <si>
+    <t>5,26</t>
+  </si>
+  <si>
+    <t>0,57</t>
+  </si>
+  <si>
+    <t>0,85</t>
+  </si>
+  <si>
+    <t>0,71</t>
+  </si>
+  <si>
+    <t>8,3</t>
+  </si>
+  <si>
+    <t>28,39</t>
+  </si>
+  <si>
+    <t>1811</t>
+  </si>
+  <si>
+    <t>MESUJI</t>
+  </si>
+  <si>
+    <t>30,32</t>
+  </si>
+  <si>
+    <t>3,25</t>
+  </si>
+  <si>
+    <t>1,42</t>
+  </si>
+  <si>
+    <t>37,84</t>
+  </si>
+  <si>
+    <t>5,55</t>
+  </si>
+  <si>
+    <t>3,93</t>
+  </si>
+  <si>
+    <t>0,49</t>
+  </si>
+  <si>
+    <t>2,92</t>
+  </si>
+  <si>
+    <t>8,05</t>
+  </si>
+  <si>
+    <t>5,13</t>
+  </si>
+  <si>
+    <t>1812</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG BARAT</t>
+  </si>
+  <si>
+    <t>17,87</t>
+  </si>
+  <si>
+    <t>1,5</t>
+  </si>
+  <si>
+    <t>1,34</t>
+  </si>
+  <si>
+    <t>32,23</t>
+  </si>
+  <si>
+    <t>17,09</t>
+  </si>
+  <si>
+    <t>6,32</t>
+  </si>
+  <si>
+    <t>0,24</t>
+  </si>
+  <si>
+    <t>0,38</t>
+  </si>
+  <si>
+    <t>18,4</t>
+  </si>
+  <si>
+    <t>1813</t>
+  </si>
+  <si>
+    <t>PESISIR BARAT</t>
+  </si>
+  <si>
+    <t>46,31</t>
+  </si>
+  <si>
+    <t>15,79</t>
+  </si>
+  <si>
+    <t>10,22</t>
+  </si>
+  <si>
+    <t>6,56</t>
+  </si>
+  <si>
+    <t>8,38</t>
+  </si>
+  <si>
+    <t>1871</t>
+  </si>
+  <si>
+    <t>BANDAR LAMPUNG</t>
+  </si>
+  <si>
+    <t>15,44</t>
+  </si>
+  <si>
+    <t>3,43</t>
+  </si>
+  <si>
+    <t>31,65</t>
+  </si>
+  <si>
+    <t>4,58</t>
+  </si>
+  <si>
+    <t>16,02</t>
+  </si>
+  <si>
+    <t>0,86</t>
+  </si>
+  <si>
+    <t>0,29</t>
+  </si>
+  <si>
+    <t>1,72</t>
+  </si>
+  <si>
+    <t>1,33</t>
+  </si>
+  <si>
+    <t>4,48</t>
+  </si>
+  <si>
+    <t>17,64</t>
+  </si>
+  <si>
+    <t>1872</t>
+  </si>
+  <si>
+    <t>METRO</t>
+  </si>
+  <si>
+    <t>16,4</t>
+  </si>
+  <si>
+    <t>5,86</t>
+  </si>
+  <si>
+    <t>30,34</t>
+  </si>
+  <si>
+    <t>3,98</t>
+  </si>
+  <si>
+    <t>3,08</t>
   </si>
   <si>
     <t>0,66</t>
   </si>
   <si>
-    <t>0,21</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>18,89</t>
-  </si>
-  <si>
-    <t>0,74</t>
-  </si>
-  <si>
-    <t>1,07</t>
-  </si>
-  <si>
-    <t>37,33</t>
-  </si>
-  <si>
-    <t>14,12</t>
-  </si>
-  <si>
-    <t>7,83</t>
-  </si>
-  <si>
-    <t>0,35</t>
-  </si>
-  <si>
-    <t>0,56</t>
-  </si>
-  <si>
-    <t>0,29</t>
-  </si>
-  <si>
-    <t>6,8</t>
-  </si>
-  <si>
-    <t>10,34</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>17,99</t>
-  </si>
-  <si>
-    <t>0,65</t>
-  </si>
-  <si>
-    <t>0,44</t>
-  </si>
-  <si>
-    <t>42,85</t>
-  </si>
-  <si>
-    <t>17,36</t>
-  </si>
-  <si>
-    <t>6,28</t>
-  </si>
-  <si>
-    <t>0,78</t>
-  </si>
-  <si>
-    <t>0,49</t>
-  </si>
-  <si>
-    <t>7,19</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>23,46</t>
-  </si>
-  <si>
-    <t>0,41</t>
-  </si>
-  <si>
-    <t>2,59</t>
-  </si>
-  <si>
-    <t>27,46</t>
-  </si>
-  <si>
-    <t>15,61</t>
-  </si>
-  <si>
-    <t>5,73</t>
-  </si>
-  <si>
-    <t>0,2</t>
-  </si>
-  <si>
-    <t>0,64</t>
-  </si>
-  <si>
-    <t>2,41</t>
-  </si>
-  <si>
-    <t>7,33</t>
-  </si>
-  <si>
-    <t>13,36</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>30,72</t>
-  </si>
-  <si>
-    <t>0,45</t>
-  </si>
-  <si>
-    <t>30,5</t>
-  </si>
-  <si>
-    <t>1,88</t>
-  </si>
-  <si>
-    <t>5,85</t>
-  </si>
-  <si>
-    <t>0,63</t>
-  </si>
-  <si>
-    <t>8,4</t>
-  </si>
-  <si>
-    <t>20,75</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>18,05</t>
-  </si>
-  <si>
-    <t>0,59</t>
-  </si>
-  <si>
-    <t>32,1</t>
-  </si>
-  <si>
-    <t>3,07</t>
-  </si>
-  <si>
-    <t>4,99</t>
-  </si>
-  <si>
-    <t>0,88</t>
-  </si>
-  <si>
-    <t>1,06</t>
-  </si>
-  <si>
-    <t>8,24</t>
-  </si>
-  <si>
-    <t>28,93</t>
-  </si>
-  <si>
-    <t>1811</t>
-  </si>
-  <si>
-    <t>MESUJI</t>
-  </si>
-  <si>
-    <t>30,21</t>
-  </si>
-  <si>
-    <t>3,8</t>
-  </si>
-  <si>
-    <t>1,51</t>
-  </si>
-  <si>
-    <t>36,72</t>
-  </si>
-  <si>
-    <t>5,6</t>
-  </si>
-  <si>
-    <t>3,62</t>
-  </si>
-  <si>
-    <t>0,52</t>
-  </si>
-  <si>
-    <t>3,09</t>
-  </si>
-  <si>
-    <t>8,37</t>
-  </si>
-  <si>
-    <t>5,4</t>
-  </si>
-  <si>
-    <t>1812</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG BARAT</t>
-  </si>
-  <si>
-    <t>16,87</t>
-  </si>
-  <si>
-    <t>1,58</t>
-  </si>
-  <si>
-    <t>1,98</t>
-  </si>
-  <si>
-    <t>31,17</t>
-  </si>
-  <si>
-    <t>17,63</t>
-  </si>
-  <si>
-    <t>0,31</t>
-  </si>
-  <si>
-    <t>0,13</t>
-  </si>
-  <si>
-    <t>4,19</t>
-  </si>
-  <si>
-    <t>19,52</t>
-  </si>
-  <si>
-    <t>1813</t>
-  </si>
-  <si>
-    <t>PESISIR BARAT</t>
-  </si>
-  <si>
-    <t>11,95</t>
-  </si>
-  <si>
-    <t>0,16</t>
-  </si>
-  <si>
-    <t>0,27</t>
-  </si>
-  <si>
-    <t>44,79</t>
-  </si>
-  <si>
-    <t>16,11</t>
-  </si>
-  <si>
-    <t>10,05</t>
-  </si>
-  <si>
-    <t>6,71</t>
-  </si>
-  <si>
-    <t>8,82</t>
-  </si>
-  <si>
-    <t>1871</t>
-  </si>
-  <si>
-    <t>BANDAR LAMPUNG</t>
-  </si>
-  <si>
-    <t>15,49</t>
-  </si>
-  <si>
-    <t>0,57</t>
-  </si>
-  <si>
-    <t>3,35</t>
-  </si>
-  <si>
-    <t>31,64</t>
-  </si>
-  <si>
-    <t>4,59</t>
-  </si>
-  <si>
-    <t>16,06</t>
-  </si>
-  <si>
-    <t>0,86</t>
-  </si>
-  <si>
-    <t>1,72</t>
-  </si>
-  <si>
-    <t>0,38</t>
-  </si>
-  <si>
-    <t>1,24</t>
-  </si>
-  <si>
-    <t>4,49</t>
-  </si>
-  <si>
-    <t>17,69</t>
-  </si>
-  <si>
-    <t>1872</t>
-  </si>
-  <si>
-    <t>METRO</t>
-  </si>
-  <si>
-    <t>16,45</t>
-  </si>
-  <si>
-    <t>5,88</t>
-  </si>
-  <si>
-    <t>30,32</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>0,67</t>
-  </si>
-  <si>
-    <t>0,71</t>
-  </si>
-  <si>
-    <t>3,76</t>
-  </si>
-  <si>
-    <t>33,8</t>
+    <t>0,7</t>
+  </si>
+  <si>
+    <t>0,9</t>
+  </si>
+  <si>
+    <t>3,79</t>
+  </si>
+  <si>
+    <t>33,7</t>
   </si>
   <si>
     <t/>
@@ -1923,148 +1920,148 @@
         <v>105</v>
       </c>
       <c r="C6" s="6">
-        <v>113814</v>
+        <v>117473</v>
       </c>
       <c r="D6" s="6">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>106</v>
       </c>
       <c r="F6" s="6">
-        <v>23252</v>
+        <v>23931</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>107</v>
       </c>
       <c r="H6" s="6">
-        <v>1450</v>
+        <v>1529</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>108</v>
       </c>
       <c r="J6" s="6">
-        <v>2565</v>
+        <v>2400</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>109</v>
       </c>
       <c r="L6" s="6">
-        <v>42111</v>
+        <v>44236</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>110</v>
       </c>
       <c r="N6" s="6">
-        <v>11727</v>
+        <v>11970</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>111</v>
       </c>
       <c r="P6" s="6">
-        <v>266</v>
+        <v>241</v>
       </c>
       <c r="Q6" s="7" t="s">
         <v>112</v>
       </c>
       <c r="R6" s="6">
-        <v>8364</v>
+        <v>8834</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>113</v>
       </c>
       <c r="T6" s="6">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="U6" s="7" t="s">
         <v>114</v>
       </c>
       <c r="V6" s="6">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="W6" s="7" t="s">
         <v>115</v>
       </c>
       <c r="X6" s="6">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="Y6" s="7" t="s">
         <v>116</v>
       </c>
       <c r="Z6" s="6">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="AA6" s="7" t="s">
         <v>117</v>
       </c>
       <c r="AB6" s="6">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="AC6" s="7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AD6" s="6">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="AE6" s="7" t="s">
         <v>118</v>
       </c>
       <c r="AF6" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG6" s="7" t="s">
         <v>119</v>
       </c>
       <c r="AH6" s="6">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="AI6" s="7" t="s">
         <v>117</v>
       </c>
       <c r="AJ6" s="6">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="AK6" s="7" t="s">
         <v>120</v>
       </c>
       <c r="AL6" s="6">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="AM6" s="7" t="s">
         <v>115</v>
       </c>
       <c r="AN6" s="6">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="AO6" s="7" t="s">
         <v>118</v>
       </c>
       <c r="AP6" s="6">
-        <v>659</v>
+        <v>678</v>
       </c>
       <c r="AQ6" s="7" t="s">
         <v>121</v>
       </c>
       <c r="AR6" s="6">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="AS6" s="7" t="s">
         <v>122</v>
       </c>
       <c r="AT6" s="6">
-        <v>1143</v>
+        <v>1087</v>
       </c>
       <c r="AU6" s="7" t="s">
         <v>123</v>
       </c>
       <c r="AV6" s="6">
-        <v>5832</v>
+        <v>5959</v>
       </c>
       <c r="AW6" s="7" t="s">
         <v>124</v>
       </c>
       <c r="AX6" s="6">
-        <v>15378</v>
+        <v>15528</v>
       </c>
       <c r="AY6" s="7" t="s">
         <v>125</v>
@@ -2078,52 +2075,52 @@
         <v>127</v>
       </c>
       <c r="C7" s="9">
-        <v>7374</v>
+        <v>7732</v>
       </c>
       <c r="D7" s="9">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>128</v>
       </c>
       <c r="F7" s="9">
-        <v>1442</v>
+        <v>1487</v>
       </c>
       <c r="G7" s="10" t="s">
         <v>129</v>
       </c>
       <c r="H7" s="9">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="I7" s="10" t="s">
         <v>130</v>
       </c>
       <c r="J7" s="9">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="K7" s="10" t="s">
         <v>131</v>
       </c>
       <c r="L7" s="9">
-        <v>3367</v>
+        <v>3678</v>
       </c>
       <c r="M7" s="10" t="s">
         <v>132</v>
       </c>
       <c r="N7" s="9">
-        <v>384</v>
+        <v>312</v>
       </c>
       <c r="O7" s="10" t="s">
         <v>133</v>
       </c>
       <c r="P7" s="9">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="Q7" s="10" t="s">
         <v>134</v>
       </c>
       <c r="R7" s="9">
-        <v>329</v>
+        <v>352</v>
       </c>
       <c r="S7" s="10" t="s">
         <v>135</v>
@@ -2141,7 +2138,7 @@
         <v>136</v>
       </c>
       <c r="X7" s="9">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Y7" s="10" t="s">
         <v>137</v>
@@ -2153,7 +2150,7 @@
         <v>115</v>
       </c>
       <c r="AB7" s="9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AC7" s="10" t="s">
         <v>114</v>
@@ -2162,7 +2159,7 @@
         <v>5</v>
       </c>
       <c r="AE7" s="10" t="s">
-        <v>138</v>
+        <v>106</v>
       </c>
       <c r="AF7" s="9">
         <v>0</v>
@@ -2180,7 +2177,7 @@
         <v>10</v>
       </c>
       <c r="AK7" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AL7" s="9">
         <v>1</v>
@@ -2189,51 +2186,51 @@
         <v>136</v>
       </c>
       <c r="AN7" s="9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AO7" s="10" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="AP7" s="9">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="AQ7" s="10" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="AR7" s="9">
         <v>3</v>
       </c>
       <c r="AS7" s="10" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="AT7" s="9">
-        <v>237</v>
+        <v>218</v>
       </c>
       <c r="AU7" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="AV7" s="9">
+        <v>272</v>
+      </c>
+      <c r="AW7" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="AV7" s="9">
-        <v>254</v>
-      </c>
-      <c r="AW7" s="10" t="s">
+      <c r="AX7" s="9">
+        <v>1159</v>
+      </c>
+      <c r="AY7" s="10" t="s">
         <v>143</v>
-      </c>
-      <c r="AX7" s="9">
-        <v>1100</v>
-      </c>
-      <c r="AY7" s="10" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="B8" s="8" t="s">
-        <v>146</v>
-      </c>
       <c r="C8" s="9">
-        <v>3343</v>
+        <v>3348</v>
       </c>
       <c r="D8" s="9">
         <v>0</v>
@@ -2245,43 +2242,43 @@
         <v>459</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H8" s="9">
         <v>18</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J8" s="9">
         <v>36</v>
       </c>
       <c r="K8" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="L8" s="9">
+        <v>883</v>
+      </c>
+      <c r="M8" s="10" t="s">
         <v>149</v>
-      </c>
-      <c r="L8" s="9">
-        <v>877</v>
-      </c>
-      <c r="M8" s="10" t="s">
-        <v>150</v>
       </c>
       <c r="N8" s="9">
         <v>1017</v>
       </c>
       <c r="O8" s="10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="P8" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q8" s="10" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="R8" s="9">
         <v>216</v>
       </c>
       <c r="S8" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="T8" s="9">
         <v>0</v>
@@ -2299,7 +2296,7 @@
         <v>6</v>
       </c>
       <c r="Y8" s="10" t="s">
-        <v>153</v>
+        <v>134</v>
       </c>
       <c r="Z8" s="9">
         <v>0</v>
@@ -2335,7 +2332,7 @@
         <v>5</v>
       </c>
       <c r="AK8" s="10" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="AL8" s="9">
         <v>0</v>
@@ -2353,7 +2350,7 @@
         <v>16</v>
       </c>
       <c r="AQ8" s="10" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="AR8" s="9">
         <v>2</v>
@@ -2365,84 +2362,84 @@
         <v>10</v>
       </c>
       <c r="AU8" s="10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="AV8" s="9">
         <v>155</v>
       </c>
       <c r="AW8" s="10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="AX8" s="9">
         <v>524</v>
       </c>
       <c r="AY8" s="10" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="C9" s="9">
+        <v>8999</v>
+      </c>
+      <c r="D9" s="9">
+        <v>0</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="F9" s="9">
+        <v>1487</v>
+      </c>
+      <c r="G9" s="10" t="s">
         <v>159</v>
-      </c>
-      <c r="C9" s="9">
-        <v>8559</v>
-      </c>
-      <c r="D9" s="9">
-        <v>0</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="F9" s="9">
-        <v>1464</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>160</v>
       </c>
       <c r="H9" s="9">
         <v>198</v>
       </c>
       <c r="I9" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="J9" s="9">
+        <v>11</v>
+      </c>
+      <c r="K9" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="J9" s="9">
-        <v>10</v>
-      </c>
-      <c r="K9" s="10" t="s">
+      <c r="L9" s="9">
+        <v>4034</v>
+      </c>
+      <c r="M9" s="10" t="s">
         <v>162</v>
       </c>
-      <c r="L9" s="9">
-        <v>3742</v>
-      </c>
-      <c r="M9" s="10" t="s">
+      <c r="N9" s="9">
+        <v>1023</v>
+      </c>
+      <c r="O9" s="10" t="s">
         <v>163</v>
       </c>
-      <c r="N9" s="9">
-        <v>1058</v>
-      </c>
-      <c r="O9" s="10" t="s">
+      <c r="P9" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="R9" s="9">
+        <v>974</v>
+      </c>
+      <c r="S9" s="10" t="s">
         <v>164</v>
       </c>
-      <c r="P9" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="R9" s="9">
-        <v>824</v>
-      </c>
-      <c r="S9" s="10" t="s">
-        <v>165</v>
-      </c>
       <c r="T9" s="9">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="U9" s="10" t="s">
-        <v>114</v>
+        <v>136</v>
       </c>
       <c r="V9" s="9">
         <v>1</v>
@@ -2451,10 +2448,10 @@
         <v>136</v>
       </c>
       <c r="X9" s="9">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="Y9" s="10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="Z9" s="9">
         <v>0</v>
@@ -2469,28 +2466,28 @@
         <v>119</v>
       </c>
       <c r="AD9" s="9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AE9" s="10" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="AF9" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG9" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="AH9" s="9">
         <v>1</v>
       </c>
-      <c r="AG9" s="10" t="s">
+      <c r="AI9" s="10" t="s">
         <v>136</v>
-      </c>
-      <c r="AH9" s="9">
-        <v>0</v>
-      </c>
-      <c r="AI9" s="10" t="s">
-        <v>119</v>
       </c>
       <c r="AJ9" s="9">
         <v>65</v>
       </c>
       <c r="AK9" s="10" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="AL9" s="9">
         <v>0</v>
@@ -2508,7 +2505,7 @@
         <v>100</v>
       </c>
       <c r="AQ9" s="10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AR9" s="9">
         <v>2</v>
@@ -2517,66 +2514,66 @@
         <v>117</v>
       </c>
       <c r="AT9" s="9">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AU9" s="10" t="s">
-        <v>138</v>
+        <v>115</v>
       </c>
       <c r="AV9" s="9">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="AW9" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="AX9" s="9">
+        <v>693</v>
+      </c>
+      <c r="AY9" s="10" t="s">
         <v>169</v>
-      </c>
-      <c r="AX9" s="9">
-        <v>687</v>
-      </c>
-      <c r="AY9" s="10" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="C10" s="9">
+        <v>19510</v>
+      </c>
+      <c r="D10" s="9">
+        <v>34</v>
+      </c>
+      <c r="E10" s="10" t="s">
         <v>172</v>
       </c>
-      <c r="C10" s="9">
-        <v>18900</v>
-      </c>
-      <c r="D10" s="9">
-        <v>35</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>137</v>
-      </c>
       <c r="F10" s="9">
-        <v>4449</v>
+        <v>4550</v>
       </c>
       <c r="G10" s="10" t="s">
         <v>173</v>
       </c>
       <c r="H10" s="9">
-        <v>49</v>
+        <v>151</v>
       </c>
       <c r="I10" s="10" t="s">
         <v>174</v>
       </c>
       <c r="J10" s="9">
-        <v>1665</v>
+        <v>1658</v>
       </c>
       <c r="K10" s="10" t="s">
         <v>175</v>
       </c>
       <c r="L10" s="9">
-        <v>6199</v>
+        <v>6493</v>
       </c>
       <c r="M10" s="10" t="s">
         <v>176</v>
       </c>
       <c r="N10" s="9">
-        <v>2212</v>
+        <v>2278</v>
       </c>
       <c r="O10" s="10" t="s">
         <v>177</v>
@@ -2588,7 +2585,7 @@
         <v>178</v>
       </c>
       <c r="R10" s="9">
-        <v>1278</v>
+        <v>1312</v>
       </c>
       <c r="S10" s="10" t="s">
         <v>179</v>
@@ -2603,13 +2600,13 @@
         <v>7</v>
       </c>
       <c r="W10" s="10" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="X10" s="9">
         <v>14</v>
       </c>
       <c r="Y10" s="10" t="s">
-        <v>138</v>
+        <v>118</v>
       </c>
       <c r="Z10" s="9">
         <v>2</v>
@@ -2627,7 +2624,7 @@
         <v>13</v>
       </c>
       <c r="AE10" s="10" t="s">
-        <v>138</v>
+        <v>118</v>
       </c>
       <c r="AF10" s="9">
         <v>0</v>
@@ -2639,13 +2636,13 @@
         <v>8</v>
       </c>
       <c r="AI10" s="10" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="AJ10" s="9">
         <v>13</v>
       </c>
       <c r="AK10" s="10" t="s">
-        <v>138</v>
+        <v>118</v>
       </c>
       <c r="AL10" s="9">
         <v>1</v>
@@ -2663,7 +2660,7 @@
         <v>28</v>
       </c>
       <c r="AQ10" s="10" t="s">
-        <v>116</v>
+        <v>182</v>
       </c>
       <c r="AR10" s="9">
         <v>10</v>
@@ -2672,105 +2669,105 @@
         <v>180</v>
       </c>
       <c r="AT10" s="9">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="AU10" s="10" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="AV10" s="9">
-        <v>423</v>
+        <v>433</v>
       </c>
       <c r="AW10" s="10" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="AX10" s="9">
-        <v>1893</v>
+        <v>1899</v>
       </c>
       <c r="AY10" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C11" s="9">
-        <v>13038</v>
+        <v>13208</v>
       </c>
       <c r="D11" s="9">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>128</v>
+        <v>180</v>
       </c>
       <c r="F11" s="9">
-        <v>2010</v>
+        <v>2053</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H11" s="9">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J11" s="9">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>189</v>
+        <v>167</v>
       </c>
       <c r="L11" s="9">
-        <v>5999</v>
+        <v>6098</v>
       </c>
       <c r="M11" s="10" t="s">
         <v>190</v>
       </c>
       <c r="N11" s="9">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="O11" s="10" t="s">
         <v>191</v>
       </c>
       <c r="P11" s="9">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="Q11" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="R11" s="9">
+        <v>1748</v>
+      </c>
+      <c r="S11" s="10" t="s">
         <v>192</v>
-      </c>
-      <c r="R11" s="9">
-        <v>1743</v>
-      </c>
-      <c r="S11" s="10" t="s">
-        <v>193</v>
       </c>
       <c r="T11" s="9">
         <v>18</v>
       </c>
       <c r="U11" s="10" t="s">
-        <v>139</v>
+        <v>182</v>
       </c>
       <c r="V11" s="9">
         <v>5</v>
       </c>
       <c r="W11" s="10" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="X11" s="9">
         <v>11</v>
       </c>
       <c r="Y11" s="10" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="Z11" s="9">
         <v>5</v>
       </c>
       <c r="AA11" s="10" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="AB11" s="9">
         <v>3</v>
@@ -2782,7 +2779,7 @@
         <v>22</v>
       </c>
       <c r="AE11" s="10" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="AF11" s="9">
         <v>0</v>
@@ -2800,7 +2797,7 @@
         <v>29</v>
       </c>
       <c r="AK11" s="10" t="s">
-        <v>134</v>
+        <v>193</v>
       </c>
       <c r="AL11" s="9">
         <v>3</v>
@@ -2812,7 +2809,7 @@
         <v>9</v>
       </c>
       <c r="AO11" s="10" t="s">
-        <v>138</v>
+        <v>118</v>
       </c>
       <c r="AP11" s="9">
         <v>86</v>
@@ -2824,36 +2821,36 @@
         <v>15</v>
       </c>
       <c r="AS11" s="10" t="s">
-        <v>162</v>
+        <v>195</v>
       </c>
       <c r="AT11" s="9">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="AU11" s="10" t="s">
-        <v>195</v>
+        <v>112</v>
       </c>
       <c r="AV11" s="9">
-        <v>419</v>
+        <v>428</v>
       </c>
       <c r="AW11" s="10" t="s">
-        <v>142</v>
+        <v>196</v>
       </c>
       <c r="AX11" s="9">
-        <v>1525</v>
+        <v>1536</v>
       </c>
       <c r="AY11" s="10" t="s">
-        <v>177</v>
+        <v>197</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C12" s="9">
-        <v>5162</v>
+        <v>5170</v>
       </c>
       <c r="D12" s="9">
         <v>0</v>
@@ -2862,34 +2859,34 @@
         <v>119</v>
       </c>
       <c r="F12" s="9">
-        <v>975</v>
+        <v>978</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="H12" s="9">
         <v>38</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="J12" s="9">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="L12" s="9">
-        <v>1927</v>
+        <v>1929</v>
       </c>
       <c r="M12" s="10" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="N12" s="9">
         <v>729</v>
       </c>
       <c r="O12" s="10" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="P12" s="9">
         <v>3</v>
@@ -2901,7 +2898,7 @@
         <v>404</v>
       </c>
       <c r="S12" s="10" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="T12" s="9">
         <v>0</v>
@@ -2913,19 +2910,19 @@
         <v>8</v>
       </c>
       <c r="W12" s="10" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="X12" s="9">
         <v>18</v>
       </c>
       <c r="Y12" s="10" t="s">
-        <v>204</v>
+        <v>139</v>
       </c>
       <c r="Z12" s="9">
         <v>2</v>
       </c>
       <c r="AA12" s="10" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="AB12" s="9">
         <v>3</v>
@@ -2937,7 +2934,7 @@
         <v>9</v>
       </c>
       <c r="AE12" s="10" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="AF12" s="9">
         <v>0</v>
@@ -2949,13 +2946,13 @@
         <v>2</v>
       </c>
       <c r="AI12" s="10" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="AJ12" s="9">
         <v>29</v>
       </c>
       <c r="AK12" s="10" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AL12" s="9">
         <v>0</v>
@@ -2967,13 +2964,13 @@
         <v>4</v>
       </c>
       <c r="AO12" s="10" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="AP12" s="9">
         <v>55</v>
       </c>
       <c r="AQ12" s="10" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="AR12" s="9">
         <v>1</v>
@@ -2982,33 +2979,33 @@
         <v>117</v>
       </c>
       <c r="AT12" s="9">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="AU12" s="10" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="AV12" s="9">
         <v>351</v>
       </c>
       <c r="AW12" s="10" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="AX12" s="9">
         <v>534</v>
       </c>
       <c r="AY12" s="10" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C13" s="9">
-        <v>4742</v>
+        <v>4759</v>
       </c>
       <c r="D13" s="9">
         <v>0</v>
@@ -3017,46 +3014,46 @@
         <v>119</v>
       </c>
       <c r="F13" s="9">
-        <v>853</v>
+        <v>856</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="H13" s="9">
         <v>31</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>212</v>
+        <v>194</v>
       </c>
       <c r="J13" s="9">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="L13" s="9">
-        <v>2032</v>
+        <v>2050</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="N13" s="9">
-        <v>823</v>
+        <v>825</v>
       </c>
       <c r="O13" s="10" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="P13" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q13" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="R13" s="9">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="S13" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="T13" s="9">
         <v>0</v>
@@ -3068,7 +3065,7 @@
         <v>2</v>
       </c>
       <c r="W13" s="10" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="X13" s="9">
         <v>3</v>
@@ -3092,7 +3089,7 @@
         <v>8</v>
       </c>
       <c r="AE13" s="10" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="AF13" s="9">
         <v>0</v>
@@ -3110,13 +3107,13 @@
         <v>31</v>
       </c>
       <c r="AK13" s="10" t="s">
-        <v>212</v>
+        <v>194</v>
       </c>
       <c r="AL13" s="9">
         <v>11</v>
       </c>
       <c r="AM13" s="10" t="s">
-        <v>112</v>
+        <v>214</v>
       </c>
       <c r="AN13" s="9">
         <v>1</v>
@@ -3128,16 +3125,16 @@
         <v>37</v>
       </c>
       <c r="AQ13" s="10" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AR13" s="9">
         <v>23</v>
       </c>
       <c r="AS13" s="10" t="s">
-        <v>218</v>
+        <v>153</v>
       </c>
       <c r="AT13" s="9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AU13" s="10" t="s">
         <v>140</v>
@@ -3146,24 +3143,24 @@
         <v>220</v>
       </c>
       <c r="AW13" s="10" t="s">
-        <v>156</v>
+        <v>219</v>
       </c>
       <c r="AX13" s="9">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="AY13" s="10" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C14" s="9">
-        <v>4395</v>
+        <v>4548</v>
       </c>
       <c r="D14" s="9">
         <v>0</v>
@@ -3172,52 +3169,52 @@
         <v>119</v>
       </c>
       <c r="F14" s="9">
-        <v>1031</v>
+        <v>1056</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="H14" s="9">
         <v>18</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>223</v>
+        <v>165</v>
       </c>
       <c r="J14" s="9">
-        <v>114</v>
+        <v>93</v>
       </c>
       <c r="K14" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="L14" s="9">
+        <v>1269</v>
+      </c>
+      <c r="M14" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="L14" s="9">
-        <v>1207</v>
-      </c>
-      <c r="M14" s="10" t="s">
+      <c r="N14" s="9">
+        <v>725</v>
+      </c>
+      <c r="O14" s="10" t="s">
         <v>225</v>
-      </c>
-      <c r="N14" s="9">
-        <v>686</v>
-      </c>
-      <c r="O14" s="10" t="s">
-        <v>226</v>
       </c>
       <c r="P14" s="9">
         <v>8</v>
       </c>
       <c r="Q14" s="10" t="s">
-        <v>153</v>
+        <v>134</v>
       </c>
       <c r="R14" s="9">
-        <v>252</v>
+        <v>267</v>
       </c>
       <c r="S14" s="10" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="T14" s="9">
         <v>2</v>
       </c>
       <c r="U14" s="10" t="s">
-        <v>180</v>
+        <v>140</v>
       </c>
       <c r="V14" s="9">
         <v>1</v>
@@ -3229,7 +3226,7 @@
         <v>9</v>
       </c>
       <c r="Y14" s="10" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="Z14" s="9">
         <v>1</v>
@@ -3247,7 +3244,7 @@
         <v>5</v>
       </c>
       <c r="AE14" s="10" t="s">
-        <v>140</v>
+        <v>195</v>
       </c>
       <c r="AF14" s="9">
         <v>0</v>
@@ -3262,10 +3259,10 @@
         <v>117</v>
       </c>
       <c r="AJ14" s="9">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="AK14" s="10" t="s">
-        <v>120</v>
+        <v>228</v>
       </c>
       <c r="AL14" s="9">
         <v>1</v>
@@ -3277,10 +3274,10 @@
         <v>3</v>
       </c>
       <c r="AO14" s="10" t="s">
-        <v>138</v>
+        <v>118</v>
       </c>
       <c r="AP14" s="9">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="AQ14" s="10" t="s">
         <v>229</v>
@@ -3292,19 +3289,19 @@
         <v>117</v>
       </c>
       <c r="AT14" s="9">
-        <v>106</v>
+        <v>86</v>
       </c>
       <c r="AU14" s="10" t="s">
         <v>230</v>
       </c>
       <c r="AV14" s="9">
-        <v>322</v>
+        <v>339</v>
       </c>
       <c r="AW14" s="10" t="s">
         <v>231</v>
       </c>
       <c r="AX14" s="9">
-        <v>587</v>
+        <v>617</v>
       </c>
       <c r="AY14" s="10" t="s">
         <v>232</v>
@@ -3318,7 +3315,7 @@
         <v>234</v>
       </c>
       <c r="C15" s="9">
-        <v>12530</v>
+        <v>12546</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
@@ -3327,13 +3324,13 @@
         <v>119</v>
       </c>
       <c r="F15" s="9">
-        <v>3849</v>
+        <v>3863</v>
       </c>
       <c r="G15" s="10" t="s">
         <v>235</v>
       </c>
       <c r="H15" s="9">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I15" s="10" t="s">
         <v>236</v>
@@ -3342,16 +3339,16 @@
         <v>5</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="L15" s="9">
-        <v>3822</v>
+        <v>3835</v>
       </c>
       <c r="M15" s="10" t="s">
         <v>237</v>
       </c>
       <c r="N15" s="9">
-        <v>236</v>
+        <v>226</v>
       </c>
       <c r="O15" s="10" t="s">
         <v>238</v>
@@ -3372,7 +3369,7 @@
         <v>41</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>166</v>
+        <v>240</v>
       </c>
       <c r="V15" s="9">
         <v>0</v>
@@ -3384,7 +3381,7 @@
         <v>15</v>
       </c>
       <c r="Y15" s="10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="Z15" s="9">
         <v>0</v>
@@ -3420,7 +3417,7 @@
         <v>11</v>
       </c>
       <c r="AK15" s="10" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="AL15" s="9">
         <v>3</v>
@@ -3438,13 +3435,13 @@
         <v>79</v>
       </c>
       <c r="AQ15" s="10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AR15" s="9">
         <v>19</v>
       </c>
       <c r="AS15" s="10" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="AT15" s="9">
         <v>3</v>
@@ -3453,60 +3450,60 @@
         <v>117</v>
       </c>
       <c r="AV15" s="9">
-        <v>1052</v>
+        <v>1053</v>
       </c>
       <c r="AW15" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AX15" s="9">
-        <v>2600</v>
+        <v>2599</v>
       </c>
       <c r="AY15" s="10" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C16" s="9">
-        <v>4891</v>
+        <v>5059</v>
       </c>
       <c r="D16" s="9">
         <v>2</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="F16" s="9">
-        <v>883</v>
+        <v>899</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="H16" s="9">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="J16" s="9">
-        <v>47</v>
+        <v>8</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="L16" s="9">
-        <v>1570</v>
+        <v>1597</v>
       </c>
       <c r="M16" s="10" t="s">
         <v>247</v>
       </c>
       <c r="N16" s="9">
-        <v>150</v>
+        <v>268</v>
       </c>
       <c r="O16" s="10" t="s">
         <v>248</v>
@@ -3518,7 +3515,7 @@
         <v>119</v>
       </c>
       <c r="R16" s="9">
-        <v>244</v>
+        <v>266</v>
       </c>
       <c r="S16" s="10" t="s">
         <v>249</v>
@@ -3530,16 +3527,16 @@
         <v>119</v>
       </c>
       <c r="V16" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W16" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="X16" s="9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Y16" s="10" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="Z16" s="9">
         <v>3</v>
@@ -3575,108 +3572,108 @@
         <v>29</v>
       </c>
       <c r="AK16" s="10" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="AL16" s="9">
         <v>4</v>
       </c>
       <c r="AM16" s="10" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="AN16" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO16" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="AP16" s="9">
         <v>43</v>
       </c>
       <c r="AQ16" s="10" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="AR16" s="9">
         <v>7</v>
       </c>
       <c r="AS16" s="10" t="s">
-        <v>139</v>
+        <v>182</v>
       </c>
       <c r="AT16" s="9">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="AU16" s="10" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="AV16" s="9">
-        <v>403</v>
+        <v>420</v>
       </c>
       <c r="AW16" s="10" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="AX16" s="9">
-        <v>1415</v>
+        <v>1436</v>
       </c>
       <c r="AY16" s="10" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C17" s="9">
-        <v>8395</v>
+        <v>8917</v>
       </c>
       <c r="D17" s="9">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>195</v>
+        <v>137</v>
       </c>
       <c r="F17" s="9">
-        <v>2536</v>
+        <v>2704</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="H17" s="9">
-        <v>319</v>
+        <v>290</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="J17" s="9">
         <v>127</v>
       </c>
       <c r="K17" s="10" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="L17" s="9">
-        <v>3083</v>
+        <v>3374</v>
       </c>
       <c r="M17" s="10" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="N17" s="9">
-        <v>470</v>
+        <v>495</v>
       </c>
       <c r="O17" s="10" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="P17" s="9">
         <v>22</v>
       </c>
       <c r="Q17" s="10" t="s">
-        <v>174</v>
+        <v>120</v>
       </c>
       <c r="R17" s="9">
-        <v>304</v>
+        <v>350</v>
       </c>
       <c r="S17" s="10" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="T17" s="9">
         <v>1</v>
@@ -3688,7 +3685,7 @@
         <v>6</v>
       </c>
       <c r="W17" s="10" t="s">
-        <v>138</v>
+        <v>118</v>
       </c>
       <c r="X17" s="9">
         <v>5</v>
@@ -3697,10 +3694,10 @@
         <v>106</v>
       </c>
       <c r="Z17" s="9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AA17" s="10" t="s">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="AB17" s="9">
         <v>2</v>
@@ -3712,7 +3709,7 @@
         <v>4</v>
       </c>
       <c r="AE17" s="10" t="s">
-        <v>180</v>
+        <v>140</v>
       </c>
       <c r="AF17" s="9">
         <v>0</v>
@@ -3730,60 +3727,60 @@
         <v>16</v>
       </c>
       <c r="AK17" s="10" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="AL17" s="9">
         <v>3</v>
       </c>
       <c r="AM17" s="10" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
       <c r="AN17" s="9">
         <v>7</v>
       </c>
       <c r="AO17" s="10" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="AP17" s="9">
         <v>44</v>
       </c>
       <c r="AQ17" s="10" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="AR17" s="9">
         <v>9</v>
       </c>
       <c r="AS17" s="10" t="s">
-        <v>140</v>
+        <v>122</v>
       </c>
       <c r="AT17" s="9">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="AU17" s="10" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="AV17" s="9">
-        <v>703</v>
+        <v>718</v>
       </c>
       <c r="AW17" s="10" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="AX17" s="9">
-        <v>453</v>
+        <v>457</v>
       </c>
       <c r="AY17" s="10" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C18" s="9">
-        <v>9389</v>
+        <v>9982</v>
       </c>
       <c r="D18" s="9">
         <v>1</v>
@@ -3792,52 +3789,52 @@
         <v>136</v>
       </c>
       <c r="F18" s="9">
-        <v>1584</v>
+        <v>1784</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="H18" s="9">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="J18" s="9">
-        <v>186</v>
+        <v>134</v>
       </c>
       <c r="K18" s="10" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="L18" s="9">
-        <v>2927</v>
+        <v>3217</v>
       </c>
       <c r="M18" s="10" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="N18" s="9">
-        <v>1655</v>
+        <v>1706</v>
       </c>
       <c r="O18" s="10" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="P18" s="9">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="Q18" s="10" t="s">
-        <v>273</v>
+        <v>106</v>
       </c>
       <c r="R18" s="9">
-        <v>538</v>
+        <v>631</v>
       </c>
       <c r="S18" s="10" t="s">
-        <v>227</v>
+        <v>274</v>
       </c>
       <c r="T18" s="9">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="U18" s="10" t="s">
-        <v>112</v>
+        <v>275</v>
       </c>
       <c r="V18" s="9">
         <v>0</v>
@@ -3858,10 +3855,10 @@
         <v>136</v>
       </c>
       <c r="AB18" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC18" s="10" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="AD18" s="9">
         <v>3</v>
@@ -3876,40 +3873,40 @@
         <v>119</v>
       </c>
       <c r="AH18" s="9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AI18" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="AJ18" s="9">
         <v>11</v>
       </c>
       <c r="AK18" s="10" t="s">
-        <v>162</v>
+        <v>195</v>
       </c>
       <c r="AL18" s="9">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="AM18" s="10" t="s">
-        <v>180</v>
+        <v>122</v>
       </c>
       <c r="AN18" s="9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AO18" s="10" t="s">
-        <v>180</v>
+        <v>117</v>
       </c>
       <c r="AP18" s="9">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="AQ18" s="10" t="s">
-        <v>181</v>
+        <v>276</v>
       </c>
       <c r="AR18" s="9">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="AS18" s="10" t="s">
-        <v>274</v>
+        <v>172</v>
       </c>
       <c r="AT18" s="9">
         <v>1</v>
@@ -3918,76 +3915,76 @@
         <v>136</v>
       </c>
       <c r="AV18" s="9">
-        <v>393</v>
+        <v>403</v>
       </c>
       <c r="AW18" s="10" t="s">
-        <v>275</v>
+        <v>133</v>
       </c>
       <c r="AX18" s="9">
-        <v>1833</v>
+        <v>1837</v>
       </c>
       <c r="AY18" s="10" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C19" s="9">
-        <v>9497</v>
+        <v>10085</v>
       </c>
       <c r="D19" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>136</v>
+        <v>119</v>
       </c>
       <c r="F19" s="9">
-        <v>1135</v>
+        <v>1173</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>279</v>
+        <v>197</v>
       </c>
       <c r="H19" s="9">
         <v>15</v>
       </c>
       <c r="I19" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="J19" s="9">
+        <v>0</v>
+      </c>
+      <c r="K19" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="L19" s="9">
+        <v>4670</v>
+      </c>
+      <c r="M19" s="10" t="s">
         <v>280</v>
       </c>
-      <c r="J19" s="9">
-        <v>26</v>
-      </c>
-      <c r="K19" s="10" t="s">
+      <c r="N19" s="9">
+        <v>1592</v>
+      </c>
+      <c r="O19" s="10" t="s">
         <v>281</v>
       </c>
-      <c r="L19" s="9">
-        <v>4254</v>
-      </c>
-      <c r="M19" s="10" t="s">
+      <c r="P19" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="R19" s="9">
+        <v>1031</v>
+      </c>
+      <c r="S19" s="10" t="s">
         <v>282</v>
       </c>
-      <c r="N19" s="9">
-        <v>1530</v>
-      </c>
-      <c r="O19" s="10" t="s">
-        <v>283</v>
-      </c>
-      <c r="P19" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="R19" s="9">
-        <v>954</v>
-      </c>
-      <c r="S19" s="10" t="s">
-        <v>284</v>
-      </c>
       <c r="T19" s="9">
         <v>0</v>
       </c>
@@ -3995,16 +3992,16 @@
         <v>119</v>
       </c>
       <c r="V19" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W19" s="10" t="s">
-        <v>136</v>
+        <v>119</v>
       </c>
       <c r="X19" s="9">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="Y19" s="10" t="s">
-        <v>153</v>
+        <v>134</v>
       </c>
       <c r="Z19" s="9">
         <v>0</v>
@@ -4040,7 +4037,7 @@
         <v>16</v>
       </c>
       <c r="AK19" s="10" t="s">
-        <v>192</v>
+        <v>116</v>
       </c>
       <c r="AL19" s="9">
         <v>0</v>
@@ -4049,16 +4046,16 @@
         <v>119</v>
       </c>
       <c r="AN19" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO19" s="10" t="s">
-        <v>136</v>
+        <v>119</v>
       </c>
       <c r="AP19" s="9">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="AQ19" s="10" t="s">
-        <v>246</v>
+        <v>121</v>
       </c>
       <c r="AR19" s="9">
         <v>1</v>
@@ -4067,33 +4064,33 @@
         <v>136</v>
       </c>
       <c r="AT19" s="9">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AU19" s="10" t="s">
-        <v>274</v>
+        <v>136</v>
       </c>
       <c r="AV19" s="9">
-        <v>637</v>
+        <v>662</v>
       </c>
       <c r="AW19" s="10" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="AX19" s="9">
-        <v>838</v>
+        <v>845</v>
       </c>
       <c r="AY19" s="10" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C20" s="9">
-        <v>1046</v>
+        <v>1049</v>
       </c>
       <c r="D20" s="9">
         <v>1</v>
@@ -4105,43 +4102,43 @@
         <v>162</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="H20" s="9">
         <v>6</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>290</v>
+        <v>250</v>
       </c>
       <c r="J20" s="9">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="L20" s="9">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="M20" s="10" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="N20" s="9">
         <v>48</v>
       </c>
       <c r="O20" s="10" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="P20" s="9">
         <v>6</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>290</v>
+        <v>250</v>
       </c>
       <c r="R20" s="9">
         <v>168</v>
       </c>
       <c r="S20" s="10" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="T20" s="9">
         <v>0</v>
@@ -4159,13 +4156,13 @@
         <v>9</v>
       </c>
       <c r="Y20" s="10" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="Z20" s="9">
         <v>3</v>
       </c>
       <c r="AA20" s="10" t="s">
-        <v>206</v>
+        <v>293</v>
       </c>
       <c r="AB20" s="9">
         <v>0</v>
@@ -4195,7 +4192,7 @@
         <v>6</v>
       </c>
       <c r="AK20" s="10" t="s">
-        <v>290</v>
+        <v>250</v>
       </c>
       <c r="AL20" s="9">
         <v>2</v>
@@ -4213,42 +4210,42 @@
         <v>18</v>
       </c>
       <c r="AQ20" s="10" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="AR20" s="9">
         <v>4</v>
       </c>
       <c r="AS20" s="10" t="s">
-        <v>297</v>
+        <v>276</v>
       </c>
       <c r="AT20" s="9">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AU20" s="10" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="AV20" s="9">
         <v>47</v>
       </c>
       <c r="AW20" s="10" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="AX20" s="9">
         <v>185</v>
       </c>
       <c r="AY20" s="10" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="C21" s="9">
-        <v>2553</v>
+        <v>2561</v>
       </c>
       <c r="D21" s="9">
         <v>0</v>
@@ -4260,43 +4257,43 @@
         <v>420</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="H21" s="9">
         <v>150</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="J21" s="9">
         <v>1</v>
       </c>
       <c r="K21" s="10" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="L21" s="9">
-        <v>774</v>
+        <v>777</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="N21" s="9">
         <v>102</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="P21" s="9">
         <v>8</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>273</v>
+        <v>228</v>
       </c>
       <c r="R21" s="9">
         <v>79</v>
       </c>
       <c r="S21" s="10" t="s">
-        <v>263</v>
+        <v>304</v>
       </c>
       <c r="T21" s="9">
         <v>0</v>
@@ -4314,13 +4311,13 @@
         <v>17</v>
       </c>
       <c r="Y21" s="10" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="Z21" s="9">
         <v>2</v>
       </c>
       <c r="AA21" s="10" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="AB21" s="9">
         <v>0</v>
@@ -4350,7 +4347,7 @@
         <v>3</v>
       </c>
       <c r="AK21" s="10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AL21" s="9">
         <v>0</v>
@@ -4368,183 +4365,183 @@
         <v>18</v>
       </c>
       <c r="AQ21" s="10" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="AR21" s="9">
         <v>1</v>
       </c>
       <c r="AS21" s="10" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="AT21" s="9">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="AU21" s="10" t="s">
-        <v>199</v>
+        <v>307</v>
       </c>
       <c r="AV21" s="9">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AW21" s="10" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="AX21" s="9">
         <v>863</v>
       </c>
       <c r="AY21" s="10" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
+        <v>310</v>
+      </c>
+      <c r="B22" s="11" t="s">
         <v>311</v>
       </c>
-      <c r="B22" s="11" t="s">
-        <v>312</v>
-      </c>
       <c r="C22" s="12">
-        <v>113814</v>
+        <v>117473</v>
       </c>
       <c r="D22" s="12">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>106</v>
       </c>
       <c r="F22" s="12">
-        <v>23252</v>
+        <v>23931</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>107</v>
       </c>
       <c r="H22" s="12">
-        <v>1450</v>
+        <v>1529</v>
       </c>
       <c r="I22" s="13" t="s">
         <v>108</v>
       </c>
       <c r="J22" s="12">
-        <v>2565</v>
+        <v>2400</v>
       </c>
       <c r="K22" s="13" t="s">
         <v>109</v>
       </c>
       <c r="L22" s="12">
-        <v>42111</v>
+        <v>44236</v>
       </c>
       <c r="M22" s="13" t="s">
         <v>110</v>
       </c>
       <c r="N22" s="12">
-        <v>11727</v>
+        <v>11970</v>
       </c>
       <c r="O22" s="13" t="s">
         <v>111</v>
       </c>
       <c r="P22" s="12">
-        <v>266</v>
+        <v>241</v>
       </c>
       <c r="Q22" s="13" t="s">
         <v>112</v>
       </c>
       <c r="R22" s="12">
-        <v>8364</v>
+        <v>8834</v>
       </c>
       <c r="S22" s="13" t="s">
         <v>113</v>
       </c>
       <c r="T22" s="12">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="U22" s="13" t="s">
         <v>114</v>
       </c>
       <c r="V22" s="12">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="W22" s="13" t="s">
         <v>115</v>
       </c>
       <c r="X22" s="12">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="Y22" s="13" t="s">
         <v>116</v>
       </c>
       <c r="Z22" s="12">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="AA22" s="13" t="s">
         <v>117</v>
       </c>
       <c r="AB22" s="12">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="AC22" s="13" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AD22" s="12">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="AE22" s="13" t="s">
         <v>118</v>
       </c>
       <c r="AF22" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG22" s="13" t="s">
         <v>119</v>
       </c>
       <c r="AH22" s="12">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="AI22" s="13" t="s">
         <v>117</v>
       </c>
       <c r="AJ22" s="12">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="AK22" s="13" t="s">
         <v>120</v>
       </c>
       <c r="AL22" s="12">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="AM22" s="13" t="s">
         <v>115</v>
       </c>
       <c r="AN22" s="12">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="AO22" s="13" t="s">
         <v>118</v>
       </c>
       <c r="AP22" s="12">
-        <v>659</v>
+        <v>678</v>
       </c>
       <c r="AQ22" s="13" t="s">
         <v>121</v>
       </c>
       <c r="AR22" s="12">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="AS22" s="13" t="s">
         <v>122</v>
       </c>
       <c r="AT22" s="12">
-        <v>1143</v>
+        <v>1087</v>
       </c>
       <c r="AU22" s="13" t="s">
         <v>123</v>
       </c>
       <c r="AV22" s="12">
-        <v>5832</v>
+        <v>5959</v>
       </c>
       <c r="AW22" s="13" t="s">
         <v>124</v>
       </c>
       <c r="AX22" s="12">
-        <v>15378</v>
+        <v>15528</v>
       </c>
       <c r="AY22" s="13" t="s">
         <v>125</v>

</xml_diff>

<commit_message>
Perbarui data SE2026 04/09/2026  8:17:13,95
</commit_message>
<xml_diff>
--- a/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
+++ b/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="307">
   <si>
     <t>DATA RADAR ANOMALI USAHA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 3 Sep 2026, 13.26</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 4 Sep 2026, 08.16</t>
   </si>
   <si>
     <t>Kode</t>
@@ -331,616 +331,601 @@
     <t>LAMPUNG</t>
   </si>
   <si>
+    <t>0,07</t>
+  </si>
+  <si>
+    <t>20,29</t>
+  </si>
+  <si>
+    <t>1,25</t>
+  </si>
+  <si>
+    <t>1,89</t>
+  </si>
+  <si>
+    <t>38,2</t>
+  </si>
+  <si>
+    <t>10,2</t>
+  </si>
+  <si>
+    <t>0,2</t>
+  </si>
+  <si>
+    <t>7,69</t>
+  </si>
+  <si>
+    <t>0,08</t>
+  </si>
+  <si>
+    <t>0,02</t>
+  </si>
+  <si>
+    <t>0,16</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>0,24</t>
+  </si>
+  <si>
+    <t>0,03</t>
+  </si>
+  <si>
+    <t>0,57</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>0,86</t>
+  </si>
+  <si>
+    <t>5,01</t>
+  </si>
+  <si>
+    <t>12,95</t>
+  </si>
+  <si>
+    <t>1801</t>
+  </si>
+  <si>
+    <t>LAMPUNG BARAT</t>
+  </si>
+  <si>
+    <t>19,17</t>
+  </si>
+  <si>
+    <t>0,95</t>
+  </si>
+  <si>
+    <t>0,99</t>
+  </si>
+  <si>
+    <t>47,84</t>
+  </si>
+  <si>
+    <t>4,02</t>
+  </si>
+  <si>
+    <t>0,14</t>
+  </si>
+  <si>
+    <t>4,52</t>
+  </si>
+  <si>
+    <t>0,01</t>
+  </si>
+  <si>
+    <t>0,19</t>
+  </si>
+  <si>
     <t>0,06</t>
   </si>
   <si>
-    <t>20,37</t>
-  </si>
-  <si>
-    <t>1,3</t>
-  </si>
-  <si>
-    <t>2,04</t>
-  </si>
-  <si>
-    <t>37,66</t>
-  </si>
-  <si>
-    <t>10,19</t>
+    <t>0,13</t>
+  </si>
+  <si>
+    <t>0,04</t>
+  </si>
+  <si>
+    <t>0,35</t>
+  </si>
+  <si>
+    <t>2,8</t>
+  </si>
+  <si>
+    <t>3,56</t>
+  </si>
+  <si>
+    <t>14,94</t>
+  </si>
+  <si>
+    <t>1802</t>
+  </si>
+  <si>
+    <t>TANGGAMUS</t>
+  </si>
+  <si>
+    <t>13,67</t>
+  </si>
+  <si>
+    <t>0,5</t>
+  </si>
+  <si>
+    <t>0,89</t>
+  </si>
+  <si>
+    <t>26,72</t>
+  </si>
+  <si>
+    <t>30,24</t>
+  </si>
+  <si>
+    <t>6,45</t>
+  </si>
+  <si>
+    <t>0,18</t>
+  </si>
+  <si>
+    <t>0,15</t>
+  </si>
+  <si>
+    <t>0,47</t>
+  </si>
+  <si>
+    <t>4,73</t>
+  </si>
+  <si>
+    <t>15,86</t>
+  </si>
+  <si>
+    <t>1803</t>
+  </si>
+  <si>
+    <t>LAMPUNG SELATAN</t>
+  </si>
+  <si>
+    <t>16,32</t>
+  </si>
+  <si>
+    <t>2,1</t>
+  </si>
+  <si>
+    <t>47,54</t>
+  </si>
+  <si>
+    <t>9,63</t>
+  </si>
+  <si>
+    <t>10,72</t>
+  </si>
+  <si>
+    <t>0,38</t>
+  </si>
+  <si>
+    <t>0,7</t>
+  </si>
+  <si>
+    <t>1,07</t>
+  </si>
+  <si>
+    <t>3,85</t>
+  </si>
+  <si>
+    <t>7,38</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>23,35</t>
+  </si>
+  <si>
+    <t>0,76</t>
+  </si>
+  <si>
+    <t>7,84</t>
+  </si>
+  <si>
+    <t>32,93</t>
+  </si>
+  <si>
+    <t>12,65</t>
+  </si>
+  <si>
+    <t>0,73</t>
+  </si>
+  <si>
+    <t>7,16</t>
+  </si>
+  <si>
+    <t>0,05</t>
+  </si>
+  <si>
+    <t>0,26</t>
+  </si>
+  <si>
+    <t>1,92</t>
+  </si>
+  <si>
+    <t>2,21</t>
+  </si>
+  <si>
+    <t>9,43</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>15,69</t>
+  </si>
+  <si>
+    <t>2,27</t>
+  </si>
+  <si>
+    <t>1,13</t>
+  </si>
+  <si>
+    <t>46,26</t>
+  </si>
+  <si>
+    <t>4,65</t>
   </si>
   <si>
     <t>0,21</t>
   </si>
   <si>
-    <t>7,52</t>
-  </si>
-  <si>
-    <t>0,08</t>
-  </si>
-  <si>
-    <t>0,03</t>
-  </si>
-  <si>
-    <t>0,16</t>
-  </si>
-  <si>
-    <t>0,02</t>
-  </si>
-  <si>
-    <t>0,07</t>
-  </si>
-  <si>
-    <t>0</t>
+    <t>13,13</t>
+  </si>
+  <si>
+    <t>0,22</t>
+  </si>
+  <si>
+    <t>0,64</t>
+  </si>
+  <si>
+    <t>0,11</t>
+  </si>
+  <si>
+    <t>0,27</t>
+  </si>
+  <si>
+    <t>3,21</t>
+  </si>
+  <si>
+    <t>11,53</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>18,9</t>
+  </si>
+  <si>
+    <t>0,98</t>
+  </si>
+  <si>
+    <t>37,62</t>
+  </si>
+  <si>
+    <t>13,98</t>
+  </si>
+  <si>
+    <t>7,85</t>
+  </si>
+  <si>
+    <t>0,59</t>
+  </si>
+  <si>
+    <t>1,15</t>
   </si>
   <si>
     <t>0,25</t>
   </si>
   <si>
-    <t>0,58</t>
-  </si>
-  <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>0,93</t>
-  </si>
-  <si>
-    <t>5,07</t>
-  </si>
-  <si>
-    <t>13,22</t>
-  </si>
-  <si>
-    <t>1801</t>
-  </si>
-  <si>
-    <t>LAMPUNG BARAT</t>
+    <t>6,81</t>
+  </si>
+  <si>
+    <t>10,38</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>17,65</t>
+  </si>
+  <si>
+    <t>0,8</t>
+  </si>
+  <si>
+    <t>43,26</t>
+  </si>
+  <si>
+    <t>16,97</t>
+  </si>
+  <si>
+    <t>6,22</t>
+  </si>
+  <si>
+    <t>0,66</t>
+  </si>
+  <si>
+    <t>0,23</t>
+  </si>
+  <si>
+    <t>7,13</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>22,82</t>
+  </si>
+  <si>
+    <t>0,37</t>
+  </si>
+  <si>
+    <t>28,36</t>
+  </si>
+  <si>
+    <t>18,09</t>
+  </si>
+  <si>
+    <t>6,07</t>
+  </si>
+  <si>
+    <t>0,33</t>
+  </si>
+  <si>
+    <t>0,55</t>
+  </si>
+  <si>
+    <t>7,44</t>
+  </si>
+  <si>
+    <t>14,13</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>30,79</t>
+  </si>
+  <si>
+    <t>0,44</t>
+  </si>
+  <si>
+    <t>30,67</t>
+  </si>
+  <si>
+    <t>1,8</t>
+  </si>
+  <si>
+    <t>5,83</t>
+  </si>
+  <si>
+    <t>0,12</t>
   </si>
   <si>
     <t>0,09</t>
   </si>
   <si>
-    <t>19,23</t>
-  </si>
-  <si>
-    <t>0,96</t>
-  </si>
-  <si>
-    <t>1,02</t>
-  </si>
-  <si>
-    <t>47,57</t>
-  </si>
-  <si>
-    <t>4,04</t>
-  </si>
-  <si>
-    <t>0,18</t>
-  </si>
-  <si>
-    <t>4,55</t>
-  </si>
-  <si>
-    <t>0,01</t>
-  </si>
-  <si>
-    <t>0,19</t>
-  </si>
-  <si>
-    <t>0,13</t>
-  </si>
-  <si>
-    <t>0,35</t>
-  </si>
-  <si>
-    <t>0,04</t>
-  </si>
-  <si>
-    <t>2,82</t>
-  </si>
-  <si>
-    <t>3,52</t>
-  </si>
-  <si>
-    <t>14,99</t>
-  </si>
-  <si>
-    <t>1802</t>
-  </si>
-  <si>
-    <t>TANGGAMUS</t>
-  </si>
-  <si>
-    <t>13,71</t>
-  </si>
-  <si>
-    <t>0,54</t>
-  </si>
-  <si>
-    <t>1,08</t>
-  </si>
-  <si>
-    <t>26,37</t>
-  </si>
-  <si>
-    <t>30,38</t>
-  </si>
-  <si>
-    <t>6,45</t>
-  </si>
-  <si>
-    <t>0,15</t>
-  </si>
-  <si>
-    <t>0,48</t>
-  </si>
-  <si>
-    <t>0,3</t>
-  </si>
-  <si>
-    <t>4,63</t>
-  </si>
-  <si>
-    <t>15,65</t>
-  </si>
-  <si>
-    <t>1803</t>
-  </si>
-  <si>
-    <t>LAMPUNG SELATAN</t>
-  </si>
-  <si>
-    <t>16,52</t>
-  </si>
-  <si>
-    <t>2,2</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>44,83</t>
-  </si>
-  <si>
-    <t>11,37</t>
-  </si>
-  <si>
-    <t>10,82</t>
-  </si>
-  <si>
-    <t>0,4</t>
-  </si>
-  <si>
-    <t>0,72</t>
-  </si>
-  <si>
-    <t>1,11</t>
-  </si>
-  <si>
-    <t>4,01</t>
-  </si>
-  <si>
-    <t>7,7</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
+    <t>0,63</t>
+  </si>
+  <si>
+    <t>8,37</t>
+  </si>
+  <si>
+    <t>20,67</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>17,74</t>
+  </si>
+  <si>
+    <t>31,59</t>
+  </si>
+  <si>
+    <t>5,35</t>
+  </si>
+  <si>
+    <t>5,25</t>
+  </si>
+  <si>
+    <t>0,85</t>
+  </si>
+  <si>
+    <t>8,29</t>
+  </si>
+  <si>
+    <t>28,33</t>
+  </si>
+  <si>
+    <t>1811</t>
+  </si>
+  <si>
+    <t>MESUJI</t>
+  </si>
+  <si>
+    <t>29,6</t>
+  </si>
+  <si>
+    <t>2,73</t>
+  </si>
+  <si>
+    <t>1,26</t>
+  </si>
+  <si>
+    <t>38,62</t>
+  </si>
+  <si>
+    <t>6,62</t>
+  </si>
+  <si>
+    <t>4,42</t>
   </si>
   <si>
     <t>0,17</t>
   </si>
   <si>
-    <t>23,32</t>
-  </si>
-  <si>
-    <t>0,77</t>
-  </si>
-  <si>
-    <t>8,5</t>
-  </si>
-  <si>
-    <t>33,28</t>
-  </si>
-  <si>
-    <t>11,68</t>
-  </si>
-  <si>
-    <t>0,76</t>
-  </si>
-  <si>
-    <t>6,72</t>
-  </si>
-  <si>
-    <t>0,05</t>
-  </si>
-  <si>
-    <t>0,27</t>
-  </si>
-  <si>
-    <t>0,14</t>
-  </si>
-  <si>
-    <t>1,96</t>
-  </si>
-  <si>
-    <t>2,22</t>
-  </si>
-  <si>
-    <t>9,73</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>15,54</t>
-  </si>
-  <si>
-    <t>2,29</t>
-  </si>
-  <si>
-    <t>46,17</t>
-  </si>
-  <si>
-    <t>4,72</t>
-  </si>
-  <si>
-    <t>13,23</t>
-  </si>
-  <si>
-    <t>0,22</t>
-  </si>
-  <si>
-    <t>0,65</t>
-  </si>
-  <si>
-    <t>0,11</t>
-  </si>
-  <si>
-    <t>3,24</t>
-  </si>
-  <si>
-    <t>11,63</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>18,92</t>
-  </si>
-  <si>
-    <t>0,74</t>
-  </si>
-  <si>
-    <t>1,04</t>
-  </si>
-  <si>
-    <t>37,31</t>
-  </si>
-  <si>
-    <t>14,1</t>
-  </si>
-  <si>
-    <t>7,81</t>
-  </si>
-  <si>
-    <t>0,56</t>
-  </si>
-  <si>
-    <t>1,06</t>
-  </si>
-  <si>
-    <t>0,37</t>
-  </si>
-  <si>
-    <t>6,79</t>
-  </si>
-  <si>
-    <t>10,33</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>17,99</t>
-  </si>
-  <si>
-    <t>0,23</t>
-  </si>
-  <si>
-    <t>43,08</t>
-  </si>
-  <si>
-    <t>17,34</t>
-  </si>
-  <si>
-    <t>6,37</t>
-  </si>
-  <si>
-    <t>0,78</t>
-  </si>
-  <si>
-    <t>4,62</t>
-  </si>
-  <si>
-    <t>7,23</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>23,22</t>
-  </si>
-  <si>
-    <t>27,9</t>
-  </si>
-  <si>
-    <t>15,94</t>
-  </si>
-  <si>
-    <t>5,87</t>
-  </si>
-  <si>
-    <t>0,2</t>
+    <t>0,45</t>
+  </si>
+  <si>
+    <t>2,78</t>
+  </si>
+  <si>
+    <t>7,6</t>
+  </si>
+  <si>
+    <t>4,8</t>
+  </si>
+  <si>
+    <t>1812</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG BARAT</t>
+  </si>
+  <si>
+    <t>18,12</t>
+  </si>
+  <si>
+    <t>1,49</t>
+  </si>
+  <si>
+    <t>1,31</t>
+  </si>
+  <si>
+    <t>33,42</t>
+  </si>
+  <si>
+    <t>15,68</t>
+  </si>
+  <si>
+    <t>6,61</t>
+  </si>
+  <si>
+    <t>4,05</t>
+  </si>
+  <si>
+    <t>18,14</t>
+  </si>
+  <si>
+    <t>1813</t>
+  </si>
+  <si>
+    <t>PESISIR BARAT</t>
+  </si>
+  <si>
+    <t>11,21</t>
+  </si>
+  <si>
+    <t>47,67</t>
+  </si>
+  <si>
+    <t>14,88</t>
+  </si>
+  <si>
+    <t>10,92</t>
+  </si>
+  <si>
+    <t>6,29</t>
+  </si>
+  <si>
+    <t>7,93</t>
+  </si>
+  <si>
+    <t>1871</t>
+  </si>
+  <si>
+    <t>BANDAR LAMPUNG</t>
+  </si>
+  <si>
+    <t>15,38</t>
+  </si>
+  <si>
+    <t>3,32</t>
+  </si>
+  <si>
+    <t>31,81</t>
+  </si>
+  <si>
+    <t>4,56</t>
+  </si>
+  <si>
+    <t>15,95</t>
+  </si>
+  <si>
+    <t>0,28</t>
+  </si>
+  <si>
+    <t>1,71</t>
+  </si>
+  <si>
+    <t>1,52</t>
+  </si>
+  <si>
+    <t>4,46</t>
+  </si>
+  <si>
+    <t>17,57</t>
+  </si>
+  <si>
+    <t>1872</t>
+  </si>
+  <si>
+    <t>METRO</t>
+  </si>
+  <si>
+    <t>16,37</t>
+  </si>
+  <si>
+    <t>5,85</t>
+  </si>
+  <si>
+    <t>30,44</t>
+  </si>
+  <si>
+    <t>3,98</t>
   </si>
   <si>
     <t>0,31</t>
   </si>
   <si>
-    <t>0,68</t>
-  </si>
-  <si>
-    <t>1,89</t>
-  </si>
-  <si>
-    <t>7,45</t>
-  </si>
-  <si>
-    <t>13,57</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>30,79</t>
-  </si>
-  <si>
-    <t>0,44</t>
-  </si>
-  <si>
-    <t>30,57</t>
-  </si>
-  <si>
-    <t>1,8</t>
-  </si>
-  <si>
-    <t>5,84</t>
-  </si>
-  <si>
-    <t>0,33</t>
-  </si>
-  <si>
-    <t>0,63</t>
-  </si>
-  <si>
-    <t>8,39</t>
-  </si>
-  <si>
-    <t>20,72</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>17,77</t>
-  </si>
-  <si>
-    <t>31,57</t>
-  </si>
-  <si>
-    <t>5,3</t>
-  </si>
-  <si>
-    <t>5,26</t>
-  </si>
-  <si>
-    <t>0,57</t>
-  </si>
-  <si>
-    <t>0,85</t>
-  </si>
-  <si>
-    <t>0,71</t>
-  </si>
-  <si>
-    <t>8,3</t>
-  </si>
-  <si>
-    <t>28,39</t>
-  </si>
-  <si>
-    <t>1811</t>
-  </si>
-  <si>
-    <t>MESUJI</t>
-  </si>
-  <si>
-    <t>30,32</t>
-  </si>
-  <si>
-    <t>3,25</t>
-  </si>
-  <si>
-    <t>1,42</t>
-  </si>
-  <si>
-    <t>37,84</t>
-  </si>
-  <si>
-    <t>5,55</t>
-  </si>
-  <si>
-    <t>3,93</t>
-  </si>
-  <si>
-    <t>0,49</t>
-  </si>
-  <si>
-    <t>2,92</t>
-  </si>
-  <si>
-    <t>8,05</t>
-  </si>
-  <si>
-    <t>5,13</t>
-  </si>
-  <si>
-    <t>1812</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG BARAT</t>
-  </si>
-  <si>
-    <t>17,87</t>
-  </si>
-  <si>
-    <t>1,5</t>
-  </si>
-  <si>
-    <t>1,34</t>
-  </si>
-  <si>
-    <t>32,23</t>
-  </si>
-  <si>
-    <t>17,09</t>
-  </si>
-  <si>
-    <t>6,32</t>
-  </si>
-  <si>
-    <t>0,24</t>
-  </si>
-  <si>
-    <t>0,38</t>
-  </si>
-  <si>
-    <t>18,4</t>
-  </si>
-  <si>
-    <t>1813</t>
-  </si>
-  <si>
-    <t>PESISIR BARAT</t>
-  </si>
-  <si>
-    <t>46,31</t>
-  </si>
-  <si>
-    <t>15,79</t>
-  </si>
-  <si>
-    <t>10,22</t>
-  </si>
-  <si>
-    <t>6,56</t>
-  </si>
-  <si>
-    <t>8,38</t>
-  </si>
-  <si>
-    <t>1871</t>
-  </si>
-  <si>
-    <t>BANDAR LAMPUNG</t>
-  </si>
-  <si>
-    <t>15,44</t>
-  </si>
-  <si>
-    <t>3,43</t>
-  </si>
-  <si>
-    <t>31,65</t>
-  </si>
-  <si>
-    <t>4,58</t>
-  </si>
-  <si>
-    <t>16,02</t>
-  </si>
-  <si>
-    <t>0,86</t>
-  </si>
-  <si>
-    <t>0,29</t>
-  </si>
-  <si>
-    <t>1,72</t>
-  </si>
-  <si>
-    <t>1,33</t>
-  </si>
-  <si>
-    <t>4,48</t>
-  </si>
-  <si>
-    <t>17,64</t>
-  </si>
-  <si>
-    <t>1872</t>
-  </si>
-  <si>
-    <t>METRO</t>
-  </si>
-  <si>
-    <t>16,4</t>
-  </si>
-  <si>
-    <t>5,86</t>
-  </si>
-  <si>
-    <t>30,34</t>
-  </si>
-  <si>
-    <t>3,98</t>
-  </si>
-  <si>
     <t>3,08</t>
   </si>
   <si>
-    <t>0,66</t>
-  </si>
-  <si>
-    <t>0,7</t>
-  </si>
-  <si>
     <t>0,9</t>
   </si>
   <si>
-    <t>3,79</t>
-  </si>
-  <si>
-    <t>33,7</t>
+    <t>3,78</t>
+  </si>
+  <si>
+    <t>33,63</t>
   </si>
   <si>
     <t/>
@@ -1920,234 +1905,234 @@
         <v>105</v>
       </c>
       <c r="C6" s="6">
-        <v>117473</v>
+        <v>120818</v>
       </c>
       <c r="D6" s="6">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>106</v>
       </c>
       <c r="F6" s="6">
-        <v>23931</v>
+        <v>24509</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>107</v>
       </c>
       <c r="H6" s="6">
-        <v>1529</v>
+        <v>1506</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>108</v>
       </c>
       <c r="J6" s="6">
-        <v>2400</v>
+        <v>2285</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>109</v>
       </c>
       <c r="L6" s="6">
-        <v>44236</v>
+        <v>46153</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>110</v>
       </c>
       <c r="N6" s="6">
-        <v>11970</v>
+        <v>12318</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>111</v>
       </c>
       <c r="P6" s="6">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="Q6" s="7" t="s">
         <v>112</v>
       </c>
       <c r="R6" s="6">
-        <v>8834</v>
+        <v>9292</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>113</v>
       </c>
       <c r="T6" s="6">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="U6" s="7" t="s">
         <v>114</v>
       </c>
       <c r="V6" s="6">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="W6" s="7" t="s">
         <v>115</v>
       </c>
       <c r="X6" s="6">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="Y6" s="7" t="s">
         <v>116</v>
       </c>
       <c r="Z6" s="6">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AA6" s="7" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AB6" s="6">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="AC6" s="7" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AD6" s="6">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AE6" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="AF6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG6" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="AH6" s="6">
+        <v>20</v>
+      </c>
+      <c r="AI6" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="AJ6" s="6">
+        <v>294</v>
+      </c>
+      <c r="AK6" s="7" t="s">
         <v>118</v>
-      </c>
-      <c r="AF6" s="6">
-        <v>0</v>
-      </c>
-      <c r="AG6" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="AH6" s="6">
-        <v>24</v>
-      </c>
-      <c r="AI6" s="7" t="s">
-        <v>117</v>
-      </c>
-      <c r="AJ6" s="6">
-        <v>288</v>
-      </c>
-      <c r="AK6" s="7" t="s">
-        <v>120</v>
       </c>
       <c r="AL6" s="6">
         <v>39</v>
       </c>
       <c r="AM6" s="7" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="AN6" s="6">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="AO6" s="7" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="AP6" s="6">
-        <v>678</v>
+        <v>689</v>
       </c>
       <c r="AQ6" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="AR6" s="6">
         <v>115</v>
       </c>
       <c r="AS6" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="AT6" s="6">
+        <v>1042</v>
+      </c>
+      <c r="AU6" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="AT6" s="6">
-        <v>1087</v>
-      </c>
-      <c r="AU6" s="7" t="s">
+      <c r="AV6" s="6">
+        <v>6047</v>
+      </c>
+      <c r="AW6" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="AV6" s="6">
-        <v>5959</v>
-      </c>
-      <c r="AW6" s="7" t="s">
+      <c r="AX6" s="6">
+        <v>15646</v>
+      </c>
+      <c r="AY6" s="7" t="s">
         <v>124</v>
-      </c>
-      <c r="AX6" s="6">
-        <v>15528</v>
-      </c>
-      <c r="AY6" s="7" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="C7" s="9">
+        <v>7783</v>
+      </c>
+      <c r="D7" s="9">
+        <v>8</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="F7" s="9">
+        <v>1492</v>
+      </c>
+      <c r="G7" s="10" t="s">
         <v>127</v>
-      </c>
-      <c r="C7" s="9">
-        <v>7732</v>
-      </c>
-      <c r="D7" s="9">
-        <v>7</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>128</v>
-      </c>
-      <c r="F7" s="9">
-        <v>1487</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>129</v>
       </c>
       <c r="H7" s="9">
         <v>74</v>
       </c>
       <c r="I7" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="J7" s="9">
+        <v>77</v>
+      </c>
+      <c r="K7" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="L7" s="9">
+        <v>3723</v>
+      </c>
+      <c r="M7" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="J7" s="9">
-        <v>79</v>
-      </c>
-      <c r="K7" s="10" t="s">
+      <c r="N7" s="9">
+        <v>313</v>
+      </c>
+      <c r="O7" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="L7" s="9">
-        <v>3678</v>
-      </c>
-      <c r="M7" s="10" t="s">
+      <c r="P7" s="9">
+        <v>11</v>
+      </c>
+      <c r="Q7" s="10" t="s">
         <v>132</v>
-      </c>
-      <c r="N7" s="9">
-        <v>312</v>
-      </c>
-      <c r="O7" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="P7" s="9">
-        <v>14</v>
-      </c>
-      <c r="Q7" s="10" t="s">
-        <v>134</v>
       </c>
       <c r="R7" s="9">
         <v>352</v>
       </c>
       <c r="S7" s="10" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="T7" s="9">
         <v>2</v>
       </c>
       <c r="U7" s="10" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="V7" s="9">
         <v>1</v>
       </c>
       <c r="W7" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="X7" s="9">
         <v>15</v>
       </c>
       <c r="Y7" s="10" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="Z7" s="9">
         <v>2</v>
       </c>
       <c r="AA7" s="10" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="AB7" s="9">
         <v>6</v>
@@ -2159,37 +2144,37 @@
         <v>5</v>
       </c>
       <c r="AE7" s="10" t="s">
-        <v>106</v>
+        <v>136</v>
       </c>
       <c r="AF7" s="9">
         <v>0</v>
       </c>
       <c r="AG7" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AH7" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI7" s="10" t="s">
-        <v>136</v>
+        <v>117</v>
       </c>
       <c r="AJ7" s="9">
         <v>10</v>
       </c>
       <c r="AK7" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AL7" s="9">
         <v>1</v>
       </c>
       <c r="AM7" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AN7" s="9">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="AO7" s="10" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="AP7" s="9">
         <v>27</v>
@@ -2201,132 +2186,132 @@
         <v>3</v>
       </c>
       <c r="AS7" s="10" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="AT7" s="9">
         <v>218</v>
       </c>
       <c r="AU7" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="AV7" s="9">
+        <v>277</v>
+      </c>
+      <c r="AW7" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="AV7" s="9">
-        <v>272</v>
-      </c>
-      <c r="AW7" s="10" t="s">
+      <c r="AX7" s="9">
+        <v>1163</v>
+      </c>
+      <c r="AY7" s="10" t="s">
         <v>142</v>
-      </c>
-      <c r="AX7" s="9">
-        <v>1159</v>
-      </c>
-      <c r="AY7" s="10" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="C8" s="9">
+        <v>3380</v>
+      </c>
+      <c r="D8" s="9">
+        <v>0</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="F8" s="9">
+        <v>462</v>
+      </c>
+      <c r="G8" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="C8" s="9">
-        <v>3348</v>
-      </c>
-      <c r="D8" s="9">
-        <v>0</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="F8" s="9">
-        <v>459</v>
-      </c>
-      <c r="G8" s="10" t="s">
+      <c r="H8" s="9">
+        <v>17</v>
+      </c>
+      <c r="I8" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="H8" s="9">
-        <v>18</v>
-      </c>
-      <c r="I8" s="10" t="s">
+      <c r="J8" s="9">
+        <v>30</v>
+      </c>
+      <c r="K8" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="J8" s="9">
-        <v>36</v>
-      </c>
-      <c r="K8" s="10" t="s">
+      <c r="L8" s="9">
+        <v>903</v>
+      </c>
+      <c r="M8" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="L8" s="9">
-        <v>883</v>
-      </c>
-      <c r="M8" s="10" t="s">
+      <c r="N8" s="9">
+        <v>1022</v>
+      </c>
+      <c r="O8" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="N8" s="9">
-        <v>1017</v>
-      </c>
-      <c r="O8" s="10" t="s">
+      <c r="P8" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="R8" s="9">
+        <v>218</v>
+      </c>
+      <c r="S8" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="P8" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="R8" s="9">
-        <v>216</v>
-      </c>
-      <c r="S8" s="10" t="s">
-        <v>151</v>
-      </c>
       <c r="T8" s="9">
         <v>0</v>
       </c>
       <c r="U8" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="V8" s="9">
         <v>0</v>
       </c>
       <c r="W8" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="X8" s="9">
         <v>6</v>
       </c>
       <c r="Y8" s="10" t="s">
-        <v>134</v>
+        <v>151</v>
       </c>
       <c r="Z8" s="9">
         <v>0</v>
       </c>
       <c r="AA8" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AB8" s="9">
         <v>0</v>
       </c>
       <c r="AC8" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AD8" s="9">
         <v>1</v>
       </c>
       <c r="AE8" s="10" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="AF8" s="9">
         <v>0</v>
       </c>
       <c r="AG8" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AH8" s="9">
         <v>0</v>
       </c>
       <c r="AI8" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AJ8" s="9">
         <v>5</v>
@@ -2338,13 +2323,13 @@
         <v>0</v>
       </c>
       <c r="AM8" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AN8" s="9">
         <v>0</v>
       </c>
       <c r="AO8" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AP8" s="9">
         <v>16</v>
@@ -2356,406 +2341,406 @@
         <v>2</v>
       </c>
       <c r="AS8" s="10" t="s">
-        <v>106</v>
+        <v>136</v>
       </c>
       <c r="AT8" s="9">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="AU8" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="AV8" s="9">
+        <v>160</v>
+      </c>
+      <c r="AW8" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="AV8" s="9">
+      <c r="AX8" s="9">
+        <v>536</v>
+      </c>
+      <c r="AY8" s="10" t="s">
         <v>155</v>
-      </c>
-      <c r="AW8" s="10" t="s">
-        <v>155</v>
-      </c>
-      <c r="AX8" s="9">
-        <v>524</v>
-      </c>
-      <c r="AY8" s="10" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="C9" s="9">
+        <v>9384</v>
+      </c>
+      <c r="D9" s="9">
+        <v>0</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="F9" s="9">
+        <v>1531</v>
+      </c>
+      <c r="G9" s="10" t="s">
         <v>158</v>
       </c>
-      <c r="C9" s="9">
-        <v>8999</v>
-      </c>
-      <c r="D9" s="9">
-        <v>0</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="F9" s="9">
-        <v>1487</v>
-      </c>
-      <c r="G9" s="10" t="s">
+      <c r="H9" s="9">
+        <v>197</v>
+      </c>
+      <c r="I9" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="H9" s="9">
-        <v>198</v>
-      </c>
-      <c r="I9" s="10" t="s">
+      <c r="J9" s="9">
+        <v>13</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="L9" s="9">
+        <v>4461</v>
+      </c>
+      <c r="M9" s="10" t="s">
         <v>160</v>
       </c>
-      <c r="J9" s="9">
-        <v>11</v>
-      </c>
-      <c r="K9" s="10" t="s">
+      <c r="N9" s="9">
+        <v>904</v>
+      </c>
+      <c r="O9" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="L9" s="9">
-        <v>4034</v>
-      </c>
-      <c r="M9" s="10" t="s">
+      <c r="P9" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="R9" s="9">
+        <v>1006</v>
+      </c>
+      <c r="S9" s="10" t="s">
         <v>162</v>
-      </c>
-      <c r="N9" s="9">
-        <v>1023</v>
-      </c>
-      <c r="O9" s="10" t="s">
-        <v>163</v>
-      </c>
-      <c r="P9" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="R9" s="9">
-        <v>974</v>
-      </c>
-      <c r="S9" s="10" t="s">
-        <v>164</v>
       </c>
       <c r="T9" s="9">
         <v>1</v>
       </c>
       <c r="U9" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="V9" s="9">
         <v>1</v>
       </c>
       <c r="W9" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="X9" s="9">
         <v>36</v>
       </c>
       <c r="Y9" s="10" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="Z9" s="9">
         <v>0</v>
       </c>
       <c r="AA9" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AB9" s="9">
         <v>0</v>
       </c>
       <c r="AC9" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AD9" s="9">
         <v>9</v>
       </c>
       <c r="AE9" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="AF9" s="9">
         <v>0</v>
       </c>
       <c r="AG9" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AH9" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI9" s="10" t="s">
-        <v>136</v>
+        <v>117</v>
       </c>
       <c r="AJ9" s="9">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="AK9" s="10" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="AL9" s="9">
         <v>0</v>
       </c>
       <c r="AM9" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AN9" s="9">
         <v>0</v>
       </c>
       <c r="AO9" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AP9" s="9">
         <v>100</v>
       </c>
       <c r="AQ9" s="10" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="AR9" s="9">
         <v>2</v>
       </c>
       <c r="AS9" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AT9" s="9">
         <v>3</v>
       </c>
       <c r="AU9" s="10" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="AV9" s="9">
         <v>361</v>
       </c>
       <c r="AW9" s="10" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="AX9" s="9">
         <v>693</v>
       </c>
       <c r="AY9" s="10" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="C10" s="9">
+        <v>20201</v>
+      </c>
+      <c r="D10" s="9">
+        <v>36</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="F10" s="9">
+        <v>4717</v>
+      </c>
+      <c r="G10" s="10" t="s">
         <v>170</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="H10" s="9">
+        <v>154</v>
+      </c>
+      <c r="I10" s="10" t="s">
         <v>171</v>
       </c>
-      <c r="C10" s="9">
-        <v>19510</v>
-      </c>
-      <c r="D10" s="9">
-        <v>34</v>
-      </c>
-      <c r="E10" s="10" t="s">
+      <c r="J10" s="9">
+        <v>1584</v>
+      </c>
+      <c r="K10" s="10" t="s">
         <v>172</v>
       </c>
-      <c r="F10" s="9">
-        <v>4550</v>
-      </c>
-      <c r="G10" s="10" t="s">
+      <c r="L10" s="9">
+        <v>6652</v>
+      </c>
+      <c r="M10" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="H10" s="9">
-        <v>151</v>
-      </c>
-      <c r="I10" s="10" t="s">
+      <c r="N10" s="9">
+        <v>2555</v>
+      </c>
+      <c r="O10" s="10" t="s">
         <v>174</v>
       </c>
-      <c r="J10" s="9">
-        <v>1658</v>
-      </c>
-      <c r="K10" s="10" t="s">
+      <c r="P10" s="9">
+        <v>148</v>
+      </c>
+      <c r="Q10" s="10" t="s">
         <v>175</v>
       </c>
-      <c r="L10" s="9">
-        <v>6493</v>
-      </c>
-      <c r="M10" s="10" t="s">
+      <c r="R10" s="9">
+        <v>1446</v>
+      </c>
+      <c r="S10" s="10" t="s">
         <v>176</v>
-      </c>
-      <c r="N10" s="9">
-        <v>2278</v>
-      </c>
-      <c r="O10" s="10" t="s">
-        <v>177</v>
-      </c>
-      <c r="P10" s="9">
-        <v>149</v>
-      </c>
-      <c r="Q10" s="10" t="s">
-        <v>178</v>
-      </c>
-      <c r="R10" s="9">
-        <v>1312</v>
-      </c>
-      <c r="S10" s="10" t="s">
-        <v>179</v>
       </c>
       <c r="T10" s="9">
         <v>10</v>
       </c>
       <c r="U10" s="10" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="V10" s="9">
         <v>7</v>
       </c>
       <c r="W10" s="10" t="s">
-        <v>140</v>
+        <v>119</v>
       </c>
       <c r="X10" s="9">
         <v>14</v>
       </c>
       <c r="Y10" s="10" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="Z10" s="9">
         <v>2</v>
       </c>
       <c r="AA10" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AB10" s="9">
         <v>12</v>
       </c>
       <c r="AC10" s="10" t="s">
-        <v>106</v>
+        <v>136</v>
       </c>
       <c r="AD10" s="9">
         <v>13</v>
       </c>
       <c r="AE10" s="10" t="s">
-        <v>118</v>
+        <v>136</v>
       </c>
       <c r="AF10" s="9">
         <v>0</v>
       </c>
       <c r="AG10" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AH10" s="9">
         <v>8</v>
       </c>
       <c r="AI10" s="10" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="AJ10" s="9">
         <v>13</v>
       </c>
       <c r="AK10" s="10" t="s">
-        <v>118</v>
+        <v>136</v>
       </c>
       <c r="AL10" s="9">
         <v>1</v>
       </c>
       <c r="AM10" s="10" t="s">
-        <v>136</v>
+        <v>117</v>
       </c>
       <c r="AN10" s="9">
         <v>52</v>
       </c>
       <c r="AO10" s="10" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="AP10" s="9">
         <v>28</v>
       </c>
       <c r="AQ10" s="10" t="s">
-        <v>182</v>
+        <v>132</v>
       </c>
       <c r="AR10" s="9">
         <v>10</v>
       </c>
       <c r="AS10" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="AT10" s="9">
+        <v>388</v>
+      </c>
+      <c r="AU10" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AV10" s="9">
+        <v>447</v>
+      </c>
+      <c r="AW10" s="10" t="s">
         <v>180</v>
       </c>
-      <c r="AT10" s="9">
-        <v>383</v>
-      </c>
-      <c r="AU10" s="10" t="s">
-        <v>183</v>
-      </c>
-      <c r="AV10" s="9">
-        <v>433</v>
-      </c>
-      <c r="AW10" s="10" t="s">
-        <v>184</v>
-      </c>
       <c r="AX10" s="9">
-        <v>1899</v>
+        <v>1904</v>
       </c>
       <c r="AY10" s="10" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="C11" s="9">
-        <v>13208</v>
+        <v>13343</v>
       </c>
       <c r="D11" s="9">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>180</v>
+        <v>106</v>
       </c>
       <c r="F11" s="9">
-        <v>2053</v>
+        <v>2093</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="H11" s="9">
         <v>303</v>
       </c>
       <c r="I11" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="J11" s="9">
+        <v>151</v>
+      </c>
+      <c r="K11" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="L11" s="9">
+        <v>6172</v>
+      </c>
+      <c r="M11" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="N11" s="9">
+        <v>620</v>
+      </c>
+      <c r="O11" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="P11" s="9">
+        <v>28</v>
+      </c>
+      <c r="Q11" s="10" t="s">
         <v>189</v>
       </c>
-      <c r="J11" s="9">
-        <v>147</v>
-      </c>
-      <c r="K11" s="10" t="s">
-        <v>167</v>
-      </c>
-      <c r="L11" s="9">
-        <v>6098</v>
-      </c>
-      <c r="M11" s="10" t="s">
+      <c r="R11" s="9">
+        <v>1752</v>
+      </c>
+      <c r="S11" s="10" t="s">
         <v>190</v>
-      </c>
-      <c r="N11" s="9">
-        <v>624</v>
-      </c>
-      <c r="O11" s="10" t="s">
-        <v>191</v>
-      </c>
-      <c r="P11" s="9">
-        <v>24</v>
-      </c>
-      <c r="Q11" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="R11" s="9">
-        <v>1748</v>
-      </c>
-      <c r="S11" s="10" t="s">
-        <v>192</v>
       </c>
       <c r="T11" s="9">
         <v>18</v>
       </c>
       <c r="U11" s="10" t="s">
-        <v>182</v>
+        <v>137</v>
       </c>
       <c r="V11" s="9">
         <v>5</v>
       </c>
       <c r="W11" s="10" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="X11" s="9">
         <v>11</v>
@@ -2767,365 +2752,365 @@
         <v>5</v>
       </c>
       <c r="AA11" s="10" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="AB11" s="9">
         <v>3</v>
       </c>
       <c r="AC11" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AD11" s="9">
         <v>22</v>
       </c>
       <c r="AE11" s="10" t="s">
-        <v>172</v>
+        <v>116</v>
       </c>
       <c r="AF11" s="9">
         <v>0</v>
       </c>
       <c r="AG11" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AH11" s="9">
         <v>6</v>
       </c>
       <c r="AI11" s="10" t="s">
-        <v>180</v>
+        <v>138</v>
       </c>
       <c r="AJ11" s="9">
         <v>29</v>
       </c>
       <c r="AK11" s="10" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="AL11" s="9">
         <v>3</v>
       </c>
       <c r="AM11" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AN11" s="9">
         <v>9</v>
       </c>
       <c r="AO11" s="10" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="AP11" s="9">
         <v>86</v>
       </c>
       <c r="AQ11" s="10" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="AR11" s="9">
         <v>15</v>
       </c>
       <c r="AS11" s="10" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="AT11" s="9">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="AU11" s="10" t="s">
-        <v>112</v>
+        <v>194</v>
       </c>
       <c r="AV11" s="9">
         <v>428</v>
       </c>
       <c r="AW11" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="AX11" s="9">
+        <v>1539</v>
+      </c>
+      <c r="AY11" s="10" t="s">
         <v>196</v>
-      </c>
-      <c r="AX11" s="9">
-        <v>1536</v>
-      </c>
-      <c r="AY11" s="10" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="C12" s="9">
+        <v>5213</v>
+      </c>
+      <c r="D12" s="9">
+        <v>0</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="F12" s="9">
+        <v>985</v>
+      </c>
+      <c r="G12" s="10" t="s">
         <v>199</v>
-      </c>
-      <c r="C12" s="9">
-        <v>5170</v>
-      </c>
-      <c r="D12" s="9">
-        <v>0</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="F12" s="9">
-        <v>978</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>200</v>
       </c>
       <c r="H12" s="9">
         <v>38</v>
       </c>
       <c r="I12" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="J12" s="9">
+        <v>51</v>
+      </c>
+      <c r="K12" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="L12" s="9">
+        <v>1961</v>
+      </c>
+      <c r="M12" s="10" t="s">
         <v>201</v>
-      </c>
-      <c r="J12" s="9">
-        <v>54</v>
-      </c>
-      <c r="K12" s="10" t="s">
-        <v>202</v>
-      </c>
-      <c r="L12" s="9">
-        <v>1929</v>
-      </c>
-      <c r="M12" s="10" t="s">
-        <v>203</v>
       </c>
       <c r="N12" s="9">
         <v>729</v>
       </c>
       <c r="O12" s="10" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="P12" s="9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Q12" s="10" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="R12" s="9">
-        <v>404</v>
+        <v>409</v>
       </c>
       <c r="S12" s="10" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="T12" s="9">
         <v>0</v>
       </c>
       <c r="U12" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="V12" s="9">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="W12" s="10" t="s">
-        <v>152</v>
+        <v>117</v>
       </c>
       <c r="X12" s="9">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="Y12" s="10" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="Z12" s="9">
         <v>2</v>
       </c>
       <c r="AA12" s="10" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="AB12" s="9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AC12" s="10" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="AD12" s="9">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AE12" s="10" t="s">
-        <v>172</v>
+        <v>135</v>
       </c>
       <c r="AF12" s="9">
         <v>0</v>
       </c>
       <c r="AG12" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AH12" s="9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AI12" s="10" t="s">
-        <v>140</v>
+        <v>117</v>
       </c>
       <c r="AJ12" s="9">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="AK12" s="10" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="AL12" s="9">
         <v>0</v>
       </c>
       <c r="AM12" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AN12" s="9">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AO12" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AP12" s="9">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="AQ12" s="10" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="AR12" s="9">
         <v>1</v>
       </c>
       <c r="AS12" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AT12" s="9">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="AU12" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="AV12" s="9">
+        <v>355</v>
+      </c>
+      <c r="AW12" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="AX12" s="9">
+        <v>541</v>
+      </c>
+      <c r="AY12" s="10" t="s">
         <v>208</v>
-      </c>
-      <c r="AV12" s="9">
-        <v>351</v>
-      </c>
-      <c r="AW12" s="10" t="s">
-        <v>209</v>
-      </c>
-      <c r="AX12" s="9">
-        <v>534</v>
-      </c>
-      <c r="AY12" s="10" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>210</v>
+      </c>
+      <c r="C13" s="9">
+        <v>4868</v>
+      </c>
+      <c r="D13" s="9">
+        <v>3</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="F13" s="9">
+        <v>859</v>
+      </c>
+      <c r="G13" s="10" t="s">
         <v>211</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="C13" s="9">
-        <v>4759</v>
-      </c>
-      <c r="D13" s="9">
-        <v>0</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="F13" s="9">
-        <v>856</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>213</v>
       </c>
       <c r="H13" s="9">
         <v>31</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="J13" s="9">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="K13" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="L13" s="9">
+        <v>2106</v>
+      </c>
+      <c r="M13" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="N13" s="9">
+        <v>826</v>
+      </c>
+      <c r="O13" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="L13" s="9">
-        <v>2050</v>
-      </c>
-      <c r="M13" s="10" t="s">
-        <v>215</v>
-      </c>
-      <c r="N13" s="9">
-        <v>825</v>
-      </c>
-      <c r="O13" s="10" t="s">
-        <v>216</v>
-      </c>
       <c r="P13" s="9">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="Q13" s="10" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="R13" s="9">
         <v>303</v>
       </c>
       <c r="S13" s="10" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="T13" s="9">
         <v>0</v>
       </c>
       <c r="U13" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="V13" s="9">
         <v>2</v>
       </c>
       <c r="W13" s="10" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="X13" s="9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Y13" s="10" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="Z13" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA13" s="10" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="AB13" s="9">
         <v>0</v>
       </c>
       <c r="AC13" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AD13" s="9">
         <v>8</v>
       </c>
       <c r="AE13" s="10" t="s">
-        <v>172</v>
+        <v>116</v>
       </c>
       <c r="AF13" s="9">
         <v>0</v>
       </c>
       <c r="AG13" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AH13" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AI13" s="10" t="s">
-        <v>117</v>
+        <v>138</v>
       </c>
       <c r="AJ13" s="9">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="AK13" s="10" t="s">
-        <v>194</v>
+        <v>216</v>
       </c>
       <c r="AL13" s="9">
         <v>11</v>
       </c>
       <c r="AM13" s="10" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="AN13" s="9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AO13" s="10" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="AP13" s="9">
         <v>37</v>
       </c>
       <c r="AQ13" s="10" t="s">
-        <v>218</v>
+        <v>171</v>
       </c>
       <c r="AR13" s="9">
         <v>23</v>
@@ -3134,90 +3119,90 @@
         <v>153</v>
       </c>
       <c r="AT13" s="9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AU13" s="10" t="s">
-        <v>140</v>
+        <v>114</v>
       </c>
       <c r="AV13" s="9">
         <v>220</v>
       </c>
       <c r="AW13" s="10" t="s">
-        <v>219</v>
+        <v>133</v>
       </c>
       <c r="AX13" s="9">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="AY13" s="10" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="C14" s="9">
+        <v>4891</v>
+      </c>
+      <c r="D14" s="9">
+        <v>0</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="F14" s="9">
+        <v>1116</v>
+      </c>
+      <c r="G14" s="10" t="s">
         <v>221</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>222</v>
-      </c>
-      <c r="C14" s="9">
-        <v>4548</v>
-      </c>
-      <c r="D14" s="9">
-        <v>0</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="F14" s="9">
-        <v>1056</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>223</v>
       </c>
       <c r="H14" s="9">
         <v>18</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>165</v>
+        <v>222</v>
       </c>
       <c r="J14" s="9">
-        <v>93</v>
+        <v>34</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>109</v>
+        <v>164</v>
       </c>
       <c r="L14" s="9">
-        <v>1269</v>
+        <v>1387</v>
       </c>
       <c r="M14" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="N14" s="9">
+        <v>885</v>
+      </c>
+      <c r="O14" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="N14" s="9">
-        <v>725</v>
-      </c>
-      <c r="O14" s="10" t="s">
+      <c r="P14" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="R14" s="9">
+        <v>297</v>
+      </c>
+      <c r="S14" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="P14" s="9">
-        <v>8</v>
-      </c>
-      <c r="Q14" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="R14" s="9">
-        <v>267</v>
-      </c>
-      <c r="S14" s="10" t="s">
-        <v>226</v>
-      </c>
       <c r="T14" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U14" s="10" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="V14" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W14" s="10" t="s">
         <v>117</v>
@@ -3226,16 +3211,16 @@
         <v>9</v>
       </c>
       <c r="Y14" s="10" t="s">
-        <v>227</v>
+        <v>151</v>
       </c>
       <c r="Z14" s="9">
         <v>1</v>
       </c>
       <c r="AA14" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AB14" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC14" s="10" t="s">
         <v>117</v>
@@ -3244,198 +3229,198 @@
         <v>5</v>
       </c>
       <c r="AE14" s="10" t="s">
-        <v>195</v>
+        <v>121</v>
       </c>
       <c r="AF14" s="9">
         <v>0</v>
       </c>
       <c r="AG14" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AH14" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI14" s="10" t="s">
         <v>117</v>
       </c>
       <c r="AJ14" s="9">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="AK14" s="10" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="AL14" s="9">
         <v>1</v>
       </c>
       <c r="AM14" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AN14" s="9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AO14" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AP14" s="9">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="AQ14" s="10" t="s">
-        <v>229</v>
+        <v>164</v>
       </c>
       <c r="AR14" s="9">
         <v>1</v>
       </c>
       <c r="AS14" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AT14" s="9">
-        <v>86</v>
+        <v>27</v>
       </c>
       <c r="AU14" s="10" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="AV14" s="9">
-        <v>339</v>
+        <v>364</v>
       </c>
       <c r="AW14" s="10" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="AX14" s="9">
-        <v>617</v>
+        <v>691</v>
       </c>
       <c r="AY14" s="10" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C15" s="9">
-        <v>12546</v>
+        <v>12580</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F15" s="9">
-        <v>3863</v>
+        <v>3873</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="H15" s="9">
         <v>55</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J15" s="9">
         <v>5</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="L15" s="9">
-        <v>3835</v>
+        <v>3858</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="N15" s="9">
         <v>226</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="P15" s="9">
         <v>1</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="R15" s="9">
         <v>733</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="T15" s="9">
         <v>41</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
       <c r="V15" s="9">
         <v>0</v>
       </c>
       <c r="W15" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="X15" s="9">
         <v>15</v>
       </c>
       <c r="Y15" s="10" t="s">
-        <v>161</v>
+        <v>237</v>
       </c>
       <c r="Z15" s="9">
         <v>0</v>
       </c>
       <c r="AA15" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AB15" s="9">
         <v>0</v>
       </c>
       <c r="AC15" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AD15" s="9">
         <v>3</v>
       </c>
       <c r="AE15" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AF15" s="9">
         <v>0</v>
       </c>
       <c r="AG15" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AH15" s="9">
         <v>1</v>
       </c>
       <c r="AI15" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AJ15" s="9">
         <v>11</v>
       </c>
       <c r="AK15" s="10" t="s">
-        <v>128</v>
+        <v>238</v>
       </c>
       <c r="AL15" s="9">
         <v>3</v>
       </c>
       <c r="AM15" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AN15" s="9">
         <v>1</v>
       </c>
       <c r="AO15" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AP15" s="9">
         <v>79</v>
       </c>
       <c r="AQ15" s="10" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="AR15" s="9">
         <v>19</v>
@@ -3447,48 +3432,48 @@
         <v>3</v>
       </c>
       <c r="AU15" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AV15" s="9">
         <v>1053</v>
       </c>
       <c r="AW15" s="10" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="AX15" s="9">
-        <v>2599</v>
+        <v>2600</v>
       </c>
       <c r="AY15" s="10" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C16" s="9">
-        <v>5059</v>
+        <v>5068</v>
       </c>
       <c r="D16" s="9">
         <v>2</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="F16" s="9">
         <v>899</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="H16" s="9">
         <v>32</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="J16" s="9">
         <v>8</v>
@@ -3497,82 +3482,82 @@
         <v>116</v>
       </c>
       <c r="L16" s="9">
-        <v>1597</v>
+        <v>1601</v>
       </c>
       <c r="M16" s="10" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="N16" s="9">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="O16" s="10" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="P16" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q16" s="10" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="R16" s="9">
         <v>266</v>
       </c>
       <c r="S16" s="10" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="T16" s="9">
         <v>0</v>
       </c>
       <c r="U16" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="V16" s="9">
         <v>0</v>
       </c>
       <c r="W16" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="X16" s="9">
         <v>5</v>
       </c>
       <c r="Y16" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="Z16" s="9">
         <v>3</v>
       </c>
       <c r="AA16" s="10" t="s">
-        <v>106</v>
+        <v>136</v>
       </c>
       <c r="AB16" s="9">
         <v>1</v>
       </c>
       <c r="AC16" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AD16" s="9">
         <v>3</v>
       </c>
       <c r="AE16" s="10" t="s">
-        <v>106</v>
+        <v>136</v>
       </c>
       <c r="AF16" s="9">
         <v>0</v>
       </c>
       <c r="AG16" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AH16" s="9">
         <v>0</v>
       </c>
       <c r="AI16" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AJ16" s="9">
         <v>29</v>
       </c>
       <c r="AK16" s="10" t="s">
-        <v>250</v>
+        <v>120</v>
       </c>
       <c r="AL16" s="9">
         <v>4</v>
@@ -3584,734 +3569,734 @@
         <v>0</v>
       </c>
       <c r="AO16" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AP16" s="9">
         <v>43</v>
       </c>
       <c r="AQ16" s="10" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="AR16" s="9">
         <v>7</v>
       </c>
       <c r="AS16" s="10" t="s">
-        <v>182</v>
+        <v>132</v>
       </c>
       <c r="AT16" s="9">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="AU16" s="10" t="s">
-        <v>252</v>
+        <v>175</v>
       </c>
       <c r="AV16" s="9">
         <v>420</v>
       </c>
       <c r="AW16" s="10" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="AX16" s="9">
         <v>1436</v>
       </c>
       <c r="AY16" s="10" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="C17" s="9">
+        <v>9692</v>
+      </c>
+      <c r="D17" s="9">
+        <v>26</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>194</v>
+      </c>
+      <c r="F17" s="9">
+        <v>2869</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>253</v>
+      </c>
+      <c r="H17" s="9">
+        <v>265</v>
+      </c>
+      <c r="I17" s="10" t="s">
+        <v>254</v>
+      </c>
+      <c r="J17" s="9">
+        <v>122</v>
+      </c>
+      <c r="K17" s="10" t="s">
         <v>255</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="L17" s="9">
+        <v>3743</v>
+      </c>
+      <c r="M17" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="C17" s="9">
-        <v>8917</v>
-      </c>
-      <c r="D17" s="9">
-        <v>17</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>137</v>
-      </c>
-      <c r="F17" s="9">
-        <v>2704</v>
-      </c>
-      <c r="G17" s="10" t="s">
+      <c r="N17" s="9">
+        <v>642</v>
+      </c>
+      <c r="O17" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="H17" s="9">
-        <v>290</v>
-      </c>
-      <c r="I17" s="10" t="s">
+      <c r="P17" s="9">
+        <v>23</v>
+      </c>
+      <c r="Q17" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="R17" s="9">
+        <v>428</v>
+      </c>
+      <c r="S17" s="10" t="s">
         <v>258</v>
-      </c>
-      <c r="J17" s="9">
-        <v>127</v>
-      </c>
-      <c r="K17" s="10" t="s">
-        <v>259</v>
-      </c>
-      <c r="L17" s="9">
-        <v>3374</v>
-      </c>
-      <c r="M17" s="10" t="s">
-        <v>260</v>
-      </c>
-      <c r="N17" s="9">
-        <v>495</v>
-      </c>
-      <c r="O17" s="10" t="s">
-        <v>261</v>
-      </c>
-      <c r="P17" s="9">
-        <v>22</v>
-      </c>
-      <c r="Q17" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="R17" s="9">
-        <v>350</v>
-      </c>
-      <c r="S17" s="10" t="s">
-        <v>262</v>
       </c>
       <c r="T17" s="9">
         <v>1</v>
       </c>
       <c r="U17" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="V17" s="9">
         <v>6</v>
       </c>
       <c r="W17" s="10" t="s">
-        <v>118</v>
+        <v>136</v>
       </c>
       <c r="X17" s="9">
         <v>5</v>
       </c>
       <c r="Y17" s="10" t="s">
-        <v>106</v>
+        <v>177</v>
       </c>
       <c r="Z17" s="9">
         <v>4</v>
       </c>
       <c r="AA17" s="10" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="AB17" s="9">
         <v>2</v>
       </c>
       <c r="AC17" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AD17" s="9">
         <v>4</v>
       </c>
       <c r="AE17" s="10" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="AF17" s="9">
         <v>0</v>
       </c>
       <c r="AG17" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AH17" s="9">
         <v>2</v>
       </c>
       <c r="AI17" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AJ17" s="9">
         <v>16</v>
       </c>
       <c r="AK17" s="10" t="s">
-        <v>134</v>
+        <v>259</v>
       </c>
       <c r="AL17" s="9">
         <v>3</v>
       </c>
       <c r="AM17" s="10" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="AN17" s="9">
         <v>7</v>
       </c>
       <c r="AO17" s="10" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="AP17" s="9">
         <v>44</v>
       </c>
       <c r="AQ17" s="10" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="AR17" s="9">
         <v>9</v>
       </c>
       <c r="AS17" s="10" t="s">
-        <v>122</v>
+        <v>238</v>
       </c>
       <c r="AT17" s="9">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="AU17" s="10" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="AV17" s="9">
-        <v>718</v>
+        <v>737</v>
       </c>
       <c r="AW17" s="10" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="AX17" s="9">
-        <v>457</v>
+        <v>465</v>
       </c>
       <c r="AY17" s="10" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C18" s="9">
-        <v>9982</v>
+        <v>10129</v>
       </c>
       <c r="D18" s="9">
         <v>1</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F18" s="9">
-        <v>1784</v>
+        <v>1835</v>
       </c>
       <c r="G18" s="10" t="s">
+        <v>266</v>
+      </c>
+      <c r="H18" s="9">
+        <v>151</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>267</v>
+      </c>
+      <c r="J18" s="9">
+        <v>133</v>
+      </c>
+      <c r="K18" s="10" t="s">
+        <v>268</v>
+      </c>
+      <c r="L18" s="9">
+        <v>3385</v>
+      </c>
+      <c r="M18" s="10" t="s">
         <v>269</v>
       </c>
-      <c r="H18" s="9">
-        <v>150</v>
-      </c>
-      <c r="I18" s="10" t="s">
+      <c r="N18" s="9">
+        <v>1588</v>
+      </c>
+      <c r="O18" s="10" t="s">
         <v>270</v>
-      </c>
-      <c r="J18" s="9">
-        <v>134</v>
-      </c>
-      <c r="K18" s="10" t="s">
-        <v>271</v>
-      </c>
-      <c r="L18" s="9">
-        <v>3217</v>
-      </c>
-      <c r="M18" s="10" t="s">
-        <v>272</v>
-      </c>
-      <c r="N18" s="9">
-        <v>1706</v>
-      </c>
-      <c r="O18" s="10" t="s">
-        <v>273</v>
       </c>
       <c r="P18" s="9">
         <v>6</v>
       </c>
       <c r="Q18" s="10" t="s">
-        <v>106</v>
+        <v>136</v>
       </c>
       <c r="R18" s="9">
-        <v>631</v>
+        <v>670</v>
       </c>
       <c r="S18" s="10" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="T18" s="9">
         <v>24</v>
       </c>
       <c r="U18" s="10" t="s">
-        <v>275</v>
+        <v>118</v>
       </c>
       <c r="V18" s="9">
         <v>0</v>
       </c>
       <c r="W18" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="X18" s="9">
         <v>5</v>
       </c>
       <c r="Y18" s="10" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="Z18" s="9">
         <v>1</v>
       </c>
       <c r="AA18" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AB18" s="9">
         <v>1</v>
       </c>
       <c r="AC18" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AD18" s="9">
         <v>3</v>
       </c>
       <c r="AE18" s="10" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="AF18" s="9">
         <v>0</v>
       </c>
       <c r="AG18" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AH18" s="9">
         <v>0</v>
       </c>
       <c r="AI18" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AJ18" s="9">
         <v>11</v>
       </c>
       <c r="AK18" s="10" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="AL18" s="9">
         <v>10</v>
       </c>
       <c r="AM18" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="AN18" s="9">
         <v>2</v>
       </c>
       <c r="AO18" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AP18" s="9">
         <v>38</v>
       </c>
       <c r="AQ18" s="10" t="s">
-        <v>276</v>
+        <v>163</v>
       </c>
       <c r="AR18" s="9">
         <v>17</v>
       </c>
       <c r="AS18" s="10" t="s">
-        <v>172</v>
+        <v>259</v>
       </c>
       <c r="AT18" s="9">
         <v>1</v>
       </c>
       <c r="AU18" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AV18" s="9">
-        <v>403</v>
+        <v>410</v>
       </c>
       <c r="AW18" s="10" t="s">
-        <v>133</v>
+        <v>272</v>
       </c>
       <c r="AX18" s="9">
         <v>1837</v>
       </c>
       <c r="AY18" s="10" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="C19" s="9">
-        <v>10085</v>
+        <v>10667</v>
       </c>
       <c r="D19" s="9">
         <v>0</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F19" s="9">
-        <v>1173</v>
+        <v>1196</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>197</v>
+        <v>276</v>
       </c>
       <c r="H19" s="9">
         <v>15</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>152</v>
+        <v>132</v>
       </c>
       <c r="J19" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K19" s="10" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="L19" s="9">
-        <v>4670</v>
+        <v>5085</v>
       </c>
       <c r="M19" s="10" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="N19" s="9">
-        <v>1592</v>
+        <v>1587</v>
       </c>
       <c r="O19" s="10" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="P19" s="9">
         <v>0</v>
       </c>
       <c r="Q19" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="R19" s="9">
-        <v>1031</v>
+        <v>1165</v>
       </c>
       <c r="S19" s="10" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="T19" s="9">
         <v>0</v>
       </c>
       <c r="U19" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="V19" s="9">
         <v>0</v>
       </c>
       <c r="W19" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="X19" s="9">
         <v>18</v>
       </c>
       <c r="Y19" s="10" t="s">
-        <v>134</v>
+        <v>259</v>
       </c>
       <c r="Z19" s="9">
         <v>0</v>
       </c>
       <c r="AA19" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AB19" s="9">
         <v>0</v>
       </c>
       <c r="AC19" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AD19" s="9">
         <v>3</v>
       </c>
       <c r="AE19" s="10" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="AF19" s="9">
         <v>0</v>
       </c>
       <c r="AG19" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AH19" s="9">
         <v>0</v>
       </c>
       <c r="AI19" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AJ19" s="9">
         <v>16</v>
       </c>
       <c r="AK19" s="10" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="AL19" s="9">
         <v>0</v>
       </c>
       <c r="AM19" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AN19" s="9">
         <v>0</v>
       </c>
       <c r="AO19" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AP19" s="9">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="AQ19" s="10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="AR19" s="9">
         <v>1</v>
       </c>
       <c r="AS19" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AT19" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU19" s="10" t="s">
-        <v>136</v>
+        <v>115</v>
       </c>
       <c r="AV19" s="9">
-        <v>662</v>
+        <v>671</v>
       </c>
       <c r="AW19" s="10" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="AX19" s="9">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="AY19" s="10" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C20" s="9">
-        <v>1049</v>
+        <v>1053</v>
       </c>
       <c r="D20" s="9">
         <v>1</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>122</v>
+        <v>238</v>
       </c>
       <c r="F20" s="9">
         <v>162</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="H20" s="9">
         <v>6</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>250</v>
+        <v>120</v>
       </c>
       <c r="J20" s="9">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="L20" s="9">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="M20" s="10" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="N20" s="9">
         <v>48</v>
       </c>
       <c r="O20" s="10" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="P20" s="9">
         <v>6</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>250</v>
+        <v>120</v>
       </c>
       <c r="R20" s="9">
         <v>168</v>
       </c>
       <c r="S20" s="10" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="T20" s="9">
         <v>0</v>
       </c>
       <c r="U20" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="V20" s="9">
         <v>0</v>
       </c>
       <c r="W20" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="X20" s="9">
         <v>9</v>
       </c>
       <c r="Y20" s="10" t="s">
-        <v>292</v>
+        <v>248</v>
       </c>
       <c r="Z20" s="9">
         <v>3</v>
       </c>
       <c r="AA20" s="10" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="AB20" s="9">
         <v>0</v>
       </c>
       <c r="AC20" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AD20" s="9">
         <v>0</v>
       </c>
       <c r="AE20" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AF20" s="9">
         <v>0</v>
       </c>
       <c r="AG20" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AH20" s="9">
         <v>1</v>
       </c>
       <c r="AI20" s="10" t="s">
-        <v>122</v>
+        <v>238</v>
       </c>
       <c r="AJ20" s="9">
         <v>6</v>
       </c>
       <c r="AK20" s="10" t="s">
-        <v>250</v>
+        <v>120</v>
       </c>
       <c r="AL20" s="9">
         <v>2</v>
       </c>
       <c r="AM20" s="10" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="AN20" s="9">
         <v>1</v>
       </c>
       <c r="AO20" s="10" t="s">
-        <v>122</v>
+        <v>238</v>
       </c>
       <c r="AP20" s="9">
         <v>18</v>
       </c>
       <c r="AQ20" s="10" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="AR20" s="9">
         <v>4</v>
       </c>
       <c r="AS20" s="10" t="s">
-        <v>276</v>
+        <v>163</v>
       </c>
       <c r="AT20" s="9">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="AU20" s="10" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="AV20" s="9">
         <v>47</v>
       </c>
       <c r="AW20" s="10" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="AX20" s="9">
         <v>185</v>
       </c>
       <c r="AY20" s="10" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="C21" s="9">
-        <v>2561</v>
+        <v>2566</v>
       </c>
       <c r="D21" s="9">
         <v>0</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F21" s="9">
         <v>420</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="H21" s="9">
         <v>150</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="J21" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K21" s="10" t="s">
-        <v>140</v>
+        <v>114</v>
       </c>
       <c r="L21" s="9">
-        <v>777</v>
+        <v>781</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="N21" s="9">
         <v>102</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="P21" s="9">
         <v>8</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>228</v>
+        <v>300</v>
       </c>
       <c r="R21" s="9">
         <v>79</v>
       </c>
       <c r="S21" s="10" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="T21" s="9">
         <v>0</v>
       </c>
       <c r="U21" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="V21" s="9">
         <v>0</v>
       </c>
       <c r="W21" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="X21" s="9">
         <v>17</v>
       </c>
       <c r="Y21" s="10" t="s">
-        <v>305</v>
+        <v>216</v>
       </c>
       <c r="Z21" s="9">
         <v>2</v>
@@ -4323,228 +4308,228 @@
         <v>0</v>
       </c>
       <c r="AC21" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AD21" s="9">
         <v>0</v>
       </c>
       <c r="AE21" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AF21" s="9">
         <v>0</v>
       </c>
       <c r="AG21" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AH21" s="9">
         <v>0</v>
       </c>
       <c r="AI21" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AJ21" s="9">
         <v>3</v>
       </c>
       <c r="AK21" s="10" t="s">
-        <v>161</v>
+        <v>237</v>
       </c>
       <c r="AL21" s="9">
         <v>0</v>
       </c>
       <c r="AM21" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AN21" s="9">
         <v>0</v>
       </c>
       <c r="AO21" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AP21" s="9">
         <v>18</v>
       </c>
       <c r="AQ21" s="10" t="s">
-        <v>306</v>
+        <v>164</v>
       </c>
       <c r="AR21" s="9">
         <v>1</v>
       </c>
       <c r="AS21" s="10" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="AT21" s="9">
         <v>23</v>
       </c>
       <c r="AU21" s="10" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="AV21" s="9">
         <v>97</v>
       </c>
       <c r="AW21" s="10" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="AX21" s="9">
         <v>863</v>
       </c>
       <c r="AY21" s="10" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="C22" s="12">
-        <v>117473</v>
+        <v>120818</v>
       </c>
       <c r="D22" s="12">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>106</v>
       </c>
       <c r="F22" s="12">
-        <v>23931</v>
+        <v>24509</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>107</v>
       </c>
       <c r="H22" s="12">
-        <v>1529</v>
+        <v>1506</v>
       </c>
       <c r="I22" s="13" t="s">
         <v>108</v>
       </c>
       <c r="J22" s="12">
-        <v>2400</v>
+        <v>2285</v>
       </c>
       <c r="K22" s="13" t="s">
         <v>109</v>
       </c>
       <c r="L22" s="12">
-        <v>44236</v>
+        <v>46153</v>
       </c>
       <c r="M22" s="13" t="s">
         <v>110</v>
       </c>
       <c r="N22" s="12">
-        <v>11970</v>
+        <v>12318</v>
       </c>
       <c r="O22" s="13" t="s">
         <v>111</v>
       </c>
       <c r="P22" s="12">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="Q22" s="13" t="s">
         <v>112</v>
       </c>
       <c r="R22" s="12">
-        <v>8834</v>
+        <v>9292</v>
       </c>
       <c r="S22" s="13" t="s">
         <v>113</v>
       </c>
       <c r="T22" s="12">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="U22" s="13" t="s">
         <v>114</v>
       </c>
       <c r="V22" s="12">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="W22" s="13" t="s">
         <v>115</v>
       </c>
       <c r="X22" s="12">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="Y22" s="13" t="s">
         <v>116</v>
       </c>
       <c r="Z22" s="12">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AA22" s="13" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AB22" s="12">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="AC22" s="13" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AD22" s="12">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AE22" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="AF22" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG22" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="AH22" s="12">
+        <v>20</v>
+      </c>
+      <c r="AI22" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="AJ22" s="12">
+        <v>294</v>
+      </c>
+      <c r="AK22" s="13" t="s">
         <v>118</v>
-      </c>
-      <c r="AF22" s="12">
-        <v>0</v>
-      </c>
-      <c r="AG22" s="13" t="s">
-        <v>119</v>
-      </c>
-      <c r="AH22" s="12">
-        <v>24</v>
-      </c>
-      <c r="AI22" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="AJ22" s="12">
-        <v>288</v>
-      </c>
-      <c r="AK22" s="13" t="s">
-        <v>120</v>
       </c>
       <c r="AL22" s="12">
         <v>39</v>
       </c>
       <c r="AM22" s="13" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="AN22" s="12">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="AO22" s="13" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="AP22" s="12">
-        <v>678</v>
+        <v>689</v>
       </c>
       <c r="AQ22" s="13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="AR22" s="12">
         <v>115</v>
       </c>
       <c r="AS22" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="AT22" s="12">
+        <v>1042</v>
+      </c>
+      <c r="AU22" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="AT22" s="12">
-        <v>1087</v>
-      </c>
-      <c r="AU22" s="13" t="s">
+      <c r="AV22" s="12">
+        <v>6047</v>
+      </c>
+      <c r="AW22" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="AV22" s="12">
-        <v>5959</v>
-      </c>
-      <c r="AW22" s="13" t="s">
+      <c r="AX22" s="12">
+        <v>15646</v>
+      </c>
+      <c r="AY22" s="13" t="s">
         <v>124</v>
-      </c>
-      <c r="AX22" s="12">
-        <v>15528</v>
-      </c>
-      <c r="AY22" s="13" t="s">
-        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Perbarui data SE2026 05/09/2026  6:53:01,88
</commit_message>
<xml_diff>
--- a/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
+++ b/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="309">
   <si>
     <t>DATA RADAR ANOMALI USAHA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 4 Sep 2026, 08.16</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 5 Sep 2026, 06.51</t>
   </si>
   <si>
     <t>Kode</t>
@@ -331,601 +331,607 @@
     <t>LAMPUNG</t>
   </si>
   <si>
+    <t>0,08</t>
+  </si>
+  <si>
+    <t>20,47</t>
+  </si>
+  <si>
+    <t>1,2</t>
+  </si>
+  <si>
+    <t>1,84</t>
+  </si>
+  <si>
+    <t>38,46</t>
+  </si>
+  <si>
+    <t>10,11</t>
+  </si>
+  <si>
+    <t>0,19</t>
+  </si>
+  <si>
+    <t>7,64</t>
+  </si>
+  <si>
+    <t>0,09</t>
+  </si>
+  <si>
+    <t>0,02</t>
+  </si>
+  <si>
+    <t>0,16</t>
+  </si>
+  <si>
     <t>0,07</t>
   </si>
   <si>
-    <t>20,29</t>
-  </si>
-  <si>
-    <t>1,25</t>
-  </si>
-  <si>
-    <t>1,89</t>
-  </si>
-  <si>
-    <t>38,2</t>
-  </si>
-  <si>
-    <t>10,2</t>
+    <t>0</t>
+  </si>
+  <si>
+    <t>0,24</t>
+  </si>
+  <si>
+    <t>0,03</t>
+  </si>
+  <si>
+    <t>0,56</t>
+  </si>
+  <si>
+    <t>0,86</t>
+  </si>
+  <si>
+    <t>4,97</t>
+  </si>
+  <si>
+    <t>12,8</t>
+  </si>
+  <si>
+    <t>1801</t>
+  </si>
+  <si>
+    <t>LAMPUNG BARAT</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>19,17</t>
+  </si>
+  <si>
+    <t>0,95</t>
+  </si>
+  <si>
+    <t>0,99</t>
+  </si>
+  <si>
+    <t>47,84</t>
+  </si>
+  <si>
+    <t>4,02</t>
+  </si>
+  <si>
+    <t>0,14</t>
+  </si>
+  <si>
+    <t>4,52</t>
+  </si>
+  <si>
+    <t>0,01</t>
+  </si>
+  <si>
+    <t>0,06</t>
+  </si>
+  <si>
+    <t>0,13</t>
+  </si>
+  <si>
+    <t>0,04</t>
+  </si>
+  <si>
+    <t>0,35</t>
+  </si>
+  <si>
+    <t>2,8</t>
+  </si>
+  <si>
+    <t>3,56</t>
+  </si>
+  <si>
+    <t>14,94</t>
+  </si>
+  <si>
+    <t>1802</t>
+  </si>
+  <si>
+    <t>TANGGAMUS</t>
+  </si>
+  <si>
+    <t>13,68</t>
+  </si>
+  <si>
+    <t>0,5</t>
+  </si>
+  <si>
+    <t>0,88</t>
+  </si>
+  <si>
+    <t>27,01</t>
+  </si>
+  <si>
+    <t>30,07</t>
+  </si>
+  <si>
+    <t>6,41</t>
+  </si>
+  <si>
+    <t>0,18</t>
+  </si>
+  <si>
+    <t>0,15</t>
+  </si>
+  <si>
+    <t>0,47</t>
+  </si>
+  <si>
+    <t>4,71</t>
+  </si>
+  <si>
+    <t>15,8</t>
+  </si>
+  <si>
+    <t>1803</t>
+  </si>
+  <si>
+    <t>LAMPUNG SELATAN</t>
+  </si>
+  <si>
+    <t>16,18</t>
+  </si>
+  <si>
+    <t>2,05</t>
   </si>
   <si>
     <t>0,2</t>
   </si>
   <si>
-    <t>7,69</t>
-  </si>
-  <si>
-    <t>0,08</t>
-  </si>
-  <si>
-    <t>0,02</t>
-  </si>
-  <si>
-    <t>0,16</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>0,24</t>
-  </si>
-  <si>
-    <t>0,03</t>
+    <t>48,61</t>
+  </si>
+  <si>
+    <t>9,05</t>
+  </si>
+  <si>
+    <t>10,55</t>
+  </si>
+  <si>
+    <t>0,38</t>
+  </si>
+  <si>
+    <t>0,72</t>
+  </si>
+  <si>
+    <t>1,04</t>
+  </si>
+  <si>
+    <t>3,79</t>
+  </si>
+  <si>
+    <t>7,23</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>24,1</t>
+  </si>
+  <si>
+    <t>0,76</t>
+  </si>
+  <si>
+    <t>7,4</t>
+  </si>
+  <si>
+    <t>33,25</t>
+  </si>
+  <si>
+    <t>12,55</t>
+  </si>
+  <si>
+    <t>0,7</t>
+  </si>
+  <si>
+    <t>7,12</t>
+  </si>
+  <si>
+    <t>0,25</t>
+  </si>
+  <si>
+    <t>0,05</t>
+  </si>
+  <si>
+    <t>1,87</t>
+  </si>
+  <si>
+    <t>2,15</t>
+  </si>
+  <si>
+    <t>9,1</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>2,2</t>
+  </si>
+  <si>
+    <t>1,11</t>
+  </si>
+  <si>
+    <t>46,34</t>
+  </si>
+  <si>
+    <t>4,59</t>
+  </si>
+  <si>
+    <t>0,22</t>
+  </si>
+  <si>
+    <t>13,01</t>
+  </si>
+  <si>
+    <t>0,64</t>
+  </si>
+  <si>
+    <t>0,11</t>
+  </si>
+  <si>
+    <t>0,3</t>
+  </si>
+  <si>
+    <t>3,19</t>
+  </si>
+  <si>
+    <t>11,59</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>18,9</t>
+  </si>
+  <si>
+    <t>0,73</t>
+  </si>
+  <si>
+    <t>0,98</t>
+  </si>
+  <si>
+    <t>37,69</t>
+  </si>
+  <si>
+    <t>13,96</t>
+  </si>
+  <si>
+    <t>7,83</t>
+  </si>
+  <si>
+    <t>0,59</t>
+  </si>
+  <si>
+    <t>1,15</t>
+  </si>
+  <si>
+    <t>6,82</t>
+  </si>
+  <si>
+    <t>10,48</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>17,64</t>
+  </si>
+  <si>
+    <t>0,63</t>
+  </si>
+  <si>
+    <t>1,24</t>
+  </si>
+  <si>
+    <t>43,12</t>
+  </si>
+  <si>
+    <t>16,74</t>
+  </si>
+  <si>
+    <t>6,18</t>
+  </si>
+  <si>
+    <t>0,65</t>
+  </si>
+  <si>
+    <t>0,75</t>
+  </si>
+  <si>
+    <t>4,46</t>
+  </si>
+  <si>
+    <t>7,1</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>22,78</t>
+  </si>
+  <si>
+    <t>0,37</t>
+  </si>
+  <si>
+    <t>0,55</t>
+  </si>
+  <si>
+    <t>28,48</t>
+  </si>
+  <si>
+    <t>18,25</t>
+  </si>
+  <si>
+    <t>6,11</t>
+  </si>
+  <si>
+    <t>0,32</t>
+  </si>
+  <si>
+    <t>0,69</t>
+  </si>
+  <si>
+    <t>7,41</t>
+  </si>
+  <si>
+    <t>14,13</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>30,79</t>
+  </si>
+  <si>
+    <t>0,44</t>
+  </si>
+  <si>
+    <t>30,67</t>
+  </si>
+  <si>
+    <t>1,79</t>
+  </si>
+  <si>
+    <t>5,82</t>
+  </si>
+  <si>
+    <t>0,33</t>
+  </si>
+  <si>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>8,38</t>
+  </si>
+  <si>
+    <t>20,64</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>17,72</t>
+  </si>
+  <si>
+    <t>31,71</t>
+  </si>
+  <si>
+    <t>5,33</t>
+  </si>
+  <si>
+    <t>5,24</t>
   </si>
   <si>
     <t>0,57</t>
   </si>
   <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>0,86</t>
-  </si>
-  <si>
-    <t>5,01</t>
-  </si>
-  <si>
-    <t>12,95</t>
-  </si>
-  <si>
-    <t>1801</t>
-  </si>
-  <si>
-    <t>LAMPUNG BARAT</t>
-  </si>
-  <si>
-    <t>19,17</t>
-  </si>
-  <si>
-    <t>0,95</t>
-  </si>
-  <si>
-    <t>0,99</t>
-  </si>
-  <si>
-    <t>47,84</t>
-  </si>
-  <si>
-    <t>4,02</t>
-  </si>
-  <si>
-    <t>0,14</t>
-  </si>
-  <si>
-    <t>4,52</t>
-  </si>
-  <si>
-    <t>0,01</t>
-  </si>
-  <si>
-    <t>0,19</t>
-  </si>
-  <si>
-    <t>0,06</t>
-  </si>
-  <si>
-    <t>0,13</t>
-  </si>
-  <si>
-    <t>0,04</t>
-  </si>
-  <si>
-    <t>0,35</t>
-  </si>
-  <si>
-    <t>2,8</t>
-  </si>
-  <si>
-    <t>3,56</t>
-  </si>
-  <si>
-    <t>14,94</t>
-  </si>
-  <si>
-    <t>1802</t>
-  </si>
-  <si>
-    <t>TANGGAMUS</t>
-  </si>
-  <si>
-    <t>13,67</t>
-  </si>
-  <si>
-    <t>0,5</t>
-  </si>
-  <si>
-    <t>0,89</t>
-  </si>
-  <si>
-    <t>26,72</t>
-  </si>
-  <si>
-    <t>30,24</t>
-  </si>
-  <si>
-    <t>6,45</t>
-  </si>
-  <si>
-    <t>0,18</t>
-  </si>
-  <si>
-    <t>0,15</t>
-  </si>
-  <si>
-    <t>0,47</t>
-  </si>
-  <si>
-    <t>4,73</t>
-  </si>
-  <si>
-    <t>15,86</t>
-  </si>
-  <si>
-    <t>1803</t>
-  </si>
-  <si>
-    <t>LAMPUNG SELATAN</t>
-  </si>
-  <si>
-    <t>16,32</t>
-  </si>
-  <si>
-    <t>2,1</t>
-  </si>
-  <si>
-    <t>47,54</t>
-  </si>
-  <si>
-    <t>9,63</t>
-  </si>
-  <si>
-    <t>10,72</t>
-  </si>
-  <si>
-    <t>0,38</t>
-  </si>
-  <si>
-    <t>0,7</t>
-  </si>
-  <si>
-    <t>1,07</t>
-  </si>
-  <si>
-    <t>3,85</t>
-  </si>
-  <si>
-    <t>7,38</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>23,35</t>
-  </si>
-  <si>
-    <t>0,76</t>
-  </si>
-  <si>
-    <t>7,84</t>
-  </si>
-  <si>
-    <t>32,93</t>
-  </si>
-  <si>
-    <t>12,65</t>
-  </si>
-  <si>
-    <t>0,73</t>
-  </si>
-  <si>
-    <t>7,16</t>
-  </si>
-  <si>
-    <t>0,05</t>
-  </si>
-  <si>
-    <t>0,26</t>
-  </si>
-  <si>
-    <t>1,92</t>
-  </si>
-  <si>
-    <t>2,21</t>
-  </si>
-  <si>
-    <t>9,43</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>15,69</t>
-  </si>
-  <si>
-    <t>2,27</t>
-  </si>
-  <si>
-    <t>1,13</t>
-  </si>
-  <si>
-    <t>46,26</t>
-  </si>
-  <si>
-    <t>4,65</t>
+    <t>0,85</t>
+  </si>
+  <si>
+    <t>8,29</t>
+  </si>
+  <si>
+    <t>28,33</t>
+  </si>
+  <si>
+    <t>1811</t>
+  </si>
+  <si>
+    <t>MESUJI</t>
+  </si>
+  <si>
+    <t>29,54</t>
+  </si>
+  <si>
+    <t>2,35</t>
+  </si>
+  <si>
+    <t>1,19</t>
+  </si>
+  <si>
+    <t>39,23</t>
+  </si>
+  <si>
+    <t>6,74</t>
   </si>
   <si>
     <t>0,21</t>
   </si>
   <si>
-    <t>13,13</t>
-  </si>
-  <si>
-    <t>0,22</t>
-  </si>
-  <si>
-    <t>0,64</t>
-  </si>
-  <si>
-    <t>0,11</t>
-  </si>
-  <si>
-    <t>0,27</t>
-  </si>
-  <si>
-    <t>3,21</t>
-  </si>
-  <si>
-    <t>11,53</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>18,9</t>
-  </si>
-  <si>
-    <t>0,98</t>
-  </si>
-  <si>
-    <t>37,62</t>
-  </si>
-  <si>
-    <t>13,98</t>
-  </si>
-  <si>
-    <t>7,85</t>
-  </si>
-  <si>
-    <t>0,59</t>
-  </si>
-  <si>
-    <t>1,15</t>
-  </si>
-  <si>
-    <t>0,25</t>
-  </si>
-  <si>
-    <t>6,81</t>
-  </si>
-  <si>
-    <t>10,38</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>17,65</t>
-  </si>
-  <si>
-    <t>0,8</t>
-  </si>
-  <si>
-    <t>43,26</t>
-  </si>
-  <si>
-    <t>16,97</t>
-  </si>
-  <si>
-    <t>6,22</t>
+    <t>4,37</t>
+  </si>
+  <si>
+    <t>2,67</t>
+  </si>
+  <si>
+    <t>7,55</t>
+  </si>
+  <si>
+    <t>4,79</t>
+  </si>
+  <si>
+    <t>1812</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG BARAT</t>
+  </si>
+  <si>
+    <t>18,6</t>
+  </si>
+  <si>
+    <t>1,47</t>
+  </si>
+  <si>
+    <t>1,14</t>
+  </si>
+  <si>
+    <t>33,54</t>
+  </si>
+  <si>
+    <t>15,52</t>
+  </si>
+  <si>
+    <t>6,55</t>
+  </si>
+  <si>
+    <t>0,29</t>
+  </si>
+  <si>
+    <t>0,17</t>
+  </si>
+  <si>
+    <t>4,07</t>
+  </si>
+  <si>
+    <t>17,91</t>
+  </si>
+  <si>
+    <t>1813</t>
+  </si>
+  <si>
+    <t>PESISIR BARAT</t>
+  </si>
+  <si>
+    <t>11,3</t>
+  </si>
+  <si>
+    <t>48,09</t>
+  </si>
+  <si>
+    <t>14,57</t>
+  </si>
+  <si>
+    <t>10,84</t>
+  </si>
+  <si>
+    <t>6,32</t>
+  </si>
+  <si>
+    <t>7,79</t>
+  </si>
+  <si>
+    <t>1871</t>
+  </si>
+  <si>
+    <t>BANDAR LAMPUNG</t>
+  </si>
+  <si>
+    <t>15,27</t>
+  </si>
+  <si>
+    <t>3,3</t>
+  </si>
+  <si>
+    <t>32,05</t>
+  </si>
+  <si>
+    <t>15,83</t>
+  </si>
+  <si>
+    <t>0,28</t>
+  </si>
+  <si>
+    <t>1,7</t>
+  </si>
+  <si>
+    <t>4,43</t>
+  </si>
+  <si>
+    <t>17,44</t>
+  </si>
+  <si>
+    <t>1872</t>
+  </si>
+  <si>
+    <t>METRO</t>
+  </si>
+  <si>
+    <t>16,36</t>
+  </si>
+  <si>
+    <t>5,84</t>
+  </si>
+  <si>
+    <t>30,45</t>
+  </si>
+  <si>
+    <t>3,97</t>
+  </si>
+  <si>
+    <t>0,31</t>
+  </si>
+  <si>
+    <t>3,08</t>
   </si>
   <si>
     <t>0,66</t>
   </si>
   <si>
-    <t>0,23</t>
-  </si>
-  <si>
-    <t>7,13</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>22,82</t>
-  </si>
-  <si>
-    <t>0,37</t>
-  </si>
-  <si>
-    <t>28,36</t>
-  </si>
-  <si>
-    <t>18,09</t>
-  </si>
-  <si>
-    <t>6,07</t>
-  </si>
-  <si>
-    <t>0,33</t>
-  </si>
-  <si>
-    <t>0,55</t>
-  </si>
-  <si>
-    <t>7,44</t>
-  </si>
-  <si>
-    <t>14,13</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>30,79</t>
-  </si>
-  <si>
-    <t>0,44</t>
-  </si>
-  <si>
-    <t>30,67</t>
-  </si>
-  <si>
-    <t>1,8</t>
-  </si>
-  <si>
-    <t>5,83</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>0,09</t>
-  </si>
-  <si>
-    <t>0,63</t>
-  </si>
-  <si>
-    <t>8,37</t>
-  </si>
-  <si>
-    <t>20,67</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>17,74</t>
-  </si>
-  <si>
-    <t>31,59</t>
-  </si>
-  <si>
-    <t>5,35</t>
-  </si>
-  <si>
-    <t>5,25</t>
-  </si>
-  <si>
-    <t>0,85</t>
-  </si>
-  <si>
-    <t>8,29</t>
-  </si>
-  <si>
-    <t>28,33</t>
-  </si>
-  <si>
-    <t>1811</t>
-  </si>
-  <si>
-    <t>MESUJI</t>
-  </si>
-  <si>
-    <t>29,6</t>
-  </si>
-  <si>
-    <t>2,73</t>
-  </si>
-  <si>
-    <t>1,26</t>
-  </si>
-  <si>
-    <t>38,62</t>
-  </si>
-  <si>
-    <t>6,62</t>
-  </si>
-  <si>
-    <t>4,42</t>
-  </si>
-  <si>
-    <t>0,17</t>
-  </si>
-  <si>
-    <t>0,45</t>
-  </si>
-  <si>
-    <t>2,78</t>
-  </si>
-  <si>
-    <t>7,6</t>
-  </si>
-  <si>
-    <t>4,8</t>
-  </si>
-  <si>
-    <t>1812</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG BARAT</t>
-  </si>
-  <si>
-    <t>18,12</t>
-  </si>
-  <si>
-    <t>1,49</t>
-  </si>
-  <si>
-    <t>1,31</t>
-  </si>
-  <si>
-    <t>33,42</t>
-  </si>
-  <si>
-    <t>15,68</t>
-  </si>
-  <si>
-    <t>6,61</t>
-  </si>
-  <si>
-    <t>4,05</t>
-  </si>
-  <si>
-    <t>18,14</t>
-  </si>
-  <si>
-    <t>1813</t>
-  </si>
-  <si>
-    <t>PESISIR BARAT</t>
-  </si>
-  <si>
-    <t>11,21</t>
-  </si>
-  <si>
-    <t>47,67</t>
-  </si>
-  <si>
-    <t>14,88</t>
-  </si>
-  <si>
-    <t>10,92</t>
-  </si>
-  <si>
-    <t>6,29</t>
-  </si>
-  <si>
-    <t>7,93</t>
-  </si>
-  <si>
-    <t>1871</t>
-  </si>
-  <si>
-    <t>BANDAR LAMPUNG</t>
-  </si>
-  <si>
-    <t>15,38</t>
-  </si>
-  <si>
-    <t>3,32</t>
-  </si>
-  <si>
-    <t>31,81</t>
-  </si>
-  <si>
-    <t>4,56</t>
-  </si>
-  <si>
-    <t>15,95</t>
-  </si>
-  <si>
-    <t>0,28</t>
-  </si>
-  <si>
-    <t>1,71</t>
-  </si>
-  <si>
-    <t>1,52</t>
-  </si>
-  <si>
-    <t>4,46</t>
-  </si>
-  <si>
-    <t>17,57</t>
-  </si>
-  <si>
-    <t>1872</t>
-  </si>
-  <si>
-    <t>METRO</t>
-  </si>
-  <si>
-    <t>16,37</t>
-  </si>
-  <si>
-    <t>5,85</t>
-  </si>
-  <si>
-    <t>30,44</t>
-  </si>
-  <si>
-    <t>3,98</t>
-  </si>
-  <si>
-    <t>0,31</t>
-  </si>
-  <si>
-    <t>3,08</t>
-  </si>
-  <si>
-    <t>0,9</t>
+    <t>0,93</t>
   </si>
   <si>
     <t>3,78</t>
   </si>
   <si>
-    <t>33,63</t>
+    <t>33,61</t>
   </si>
   <si>
     <t/>
@@ -1905,70 +1911,70 @@
         <v>105</v>
       </c>
       <c r="C6" s="6">
-        <v>120818</v>
+        <v>122688</v>
       </c>
       <c r="D6" s="6">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>106</v>
       </c>
       <c r="F6" s="6">
-        <v>24509</v>
+        <v>25110</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>107</v>
       </c>
       <c r="H6" s="6">
-        <v>1506</v>
+        <v>1473</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>108</v>
       </c>
       <c r="J6" s="6">
-        <v>2285</v>
+        <v>2256</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>109</v>
       </c>
       <c r="L6" s="6">
-        <v>46153</v>
+        <v>47186</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>110</v>
       </c>
       <c r="N6" s="6">
-        <v>12318</v>
+        <v>12401</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>111</v>
       </c>
       <c r="P6" s="6">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="Q6" s="7" t="s">
         <v>112</v>
       </c>
       <c r="R6" s="6">
-        <v>9292</v>
+        <v>9373</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>113</v>
       </c>
       <c r="T6" s="6">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="U6" s="7" t="s">
         <v>114</v>
       </c>
       <c r="V6" s="6">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="W6" s="7" t="s">
         <v>115</v>
       </c>
       <c r="X6" s="6">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="Y6" s="7" t="s">
         <v>116</v>
@@ -1980,7 +1986,7 @@
         <v>115</v>
       </c>
       <c r="AB6" s="6">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="AC6" s="7" t="s">
         <v>115</v>
@@ -1989,13 +1995,13 @@
         <v>89</v>
       </c>
       <c r="AE6" s="7" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="AF6" s="6">
         <v>0</v>
       </c>
       <c r="AG6" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH6" s="6">
         <v>20</v>
@@ -2004,49 +2010,49 @@
         <v>115</v>
       </c>
       <c r="AJ6" s="6">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="AK6" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AL6" s="6">
         <v>39</v>
       </c>
       <c r="AM6" s="7" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AN6" s="6">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="AO6" s="7" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="AP6" s="6">
         <v>689</v>
       </c>
       <c r="AQ6" s="7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AR6" s="6">
         <v>115</v>
       </c>
       <c r="AS6" s="7" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="AT6" s="6">
-        <v>1042</v>
+        <v>1049</v>
       </c>
       <c r="AU6" s="7" t="s">
         <v>122</v>
       </c>
       <c r="AV6" s="6">
-        <v>6047</v>
+        <v>6099</v>
       </c>
       <c r="AW6" s="7" t="s">
         <v>123</v>
       </c>
       <c r="AX6" s="6">
-        <v>15646</v>
+        <v>15703</v>
       </c>
       <c r="AY6" s="7" t="s">
         <v>124</v>
@@ -2066,79 +2072,79 @@
         <v>8</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="F7" s="9">
         <v>1492</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H7" s="9">
         <v>74</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J7" s="9">
         <v>77</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="L7" s="9">
         <v>3723</v>
       </c>
       <c r="M7" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="N7" s="9">
         <v>313</v>
       </c>
       <c r="O7" s="10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="P7" s="9">
         <v>11</v>
       </c>
       <c r="Q7" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="R7" s="9">
         <v>352</v>
       </c>
       <c r="S7" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="T7" s="9">
         <v>2</v>
       </c>
       <c r="U7" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="V7" s="9">
         <v>1</v>
       </c>
       <c r="W7" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="X7" s="9">
         <v>15</v>
       </c>
       <c r="Y7" s="10" t="s">
-        <v>135</v>
+        <v>112</v>
       </c>
       <c r="Z7" s="9">
         <v>2</v>
       </c>
       <c r="AA7" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AB7" s="9">
         <v>6</v>
       </c>
       <c r="AC7" s="10" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="AD7" s="9">
         <v>5</v>
@@ -2150,13 +2156,13 @@
         <v>0</v>
       </c>
       <c r="AG7" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH7" s="9">
         <v>0</v>
       </c>
       <c r="AI7" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ7" s="9">
         <v>10</v>
@@ -2168,7 +2174,7 @@
         <v>1</v>
       </c>
       <c r="AM7" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="AN7" s="9">
         <v>3</v>
@@ -2215,16 +2221,16 @@
         <v>144</v>
       </c>
       <c r="C8" s="9">
-        <v>3380</v>
+        <v>3399</v>
       </c>
       <c r="D8" s="9">
         <v>0</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F8" s="9">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>145</v>
@@ -2242,7 +2248,7 @@
         <v>147</v>
       </c>
       <c r="L8" s="9">
-        <v>903</v>
+        <v>918</v>
       </c>
       <c r="M8" s="10" t="s">
         <v>148</v>
@@ -2257,7 +2263,7 @@
         <v>0</v>
       </c>
       <c r="Q8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="R8" s="9">
         <v>218</v>
@@ -2269,13 +2275,13 @@
         <v>0</v>
       </c>
       <c r="U8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V8" s="9">
         <v>0</v>
       </c>
       <c r="W8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X8" s="9">
         <v>6</v>
@@ -2287,31 +2293,31 @@
         <v>0</v>
       </c>
       <c r="AA8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AB8" s="9">
         <v>0</v>
       </c>
       <c r="AC8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD8" s="9">
         <v>1</v>
       </c>
       <c r="AE8" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AF8" s="9">
         <v>0</v>
       </c>
       <c r="AG8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH8" s="9">
         <v>0</v>
       </c>
       <c r="AI8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ8" s="9">
         <v>5</v>
@@ -2323,13 +2329,13 @@
         <v>0</v>
       </c>
       <c r="AM8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AN8" s="9">
         <v>0</v>
       </c>
       <c r="AO8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AP8" s="9">
         <v>16</v>
@@ -2356,7 +2362,7 @@
         <v>154</v>
       </c>
       <c r="AX8" s="9">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="AY8" s="10" t="s">
         <v>155</v>
@@ -2370,16 +2376,16 @@
         <v>157</v>
       </c>
       <c r="C9" s="9">
-        <v>9384</v>
+        <v>9593</v>
       </c>
       <c r="D9" s="9">
         <v>0</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F9" s="9">
-        <v>1531</v>
+        <v>1552</v>
       </c>
       <c r="G9" s="10" t="s">
         <v>158</v>
@@ -2391,106 +2397,106 @@
         <v>159</v>
       </c>
       <c r="J9" s="9">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>132</v>
+        <v>160</v>
       </c>
       <c r="L9" s="9">
-        <v>4461</v>
+        <v>4663</v>
       </c>
       <c r="M9" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="N9" s="9">
-        <v>904</v>
+        <v>868</v>
       </c>
       <c r="O9" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="P9" s="9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="R9" s="9">
-        <v>1006</v>
+        <v>1012</v>
       </c>
       <c r="S9" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T9" s="9">
         <v>1</v>
       </c>
       <c r="U9" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="V9" s="9">
         <v>1</v>
       </c>
       <c r="W9" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="X9" s="9">
         <v>36</v>
       </c>
       <c r="Y9" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="Z9" s="9">
         <v>0</v>
       </c>
       <c r="AA9" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AB9" s="9">
         <v>0</v>
       </c>
       <c r="AC9" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD9" s="9">
         <v>9</v>
       </c>
       <c r="AE9" s="10" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="AF9" s="9">
         <v>0</v>
       </c>
       <c r="AG9" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH9" s="9">
         <v>0</v>
       </c>
       <c r="AI9" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ9" s="9">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="AK9" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="AL9" s="9">
         <v>0</v>
       </c>
       <c r="AM9" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AN9" s="9">
         <v>0</v>
       </c>
       <c r="AO9" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AP9" s="9">
         <v>100</v>
       </c>
       <c r="AQ9" s="10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="AR9" s="9">
         <v>2</v>
@@ -2502,102 +2508,102 @@
         <v>3</v>
       </c>
       <c r="AU9" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AV9" s="9">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="AW9" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AX9" s="9">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="AY9" s="10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C10" s="9">
-        <v>20201</v>
+        <v>20976</v>
       </c>
       <c r="D10" s="9">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>151</v>
       </c>
       <c r="F10" s="9">
-        <v>4717</v>
+        <v>5055</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H10" s="9">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J10" s="9">
-        <v>1584</v>
+        <v>1553</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="L10" s="9">
-        <v>6652</v>
+        <v>6974</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="N10" s="9">
-        <v>2555</v>
+        <v>2632</v>
       </c>
       <c r="O10" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P10" s="9">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="Q10" s="10" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="R10" s="9">
-        <v>1446</v>
+        <v>1493</v>
       </c>
       <c r="S10" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="T10" s="9">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="U10" s="10" t="s">
-        <v>177</v>
+        <v>136</v>
       </c>
       <c r="V10" s="9">
         <v>7</v>
       </c>
       <c r="W10" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="X10" s="9">
         <v>14</v>
       </c>
       <c r="Y10" s="10" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="Z10" s="9">
         <v>2</v>
       </c>
       <c r="AA10" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="AB10" s="9">
         <v>12</v>
@@ -2615,7 +2621,7 @@
         <v>0</v>
       </c>
       <c r="AG10" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH10" s="9">
         <v>8</v>
@@ -2633,7 +2639,7 @@
         <v>1</v>
       </c>
       <c r="AM10" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AN10" s="9">
         <v>52</v>
@@ -2645,81 +2651,81 @@
         <v>28</v>
       </c>
       <c r="AQ10" s="10" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="AR10" s="9">
         <v>10</v>
       </c>
       <c r="AS10" s="10" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AT10" s="9">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="AU10" s="10" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="AV10" s="9">
-        <v>447</v>
+        <v>452</v>
       </c>
       <c r="AW10" s="10" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="AX10" s="9">
-        <v>1904</v>
+        <v>1909</v>
       </c>
       <c r="AY10" s="10" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C11" s="9">
-        <v>13343</v>
+        <v>13465</v>
       </c>
       <c r="D11" s="9">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>106</v>
       </c>
       <c r="F11" s="9">
-        <v>2093</v>
+        <v>2128</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>184</v>
+        <v>155</v>
       </c>
       <c r="H11" s="9">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="I11" s="10" t="s">
         <v>185</v>
       </c>
       <c r="J11" s="9">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K11" s="10" t="s">
         <v>186</v>
       </c>
       <c r="L11" s="9">
-        <v>6172</v>
+        <v>6240</v>
       </c>
       <c r="M11" s="10" t="s">
         <v>187</v>
       </c>
       <c r="N11" s="9">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="O11" s="10" t="s">
         <v>188</v>
       </c>
       <c r="P11" s="9">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q11" s="10" t="s">
         <v>189</v>
@@ -2746,7 +2752,7 @@
         <v>11</v>
       </c>
       <c r="Y11" s="10" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="Z11" s="9">
         <v>5</v>
@@ -2770,7 +2776,7 @@
         <v>0</v>
       </c>
       <c r="AG11" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH11" s="9">
         <v>6</v>
@@ -2782,7 +2788,7 @@
         <v>29</v>
       </c>
       <c r="AK11" s="10" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="AL11" s="9">
         <v>3</v>
@@ -2794,66 +2800,66 @@
         <v>9</v>
       </c>
       <c r="AO11" s="10" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="AP11" s="9">
         <v>86</v>
       </c>
       <c r="AQ11" s="10" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="AR11" s="9">
         <v>15</v>
       </c>
       <c r="AS11" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="AT11" s="9">
+        <v>40</v>
+      </c>
+      <c r="AU11" s="10" t="s">
         <v>193</v>
       </c>
-      <c r="AT11" s="9">
-        <v>36</v>
-      </c>
-      <c r="AU11" s="10" t="s">
+      <c r="AV11" s="9">
+        <v>429</v>
+      </c>
+      <c r="AW11" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="AV11" s="9">
-        <v>428</v>
-      </c>
-      <c r="AW11" s="10" t="s">
+      <c r="AX11" s="9">
+        <v>1560</v>
+      </c>
+      <c r="AY11" s="10" t="s">
         <v>195</v>
-      </c>
-      <c r="AX11" s="9">
-        <v>1539</v>
-      </c>
-      <c r="AY11" s="10" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="C12" s="9">
+        <v>5221</v>
+      </c>
+      <c r="D12" s="9">
+        <v>0</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F12" s="9">
+        <v>987</v>
+      </c>
+      <c r="G12" s="10" t="s">
         <v>198</v>
-      </c>
-      <c r="C12" s="9">
-        <v>5213</v>
-      </c>
-      <c r="D12" s="9">
-        <v>0</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="F12" s="9">
-        <v>985</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>199</v>
       </c>
       <c r="H12" s="9">
         <v>38</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>175</v>
+        <v>199</v>
       </c>
       <c r="J12" s="9">
         <v>51</v>
@@ -2862,7 +2868,7 @@
         <v>200</v>
       </c>
       <c r="L12" s="9">
-        <v>1961</v>
+        <v>1968</v>
       </c>
       <c r="M12" s="10" t="s">
         <v>201</v>
@@ -2877,7 +2883,7 @@
         <v>0</v>
       </c>
       <c r="Q12" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="R12" s="9">
         <v>409</v>
@@ -2889,13 +2895,13 @@
         <v>0</v>
       </c>
       <c r="U12" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V12" s="9">
         <v>0</v>
       </c>
       <c r="W12" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X12" s="9">
         <v>26</v>
@@ -2910,28 +2916,28 @@
         <v>138</v>
       </c>
       <c r="AB12" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC12" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AD12" s="9">
         <v>10</v>
       </c>
       <c r="AE12" s="10" t="s">
-        <v>135</v>
+        <v>112</v>
       </c>
       <c r="AF12" s="9">
         <v>0</v>
       </c>
       <c r="AG12" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH12" s="9">
         <v>0</v>
       </c>
       <c r="AI12" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ12" s="9">
         <v>31</v>
@@ -2943,13 +2949,13 @@
         <v>0</v>
       </c>
       <c r="AM12" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AN12" s="9">
         <v>0</v>
       </c>
       <c r="AO12" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AP12" s="9">
         <v>60</v>
@@ -2964,60 +2970,60 @@
         <v>115</v>
       </c>
       <c r="AT12" s="9">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="AU12" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="AV12" s="9">
+        <v>356</v>
+      </c>
+      <c r="AW12" s="10" t="s">
         <v>206</v>
       </c>
-      <c r="AV12" s="9">
-        <v>355</v>
-      </c>
-      <c r="AW12" s="10" t="s">
+      <c r="AX12" s="9">
+        <v>547</v>
+      </c>
+      <c r="AY12" s="10" t="s">
         <v>207</v>
-      </c>
-      <c r="AX12" s="9">
-        <v>541</v>
-      </c>
-      <c r="AY12" s="10" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="C13" s="9">
+        <v>4933</v>
+      </c>
+      <c r="D13" s="9">
+        <v>1</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="F13" s="9">
+        <v>870</v>
+      </c>
+      <c r="G13" s="10" t="s">
         <v>210</v>
-      </c>
-      <c r="C13" s="9">
-        <v>4868</v>
-      </c>
-      <c r="D13" s="9">
-        <v>3</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>136</v>
-      </c>
-      <c r="F13" s="9">
-        <v>859</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>211</v>
       </c>
       <c r="H13" s="9">
         <v>31</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>192</v>
+        <v>211</v>
       </c>
       <c r="J13" s="9">
-        <v>39</v>
+        <v>61</v>
       </c>
       <c r="K13" s="10" t="s">
         <v>212</v>
       </c>
       <c r="L13" s="9">
-        <v>2106</v>
+        <v>2127</v>
       </c>
       <c r="M13" s="10" t="s">
         <v>213</v>
@@ -3029,13 +3035,13 @@
         <v>214</v>
       </c>
       <c r="P13" s="9">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q13" s="10" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="R13" s="9">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="S13" s="10" t="s">
         <v>215</v>
@@ -3044,19 +3050,19 @@
         <v>0</v>
       </c>
       <c r="U13" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V13" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W13" s="10" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="X13" s="9">
         <v>4</v>
       </c>
       <c r="Y13" s="10" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="Z13" s="9">
         <v>1</v>
@@ -3068,7 +3074,7 @@
         <v>0</v>
       </c>
       <c r="AC13" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD13" s="9">
         <v>8</v>
@@ -3080,7 +3086,7 @@
         <v>0</v>
       </c>
       <c r="AG13" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH13" s="9">
         <v>2</v>
@@ -3098,19 +3104,19 @@
         <v>11</v>
       </c>
       <c r="AM13" s="10" t="s">
-        <v>217</v>
+        <v>189</v>
       </c>
       <c r="AN13" s="9">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AO13" s="10" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="AP13" s="9">
         <v>37</v>
       </c>
       <c r="AQ13" s="10" t="s">
-        <v>171</v>
+        <v>217</v>
       </c>
       <c r="AR13" s="9">
         <v>23</v>
@@ -3119,69 +3125,69 @@
         <v>153</v>
       </c>
       <c r="AT13" s="9">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="AU13" s="10" t="s">
-        <v>114</v>
+        <v>189</v>
       </c>
       <c r="AV13" s="9">
         <v>220</v>
       </c>
       <c r="AW13" s="10" t="s">
-        <v>133</v>
+        <v>218</v>
       </c>
       <c r="AX13" s="9">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="AY13" s="10" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C14" s="9">
-        <v>4891</v>
+        <v>4926</v>
       </c>
       <c r="D14" s="9">
         <v>0</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F14" s="9">
-        <v>1116</v>
+        <v>1122</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="H14" s="9">
         <v>18</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="J14" s="9">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>164</v>
+        <v>224</v>
       </c>
       <c r="L14" s="9">
-        <v>1387</v>
+        <v>1403</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="N14" s="9">
-        <v>885</v>
+        <v>899</v>
       </c>
       <c r="O14" s="10" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="P14" s="9">
         <v>1</v>
@@ -3190,10 +3196,10 @@
         <v>115</v>
       </c>
       <c r="R14" s="9">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="S14" s="10" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="T14" s="9">
         <v>3</v>
@@ -3205,7 +3211,7 @@
         <v>0</v>
       </c>
       <c r="W14" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X14" s="9">
         <v>9</v>
@@ -3223,31 +3229,31 @@
         <v>0</v>
       </c>
       <c r="AC14" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD14" s="9">
         <v>5</v>
       </c>
       <c r="AE14" s="10" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="AF14" s="9">
         <v>0</v>
       </c>
       <c r="AG14" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH14" s="9">
         <v>0</v>
       </c>
       <c r="AI14" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ14" s="9">
         <v>16</v>
       </c>
       <c r="AK14" s="10" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="AL14" s="9">
         <v>1</v>
@@ -3265,7 +3271,7 @@
         <v>34</v>
       </c>
       <c r="AQ14" s="10" t="s">
-        <v>164</v>
+        <v>229</v>
       </c>
       <c r="AR14" s="9">
         <v>1</v>
@@ -3274,111 +3280,111 @@
         <v>115</v>
       </c>
       <c r="AT14" s="9">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="AU14" s="10" t="s">
-        <v>227</v>
+        <v>153</v>
       </c>
       <c r="AV14" s="9">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="AW14" s="10" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="AX14" s="9">
-        <v>691</v>
+        <v>696</v>
       </c>
       <c r="AY14" s="10" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C15" s="9">
-        <v>12580</v>
+        <v>12596</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F15" s="9">
-        <v>3873</v>
+        <v>3878</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="H15" s="9">
         <v>55</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="J15" s="9">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>138</v>
+        <v>179</v>
       </c>
       <c r="L15" s="9">
-        <v>3858</v>
+        <v>3863</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="N15" s="9">
         <v>226</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="P15" s="9">
         <v>1</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="R15" s="9">
         <v>733</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="T15" s="9">
         <v>41</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="V15" s="9">
         <v>0</v>
       </c>
       <c r="W15" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X15" s="9">
         <v>15</v>
       </c>
       <c r="Y15" s="10" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="Z15" s="9">
         <v>0</v>
       </c>
       <c r="AA15" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AB15" s="9">
         <v>0</v>
       </c>
       <c r="AC15" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD15" s="9">
         <v>3</v>
@@ -3390,19 +3396,19 @@
         <v>0</v>
       </c>
       <c r="AG15" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH15" s="9">
         <v>1</v>
       </c>
       <c r="AI15" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="AJ15" s="9">
         <v>11</v>
       </c>
       <c r="AK15" s="10" t="s">
-        <v>238</v>
+        <v>114</v>
       </c>
       <c r="AL15" s="9">
         <v>3</v>
@@ -3414,13 +3420,13 @@
         <v>1</v>
       </c>
       <c r="AO15" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="AP15" s="9">
         <v>79</v>
       </c>
       <c r="AQ15" s="10" t="s">
-        <v>239</v>
+        <v>211</v>
       </c>
       <c r="AR15" s="9">
         <v>19</v>
@@ -3429,33 +3435,33 @@
         <v>152</v>
       </c>
       <c r="AT15" s="9">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AU15" s="10" t="s">
-        <v>115</v>
+        <v>179</v>
       </c>
       <c r="AV15" s="9">
-        <v>1053</v>
+        <v>1055</v>
       </c>
       <c r="AW15" s="10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AX15" s="9">
         <v>2600</v>
       </c>
       <c r="AY15" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C16" s="9">
-        <v>5068</v>
+        <v>5080</v>
       </c>
       <c r="D16" s="9">
         <v>2</v>
@@ -3464,16 +3470,16 @@
         <v>138</v>
       </c>
       <c r="F16" s="9">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="H16" s="9">
         <v>32</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>239</v>
+        <v>211</v>
       </c>
       <c r="J16" s="9">
         <v>8</v>
@@ -3482,16 +3488,16 @@
         <v>116</v>
       </c>
       <c r="L16" s="9">
-        <v>1601</v>
+        <v>1611</v>
       </c>
       <c r="M16" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="N16" s="9">
         <v>271</v>
       </c>
       <c r="O16" s="10" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="P16" s="9">
         <v>1</v>
@@ -3503,25 +3509,25 @@
         <v>266</v>
       </c>
       <c r="S16" s="10" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="T16" s="9">
         <v>0</v>
       </c>
       <c r="U16" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V16" s="9">
         <v>0</v>
       </c>
       <c r="W16" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X16" s="9">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y16" s="10" t="s">
-        <v>121</v>
+        <v>240</v>
       </c>
       <c r="Z16" s="9">
         <v>3</v>
@@ -3545,138 +3551,138 @@
         <v>0</v>
       </c>
       <c r="AG16" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH16" s="9">
         <v>0</v>
       </c>
       <c r="AI16" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ16" s="9">
         <v>29</v>
       </c>
       <c r="AK16" s="10" t="s">
-        <v>120</v>
+        <v>249</v>
       </c>
       <c r="AL16" s="9">
         <v>4</v>
       </c>
       <c r="AM16" s="10" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="AN16" s="9">
         <v>0</v>
       </c>
       <c r="AO16" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AP16" s="9">
         <v>43</v>
       </c>
       <c r="AQ16" s="10" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="AR16" s="9">
         <v>7</v>
       </c>
       <c r="AS16" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="AT16" s="9">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="AU16" s="10" t="s">
-        <v>175</v>
+        <v>216</v>
       </c>
       <c r="AV16" s="9">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="AW16" s="10" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="AX16" s="9">
-        <v>1436</v>
+        <v>1439</v>
       </c>
       <c r="AY16" s="10" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C17" s="9">
-        <v>9692</v>
+        <v>9963</v>
       </c>
       <c r="D17" s="9">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>194</v>
+        <v>228</v>
       </c>
       <c r="F17" s="9">
-        <v>2869</v>
+        <v>2943</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="H17" s="9">
-        <v>265</v>
+        <v>234</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="J17" s="9">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="K17" s="10" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="L17" s="9">
-        <v>3743</v>
+        <v>3908</v>
       </c>
       <c r="M17" s="10" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="N17" s="9">
-        <v>642</v>
+        <v>672</v>
       </c>
       <c r="O17" s="10" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="P17" s="9">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="Q17" s="10" t="s">
-        <v>118</v>
+        <v>260</v>
       </c>
       <c r="R17" s="9">
-        <v>428</v>
+        <v>435</v>
       </c>
       <c r="S17" s="10" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="T17" s="9">
         <v>1</v>
       </c>
       <c r="U17" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="V17" s="9">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="W17" s="10" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="X17" s="9">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="Y17" s="10" t="s">
-        <v>177</v>
+        <v>106</v>
       </c>
       <c r="Z17" s="9">
         <v>4</v>
@@ -3700,7 +3706,7 @@
         <v>0</v>
       </c>
       <c r="AG17" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH17" s="9">
         <v>2</v>
@@ -3712,168 +3718,168 @@
         <v>16</v>
       </c>
       <c r="AK17" s="10" t="s">
-        <v>259</v>
+        <v>116</v>
       </c>
       <c r="AL17" s="9">
         <v>3</v>
       </c>
       <c r="AM17" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AN17" s="9">
         <v>7</v>
       </c>
       <c r="AO17" s="10" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="AP17" s="9">
         <v>44</v>
       </c>
       <c r="AQ17" s="10" t="s">
-        <v>260</v>
+        <v>235</v>
       </c>
       <c r="AR17" s="9">
         <v>9</v>
       </c>
       <c r="AS17" s="10" t="s">
-        <v>238</v>
+        <v>114</v>
       </c>
       <c r="AT17" s="9">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="AU17" s="10" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AV17" s="9">
-        <v>737</v>
+        <v>752</v>
       </c>
       <c r="AW17" s="10" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="AX17" s="9">
-        <v>465</v>
+        <v>477</v>
       </c>
       <c r="AY17" s="10" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C18" s="9">
-        <v>10129</v>
+        <v>10258</v>
       </c>
       <c r="D18" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>134</v>
+        <v>115</v>
       </c>
       <c r="F18" s="9">
-        <v>1835</v>
+        <v>1908</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H18" s="9">
         <v>151</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="J18" s="9">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="K18" s="10" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="L18" s="9">
-        <v>3385</v>
+        <v>3441</v>
       </c>
       <c r="M18" s="10" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="N18" s="9">
-        <v>1588</v>
+        <v>1592</v>
       </c>
       <c r="O18" s="10" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="P18" s="9">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q18" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="R18" s="9">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="S18" s="10" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="T18" s="9">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="U18" s="10" t="s">
-        <v>118</v>
+        <v>273</v>
       </c>
       <c r="V18" s="9">
         <v>0</v>
       </c>
       <c r="W18" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X18" s="9">
         <v>5</v>
       </c>
       <c r="Y18" s="10" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="Z18" s="9">
         <v>1</v>
       </c>
       <c r="AA18" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="AB18" s="9">
         <v>1</v>
       </c>
       <c r="AC18" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="AD18" s="9">
         <v>3</v>
       </c>
       <c r="AE18" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AF18" s="9">
         <v>0</v>
       </c>
       <c r="AG18" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH18" s="9">
         <v>0</v>
       </c>
       <c r="AI18" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ18" s="9">
         <v>11</v>
       </c>
       <c r="AK18" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="AL18" s="9">
         <v>10</v>
       </c>
       <c r="AM18" s="10" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="AN18" s="9">
         <v>2</v>
@@ -3885,138 +3891,138 @@
         <v>38</v>
       </c>
       <c r="AQ18" s="10" t="s">
-        <v>163</v>
+        <v>223</v>
       </c>
       <c r="AR18" s="9">
         <v>17</v>
       </c>
       <c r="AS18" s="10" t="s">
-        <v>259</v>
+        <v>274</v>
       </c>
       <c r="AT18" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU18" s="10" t="s">
-        <v>134</v>
+        <v>115</v>
       </c>
       <c r="AV18" s="9">
-        <v>410</v>
+        <v>417</v>
       </c>
       <c r="AW18" s="10" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="AX18" s="9">
         <v>1837</v>
       </c>
       <c r="AY18" s="10" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C19" s="9">
-        <v>10667</v>
+        <v>10866</v>
       </c>
       <c r="D19" s="9">
         <v>0</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F19" s="9">
-        <v>1196</v>
+        <v>1228</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="H19" s="9">
         <v>15</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="J19" s="9">
         <v>1</v>
       </c>
       <c r="K19" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="L19" s="9">
-        <v>5085</v>
+        <v>5225</v>
       </c>
       <c r="M19" s="10" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="N19" s="9">
-        <v>1587</v>
+        <v>1583</v>
       </c>
       <c r="O19" s="10" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="P19" s="9">
         <v>0</v>
       </c>
       <c r="Q19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="R19" s="9">
-        <v>1165</v>
+        <v>1178</v>
       </c>
       <c r="S19" s="10" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="T19" s="9">
         <v>0</v>
       </c>
       <c r="U19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V19" s="9">
         <v>0</v>
       </c>
       <c r="W19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X19" s="9">
         <v>18</v>
       </c>
       <c r="Y19" s="10" t="s">
-        <v>259</v>
+        <v>274</v>
       </c>
       <c r="Z19" s="9">
         <v>0</v>
       </c>
       <c r="AA19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AB19" s="9">
         <v>0</v>
       </c>
       <c r="AC19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD19" s="9">
         <v>3</v>
       </c>
       <c r="AE19" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AF19" s="9">
         <v>0</v>
       </c>
       <c r="AG19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH19" s="9">
         <v>0</v>
       </c>
       <c r="AI19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ19" s="9">
         <v>16</v>
@@ -4028,329 +4034,329 @@
         <v>0</v>
       </c>
       <c r="AM19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AN19" s="9">
         <v>0</v>
       </c>
       <c r="AO19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AP19" s="9">
         <v>61</v>
       </c>
       <c r="AQ19" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AR19" s="9">
         <v>1</v>
       </c>
       <c r="AS19" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="AT19" s="9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AU19" s="10" t="s">
-        <v>115</v>
+        <v>138</v>
       </c>
       <c r="AV19" s="9">
-        <v>671</v>
+        <v>687</v>
       </c>
       <c r="AW19" s="10" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="AX19" s="9">
         <v>846</v>
       </c>
       <c r="AY19" s="10" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="C20" s="9">
-        <v>1053</v>
+        <v>1061</v>
       </c>
       <c r="D20" s="9">
         <v>1</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>238</v>
+        <v>114</v>
       </c>
       <c r="F20" s="9">
         <v>162</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="H20" s="9">
         <v>6</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>120</v>
+        <v>249</v>
       </c>
       <c r="J20" s="9">
         <v>35</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="L20" s="9">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="M20" s="10" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="N20" s="9">
         <v>48</v>
       </c>
       <c r="O20" s="10" t="s">
-        <v>287</v>
+        <v>134</v>
       </c>
       <c r="P20" s="9">
         <v>6</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>120</v>
+        <v>249</v>
       </c>
       <c r="R20" s="9">
         <v>168</v>
       </c>
       <c r="S20" s="10" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="T20" s="9">
         <v>0</v>
       </c>
       <c r="U20" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V20" s="9">
         <v>0</v>
       </c>
       <c r="W20" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X20" s="9">
         <v>9</v>
       </c>
       <c r="Y20" s="10" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="Z20" s="9">
         <v>3</v>
       </c>
       <c r="AA20" s="10" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="AB20" s="9">
         <v>0</v>
       </c>
       <c r="AC20" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD20" s="9">
         <v>0</v>
       </c>
       <c r="AE20" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AF20" s="9">
         <v>0</v>
       </c>
       <c r="AG20" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH20" s="9">
         <v>1</v>
       </c>
       <c r="AI20" s="10" t="s">
-        <v>238</v>
+        <v>114</v>
       </c>
       <c r="AJ20" s="9">
         <v>6</v>
       </c>
       <c r="AK20" s="10" t="s">
-        <v>120</v>
+        <v>249</v>
       </c>
       <c r="AL20" s="9">
         <v>2</v>
       </c>
       <c r="AM20" s="10" t="s">
-        <v>135</v>
+        <v>112</v>
       </c>
       <c r="AN20" s="9">
         <v>1</v>
       </c>
       <c r="AO20" s="10" t="s">
-        <v>238</v>
+        <v>114</v>
       </c>
       <c r="AP20" s="9">
         <v>18</v>
       </c>
       <c r="AQ20" s="10" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="AR20" s="9">
         <v>4</v>
       </c>
       <c r="AS20" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="AT20" s="9">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="AU20" s="10" t="s">
-        <v>291</v>
+        <v>237</v>
       </c>
       <c r="AV20" s="9">
         <v>47</v>
       </c>
       <c r="AW20" s="10" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="AX20" s="9">
         <v>185</v>
       </c>
       <c r="AY20" s="10" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C21" s="9">
-        <v>2566</v>
+        <v>2568</v>
       </c>
       <c r="D21" s="9">
         <v>0</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F21" s="9">
         <v>420</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="H21" s="9">
         <v>150</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="J21" s="9">
         <v>2</v>
       </c>
       <c r="K21" s="10" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="L21" s="9">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="N21" s="9">
         <v>102</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="P21" s="9">
         <v>8</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="R21" s="9">
         <v>79</v>
       </c>
       <c r="S21" s="10" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="T21" s="9">
         <v>0</v>
       </c>
       <c r="U21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V21" s="9">
         <v>0</v>
       </c>
       <c r="W21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X21" s="9">
         <v>17</v>
       </c>
       <c r="Y21" s="10" t="s">
-        <v>216</v>
+        <v>303</v>
       </c>
       <c r="Z21" s="9">
         <v>2</v>
       </c>
       <c r="AA21" s="10" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="AB21" s="9">
         <v>0</v>
       </c>
       <c r="AC21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD21" s="9">
         <v>0</v>
       </c>
       <c r="AE21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AF21" s="9">
         <v>0</v>
       </c>
       <c r="AG21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH21" s="9">
         <v>0</v>
       </c>
       <c r="AI21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ21" s="9">
         <v>3</v>
       </c>
       <c r="AK21" s="10" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="AL21" s="9">
         <v>0</v>
       </c>
       <c r="AM21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AN21" s="9">
         <v>0</v>
       </c>
       <c r="AO21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AP21" s="9">
         <v>18</v>
       </c>
       <c r="AQ21" s="10" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="AR21" s="9">
         <v>1</v>
@@ -4359,96 +4365,96 @@
         <v>138</v>
       </c>
       <c r="AT21" s="9">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AU21" s="10" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="AV21" s="9">
         <v>97</v>
       </c>
       <c r="AW21" s="10" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="AX21" s="9">
         <v>863</v>
       </c>
       <c r="AY21" s="10" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="C22" s="12">
-        <v>120818</v>
+        <v>122688</v>
       </c>
       <c r="D22" s="12">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>106</v>
       </c>
       <c r="F22" s="12">
-        <v>24509</v>
+        <v>25110</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>107</v>
       </c>
       <c r="H22" s="12">
-        <v>1506</v>
+        <v>1473</v>
       </c>
       <c r="I22" s="13" t="s">
         <v>108</v>
       </c>
       <c r="J22" s="12">
-        <v>2285</v>
+        <v>2256</v>
       </c>
       <c r="K22" s="13" t="s">
         <v>109</v>
       </c>
       <c r="L22" s="12">
-        <v>46153</v>
+        <v>47186</v>
       </c>
       <c r="M22" s="13" t="s">
         <v>110</v>
       </c>
       <c r="N22" s="12">
-        <v>12318</v>
+        <v>12401</v>
       </c>
       <c r="O22" s="13" t="s">
         <v>111</v>
       </c>
       <c r="P22" s="12">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="Q22" s="13" t="s">
         <v>112</v>
       </c>
       <c r="R22" s="12">
-        <v>9292</v>
+        <v>9373</v>
       </c>
       <c r="S22" s="13" t="s">
         <v>113</v>
       </c>
       <c r="T22" s="12">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="U22" s="13" t="s">
         <v>114</v>
       </c>
       <c r="V22" s="12">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="W22" s="13" t="s">
         <v>115</v>
       </c>
       <c r="X22" s="12">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="Y22" s="13" t="s">
         <v>116</v>
@@ -4460,7 +4466,7 @@
         <v>115</v>
       </c>
       <c r="AB22" s="12">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="AC22" s="13" t="s">
         <v>115</v>
@@ -4469,13 +4475,13 @@
         <v>89</v>
       </c>
       <c r="AE22" s="13" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="AF22" s="12">
         <v>0</v>
       </c>
       <c r="AG22" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH22" s="12">
         <v>20</v>
@@ -4484,49 +4490,49 @@
         <v>115</v>
       </c>
       <c r="AJ22" s="12">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="AK22" s="13" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AL22" s="12">
         <v>39</v>
       </c>
       <c r="AM22" s="13" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AN22" s="12">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="AO22" s="13" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="AP22" s="12">
         <v>689</v>
       </c>
       <c r="AQ22" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AR22" s="12">
         <v>115</v>
       </c>
       <c r="AS22" s="13" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="AT22" s="12">
-        <v>1042</v>
+        <v>1049</v>
       </c>
       <c r="AU22" s="13" t="s">
         <v>122</v>
       </c>
       <c r="AV22" s="12">
-        <v>6047</v>
+        <v>6099</v>
       </c>
       <c r="AW22" s="13" t="s">
         <v>123</v>
       </c>
       <c r="AX22" s="12">
-        <v>15646</v>
+        <v>15703</v>
       </c>
       <c r="AY22" s="13" t="s">
         <v>124</v>

</xml_diff>